<commit_message>
Fix detail-page extraction for furnishing/outdoor; commit config
Cross-checking against live listings showed furnishing read as "unknown"
(e.g. OTM 19852978 is clearly furnished) and Rightmove outdoor space missed
or false-positived on glossary text. Fixes:

- OnTheMarket enrich: read the real property node — furnishing from
  lettingDetails.items, description + features[].feature, size from
  minimumAreaSqFt (was grabbing a generic agent blurb)
- Rightmove: add detail-page enrich reading keyFeatures + the
  "Furnish type:" label; scoped to keyFeatures to avoid the standing
  glossary ("GARDEN: a property has access to…") false-positives
- Commit config.md (un-ignored; not sensitive) so scheduled runs have it

Verified: furnishing/outdoor/size now match the live listings on sampled
rows across platforms.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X41km7yJ316R9txmxhg6Ko
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -587,7 +587,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Part Furnished</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -633,7 +633,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>https://www.rightmove.co.uk/properties/90432648</t>
+          <t>https://www.rightmove.co.uk/properties/90435384</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -647,7 +647,7 @@
         </is>
       </c>
       <c r="F3" s="4" t="n">
-        <v>3000</v>
+        <v>4250</v>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
@@ -656,7 +656,7 @@
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Part Furnished</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
@@ -670,7 +670,7 @@
       <c r="K3" s="4" t="inlineStr"/>
       <c r="L3" s="4" t="inlineStr">
         <is>
-          <t>ZERO DEPOSIT AVAILABLE. LONG LET. Set on the 21st floor, this 1 bedroom flat boasts well arranged interiors including a large reception room, a modern open-plan; verify balcony/terrace; under 650 sq ft</t>
+          <t>ZERO DEPOSIT AVAILABLE. SHORT LET. Set on the 21st floor, this 1 bedroom flat boasts well arranged interiors including a large reception room, a modern open-pla; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M3" s="4" t="inlineStr">
@@ -702,7 +702,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>https://www.rightmove.co.uk/properties/90435384</t>
+          <t>https://www.rightmove.co.uk/properties/90432648</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="F4" s="4" t="n">
-        <v>4250</v>
+        <v>3000</v>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
@@ -725,7 +725,7 @@
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Part Furnished</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
@@ -739,7 +739,7 @@
       <c r="K4" s="4" t="inlineStr"/>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>ZERO DEPOSIT AVAILABLE. SHORT LET. Set on the 21st floor, this 1 bedroom flat boasts well arranged interiors including a large reception room, a modern open-pla; verify balcony/terrace; under 650 sq ft</t>
+          <t>ZERO DEPOSIT AVAILABLE. LONG LET. Set on the 21st floor, this 1 bedroom flat boasts well arranged interiors including a large reception room, a modern open-plan; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M4" s="4" t="inlineStr">
@@ -802,11 +802,13 @@
           <t>Not stated</t>
         </is>
       </c>
-      <c r="J5" s="4" t="n"/>
+      <c r="J5" s="4" t="n">
+        <v>553</v>
+      </c>
       <c r="K5" s="4" t="inlineStr"/>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>One bedroom apartment Newly refurbished; verify balcony/terrace; size not stated</t>
+          <t>One bedroom apartment Newly refurbished; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M5" s="4" t="inlineStr">
@@ -866,7 +868,7 @@
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J6" s="4" t="n">
@@ -875,7 +877,7 @@
       <c r="K6" s="4" t="inlineStr"/>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>608 sq ft floor area Nearest station 0.1mi.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>608 sq ft floor area Nearest station 0.1mi.; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M6" s="4" t="inlineStr">
@@ -895,67 +897,69 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>2 bedroom flat to rent</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>https://www.onthemarket.com/details/19852978/</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Newport Court, Covent Garden, London, WC2H</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>WC2H</t>
         </is>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="F7" s="4" t="n">
         <v>4334</v>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>2-Bed</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>Private balcony/terrace</t>
         </is>
       </c>
-      <c r="J7" s="2" t="n"/>
-      <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>Splendid two bedroom flat Ample interiors; size not stated</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="O7" s="2" t="inlineStr">
+      <c r="J7" s="4" t="n">
+        <v>858</v>
+      </c>
+      <c r="K7" s="4" t="inlineStr"/>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>Splendid two bedroom flat Ample interiors; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O7" s="4" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
@@ -1066,7 +1070,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Furnished</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -1080,7 +1084,7 @@
       <c r="K9" s="4" t="inlineStr"/>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>Council tax band: F 521 sq ft floor area; verify balcony/terrace; under 650 sq ft</t>
+          <t>Council tax band: F 521 sq ft floor area; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M9" s="4" t="inlineStr">
@@ -1140,7 +1144,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J10" s="4" t="n">
@@ -1149,7 +1153,7 @@
       <c r="K10" s="4" t="inlineStr"/>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>432 sq ft floor area Nearest station 0.1mi. Furnished Nearest school 0.2mi.; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>432 sq ft floor area Nearest station 0.1mi. Furnished Nearest school 0.2mi.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M10" s="4" t="inlineStr">
@@ -1204,7 +1208,7 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Furnished</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
@@ -1212,11 +1216,13 @@
           <t>Not stated</t>
         </is>
       </c>
-      <c r="J11" s="4" t="n"/>
+      <c r="J11" s="4" t="n">
+        <v>656</v>
+      </c>
       <c r="K11" s="4" t="inlineStr"/>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>Concierge service Highly sought-after Zone 1 location; verify balcony/terrace; size not stated</t>
+          <t>Concierge service Highly sought-after Zone 1 location; verify balcony/terrace; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M11" s="4" t="inlineStr">
@@ -1348,11 +1354,13 @@
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J13" s="6" t="n"/>
+      <c r="J13" s="6" t="n">
+        <v>603</v>
+      </c>
       <c r="K13" s="6" t="inlineStr"/>
       <c r="L13" s="6" t="inlineStr">
         <is>
-          <t>Beautifully Refurbished Secondary Glazing; outdoor space is communal/shared; size not stated</t>
+          <t>Beautifully Refurbished Secondary Glazing; outdoor space is communal/shared; under 650 sq ft</t>
         </is>
       </c>
       <c r="M13" s="6" t="inlineStr">
@@ -1407,7 +1415,7 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
@@ -1415,11 +1423,13 @@
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J14" s="6" t="n"/>
+      <c r="J14" s="6" t="n">
+        <v>671</v>
+      </c>
       <c r="K14" s="6" t="inlineStr"/>
       <c r="L14" s="6" t="inlineStr">
         <is>
-          <t>Pet friendly Wooden Floors Student; outdoor space is communal/shared; size not stated</t>
+          <t>Pet friendly Wooden Floors Student; outdoor space is communal/shared</t>
         </is>
       </c>
       <c r="M14" s="6" t="inlineStr">
@@ -1549,11 +1559,13 @@
           <t>Not stated</t>
         </is>
       </c>
-      <c r="J16" s="4" t="n"/>
+      <c r="J16" s="4" t="n">
+        <v>549</v>
+      </c>
       <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr">
         <is>
-          <t>One bedroom One shower room, ensuite; verify balcony/terrace; size not stated</t>
+          <t>One bedroom One shower room, ensuite; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M16" s="4" t="inlineStr">
@@ -1573,67 +1585,69 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>1 bedroom apartment to rent</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>https://www.onthemarket.com/details/13524814/</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>Carnaby Street, Soho, W1F</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>W1F</t>
         </is>
       </c>
-      <c r="F17" s="6" t="n">
+      <c r="F17" s="4" t="n">
         <v>3640</v>
       </c>
-      <c r="G17" s="6" t="inlineStr">
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>1-Bed</t>
         </is>
       </c>
-      <c r="H17" s="6" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>Flexible</t>
         </is>
       </c>
-      <c r="I17" s="6" t="inlineStr">
-        <is>
-          <t>Communal / shared</t>
-        </is>
-      </c>
-      <c r="J17" s="6" t="n"/>
-      <c r="K17" s="6" t="inlineStr"/>
-      <c r="L17" s="6" t="inlineStr">
-        <is>
-          <t>Recently Refurbished Apartment Original Features Student; outdoor space is communal/shared; size not stated</t>
-        </is>
-      </c>
-      <c r="M17" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N17" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O17" s="6" t="inlineStr">
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="n">
+        <v>552</v>
+      </c>
+      <c r="K17" s="4" t="inlineStr"/>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Recently Refurbished Apartment Original Features Student; verify balcony/terrace; under 650 sq ft</t>
+        </is>
+      </c>
+      <c r="M17" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N17" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O17" s="4" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
@@ -1683,11 +1697,13 @@
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J18" s="6" t="n"/>
+      <c r="J18" s="6" t="n">
+        <v>802</v>
+      </c>
       <c r="K18" s="6" t="inlineStr"/>
       <c r="L18" s="6" t="inlineStr">
         <is>
-          <t>Built in Storage Pet Friendly; outdoor space is communal/shared; size not stated</t>
+          <t>Built in Storage Pet Friendly; outdoor space is communal/shared</t>
         </is>
       </c>
       <c r="M18" s="6" t="inlineStr">
@@ -1817,11 +1833,13 @@
           <t>Not stated</t>
         </is>
       </c>
-      <c r="J20" s="4" t="n"/>
+      <c r="J20" s="4" t="n">
+        <v>581</v>
+      </c>
       <c r="K20" s="4" t="inlineStr"/>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t>One bedroom One bathroom; verify balcony/terrace; size not stated</t>
+          <t>One bedroom One bathroom; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M20" s="4" t="inlineStr">
@@ -1884,11 +1902,13 @@
           <t>Not stated</t>
         </is>
       </c>
-      <c r="J21" s="4" t="n"/>
+      <c r="J21" s="4" t="n">
+        <v>580</v>
+      </c>
       <c r="K21" s="4" t="inlineStr"/>
       <c r="L21" s="4" t="inlineStr">
         <is>
-          <t>One Double bedroom Quaint Road; verify balcony/terrace; size not stated</t>
+          <t>One Double bedroom Quaint Road; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M21" s="4" t="inlineStr">
@@ -1908,67 +1928,69 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>1 bedroom apartment to rent</t>
         </is>
       </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>https://www.onthemarket.com/details/18680649/</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>Duck Lane, Soho W1F</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>W1F</t>
         </is>
       </c>
-      <c r="F22" s="6" t="n">
+      <c r="F22" s="4" t="n">
         <v>3077</v>
       </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>1-Bed</t>
         </is>
       </c>
-      <c r="H22" s="6" t="inlineStr">
+      <c r="H22" s="4" t="inlineStr">
         <is>
           <t>Flexible</t>
         </is>
       </c>
-      <c r="I22" s="6" t="inlineStr">
-        <is>
-          <t>Communal / shared</t>
-        </is>
-      </c>
-      <c r="J22" s="6" t="n"/>
-      <c r="K22" s="6" t="inlineStr"/>
-      <c r="L22" s="6" t="inlineStr">
-        <is>
-          <t>Modern Throughout Wooden Flooring Throughout; outdoor space is communal/shared; size not stated</t>
-        </is>
-      </c>
-      <c r="M22" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N22" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O22" s="6" t="inlineStr">
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>575</v>
+      </c>
+      <c r="K22" s="4" t="inlineStr"/>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>Modern Throughout Wooden Flooring Throughout; verify balcony/terrace; under 650 sq ft</t>
+        </is>
+      </c>
+      <c r="M22" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N22" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O22" s="4" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
@@ -2018,11 +2040,13 @@
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J23" s="6" t="n"/>
+      <c r="J23" s="6" t="n">
+        <v>603</v>
+      </c>
       <c r="K23" s="6" t="inlineStr"/>
       <c r="L23" s="6" t="inlineStr">
         <is>
-          <t>One bedroom One shower room; outdoor space is communal/shared; size not stated</t>
+          <t>One bedroom One shower room; outdoor space is communal/shared; under 650 sq ft</t>
         </is>
       </c>
       <c r="M23" s="6" t="inlineStr">
@@ -2042,136 +2066,138 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>1 bedroom apartment to rent</t>
         </is>
       </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>https://www.onthemarket.com/details/15707269/</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>Casson Square, London, Waterloo, United Kingdom, SE1</t>
         </is>
       </c>
-      <c r="E24" s="6" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
         <is>
           <t>SE1</t>
         </is>
       </c>
-      <c r="F24" s="6" t="n">
+      <c r="F24" s="4" t="n">
         <v>4050</v>
       </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="G24" s="4" t="inlineStr">
         <is>
           <t>1-Bed</t>
         </is>
       </c>
-      <c r="H24" s="6" t="inlineStr">
-        <is>
-          <t>Flexible</t>
-        </is>
-      </c>
-      <c r="I24" s="6" t="inlineStr">
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
         <is>
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J24" s="6" t="n">
+      <c r="J24" s="4" t="n">
         <v>514</v>
       </c>
-      <c r="K24" s="6" t="inlineStr"/>
-      <c r="L24" s="6" t="inlineStr">
-        <is>
-          <t>Bedroom Bathroom Open-plan reception/kitchen 24 hour concierge; outdoor space is communal/shared; under 650 sq ft</t>
-        </is>
-      </c>
-      <c r="M24" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N24" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O24" s="6" t="inlineStr">
+      <c r="K24" s="4" t="inlineStr"/>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Bedroom Bathroom Open-plan reception/kitchen 24 hour concierge; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M24" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N24" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O24" s="4" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>1 bedroom apartment to rent</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>https://www.onthemarket.com/details/9568931/</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>Casson Square, Waterloo, Southbank Place, London, SE1</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>SE1</t>
         </is>
       </c>
-      <c r="F25" s="2" t="n">
+      <c r="F25" s="4" t="n">
         <v>4250</v>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="G25" s="4" t="inlineStr">
         <is>
           <t>1-Bed</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>Flexible</t>
-        </is>
-      </c>
-      <c r="I25" s="2" t="inlineStr">
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
         <is>
           <t>Private balcony/terrace</t>
         </is>
       </c>
-      <c r="J25" s="2" t="n"/>
-      <c r="K25" s="2" t="inlineStr"/>
-      <c r="L25" s="2" t="inlineStr">
-        <is>
-          <t>1 bedroom 1 bathroom Open-plan reception kitchen 24-hour five-star concierge; size not stated</t>
-        </is>
-      </c>
-      <c r="M25" s="2" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N25" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="O25" s="2" t="inlineStr">
+      <c r="J25" s="4" t="n">
+        <v>644</v>
+      </c>
+      <c r="K25" s="4" t="inlineStr"/>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>1 bedroom 1 bathroom Open-plan reception kitchen 24-hour five-star concierge; under 650 sq ft; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M25" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N25" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O25" s="4" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
@@ -2213,7 +2239,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Part Furnished</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -2221,11 +2247,13 @@
           <t>Private balcony/terrace</t>
         </is>
       </c>
-      <c r="J26" s="2" t="n"/>
+      <c r="J26" s="2" t="n">
+        <v>1385</v>
+      </c>
       <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>Spectacular Views Waterloo; size not stated</t>
+          <t>Spectacular Views Waterloo</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
@@ -2245,63 +2273,65 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>2 bedroom end of terrace house to rent</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>https://www.onthemarket.com/details/19811489/</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>Carlisle Lane, Waterloo</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr"/>
-      <c r="F27" s="2" t="n">
+      <c r="E27" s="4" t="inlineStr"/>
+      <c r="F27" s="4" t="n">
         <v>3575</v>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="G27" s="4" t="inlineStr">
         <is>
           <t>2-Bed</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="I27" s="2" t="inlineStr">
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
         <is>
           <t>Private balcony/terrace</t>
         </is>
       </c>
-      <c r="J27" s="2" t="n"/>
-      <c r="K27" s="2" t="inlineStr"/>
-      <c r="L27" s="2" t="inlineStr">
-        <is>
-          <t>End of Terrace Shared Garden; size not stated</t>
-        </is>
-      </c>
-      <c r="M27" s="2" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N27" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="O27" s="2" t="inlineStr">
+      <c r="J27" s="4" t="n">
+        <v>904</v>
+      </c>
+      <c r="K27" s="4" t="inlineStr"/>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>End of Terrace Shared Garden; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M27" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N27" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O27" s="4" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
@@ -2351,11 +2381,13 @@
           <t>Private balcony/terrace</t>
         </is>
       </c>
-      <c r="J28" s="2" t="n"/>
+      <c r="J28" s="2" t="n">
+        <v>1140</v>
+      </c>
       <c r="K28" s="2" t="inlineStr"/>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>Two Bedrooms Two Bathrooms; size not stated</t>
+          <t>Two Bedrooms Two Bathrooms</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
@@ -2444,138 +2476,138 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="inlineStr">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>2 bedroom apartment to rent</t>
         </is>
       </c>
-      <c r="B30" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C30" s="7" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>https://www.onthemarket.com/details/7516361/</t>
         </is>
       </c>
-      <c r="D30" s="6" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>Belvedere Road, Waterloo, London, SE1</t>
         </is>
       </c>
-      <c r="E30" s="6" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
         <is>
           <t>SE1</t>
         </is>
       </c>
-      <c r="F30" s="6" t="n">
+      <c r="F30" s="4" t="n">
         <v>3350</v>
       </c>
-      <c r="G30" s="6" t="inlineStr">
+      <c r="G30" s="4" t="inlineStr">
         <is>
           <t>2-Bed</t>
         </is>
       </c>
-      <c r="H30" s="6" t="inlineStr">
-        <is>
-          <t>Flexible</t>
-        </is>
-      </c>
-      <c r="I30" s="6" t="inlineStr">
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="inlineStr">
         <is>
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J30" s="6" t="n">
+      <c r="J30" s="4" t="n">
         <v>544</v>
       </c>
-      <c r="K30" s="6" t="inlineStr"/>
-      <c r="L30" s="6" t="inlineStr">
-        <is>
-          <t>Residents' swimming pool and gym. Grade II listed period building. 24 hour porters. Set close to the iconic Southbank and London Eye.; outdoor space is communal/shared; under 650 sq ft</t>
-        </is>
-      </c>
-      <c r="M30" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N30" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O30" s="6" t="inlineStr">
+      <c r="K30" s="4" t="inlineStr"/>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>Residents' swimming pool and gym. Grade II listed period building. 24 hour porters. Set close to the iconic Southbank and London Eye.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M30" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N30" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O30" s="4" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="inlineStr">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>1 bedroom apartment to rent</t>
         </is>
       </c>
-      <c r="B31" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C31" s="7" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>https://www.onthemarket.com/details/7589011/</t>
         </is>
       </c>
-      <c r="D31" s="6" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>Belvedere Road, London, Waterloo, SE1</t>
         </is>
       </c>
-      <c r="E31" s="6" t="inlineStr">
+      <c r="E31" s="4" t="inlineStr">
         <is>
           <t>SE1</t>
         </is>
       </c>
-      <c r="F31" s="6" t="n">
+      <c r="F31" s="4" t="n">
         <v>4200</v>
       </c>
-      <c r="G31" s="6" t="inlineStr">
+      <c r="G31" s="4" t="inlineStr">
         <is>
           <t>1-Bed</t>
         </is>
       </c>
-      <c r="H31" s="6" t="inlineStr">
-        <is>
-          <t>Flexible</t>
-        </is>
-      </c>
-      <c r="I31" s="6" t="inlineStr">
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I31" s="4" t="inlineStr">
         <is>
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J31" s="6" t="n">
+      <c r="J31" s="4" t="n">
         <v>671</v>
       </c>
-      <c r="K31" s="6" t="inlineStr"/>
-      <c r="L31" s="6" t="inlineStr">
-        <is>
-          <t>24-hour five-star concierge 18,000 sq ft gym and spa facilities Set in one of London's most connected locations, opposite Westminster and the Houses of Parliame; outdoor space is communal/shared</t>
-        </is>
-      </c>
-      <c r="M31" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N31" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O31" s="6" t="inlineStr">
+      <c r="K31" s="4" t="inlineStr"/>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>24-hour five-star concierge 18,000 sq ft gym and spa facilities Set in one of London's most connected locations, opposite Westminster and the Houses of Parliame; outdoor space is communal/shared; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M31" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N31" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O31" s="4" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
@@ -2617,7 +2649,7 @@
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Furnished</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
@@ -2631,7 +2663,7 @@
       <c r="K32" s="4" t="inlineStr"/>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Two bedrooms Two bathrooms 841 sq. ft. Excellent transport links; verify balcony/terrace</t>
+          <t>Two bedrooms Two bathrooms 841 sq. ft. Excellent transport links; verify balcony/terrace; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
@@ -2651,67 +2683,69 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>1 bedroom flat to rent</t>
         </is>
       </c>
-      <c r="B33" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C33" s="7" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
         <is>
           <t>https://www.onthemarket.com/details/19863550/</t>
         </is>
       </c>
-      <c r="D33" s="6" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr">
         <is>
           <t>King Street, Covent Garden, London, WC2E</t>
         </is>
       </c>
-      <c r="E33" s="6" t="inlineStr">
+      <c r="E33" s="4" t="inlineStr">
         <is>
           <t>WC2E</t>
         </is>
       </c>
-      <c r="F33" s="6" t="n">
+      <c r="F33" s="4" t="n">
         <v>3358</v>
       </c>
-      <c r="G33" s="6" t="inlineStr">
+      <c r="G33" s="4" t="inlineStr">
         <is>
           <t>1-Bed</t>
         </is>
       </c>
-      <c r="H33" s="6" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="I33" s="6" t="inlineStr">
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr">
         <is>
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J33" s="6" t="n"/>
-      <c r="K33" s="6" t="inlineStr"/>
-      <c r="L33" s="6" t="inlineStr">
-        <is>
-          <t>Iconic Covent Garden location Finished to an excellent standard throughout High ceilings Wooden flooring throughout; outdoor space is communal/shared; size not stated</t>
-        </is>
-      </c>
-      <c r="M33" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N33" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O33" s="6" t="inlineStr">
+      <c r="J33" s="4" t="n">
+        <v>455</v>
+      </c>
+      <c r="K33" s="4" t="inlineStr"/>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>Iconic Covent Garden location Finished to an excellent standard throughout High ceilings Wooden flooring throughout; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M33" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N33" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O33" s="4" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
@@ -2761,11 +2795,13 @@
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J34" s="4" t="n"/>
+      <c r="J34" s="4" t="n">
+        <v>495</v>
+      </c>
       <c r="K34" s="4" t="inlineStr"/>
       <c r="L34" s="4" t="inlineStr">
         <is>
-          <t>One bedroom One bathroom, ensuite; outdoor space is communal/shared; size not stated; listed furnished — check if flexible</t>
+          <t>One bedroom One bathroom, ensuite; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M34" s="4" t="inlineStr">
@@ -2828,11 +2864,13 @@
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J35" s="6" t="n"/>
+      <c r="J35" s="6" t="n">
+        <v>480</v>
+      </c>
       <c r="K35" s="6" t="inlineStr"/>
       <c r="L35" s="6" t="inlineStr">
         <is>
-          <t>Superb one bedroom flat arranged on the second floor Spacious reception/kitchen with ample dining space; outdoor space is communal/shared; size not stated</t>
+          <t>Superb one bedroom flat arranged on the second floor Spacious reception/kitchen with ample dining space; outdoor space is communal/shared; under 650 sq ft</t>
         </is>
       </c>
       <c r="M35" s="6" t="inlineStr">
@@ -2895,11 +2933,13 @@
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J36" s="4" t="n"/>
+      <c r="J36" s="4" t="n">
+        <v>455</v>
+      </c>
       <c r="K36" s="4" t="inlineStr"/>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Furnished Recently refurbished; outdoor space is communal/shared; size not stated; listed furnished — check if flexible</t>
+          <t>Furnished Recently refurbished; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
@@ -2962,11 +3002,13 @@
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J37" s="4" t="n"/>
+      <c r="J37" s="4" t="n">
+        <v>398</v>
+      </c>
       <c r="K37" s="4" t="inlineStr"/>
       <c r="L37" s="4" t="inlineStr">
         <is>
-          <t>Newly Refurbished Central Location; outdoor space is communal/shared; size not stated; listed furnished — check if flexible</t>
+          <t>Newly Refurbished Central Location; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M37" s="4" t="inlineStr">
@@ -2986,203 +3028,207 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="6" t="inlineStr">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>2 bedroom apartment to rent</t>
         </is>
       </c>
-      <c r="B38" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C38" s="7" t="inlineStr">
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
         <is>
           <t>https://www.onthemarket.com/details/3102769/</t>
         </is>
       </c>
-      <c r="D38" s="6" t="inlineStr">
+      <c r="D38" s="4" t="inlineStr">
         <is>
           <t>John Adam Street, Covent Garden, WC2N</t>
         </is>
       </c>
-      <c r="E38" s="6" t="inlineStr">
+      <c r="E38" s="4" t="inlineStr">
         <is>
           <t>WC2N</t>
         </is>
       </c>
-      <c r="F38" s="6" t="n">
+      <c r="F38" s="4" t="n">
         <v>3185</v>
       </c>
-      <c r="G38" s="6" t="inlineStr">
+      <c r="G38" s="4" t="inlineStr">
         <is>
           <t>2-Bed</t>
         </is>
       </c>
-      <c r="H38" s="6" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="I38" s="6" t="inlineStr">
+      <c r="H38" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I38" s="4" t="inlineStr">
         <is>
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J38" s="6" t="n">
+      <c r="J38" s="4" t="n">
         <v>655</v>
       </c>
-      <c r="K38" s="6" t="inlineStr"/>
-      <c r="L38" s="6" t="inlineStr">
-        <is>
-          <t>Concierge Close to the area's Universities for students and academics; outdoor space is communal/shared</t>
-        </is>
-      </c>
-      <c r="M38" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N38" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O38" s="6" t="inlineStr">
+      <c r="K38" s="4" t="inlineStr"/>
+      <c r="L38" s="4" t="inlineStr">
+        <is>
+          <t>Concierge Close to the area's Universities for students and academics; outdoor space is communal/shared; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M38" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N38" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O38" s="4" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="6" t="inlineStr">
+      <c r="A39" s="4" t="inlineStr">
         <is>
           <t>1 bedroom flat to rent</t>
         </is>
       </c>
-      <c r="B39" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C39" s="7" t="inlineStr">
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
         <is>
           <t>https://www.onthemarket.com/details/19733694/</t>
         </is>
       </c>
-      <c r="D39" s="6" t="inlineStr">
+      <c r="D39" s="4" t="inlineStr">
         <is>
           <t>Maiden Lane, Covent Garden, London, WC2E</t>
         </is>
       </c>
-      <c r="E39" s="6" t="inlineStr">
+      <c r="E39" s="4" t="inlineStr">
         <is>
           <t>WC2E</t>
         </is>
       </c>
-      <c r="F39" s="6" t="n">
+      <c r="F39" s="4" t="n">
         <v>3684</v>
       </c>
-      <c r="G39" s="6" t="inlineStr">
+      <c r="G39" s="4" t="inlineStr">
         <is>
           <t>1-Bed</t>
         </is>
       </c>
-      <c r="H39" s="6" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="I39" s="6" t="inlineStr">
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I39" s="4" t="inlineStr">
         <is>
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J39" s="6" t="n"/>
-      <c r="K39" s="6" t="inlineStr"/>
-      <c r="L39" s="6" t="inlineStr">
-        <is>
-          <t>1 bedroom flat arranged on the 4th floor Bright and spacious reception room; outdoor space is communal/shared; size not stated</t>
-        </is>
-      </c>
-      <c r="M39" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N39" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O39" s="6" t="inlineStr">
+      <c r="J39" s="4" t="n">
+        <v>630</v>
+      </c>
+      <c r="K39" s="4" t="inlineStr"/>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>1 bedroom flat arranged on the 4th floor Bright and spacious reception room; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M39" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N39" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O39" s="4" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>1 bedroom flat to rent</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr">
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
         <is>
           <t>https://www.onthemarket.com/details/19725776/</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="D40" s="4" t="inlineStr">
         <is>
           <t>Shelton Street, Covent Garden, London, WC2H</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E40" s="4" t="inlineStr">
         <is>
           <t>WC2H</t>
         </is>
       </c>
-      <c r="F40" s="2" t="n">
+      <c r="F40" s="4" t="n">
         <v>3500</v>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G40" s="4" t="inlineStr">
         <is>
           <t>1-Bed</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="I40" s="2" t="inlineStr">
+      <c r="H40" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I40" s="4" t="inlineStr">
         <is>
           <t>Private balcony/terrace</t>
         </is>
       </c>
-      <c r="J40" s="2" t="n"/>
-      <c r="K40" s="2" t="inlineStr"/>
-      <c r="L40" s="2" t="inlineStr">
-        <is>
-          <t>Stylish one bedroom, third floor apartment Beautifully proportioned open plan reception with balcony access; size not stated</t>
-        </is>
-      </c>
-      <c r="M40" s="2" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N40" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="O40" s="2" t="inlineStr">
+      <c r="J40" s="4" t="n">
+        <v>608</v>
+      </c>
+      <c r="K40" s="4" t="inlineStr"/>
+      <c r="L40" s="4" t="inlineStr">
+        <is>
+          <t>Stylish one bedroom, third floor apartment Beautifully proportioned open plan reception with balcony access; under 650 sq ft; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M40" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N40" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O40" s="4" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
@@ -3301,11 +3347,13 @@
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J42" s="4" t="n"/>
+      <c r="J42" s="4" t="n">
+        <v>441</v>
+      </c>
       <c r="K42" s="4" t="inlineStr"/>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>One double bedroom One bathroom; outdoor space is communal/shared; size not stated; listed furnished — check if flexible</t>
+          <t>One double bedroom One bathroom; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
@@ -3368,11 +3416,13 @@
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J43" s="4" t="n"/>
+      <c r="J43" s="4" t="n">
+        <v>667</v>
+      </c>
       <c r="K43" s="4" t="inlineStr"/>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>One bedroom One bathroom; outdoor space is communal/shared; size not stated; listed furnished — check if flexible</t>
+          <t>One bedroom One bathroom; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
@@ -3392,67 +3442,69 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="6" t="inlineStr">
+      <c r="A44" s="4" t="inlineStr">
         <is>
           <t>2 bedroom flat to rent</t>
         </is>
       </c>
-      <c r="B44" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C44" s="7" t="inlineStr">
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
         <is>
           <t>https://www.onthemarket.com/details/19511649/</t>
         </is>
       </c>
-      <c r="D44" s="6" t="inlineStr">
+      <c r="D44" s="4" t="inlineStr">
         <is>
           <t>Broad Court, Covent Garden, London, WC2B</t>
         </is>
       </c>
-      <c r="E44" s="6" t="inlineStr">
+      <c r="E44" s="4" t="inlineStr">
         <is>
           <t>WC2B</t>
         </is>
       </c>
-      <c r="F44" s="6" t="n">
+      <c r="F44" s="4" t="n">
         <v>3684</v>
       </c>
-      <c r="G44" s="6" t="inlineStr">
+      <c r="G44" s="4" t="inlineStr">
         <is>
           <t>2-Bed</t>
         </is>
       </c>
-      <c r="H44" s="6" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="I44" s="6" t="inlineStr">
+      <c r="H44" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I44" s="4" t="inlineStr">
         <is>
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J44" s="6" t="n"/>
-      <c r="K44" s="6" t="inlineStr"/>
-      <c r="L44" s="6" t="inlineStr">
-        <is>
-          <t>2 bedroom flat arranged on raised ground floor Attractive period building with a sought-after location; outdoor space is communal/shared; size not stated</t>
-        </is>
-      </c>
-      <c r="M44" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N44" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O44" s="6" t="inlineStr">
+      <c r="J44" s="4" t="n">
+        <v>811</v>
+      </c>
+      <c r="K44" s="4" t="inlineStr"/>
+      <c r="L44" s="4" t="inlineStr">
+        <is>
+          <t>2 bedroom flat arranged on raised ground floor Attractive period building with a sought-after location; outdoor space is communal/shared; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M44" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N44" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O44" s="4" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
@@ -3526,67 +3578,69 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="A46" s="4" t="inlineStr">
         <is>
           <t>1 bedroom apartment to rent</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C46" s="3" t="inlineStr">
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
         <is>
           <t>https://www.onthemarket.com/details/9591535/</t>
         </is>
       </c>
-      <c r="D46" s="2" t="inlineStr">
+      <c r="D46" s="4" t="inlineStr">
         <is>
           <t>Casson Square, Waterloo, Southbank Place, London, SE1</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="E46" s="4" t="inlineStr">
         <is>
           <t>SE1</t>
         </is>
       </c>
-      <c r="F46" s="2" t="n">
+      <c r="F46" s="4" t="n">
         <v>4075</v>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="G46" s="4" t="inlineStr">
         <is>
           <t>1-Bed</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr">
-        <is>
-          <t>Flexible</t>
-        </is>
-      </c>
-      <c r="I46" s="2" t="inlineStr">
+      <c r="H46" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I46" s="4" t="inlineStr">
         <is>
           <t>Private balcony/terrace</t>
         </is>
       </c>
-      <c r="J46" s="2" t="n"/>
-      <c r="K46" s="2" t="inlineStr"/>
-      <c r="L46" s="2" t="inlineStr">
-        <is>
-          <t>*video viewing available* 24-hour five-star concierge 18,000 sq ft gym, pool and spa facilities Bedroom; size not stated</t>
-        </is>
-      </c>
-      <c r="M46" s="2" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N46" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="O46" s="2" t="inlineStr">
+      <c r="J46" s="4" t="n">
+        <v>641</v>
+      </c>
+      <c r="K46" s="4" t="inlineStr"/>
+      <c r="L46" s="4" t="inlineStr">
+        <is>
+          <t>*video viewing available* 24-hour five-star concierge 18,000 sq ft gym, pool and spa facilities Bedroom; under 650 sq ft; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M46" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N46" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O46" s="4" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
@@ -3628,7 +3682,7 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Part Furnished</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
@@ -3636,11 +3690,13 @@
           <t>Private balcony/terrace</t>
         </is>
       </c>
-      <c r="J47" s="2" t="n"/>
+      <c r="J47" s="2" t="n">
+        <v>691</v>
+      </c>
       <c r="K47" s="2" t="inlineStr"/>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>Superb 2 bedroom flat on lower ground floor Modern open-plan kitchen with integrated appliance Spacious reception room leading to lovely private patio 2 well-pr; size not stated</t>
+          <t>Superb 2 bedroom flat on lower ground floor Modern open-plan kitchen with integrated appliance Spacious reception room leading to lovely private patio 2 well-pr</t>
         </is>
       </c>
       <c r="M47" s="2" t="inlineStr">
@@ -3764,7 +3820,7 @@
       </c>
       <c r="H49" s="4" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Furnished</t>
         </is>
       </c>
       <c r="I49" s="4" t="inlineStr">
@@ -3778,7 +3834,7 @@
       <c r="K49" s="4" t="inlineStr"/>
       <c r="L49" s="4" t="inlineStr">
         <is>
-          <t>Two double bedrooms Dine-in kitchen; verify balcony/terrace</t>
+          <t>Two double bedrooms Dine-in kitchen; verify balcony/terrace; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M49" s="4" t="inlineStr">
@@ -3798,201 +3854,207 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="4" t="inlineStr">
+      <c r="A50" s="6" t="inlineStr">
         <is>
           <t>1 bedroom flat to rent</t>
         </is>
       </c>
-      <c r="B50" s="4" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
         <is>
           <t>https://www.onthemarket.com/details/14179323/</t>
         </is>
       </c>
-      <c r="D50" s="4" t="inlineStr">
+      <c r="D50" s="6" t="inlineStr">
         <is>
           <t>Bloomsbury Square, Bloomsbury, Covent Garden, London, WC1A</t>
         </is>
       </c>
-      <c r="E50" s="4" t="inlineStr">
+      <c r="E50" s="6" t="inlineStr">
         <is>
           <t>WC1A</t>
         </is>
       </c>
-      <c r="F50" s="4" t="n">
+      <c r="F50" s="6" t="n">
         <v>3500</v>
       </c>
-      <c r="G50" s="4" t="inlineStr">
+      <c r="G50" s="6" t="inlineStr">
         <is>
           <t>1-Bed</t>
         </is>
       </c>
-      <c r="H50" s="4" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="I50" s="4" t="inlineStr">
+      <c r="H50" s="6" t="inlineStr">
+        <is>
+          <t>Part Furnished</t>
+        </is>
+      </c>
+      <c r="I50" s="6" t="inlineStr">
+        <is>
+          <t>Communal / shared</t>
+        </is>
+      </c>
+      <c r="J50" s="6" t="n">
+        <v>734</v>
+      </c>
+      <c r="K50" s="6" t="inlineStr"/>
+      <c r="L50" s="6" t="inlineStr">
+        <is>
+          <t>Stunning Period Conversion Hardwood Flooring Multi-Room Sound System and Mood Lighting Throughout Contemporary Kitchen &amp; Bathroom; outdoor space is communal/shared</t>
+        </is>
+      </c>
+      <c r="M50" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N50" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O50" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>1 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19823664/</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>Bedford Court Mansions, Adeline Place, Bloomsbury, London, WC1B</t>
+        </is>
+      </c>
+      <c r="E51" s="6" t="inlineStr">
+        <is>
+          <t>WC1B</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="n">
+        <v>3141</v>
+      </c>
+      <c r="G51" s="6" t="inlineStr">
+        <is>
+          <t>1-Bed</t>
+        </is>
+      </c>
+      <c r="H51" s="6" t="inlineStr">
+        <is>
+          <t>Flexible</t>
+        </is>
+      </c>
+      <c r="I51" s="6" t="inlineStr">
+        <is>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J51" s="6" t="n">
+        <v>573</v>
+      </c>
+      <c r="K51" s="6" t="inlineStr"/>
+      <c r="L51" s="6" t="inlineStr">
+        <is>
+          <t>One Bedroom Finished to high standard Lift Access Separate Kitchen; under 650 sq ft</t>
+        </is>
+      </c>
+      <c r="M51" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N51" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O51" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>1 bedroom apartment to rent</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/13502768/</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>Bedford Court Mansions, Bloomsbury, WC1B</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>WC1B</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="n">
+        <v>3142</v>
+      </c>
+      <c r="G52" s="4" t="inlineStr">
+        <is>
+          <t>1-Bed</t>
+        </is>
+      </c>
+      <c r="H52" s="4" t="inlineStr">
+        <is>
+          <t>Flexible</t>
+        </is>
+      </c>
+      <c r="I52" s="4" t="inlineStr">
         <is>
           <t>Not stated</t>
         </is>
       </c>
-      <c r="J50" s="4" t="n"/>
-      <c r="K50" s="4" t="inlineStr"/>
-      <c r="L50" s="4" t="inlineStr">
-        <is>
-          <t>Stunning Period Conversion Hardwood Flooring Multi-Room Sound System and Mood Lighting Throughout Contemporary Kitchen &amp; Bathroom; verify balcony/terrace; size not stated</t>
-        </is>
-      </c>
-      <c r="M50" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N50" s="4" t="inlineStr">
+      <c r="J52" s="4" t="n">
+        <v>587</v>
+      </c>
+      <c r="K52" s="4" t="inlineStr"/>
+      <c r="L52" s="4" t="inlineStr">
+        <is>
+          <t>One Bedroom Professionally Managed; verify balcony/terrace; under 650 sq ft</t>
+        </is>
+      </c>
+      <c r="M52" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N52" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="O50" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="4" t="inlineStr">
-        <is>
-          <t>1 bedroom flat to rent</t>
-        </is>
-      </c>
-      <c r="B51" s="4" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/19823664/</t>
-        </is>
-      </c>
-      <c r="D51" s="4" t="inlineStr">
-        <is>
-          <t>Bedford Court Mansions, Adeline Place, Bloomsbury, London, WC1B</t>
-        </is>
-      </c>
-      <c r="E51" s="4" t="inlineStr">
-        <is>
-          <t>WC1B</t>
-        </is>
-      </c>
-      <c r="F51" s="4" t="n">
-        <v>3141</v>
-      </c>
-      <c r="G51" s="4" t="inlineStr">
-        <is>
-          <t>1-Bed</t>
-        </is>
-      </c>
-      <c r="H51" s="4" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="I51" s="4" t="inlineStr">
-        <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="J51" s="4" t="n"/>
-      <c r="K51" s="4" t="inlineStr"/>
-      <c r="L51" s="4" t="inlineStr">
-        <is>
-          <t>One Bedroom Finished to high standard Lift Access Separate Kitchen; verify balcony/terrace; size not stated</t>
-        </is>
-      </c>
-      <c r="M51" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N51" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="O51" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="6" t="inlineStr">
-        <is>
-          <t>1 bedroom apartment to rent</t>
-        </is>
-      </c>
-      <c r="B52" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C52" s="7" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/13502768/</t>
-        </is>
-      </c>
-      <c r="D52" s="6" t="inlineStr">
-        <is>
-          <t>Bedford Court Mansions, Bloomsbury, WC1B</t>
-        </is>
-      </c>
-      <c r="E52" s="6" t="inlineStr">
-        <is>
-          <t>WC1B</t>
-        </is>
-      </c>
-      <c r="F52" s="6" t="n">
-        <v>3142</v>
-      </c>
-      <c r="G52" s="6" t="inlineStr">
-        <is>
-          <t>1-Bed</t>
-        </is>
-      </c>
-      <c r="H52" s="6" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="I52" s="6" t="inlineStr">
-        <is>
-          <t>Communal / shared</t>
-        </is>
-      </c>
-      <c r="J52" s="6" t="n"/>
-      <c r="K52" s="6" t="inlineStr"/>
-      <c r="L52" s="6" t="inlineStr">
-        <is>
-          <t>One Bedroom Professionally Managed; outdoor space is communal/shared; size not stated</t>
-        </is>
-      </c>
-      <c r="M52" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N52" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O52" s="6" t="inlineStr">
+      <c r="O52" s="4" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
@@ -4101,7 +4163,7 @@
       </c>
       <c r="H54" s="4" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I54" s="4" t="inlineStr">
@@ -4109,11 +4171,13 @@
           <t>Not stated</t>
         </is>
       </c>
-      <c r="J54" s="4" t="n"/>
+      <c r="J54" s="4" t="n">
+        <v>609</v>
+      </c>
       <c r="K54" s="4" t="inlineStr"/>
       <c r="L54" s="4" t="inlineStr">
         <is>
-          <t>One Bedroom High Ceilings Views of Bloomsbury Square Wow Factor; verify balcony/terrace; size not stated</t>
+          <t>One Bedroom High Ceilings Views of Bloomsbury Square Wow Factor; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M54" s="4" t="inlineStr">
@@ -4168,7 +4232,7 @@
       </c>
       <c r="H55" s="6" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I55" s="6" t="inlineStr">
@@ -4237,7 +4301,7 @@
       </c>
       <c r="H56" s="4" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Part Furnished</t>
         </is>
       </c>
       <c r="I56" s="4" t="inlineStr">
@@ -4245,11 +4309,13 @@
           <t>Not stated</t>
         </is>
       </c>
-      <c r="J56" s="4" t="n"/>
+      <c r="J56" s="4" t="n">
+        <v>602</v>
+      </c>
       <c r="K56" s="4" t="inlineStr"/>
       <c r="L56" s="4" t="inlineStr">
         <is>
-          <t>Superb 2 bedroom flat Spacious arrangement; verify balcony/terrace; size not stated</t>
+          <t>Superb 2 bedroom flat Spacious arrangement; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M56" s="4" t="inlineStr">
@@ -4269,134 +4335,138 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="inlineStr">
+      <c r="A57" s="6" t="inlineStr">
         <is>
           <t>1 bedroom flat to rent</t>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C57" s="3" t="inlineStr">
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
         <is>
           <t>https://www.onthemarket.com/details/19736445/</t>
         </is>
       </c>
-      <c r="D57" s="2" t="inlineStr">
+      <c r="D57" s="6" t="inlineStr">
         <is>
           <t>Millman Street, Bloomsbury, London, WC1N</t>
         </is>
       </c>
-      <c r="E57" s="2" t="inlineStr">
+      <c r="E57" s="6" t="inlineStr">
         <is>
           <t>WC1N</t>
         </is>
       </c>
-      <c r="F57" s="2" t="n">
+      <c r="F57" s="6" t="n">
         <v>3142</v>
       </c>
-      <c r="G57" s="2" t="inlineStr">
+      <c r="G57" s="6" t="inlineStr">
         <is>
           <t>1-Bed</t>
         </is>
       </c>
-      <c r="H57" s="2" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="I57" s="2" t="inlineStr">
+      <c r="H57" s="6" t="inlineStr">
+        <is>
+          <t>Part Furnished</t>
+        </is>
+      </c>
+      <c r="I57" s="6" t="inlineStr">
         <is>
           <t>Private balcony/terrace</t>
         </is>
       </c>
-      <c r="J57" s="2" t="n"/>
-      <c r="K57" s="2" t="inlineStr"/>
-      <c r="L57" s="2" t="inlineStr">
-        <is>
-          <t>Fantastic 1 bedroom flat arranged on the ground floor Set within a lovely residential block; size not stated</t>
-        </is>
-      </c>
-      <c r="M57" s="2" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N57" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="O57" s="2" t="inlineStr">
+      <c r="J57" s="6" t="n">
+        <v>542</v>
+      </c>
+      <c r="K57" s="6" t="inlineStr"/>
+      <c r="L57" s="6" t="inlineStr">
+        <is>
+          <t>Fantastic 1 bedroom flat arranged on the ground floor Set within a lovely residential block; under 650 sq ft</t>
+        </is>
+      </c>
+      <c r="M57" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N57" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O57" s="6" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="6" t="inlineStr">
+      <c r="A58" s="4" t="inlineStr">
         <is>
           <t>1 bedroom flat to rent</t>
         </is>
       </c>
-      <c r="B58" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C58" s="7" t="inlineStr">
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
         <is>
           <t>https://www.onthemarket.com/details/19715608/</t>
         </is>
       </c>
-      <c r="D58" s="6" t="inlineStr">
+      <c r="D58" s="4" t="inlineStr">
         <is>
           <t>Bloomsbury Square, London WC1A</t>
         </is>
       </c>
-      <c r="E58" s="6" t="inlineStr">
+      <c r="E58" s="4" t="inlineStr">
         <is>
           <t>WC1A</t>
         </is>
       </c>
-      <c r="F58" s="6" t="n">
+      <c r="F58" s="4" t="n">
         <v>3000</v>
       </c>
-      <c r="G58" s="6" t="inlineStr">
+      <c r="G58" s="4" t="inlineStr">
         <is>
           <t>1-Bed</t>
         </is>
       </c>
-      <c r="H58" s="6" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="I58" s="6" t="inlineStr">
+      <c r="H58" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I58" s="4" t="inlineStr">
         <is>
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J58" s="6" t="n"/>
-      <c r="K58" s="6" t="inlineStr"/>
-      <c r="L58" s="6" t="inlineStr">
-        <is>
-          <t>Period Building Concierge; outdoor space is communal/shared; size not stated</t>
-        </is>
-      </c>
-      <c r="M58" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N58" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O58" s="6" t="inlineStr">
+      <c r="J58" s="4" t="n">
+        <v>581</v>
+      </c>
+      <c r="K58" s="4" t="inlineStr"/>
+      <c r="L58" s="4" t="inlineStr">
+        <is>
+          <t>Period Building Concierge; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M58" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N58" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O58" s="4" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>

</xml_diff>

<commit_message>
Daily tracker update 2026-07-06
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Flats" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Flats'!$A$1:$O$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Flats'!$A$1:$O$61</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O58"/>
+  <dimension ref="A1:O61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -552,231 +552,231 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Apartment</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Rightmove</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>https://www.rightmove.co.uk/properties/89143989</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Waterloo Road, Southwark, SE1</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>2 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19194043/</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Great Suffolk Street, Southwark, London, SE1</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>SE1</t>
         </is>
       </c>
-      <c r="F2" s="2" t="n">
-        <v>4346</v>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="F2" s="4" t="n">
+        <v>3100</v>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>2-Bed</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Part Furnished</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>Juliet only</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="n">
+        <v>638</v>
+      </c>
+      <c r="K2" s="4" t="inlineStr"/>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>Stylish 2 bedroom flat set on the 5th floor Large reception room with Juliet balcony Modern kitchen 2 lovely double bedroom; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M2" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N2" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O2" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>1 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19099769/</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Fletcher Buildings,, Covent Garden, London, WC2B</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>WC2B</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>3792</v>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>1-Bed</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>Communal / shared</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>320</v>
+      </c>
+      <c r="K3" s="4" t="inlineStr"/>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>Bright and airy one bedroom apartment in a prime Central London location Well proportioned reception with high ceilings and neutral décor Generous double bedroo; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M3" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N3" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O3" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>2 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/6356511/</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Great James Street, Bloomsbury, London, WC1N</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>WC1N</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>3683</v>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>2-Bed</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Private balcony/terrace</t>
         </is>
       </c>
-      <c r="J2" s="2" t="n">
-        <v>1385</v>
-      </c>
-      <c r="K2" s="2" t="n"/>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>Two bedroom apartment with incredible views Waterloo Road SE1 250 Waterloo Road is an exciting new rental development conveniently located on Waterloo Road, SE1</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>2 bedroom apartment to rent</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/4473051/</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Waterloo Road, Southwark, SE1</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>SE1</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>4346</v>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>2-Bed</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Part Furnished</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Private balcony/terrace</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="n">
-        <v>1385</v>
-      </c>
-      <c r="K3" s="2" t="n"/>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>Spectacular Views Waterloo</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>2 bedroom flat to rent</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/19728858/</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Waterloo Road, London SE1</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>SE1</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>4350</v>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>2-Bed</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Flexible</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Private balcony/terrace</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="n">
-        <v>1140</v>
-      </c>
-      <c r="K4" s="2" t="n"/>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>Two Bedrooms Two Bathrooms</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
+      <c r="J4" s="4" t="n">
+        <v>928</v>
+      </c>
+      <c r="K4" s="4" t="inlineStr"/>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>Spacious Split Level Apartment Large Terrace Wooden Flooring Nearest tubes: Chancery Lane, Russell Square &amp; Holborn; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O4" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>Apartment</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>OnTheMarket</t>
+          <t>Rightmove</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/6248222/</t>
+          <t>https://www.rightmove.co.uk/properties/89143989</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Nelson Square, Southwark, London, SE1</t>
+          <t>Waterloo Road, Southwark, SE1</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -785,7 +785,7 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>3150</v>
+        <v>4346</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
@@ -794,7 +794,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Part Furnished</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -803,12 +803,12 @@
         </is>
       </c>
       <c r="J5" s="2" t="n">
-        <v>809</v>
+        <v>1385</v>
       </c>
       <c r="K5" s="2" t="n"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Dishwasher Range / Oven</t>
+          <t>Two bedroom apartment with incredible views Waterloo Road SE1 250 Waterloo Road is an exciting new rental development conveniently located on Waterloo Road, SE1</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -830,7 +830,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -840,21 +840,21 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19663010/</t>
+          <t>https://www.onthemarket.com/details/4473051/</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Guilford Street, Bloomsbury, London, WC1N</t>
+          <t>Waterloo Road, Southwark, SE1</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>WC1N</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>3684</v>
+        <v>4346</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
@@ -872,232 +872,232 @@
         </is>
       </c>
       <c r="J6" s="2" t="n">
-        <v>691</v>
+        <v>1385</v>
       </c>
       <c r="K6" s="2" t="n"/>
       <c r="L6" s="2" t="inlineStr">
         <is>
+          <t>Spectacular Views Waterloo</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19728858/</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Waterloo Road, London SE1</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>SE1</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>4350</v>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>2-Bed</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Flexible</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>1140</v>
+      </c>
+      <c r="K7" s="2" t="n"/>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Two Bedrooms Two Bathrooms</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2 bedroom apartment to rent</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/6248222/</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Nelson Square, Southwark, London, SE1</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>SE1</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>3150</v>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>2-Bed</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Unfurnished</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>809</v>
+      </c>
+      <c r="K8" s="2" t="n"/>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Dishwasher Range / Oven</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19663010/</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Guilford Street, Bloomsbury, London, WC1N</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>WC1N</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>3684</v>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>2-Bed</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Part Furnished</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>691</v>
+      </c>
+      <c r="K9" s="2" t="n"/>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
           <t>Superb 2 bedroom flat on lower ground floor Modern open-plan kitchen with integrated appliance Spacious reception room leading to lovely private patio 2 well-pr</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="O6" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>2 bedroom apartment to rent</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/19809694/</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>Shaftesbury Avenue, Soho, W1D</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>W1D</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="n">
-        <v>3553</v>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>2-Bed</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>Flexible</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="inlineStr">
-        <is>
-          <t>Communal / shared</t>
-        </is>
-      </c>
-      <c r="J7" s="6" t="n">
-        <v>603</v>
-      </c>
-      <c r="K7" s="6" t="n"/>
-      <c r="L7" s="6" t="inlineStr">
-        <is>
-          <t>Beautifully Refurbished Secondary Glazing; outdoor space is communal/shared; under 650 sq ft</t>
-        </is>
-      </c>
-      <c r="M7" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N7" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O7" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>2 bedroom apartment to rent</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/13368018/</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>Shaftesbury Avenue , Soho, W1D</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>W1D</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="n">
-        <v>3987</v>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>2-Bed</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>Flexible</t>
-        </is>
-      </c>
-      <c r="I8" s="6" t="inlineStr">
-        <is>
-          <t>Communal / shared</t>
-        </is>
-      </c>
-      <c r="J8" s="6" t="n">
-        <v>671</v>
-      </c>
-      <c r="K8" s="6" t="n"/>
-      <c r="L8" s="6" t="inlineStr">
-        <is>
-          <t>Pet friendly Wooden Floors Student; outdoor space is communal/shared</t>
-        </is>
-      </c>
-      <c r="M8" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N8" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O8" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>2 bedroom apartment to rent</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/19627828/</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>Shaftesbury Avenue, Soho, W1D</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>W1D</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="n">
-        <v>3987</v>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>2-Bed</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>Flexible</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="inlineStr">
-        <is>
-          <t>Communal / shared</t>
-        </is>
-      </c>
-      <c r="J9" s="6" t="n">
-        <v>802</v>
-      </c>
-      <c r="K9" s="6" t="n"/>
-      <c r="L9" s="6" t="inlineStr">
-        <is>
-          <t>Built in Storage Pet Friendly; outdoor space is communal/shared</t>
-        </is>
-      </c>
-      <c r="M9" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N9" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O9" s="6" t="inlineStr">
+      <c r="O9" s="2" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
@@ -1106,7 +1106,7 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -1116,12 +1116,12 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19600564/</t>
+          <t>https://www.onthemarket.com/details/19809694/</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>Rupert Court, Soho, W1D</t>
+          <t>Shaftesbury Avenue, Soho, W1D</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
@@ -1130,11 +1130,11 @@
         </is>
       </c>
       <c r="F10" s="6" t="n">
-        <v>3163</v>
+        <v>3553</v>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
@@ -1147,11 +1147,13 @@
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J10" s="6" t="n"/>
+      <c r="J10" s="6" t="n">
+        <v>603</v>
+      </c>
       <c r="K10" s="6" t="n"/>
       <c r="L10" s="6" t="inlineStr">
         <is>
-          <t>Beautifully Refurbished Pet friendly; outdoor space is communal/shared; size not stated</t>
+          <t>Beautifully Refurbished Secondary Glazing; outdoor space is communal/shared; under 650 sq ft</t>
         </is>
       </c>
       <c r="M10" s="6" t="inlineStr">
@@ -1173,7 +1175,7 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
@@ -1183,30 +1185,30 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/10862827/</t>
+          <t>https://www.onthemarket.com/details/13368018/</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Rupert Court, Soho W1</t>
+          <t>Shaftesbury Avenue , Soho, W1D</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>W1D</t>
         </is>
       </c>
       <c r="F11" s="6" t="n">
-        <v>3163</v>
+        <v>3987</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
@@ -1215,12 +1217,12 @@
         </is>
       </c>
       <c r="J11" s="6" t="n">
-        <v>603</v>
+        <v>671</v>
       </c>
       <c r="K11" s="6" t="n"/>
       <c r="L11" s="6" t="inlineStr">
         <is>
-          <t>One bedroom One shower room; outdoor space is communal/shared; under 650 sq ft</t>
+          <t>Pet friendly Wooden Floors Student; outdoor space is communal/shared</t>
         </is>
       </c>
       <c r="M11" s="6" t="inlineStr">
@@ -1242,7 +1244,7 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -1252,30 +1254,30 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19845642/</t>
+          <t>https://www.onthemarket.com/details/19627828/</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>Shelton Street, Covent Garden, London, WC2H</t>
+          <t>Shaftesbury Avenue, Soho, W1D</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>WC2H</t>
+          <t>W1D</t>
         </is>
       </c>
       <c r="F12" s="6" t="n">
-        <v>3142</v>
+        <v>3987</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
@@ -1284,12 +1286,12 @@
         </is>
       </c>
       <c r="J12" s="6" t="n">
-        <v>480</v>
+        <v>802</v>
       </c>
       <c r="K12" s="6" t="n"/>
       <c r="L12" s="6" t="inlineStr">
         <is>
-          <t>Superb one bedroom flat arranged on the second floor Spacious reception/kitchen with ample dining space; outdoor space is communal/shared; under 650 sq ft</t>
+          <t>Built in Storage Pet Friendly; outdoor space is communal/shared</t>
         </is>
       </c>
       <c r="M12" s="6" t="inlineStr">
@@ -1321,21 +1323,21 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19603496/</t>
+          <t>https://www.onthemarket.com/details/19600564/</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Arne Street, Covent Garden, WC2E</t>
+          <t>Rupert Court, Soho, W1D</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>WC2E</t>
+          <t>W1D</t>
         </is>
       </c>
       <c r="F13" s="6" t="n">
-        <v>3250</v>
+        <v>3163</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -1344,7 +1346,7 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
@@ -1352,13 +1354,11 @@
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J13" s="6" t="n">
-        <v>514</v>
-      </c>
+      <c r="J13" s="6" t="n"/>
       <c r="K13" s="6" t="n"/>
       <c r="L13" s="6" t="inlineStr">
         <is>
-          <t>Council Tax Band G 514 sq ft floor area; outdoor space is communal/shared; under 650 sq ft</t>
+          <t>Beautifully Refurbished Pet friendly; outdoor space is communal/shared; size not stated</t>
         </is>
       </c>
       <c r="M13" s="6" t="inlineStr">
@@ -1380,7 +1380,7 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1390,21 +1390,21 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/14179323/</t>
+          <t>https://www.onthemarket.com/details/10862827/</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>Bloomsbury Square, Bloomsbury, Covent Garden, London, WC1A</t>
+          <t>Rupert Court, Soho W1</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>WC1A</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="F14" s="6" t="n">
-        <v>3500</v>
+        <v>3163</v>
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
@@ -1413,7 +1413,7 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>Part Furnished</t>
+          <t>Unfurnished</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
@@ -1422,12 +1422,12 @@
         </is>
       </c>
       <c r="J14" s="6" t="n">
-        <v>734</v>
+        <v>603</v>
       </c>
       <c r="K14" s="6" t="n"/>
       <c r="L14" s="6" t="inlineStr">
         <is>
-          <t>Stunning Period Conversion Hardwood Flooring Multi-Room Sound System and Mood Lighting Throughout Contemporary Kitchen &amp; Bathroom; outdoor space is communal/shared</t>
+          <t>One bedroom One shower room; outdoor space is communal/shared; under 650 sq ft</t>
         </is>
       </c>
       <c r="M14" s="6" t="inlineStr">
@@ -1459,21 +1459,21 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19823664/</t>
+          <t>https://www.onthemarket.com/details/19845642/</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Bedford Court Mansions, Adeline Place, Bloomsbury, London, WC1B</t>
+          <t>Shelton Street, Covent Garden, London, WC2H</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>WC1B</t>
+          <t>WC2H</t>
         </is>
       </c>
       <c r="F15" s="6" t="n">
-        <v>3141</v>
+        <v>3142</v>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
@@ -1482,21 +1482,21 @@
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J15" s="6" t="n">
-        <v>573</v>
+        <v>480</v>
       </c>
       <c r="K15" s="6" t="n"/>
       <c r="L15" s="6" t="inlineStr">
         <is>
-          <t>One Bedroom Finished to high standard Lift Access Separate Kitchen; under 650 sq ft</t>
+          <t>Superb one bedroom flat arranged on the second floor Spacious reception/kitchen with ample dining space; outdoor space is communal/shared; under 650 sq ft</t>
         </is>
       </c>
       <c r="M15" s="6" t="inlineStr">
@@ -1528,21 +1528,21 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/15813612/</t>
+          <t>https://www.onthemarket.com/details/19603496/</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>Bloomsbury Square, Bloomsbury, WC1A</t>
+          <t>Arne Street, Covent Garden, WC2E</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>WC1A</t>
+          <t>WC2E</t>
         </is>
       </c>
       <c r="F16" s="6" t="n">
-        <v>3142</v>
+        <v>3250</v>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
@@ -1551,21 +1551,21 @@
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Unfurnished</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J16" s="6" t="n">
-        <v>539</v>
+        <v>514</v>
       </c>
       <c r="K16" s="6" t="n"/>
       <c r="L16" s="6" t="inlineStr">
         <is>
-          <t>Large Double Bedroom Period Features Student; under 650 sq ft</t>
+          <t>Council Tax Band G 514 sq ft floor area; outdoor space is communal/shared; under 650 sq ft</t>
         </is>
       </c>
       <c r="M16" s="6" t="inlineStr">
@@ -1597,21 +1597,21 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19736445/</t>
+          <t>https://www.onthemarket.com/details/14179323/</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>Millman Street, Bloomsbury, London, WC1N</t>
+          <t>Bloomsbury Square, Bloomsbury, Covent Garden, London, WC1A</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>WC1N</t>
+          <t>WC1A</t>
         </is>
       </c>
       <c r="F17" s="6" t="n">
-        <v>3142</v>
+        <v>3500</v>
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
@@ -1625,236 +1625,236 @@
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J17" s="6" t="n">
-        <v>542</v>
+        <v>734</v>
       </c>
       <c r="K17" s="6" t="n"/>
       <c r="L17" s="6" t="inlineStr">
         <is>
+          <t>Stunning Period Conversion Hardwood Flooring Multi-Room Sound System and Mood Lighting Throughout Contemporary Kitchen &amp; Bathroom; outdoor space is communal/shared</t>
+        </is>
+      </c>
+      <c r="M17" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N17" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O17" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>1 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19823664/</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>Bedford Court Mansions, Adeline Place, Bloomsbury, London, WC1B</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>WC1B</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>3141</v>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>1-Bed</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>Flexible</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J18" s="6" t="n">
+        <v>573</v>
+      </c>
+      <c r="K18" s="6" t="n"/>
+      <c r="L18" s="6" t="inlineStr">
+        <is>
+          <t>One Bedroom Finished to high standard Lift Access Separate Kitchen; under 650 sq ft</t>
+        </is>
+      </c>
+      <c r="M18" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N18" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O18" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>1 bedroom apartment to rent</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/15813612/</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>Bloomsbury Square, Bloomsbury, WC1A</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>WC1A</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>3142</v>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>1-Bed</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>Flexible</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="n">
+        <v>539</v>
+      </c>
+      <c r="K19" s="6" t="n"/>
+      <c r="L19" s="6" t="inlineStr">
+        <is>
+          <t>Large Double Bedroom Period Features Student; under 650 sq ft</t>
+        </is>
+      </c>
+      <c r="M19" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N19" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O19" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>1 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19736445/</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>Millman Street, Bloomsbury, London, WC1N</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>WC1N</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>3142</v>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>1-Bed</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>Part Furnished</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J20" s="6" t="n">
+        <v>542</v>
+      </c>
+      <c r="K20" s="6" t="n"/>
+      <c r="L20" s="6" t="inlineStr">
+        <is>
           <t>Fantastic 1 bedroom flat arranged on the ground floor Set within a lovely residential block; under 650 sq ft</t>
         </is>
       </c>
-      <c r="M17" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N17" s="6" t="inlineStr">
+      <c r="M20" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N20" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="O17" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>Flat</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Rightmove</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>https://www.rightmove.co.uk/properties/90435384</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>251 SOUTHWARK BRIDGE ROAD, LONDON, SE1, Elephant and Castle, London, SE1</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>SE1</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="n">
-        <v>4250</v>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>1-Bed</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>Part Furnished</t>
-        </is>
-      </c>
-      <c r="I18" s="4" t="inlineStr">
-        <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="J18" s="4" t="n">
-        <v>520</v>
-      </c>
-      <c r="K18" s="4" t="n"/>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t>ZERO DEPOSIT AVAILABLE. SHORT LET. Set on the 21st floor, this 1 bedroom flat boasts well arranged interiors including a large reception room, a modern open-pla; verify balcony/terrace; under 650 sq ft</t>
-        </is>
-      </c>
-      <c r="M18" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N18" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="O18" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Flat</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Rightmove</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>https://www.rightmove.co.uk/properties/90432648</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>251 SOUTHWARK BRIDGE ROAD, LONDON, SE1, Elephant and Castle, London, SE1</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>SE1</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="n">
-        <v>3000</v>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>1-Bed</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>Part Furnished</t>
-        </is>
-      </c>
-      <c r="I19" s="4" t="inlineStr">
-        <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="J19" s="4" t="n">
-        <v>520</v>
-      </c>
-      <c r="K19" s="4" t="n"/>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>ZERO DEPOSIT AVAILABLE. LONG LET. Set on the 21st floor, this 1 bedroom flat boasts well arranged interiors including a large reception room, a modern open-plan; verify balcony/terrace; under 650 sq ft</t>
-        </is>
-      </c>
-      <c r="M19" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N19" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="O19" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>1 bedroom apartment to rent</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/4220060/</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>Carnaby Street, Soho, W1F</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>W1F</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="n">
-        <v>3640</v>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>1-Bed</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>Unfurnished</t>
-        </is>
-      </c>
-      <c r="I20" s="4" t="inlineStr">
-        <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="J20" s="4" t="n">
-        <v>553</v>
-      </c>
-      <c r="K20" s="4" t="n"/>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t>One bedroom apartment Newly refurbished; verify balcony/terrace; under 650 sq ft</t>
-        </is>
-      </c>
-      <c r="M20" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N20" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="O20" s="4" t="inlineStr">
+      <c r="O20" s="6" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
@@ -1863,31 +1863,31 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>Flat</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>OnTheMarket</t>
+          <t>Rightmove</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/8022324/</t>
+          <t>https://www.rightmove.co.uk/properties/90435384</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Golden Square, Soho, London, W1F</t>
+          <t>251 SOUTHWARK BRIDGE ROAD, LONDON, SE1, Elephant and Castle, London, SE1</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>W1F</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F21" s="4" t="n">
-        <v>3467</v>
+        <v>4250</v>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
@@ -1896,7 +1896,7 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>Furnished</t>
+          <t>Part Furnished</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -1905,12 +1905,12 @@
         </is>
       </c>
       <c r="J21" s="4" t="n">
-        <v>608</v>
+        <v>520</v>
       </c>
       <c r="K21" s="4" t="n"/>
       <c r="L21" s="4" t="inlineStr">
         <is>
-          <t>608 sq ft floor area Nearest station 0.1mi.; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>ZERO DEPOSIT AVAILABLE. SHORT LET. Set on the 21st floor, this 1 bedroom flat boasts well arranged interiors including a large reception room, a modern open-pla; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M21" s="4" t="inlineStr">
@@ -1932,54 +1932,54 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>Flat</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>OnTheMarket</t>
+          <t>Rightmove</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19852978/</t>
+          <t>https://www.rightmove.co.uk/properties/90432648</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Newport Court, Covent Garden, London, WC2H</t>
+          <t>251 SOUTHWARK BRIDGE ROAD, LONDON, SE1, Elephant and Castle, London, SE1</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>WC2H</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F22" s="4" t="n">
-        <v>4334</v>
+        <v>3000</v>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>Furnished</t>
+          <t>Part Furnished</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J22" s="4" t="n">
-        <v>858</v>
+        <v>520</v>
       </c>
       <c r="K22" s="4" t="n"/>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Splendid two bedroom flat Ample interiors; listed furnished — check if flexible</t>
+          <t>ZERO DEPOSIT AVAILABLE. LONG LET. Set on the 21st floor, this 1 bedroom flat boasts well arranged interiors including a large reception room, a modern open-plan; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
@@ -2001,7 +2001,7 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -2011,12 +2011,12 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/16157050/</t>
+          <t>https://www.onthemarket.com/details/4220060/</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Brewer Street, Soho, W1F</t>
+          <t>Carnaby Street, Soho, W1F</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
@@ -2025,30 +2025,30 @@
         </is>
       </c>
       <c r="F23" s="4" t="n">
-        <v>3142</v>
+        <v>3640</v>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>Furnished</t>
+          <t>Unfurnished</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J23" s="4" t="n">
-        <v>730</v>
+        <v>553</v>
       </c>
       <c r="K23" s="4" t="n"/>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>730 sqft Secure Entrance; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>One bedroom apartment Newly refurbished; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
@@ -2070,7 +2070,7 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
@@ -2080,21 +2080,21 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/9956499/</t>
+          <t>https://www.onthemarket.com/details/8022324/</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Richmond Buildings, Soho, W1D</t>
+          <t>Golden Square, Soho, London, W1F</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>W1D</t>
+          <t>W1F</t>
         </is>
       </c>
       <c r="F24" s="4" t="n">
-        <v>3835</v>
+        <v>3467</v>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
@@ -2112,12 +2112,12 @@
         </is>
       </c>
       <c r="J24" s="4" t="n">
-        <v>521</v>
+        <v>608</v>
       </c>
       <c r="K24" s="4" t="n"/>
       <c r="L24" s="4" t="inlineStr">
         <is>
-          <t>Council tax band: F 521 sq ft floor area; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>608 sq ft floor area Nearest station 0.1mi.; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M24" s="4" t="inlineStr">
@@ -2139,7 +2139,7 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -2149,25 +2149,25 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19786051/</t>
+          <t>https://www.onthemarket.com/details/19852978/</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Old Compton Street, Soho, London, W1D</t>
+          <t>Newport Court, Covent Garden, London, WC2H</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>W1D</t>
+          <t>WC2H</t>
         </is>
       </c>
       <c r="F25" s="4" t="n">
-        <v>3600</v>
+        <v>4334</v>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -2177,16 +2177,16 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Private balcony/terrace</t>
         </is>
       </c>
       <c r="J25" s="4" t="n">
-        <v>432</v>
+        <v>858</v>
       </c>
       <c r="K25" s="4" t="n"/>
       <c r="L25" s="4" t="inlineStr">
         <is>
-          <t>432 sq ft floor area Nearest station 0.1mi. Furnished Nearest school 0.2mi.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Splendid two bedroom flat Ample interiors; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M25" s="4" t="inlineStr">
@@ -2208,7 +2208,7 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
@@ -2218,12 +2218,12 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19828226/</t>
+          <t>https://www.onthemarket.com/details/16157050/</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>TCRW SOHO, Fareham Street, W1F</t>
+          <t>Brewer Street, Soho, W1F</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
@@ -2232,11 +2232,11 @@
         </is>
       </c>
       <c r="F26" s="4" t="n">
-        <v>3600</v>
+        <v>3142</v>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -2246,16 +2246,16 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J26" s="4" t="n">
-        <v>656</v>
+        <v>730</v>
       </c>
       <c r="K26" s="4" t="n"/>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Concierge service Highly sought-after Zone 1 location; verify balcony/terrace; listed furnished — check if flexible</t>
+          <t>730 sqft Secure Entrance; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
@@ -2277,7 +2277,7 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
@@ -2287,25 +2287,25 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/11345150/</t>
+          <t>https://www.onthemarket.com/details/9956499/</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Shaftesbury Avenue, Covent Garden, London, WC2H</t>
+          <t>Richmond Buildings, Soho, W1D</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>WC2H</t>
+          <t>W1D</t>
         </is>
       </c>
       <c r="F27" s="4" t="n">
-        <v>3575</v>
+        <v>3835</v>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
@@ -2315,16 +2315,16 @@
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J27" s="4" t="n">
-        <v>870</v>
+        <v>521</v>
       </c>
       <c r="K27" s="4" t="n"/>
       <c r="L27" s="4" t="inlineStr">
         <is>
-          <t>870 sq ft floor area Nearest station 0.1mi.; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>Council tax band: F 521 sq ft floor area; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M27" s="4" t="inlineStr">
@@ -2346,7 +2346,7 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
@@ -2356,12 +2356,12 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/4747672/</t>
+          <t>https://www.onthemarket.com/details/19786051/</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Townsend House, Deans Street, Soho W1D</t>
+          <t>Old Compton Street, Soho, London, W1D</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
@@ -2370,11 +2370,11 @@
         </is>
       </c>
       <c r="F28" s="4" t="n">
-        <v>3850</v>
+        <v>3600</v>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
@@ -2384,14 +2384,16 @@
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="J28" s="4" t="n"/>
+          <t>Communal / shared</t>
+        </is>
+      </c>
+      <c r="J28" s="4" t="n">
+        <v>432</v>
+      </c>
       <c r="K28" s="4" t="n"/>
       <c r="L28" s="4" t="inlineStr">
         <is>
-          <t>Close to Local Shops Close to Public Transport; verify balcony/terrace; size not stated; listed furnished — check if flexible</t>
+          <t>432 sq ft floor area Nearest station 0.1mi. Furnished Nearest school 0.2mi.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M28" s="4" t="inlineStr">
@@ -2423,21 +2425,21 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19628367/</t>
+          <t>https://www.onthemarket.com/details/19828226/</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Carnaby Street, Soho W1</t>
+          <t>TCRW SOHO, Fareham Street, W1F</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>W1F</t>
         </is>
       </c>
       <c r="F29" s="4" t="n">
-        <v>3640</v>
+        <v>3600</v>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
@@ -2446,7 +2448,7 @@
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Furnished</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
@@ -2455,12 +2457,12 @@
         </is>
       </c>
       <c r="J29" s="4" t="n">
-        <v>549</v>
+        <v>656</v>
       </c>
       <c r="K29" s="4" t="n"/>
       <c r="L29" s="4" t="inlineStr">
         <is>
-          <t>One bedroom One shower room, ensuite; verify balcony/terrace; under 650 sq ft</t>
+          <t>Concierge service Highly sought-after Zone 1 location; verify balcony/terrace; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M29" s="4" t="inlineStr">
@@ -2482,7 +2484,7 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -2492,44 +2494,44 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/13524814/</t>
+          <t>https://www.onthemarket.com/details/11345150/</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Carnaby Street, Soho, W1F</t>
+          <t>Shaftesbury Avenue, Covent Garden, London, WC2H</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>W1F</t>
+          <t>WC2H</t>
         </is>
       </c>
       <c r="F30" s="4" t="n">
-        <v>3640</v>
+        <v>3575</v>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Furnished</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J30" s="4" t="n">
-        <v>552</v>
+        <v>870</v>
       </c>
       <c r="K30" s="4" t="n"/>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Recently Refurbished Apartment Original Features Student; verify balcony/terrace; under 650 sq ft</t>
+          <t>870 sq ft floor area Nearest station 0.1mi.; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
@@ -2551,7 +2553,7 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
@@ -2561,30 +2563,30 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/18690047/</t>
+          <t>https://www.onthemarket.com/details/4747672/</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Duck Lane, Soho W1</t>
+          <t>Townsend House, Deans Street, Soho W1D</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>W1D</t>
         </is>
       </c>
       <c r="F31" s="4" t="n">
-        <v>3077</v>
+        <v>3850</v>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Furnished</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
@@ -2592,13 +2594,11 @@
           <t>Not stated</t>
         </is>
       </c>
-      <c r="J31" s="4" t="n">
-        <v>581</v>
-      </c>
+      <c r="J31" s="4" t="n"/>
       <c r="K31" s="4" t="n"/>
       <c r="L31" s="4" t="inlineStr">
         <is>
-          <t>One bedroom One bathroom; verify balcony/terrace; under 650 sq ft</t>
+          <t>Close to Local Shops Close to Public Transport; verify balcony/terrace; size not stated; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M31" s="4" t="inlineStr">
@@ -2630,21 +2630,21 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/18690128/</t>
+          <t>https://www.onthemarket.com/details/19628367/</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Duck Lane, Soho, W1F</t>
+          <t>Carnaby Street, Soho W1</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>W1F</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="F32" s="4" t="n">
-        <v>3077</v>
+        <v>3640</v>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
@@ -2662,12 +2662,12 @@
         </is>
       </c>
       <c r="J32" s="4" t="n">
-        <v>580</v>
+        <v>549</v>
       </c>
       <c r="K32" s="4" t="n"/>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>One Double bedroom Quaint Road; verify balcony/terrace; under 650 sq ft</t>
+          <t>One bedroom One shower room, ensuite; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
@@ -2699,12 +2699,12 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/18680649/</t>
+          <t>https://www.onthemarket.com/details/13524814/</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Duck Lane, Soho W1F</t>
+          <t>Carnaby Street, Soho, W1F</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
@@ -2713,7 +2713,7 @@
         </is>
       </c>
       <c r="F33" s="4" t="n">
-        <v>3077</v>
+        <v>3640</v>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
@@ -2731,12 +2731,12 @@
         </is>
       </c>
       <c r="J33" s="4" t="n">
-        <v>575</v>
+        <v>552</v>
       </c>
       <c r="K33" s="4" t="n"/>
       <c r="L33" s="4" t="inlineStr">
         <is>
-          <t>Modern Throughout Wooden Flooring Throughout; verify balcony/terrace; under 650 sq ft</t>
+          <t>Recently Refurbished Apartment Original Features Student; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M33" s="4" t="inlineStr">
@@ -2768,21 +2768,21 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/15707269/</t>
+          <t>https://www.onthemarket.com/details/18690047/</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Casson Square, London, Waterloo, United Kingdom, SE1</t>
+          <t>Duck Lane, Soho W1</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>SE1</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="F34" s="4" t="n">
-        <v>4050</v>
+        <v>3077</v>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
@@ -2791,21 +2791,21 @@
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>Furnished</t>
+          <t>Unfurnished</t>
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J34" s="4" t="n">
-        <v>514</v>
+        <v>581</v>
       </c>
       <c r="K34" s="4" t="n"/>
       <c r="L34" s="4" t="inlineStr">
         <is>
-          <t>Bedroom Bathroom Open-plan reception/kitchen 24 hour concierge; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>One bedroom One bathroom; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M34" s="4" t="inlineStr">
@@ -2837,21 +2837,21 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/9568931/</t>
+          <t>https://www.onthemarket.com/details/18690128/</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Casson Square, Waterloo, Southbank Place, London, SE1</t>
+          <t>Duck Lane, Soho, W1F</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>SE1</t>
+          <t>W1F</t>
         </is>
       </c>
       <c r="F35" s="4" t="n">
-        <v>4250</v>
+        <v>3077</v>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
@@ -2860,21 +2860,21 @@
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>Furnished</t>
+          <t>Unfurnished</t>
         </is>
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J35" s="4" t="n">
-        <v>644</v>
+        <v>580</v>
       </c>
       <c r="K35" s="4" t="n"/>
       <c r="L35" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom 1 bathroom Open-plan reception kitchen 24-hour five-star concierge; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>One Double bedroom Quaint Road; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M35" s="4" t="inlineStr">
@@ -2896,7 +2896,7 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom end of terrace house to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -2906,40 +2906,44 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19811489/</t>
+          <t>https://www.onthemarket.com/details/18680649/</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Carlisle Lane, Waterloo</t>
-        </is>
-      </c>
-      <c r="E36" s="4" t="n"/>
+          <t>Duck Lane, Soho W1F</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>W1F</t>
+        </is>
+      </c>
       <c r="F36" s="4" t="n">
-        <v>3575</v>
+        <v>3077</v>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>Furnished</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J36" s="4" t="n">
-        <v>904</v>
+        <v>575</v>
       </c>
       <c r="K36" s="4" t="n"/>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>End of Terrace Shared Garden; listed furnished — check if flexible</t>
+          <t>Modern Throughout Wooden Flooring Throughout; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
@@ -2961,7 +2965,7 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
@@ -2971,12 +2975,12 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/7516361/</t>
+          <t>https://www.onthemarket.com/details/15707269/</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Belvedere Road, Waterloo, London, SE1</t>
+          <t>Casson Square, London, Waterloo, United Kingdom, SE1</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
@@ -2985,11 +2989,11 @@
         </is>
       </c>
       <c r="F37" s="4" t="n">
-        <v>3350</v>
+        <v>4050</v>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
@@ -3003,12 +3007,12 @@
         </is>
       </c>
       <c r="J37" s="4" t="n">
-        <v>544</v>
+        <v>514</v>
       </c>
       <c r="K37" s="4" t="n"/>
       <c r="L37" s="4" t="inlineStr">
         <is>
-          <t>Residents' swimming pool and gym. Grade II listed period building. 24 hour porters. Set close to the iconic Southbank and London Eye.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Bedroom Bathroom Open-plan reception/kitchen 24 hour concierge; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M37" s="4" t="inlineStr">
@@ -3040,12 +3044,12 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/7589011/</t>
+          <t>https://www.onthemarket.com/details/9568931/</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Belvedere Road, London, Waterloo, SE1</t>
+          <t>Casson Square, Waterloo, Southbank Place, London, SE1</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
@@ -3054,7 +3058,7 @@
         </is>
       </c>
       <c r="F38" s="4" t="n">
-        <v>4200</v>
+        <v>4250</v>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
@@ -3068,16 +3072,16 @@
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Private balcony/terrace</t>
         </is>
       </c>
       <c r="J38" s="4" t="n">
-        <v>671</v>
+        <v>644</v>
       </c>
       <c r="K38" s="4" t="n"/>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>24-hour five-star concierge 18,000 sq ft gym and spa facilities Set in one of London's most connected locations, opposite Westminster and the Houses of Parliame; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>1 bedroom 1 bathroom Open-plan reception kitchen 24-hour five-star concierge; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
@@ -3099,7 +3103,7 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>2 bedroom end of terrace house to rent</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
@@ -3109,21 +3113,17 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/17616661/</t>
+          <t>https://www.onthemarket.com/details/19811489/</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>The Music Box, 237 Union Street, Southwark, London, SE1</t>
-        </is>
-      </c>
-      <c r="E39" s="4" t="inlineStr">
-        <is>
-          <t>SE1</t>
-        </is>
-      </c>
+          <t>Carlisle Lane, Waterloo</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="n"/>
       <c r="F39" s="4" t="n">
-        <v>3800</v>
+        <v>3575</v>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
@@ -3137,16 +3137,16 @@
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Private balcony/terrace</t>
         </is>
       </c>
       <c r="J39" s="4" t="n">
-        <v>841</v>
+        <v>904</v>
       </c>
       <c r="K39" s="4" t="n"/>
       <c r="L39" s="4" t="inlineStr">
         <is>
-          <t>Two bedrooms Two bathrooms 841 sq. ft. Excellent transport links; verify balcony/terrace; listed furnished — check if flexible</t>
+          <t>End of Terrace Shared Garden; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M39" s="4" t="inlineStr">
@@ -3168,7 +3168,7 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
@@ -3178,25 +3178,25 @@
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19863550/</t>
+          <t>https://www.onthemarket.com/details/7516361/</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>King Street, Covent Garden, London, WC2E</t>
+          <t>Belvedere Road, Waterloo, London, SE1</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>WC2E</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F40" s="4" t="n">
-        <v>3358</v>
+        <v>3350</v>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
@@ -3210,12 +3210,12 @@
         </is>
       </c>
       <c r="J40" s="4" t="n">
-        <v>455</v>
+        <v>544</v>
       </c>
       <c r="K40" s="4" t="n"/>
       <c r="L40" s="4" t="inlineStr">
         <is>
-          <t>Iconic Covent Garden location Finished to an excellent standard throughout High ceilings Wooden flooring throughout; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Residents' swimming pool and gym. Grade II listed period building. 24 hour porters. Set close to the iconic Southbank and London Eye.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M40" s="4" t="inlineStr">
@@ -3247,21 +3247,21 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19860280/</t>
+          <t>https://www.onthemarket.com/details/7589011/</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Floral Street, Covent Garden WC2</t>
+          <t>Belvedere Road, London, Waterloo, SE1</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>WC2</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F41" s="4" t="n">
-        <v>3380</v>
+        <v>4200</v>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
@@ -3279,12 +3279,12 @@
         </is>
       </c>
       <c r="J41" s="4" t="n">
-        <v>495</v>
+        <v>671</v>
       </c>
       <c r="K41" s="4" t="n"/>
       <c r="L41" s="4" t="inlineStr">
         <is>
-          <t>One bedroom One bathroom, ensuite; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>24-hour five-star concierge 18,000 sq ft gym and spa facilities Set in one of London's most connected locations, opposite Westminster and the Houses of Parliame; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M41" s="4" t="inlineStr">
@@ -3306,7 +3306,7 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
@@ -3316,25 +3316,25 @@
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/1837052/</t>
+          <t>https://www.onthemarket.com/details/17616661/</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>King Street, Covent Garden, WC2E</t>
+          <t>The Music Box, 237 Union Street, Southwark, London, SE1</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>WC2E</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F42" s="4" t="n">
-        <v>3358</v>
+        <v>3800</v>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
@@ -3344,16 +3344,16 @@
       </c>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J42" s="4" t="n">
-        <v>455</v>
+        <v>841</v>
       </c>
       <c r="K42" s="4" t="n"/>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Furnished Recently refurbished; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Two bedrooms Two bathrooms 841 sq. ft. Excellent transport links; verify balcony/terrace; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
@@ -3375,7 +3375,7 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
@@ -3385,12 +3385,12 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/3408032/</t>
+          <t>https://www.onthemarket.com/details/19863550/</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Floral Street, Covent Garden, WC2E</t>
+          <t>King Street, Covent Garden, London, WC2E</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
@@ -3399,7 +3399,7 @@
         </is>
       </c>
       <c r="F43" s="4" t="n">
-        <v>3380</v>
+        <v>3358</v>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
@@ -3417,12 +3417,12 @@
         </is>
       </c>
       <c r="J43" s="4" t="n">
-        <v>398</v>
+        <v>455</v>
       </c>
       <c r="K43" s="4" t="n"/>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Newly Refurbished Central Location; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Iconic Covent Garden location Finished to an excellent standard throughout High ceilings Wooden flooring throughout; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
@@ -3444,7 +3444,7 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
@@ -3454,25 +3454,25 @@
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/3102769/</t>
+          <t>https://www.onthemarket.com/details/19860280/</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>John Adam Street, Covent Garden, WC2N</t>
+          <t>Floral Street, Covent Garden WC2</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>WC2N</t>
+          <t>WC2</t>
         </is>
       </c>
       <c r="F44" s="4" t="n">
-        <v>3185</v>
+        <v>3380</v>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
@@ -3486,12 +3486,12 @@
         </is>
       </c>
       <c r="J44" s="4" t="n">
-        <v>655</v>
+        <v>495</v>
       </c>
       <c r="K44" s="4" t="n"/>
       <c r="L44" s="4" t="inlineStr">
         <is>
-          <t>Concierge Close to the area's Universities for students and academics; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>One bedroom One bathroom, ensuite; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M44" s="4" t="inlineStr">
@@ -3513,7 +3513,7 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
@@ -3523,12 +3523,12 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19733694/</t>
+          <t>https://www.onthemarket.com/details/1837052/</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Maiden Lane, Covent Garden, London, WC2E</t>
+          <t>King Street, Covent Garden, WC2E</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
@@ -3537,7 +3537,7 @@
         </is>
       </c>
       <c r="F45" s="4" t="n">
-        <v>3684</v>
+        <v>3358</v>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
@@ -3555,12 +3555,12 @@
         </is>
       </c>
       <c r="J45" s="4" t="n">
-        <v>630</v>
+        <v>455</v>
       </c>
       <c r="K45" s="4" t="n"/>
       <c r="L45" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat arranged on the 4th floor Bright and spacious reception room; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Furnished Recently refurbished; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M45" s="4" t="inlineStr">
@@ -3582,7 +3582,7 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
@@ -3592,21 +3592,21 @@
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19725776/</t>
+          <t>https://www.onthemarket.com/details/3408032/</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Shelton Street, Covent Garden, London, WC2H</t>
+          <t>Floral Street, Covent Garden, WC2E</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>WC2H</t>
+          <t>WC2E</t>
         </is>
       </c>
       <c r="F46" s="4" t="n">
-        <v>3500</v>
+        <v>3380</v>
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
@@ -3620,16 +3620,16 @@
       </c>
       <c r="I46" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J46" s="4" t="n">
-        <v>608</v>
+        <v>398</v>
       </c>
       <c r="K46" s="4" t="n"/>
       <c r="L46" s="4" t="inlineStr">
         <is>
-          <t>Stylish one bedroom, third floor apartment Beautifully proportioned open plan reception with balcony access; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Newly Refurbished Central Location; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M46" s="4" t="inlineStr">
@@ -3651,7 +3651,7 @@
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
@@ -3661,25 +3661,25 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19591709/</t>
+          <t>https://www.onthemarket.com/details/3102769/</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>King Street, Covent Garden WC2</t>
+          <t>John Adam Street, Covent Garden, WC2N</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>WC2</t>
+          <t>WC2N</t>
         </is>
       </c>
       <c r="F47" s="4" t="n">
-        <v>3575</v>
+        <v>3185</v>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr">
@@ -3693,12 +3693,12 @@
         </is>
       </c>
       <c r="J47" s="4" t="n">
-        <v>441</v>
+        <v>655</v>
       </c>
       <c r="K47" s="4" t="n"/>
       <c r="L47" s="4" t="inlineStr">
         <is>
-          <t>One double bedroom One bathroom; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Concierge Close to the area's Universities for students and academics; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M47" s="4" t="inlineStr">
@@ -3720,7 +3720,7 @@
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
@@ -3730,21 +3730,21 @@
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19591720/</t>
+          <t>https://www.onthemarket.com/details/19733694/</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>King Street, Covent Garden WC2</t>
+          <t>Maiden Lane, Covent Garden, London, WC2E</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>WC2</t>
+          <t>WC2E</t>
         </is>
       </c>
       <c r="F48" s="4" t="n">
-        <v>4333</v>
+        <v>3684</v>
       </c>
       <c r="G48" s="4" t="inlineStr">
         <is>
@@ -3762,12 +3762,12 @@
         </is>
       </c>
       <c r="J48" s="4" t="n">
-        <v>667</v>
+        <v>630</v>
       </c>
       <c r="K48" s="4" t="n"/>
       <c r="L48" s="4" t="inlineStr">
         <is>
-          <t>One bedroom One bathroom; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>1 bedroom flat arranged on the 4th floor Bright and spacious reception room; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M48" s="4" t="inlineStr">
@@ -3789,7 +3789,7 @@
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
@@ -3799,25 +3799,25 @@
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19511649/</t>
+          <t>https://www.onthemarket.com/details/19725776/</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>Broad Court, Covent Garden, London, WC2B</t>
+          <t>Shelton Street, Covent Garden, London, WC2H</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>WC2B</t>
+          <t>WC2H</t>
         </is>
       </c>
       <c r="F49" s="4" t="n">
-        <v>3684</v>
+        <v>3500</v>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H49" s="4" t="inlineStr">
@@ -3827,16 +3827,16 @@
       </c>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Private balcony/terrace</t>
         </is>
       </c>
       <c r="J49" s="4" t="n">
-        <v>811</v>
+        <v>608</v>
       </c>
       <c r="K49" s="4" t="n"/>
       <c r="L49" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat arranged on raised ground floor Attractive period building with a sought-after location; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>Stylish one bedroom, third floor apartment Beautifully proportioned open plan reception with balcony access; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M49" s="4" t="inlineStr">
@@ -3858,7 +3858,7 @@
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
@@ -3868,21 +3868,21 @@
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19500342/</t>
+          <t>https://www.onthemarket.com/details/19591709/</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>Covent Garden, West End, London, WC2E</t>
+          <t>King Street, Covent Garden WC2</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>WC2E</t>
+          <t>WC2</t>
         </is>
       </c>
       <c r="F50" s="4" t="n">
-        <v>3700</v>
+        <v>3575</v>
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
@@ -3899,11 +3899,13 @@
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J50" s="4" t="n"/>
+      <c r="J50" s="4" t="n">
+        <v>441</v>
+      </c>
       <c r="K50" s="4" t="n"/>
       <c r="L50" s="4" t="inlineStr">
         <is>
-          <t>Short Term Stay between 1-6 months Furnished Ground Floor of secure block Heart of Covent Garden; outdoor space is communal/shared; size not stated; listed furnished — check if flexible</t>
+          <t>One double bedroom One bathroom; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M50" s="4" t="inlineStr">
@@ -3935,21 +3937,21 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/9591535/</t>
+          <t>https://www.onthemarket.com/details/19591720/</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>Casson Square, Waterloo, Southbank Place, London, SE1</t>
+          <t>King Street, Covent Garden WC2</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>SE1</t>
+          <t>WC2</t>
         </is>
       </c>
       <c r="F51" s="4" t="n">
-        <v>4075</v>
+        <v>4333</v>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
@@ -3963,16 +3965,16 @@
       </c>
       <c r="I51" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J51" s="4" t="n">
-        <v>641</v>
+        <v>667</v>
       </c>
       <c r="K51" s="4" t="n"/>
       <c r="L51" s="4" t="inlineStr">
         <is>
-          <t>*video viewing available* 24-hour five-star concierge 18,000 sq ft gym, pool and spa facilities Bedroom; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>One bedroom One bathroom; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M51" s="4" t="inlineStr">
@@ -4004,21 +4006,21 @@
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/5166551/</t>
+          <t>https://www.onthemarket.com/details/19511649/</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>Grafton Way, Bloomsbury, London WC1E</t>
+          <t>Broad Court, Covent Garden, London, WC2B</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>WC1E</t>
+          <t>WC2B</t>
         </is>
       </c>
       <c r="F52" s="4" t="n">
-        <v>3142</v>
+        <v>3684</v>
       </c>
       <c r="G52" s="4" t="inlineStr">
         <is>
@@ -4032,16 +4034,16 @@
       </c>
       <c r="I52" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J52" s="4" t="n">
-        <v>592</v>
+        <v>811</v>
       </c>
       <c r="K52" s="4" t="n"/>
       <c r="L52" s="4" t="inlineStr">
         <is>
-          <t>592 sq ft floor area Nearest station 0.1mi.; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>2 bedroom flat arranged on raised ground floor Attractive period building with a sought-after location; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M52" s="4" t="inlineStr">
@@ -4063,7 +4065,7 @@
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
@@ -4073,25 +4075,25 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/10453057/</t>
+          <t>https://www.onthemarket.com/details/19500342/</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>Doughty Street, Bloomsbury, London, WC1N</t>
+          <t>Covent Garden, West End, London, WC2E</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>WC1N</t>
+          <t>WC2E</t>
         </is>
       </c>
       <c r="F53" s="4" t="n">
-        <v>3250</v>
+        <v>3700</v>
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H53" s="4" t="inlineStr">
@@ -4101,16 +4103,14 @@
       </c>
       <c r="I53" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="J53" s="4" t="n">
-        <v>787</v>
-      </c>
+          <t>Communal / shared</t>
+        </is>
+      </c>
+      <c r="J53" s="4" t="n"/>
       <c r="K53" s="4" t="n"/>
       <c r="L53" s="4" t="inlineStr">
         <is>
-          <t>Two double bedrooms Dine-in kitchen; verify balcony/terrace; listed furnished — check if flexible</t>
+          <t>Short Term Stay between 1-6 months Furnished Ground Floor of secure block Heart of Covent Garden; outdoor space is communal/shared; size not stated; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M53" s="4" t="inlineStr">
@@ -4142,21 +4142,21 @@
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/13502768/</t>
+          <t>https://www.onthemarket.com/details/9591535/</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>Bedford Court Mansions, Bloomsbury, WC1B</t>
+          <t>Casson Square, Waterloo, Southbank Place, London, SE1</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>WC1B</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F54" s="4" t="n">
-        <v>3142</v>
+        <v>4075</v>
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
@@ -4165,21 +4165,21 @@
       </c>
       <c r="H54" s="4" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Furnished</t>
         </is>
       </c>
       <c r="I54" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Private balcony/terrace</t>
         </is>
       </c>
       <c r="J54" s="4" t="n">
-        <v>587</v>
+        <v>641</v>
       </c>
       <c r="K54" s="4" t="n"/>
       <c r="L54" s="4" t="inlineStr">
         <is>
-          <t>One Bedroom Professionally Managed; verify balcony/terrace; under 650 sq ft</t>
+          <t>*video viewing available* 24-hour five-star concierge 18,000 sq ft gym, pool and spa facilities Bedroom; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M54" s="4" t="inlineStr">
@@ -4201,7 +4201,7 @@
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
@@ -4211,25 +4211,25 @@
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19815346/</t>
+          <t>https://www.onthemarket.com/details/5166551/</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>Bloomsbury, London, WC1N</t>
+          <t>Grafton Way, Bloomsbury, London WC1E</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>WC1N</t>
+          <t>WC1E</t>
         </is>
       </c>
       <c r="F55" s="4" t="n">
-        <v>3000</v>
+        <v>3142</v>
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H55" s="4" t="inlineStr">
@@ -4239,14 +4239,16 @@
       </c>
       <c r="I55" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
-        </is>
-      </c>
-      <c r="J55" s="4" t="n"/>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="J55" s="4" t="n">
+        <v>592</v>
+      </c>
       <c r="K55" s="4" t="n"/>
       <c r="L55" s="4" t="inlineStr">
         <is>
-          <t>No Agent Fees Property Reference Number: 2942192; size not stated; listed furnished — check if flexible</t>
+          <t>592 sq ft floor area Nearest station 0.1mi.; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M55" s="4" t="inlineStr">
@@ -4268,7 +4270,7 @@
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
@@ -4278,30 +4280,30 @@
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/3952850/</t>
+          <t>https://www.onthemarket.com/details/10453057/</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>Bloomsbury Square, Bloomsbury, London, WC1A</t>
+          <t>Doughty Street, Bloomsbury, London, WC1N</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>WC1A</t>
+          <t>WC1N</t>
         </is>
       </c>
       <c r="F56" s="4" t="n">
-        <v>3141</v>
+        <v>3250</v>
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H56" s="4" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Furnished</t>
         </is>
       </c>
       <c r="I56" s="4" t="inlineStr">
@@ -4310,12 +4312,12 @@
         </is>
       </c>
       <c r="J56" s="4" t="n">
-        <v>609</v>
+        <v>787</v>
       </c>
       <c r="K56" s="4" t="n"/>
       <c r="L56" s="4" t="inlineStr">
         <is>
-          <t>One Bedroom High Ceilings Views of Bloomsbury Square Wow Factor; verify balcony/terrace; under 650 sq ft</t>
+          <t>Two double bedrooms Dine-in kitchen; verify balcony/terrace; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M56" s="4" t="inlineStr">
@@ -4337,7 +4339,7 @@
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
@@ -4347,30 +4349,30 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19723779/</t>
+          <t>https://www.onthemarket.com/details/13502768/</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>Mecklenburgh Square, Bloomsbury, London, WC1N</t>
+          <t>Bedford Court Mansions, Bloomsbury, WC1B</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>WC1N</t>
+          <t>WC1B</t>
         </is>
       </c>
       <c r="F57" s="4" t="n">
-        <v>3684</v>
+        <v>3142</v>
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H57" s="4" t="inlineStr">
         <is>
-          <t>Part Furnished</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I57" s="4" t="inlineStr">
@@ -4379,12 +4381,12 @@
         </is>
       </c>
       <c r="J57" s="4" t="n">
-        <v>602</v>
+        <v>587</v>
       </c>
       <c r="K57" s="4" t="n"/>
       <c r="L57" s="4" t="inlineStr">
         <is>
-          <t>Superb 2 bedroom flat Spacious arrangement; verify balcony/terrace; under 650 sq ft</t>
+          <t>One Bedroom Professionally Managed; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M57" s="4" t="inlineStr">
@@ -4416,17 +4418,17 @@
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19715608/</t>
+          <t>https://www.onthemarket.com/details/19815346/</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>Bloomsbury Square, London WC1A</t>
+          <t>Bloomsbury, London, WC1N</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>WC1A</t>
+          <t>WC1N</t>
         </is>
       </c>
       <c r="F58" s="4" t="n">
@@ -4444,36 +4446,241 @@
       </c>
       <c r="I58" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
-        </is>
-      </c>
-      <c r="J58" s="4" t="n">
-        <v>581</v>
-      </c>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J58" s="4" t="n"/>
       <c r="K58" s="4" t="n"/>
       <c r="L58" s="4" t="inlineStr">
         <is>
+          <t>No Agent Fees Property Reference Number: 2942192; size not stated; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M58" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N58" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O58" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>1 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/3952850/</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>Bloomsbury Square, Bloomsbury, London, WC1A</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>WC1A</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="n">
+        <v>3141</v>
+      </c>
+      <c r="G59" s="4" t="inlineStr">
+        <is>
+          <t>1-Bed</t>
+        </is>
+      </c>
+      <c r="H59" s="4" t="inlineStr">
+        <is>
+          <t>Flexible</t>
+        </is>
+      </c>
+      <c r="I59" s="4" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="J59" s="4" t="n">
+        <v>609</v>
+      </c>
+      <c r="K59" s="4" t="n"/>
+      <c r="L59" s="4" t="inlineStr">
+        <is>
+          <t>One Bedroom High Ceilings Views of Bloomsbury Square Wow Factor; verify balcony/terrace; under 650 sq ft</t>
+        </is>
+      </c>
+      <c r="M59" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N59" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O59" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>2 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19723779/</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>Mecklenburgh Square, Bloomsbury, London, WC1N</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>WC1N</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="n">
+        <v>3684</v>
+      </c>
+      <c r="G60" s="4" t="inlineStr">
+        <is>
+          <t>2-Bed</t>
+        </is>
+      </c>
+      <c r="H60" s="4" t="inlineStr">
+        <is>
+          <t>Part Furnished</t>
+        </is>
+      </c>
+      <c r="I60" s="4" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="J60" s="4" t="n">
+        <v>602</v>
+      </c>
+      <c r="K60" s="4" t="n"/>
+      <c r="L60" s="4" t="inlineStr">
+        <is>
+          <t>Superb 2 bedroom flat Spacious arrangement; verify balcony/terrace; under 650 sq ft</t>
+        </is>
+      </c>
+      <c r="M60" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N60" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O60" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>1 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19715608/</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>Bloomsbury Square, London WC1A</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>WC1A</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G61" s="4" t="inlineStr">
+        <is>
+          <t>1-Bed</t>
+        </is>
+      </c>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I61" s="4" t="inlineStr">
+        <is>
+          <t>Communal / shared</t>
+        </is>
+      </c>
+      <c r="J61" s="4" t="n">
+        <v>581</v>
+      </c>
+      <c r="K61" s="4" t="n"/>
+      <c r="L61" s="4" t="inlineStr">
+        <is>
           <t>Period Building Concierge; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
-      <c r="M58" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N58" s="4" t="inlineStr">
+      <c r="M61" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N61" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="O58" s="4" t="inlineStr">
+      <c r="O61" s="4" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O58"/>
+  <autoFilter ref="A1:O61"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
@@ -4532,6 +4739,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C56" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C61" r:id="rId60"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily tracker update 2026-07-07
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Flats" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Flats'!$A$1:$O$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Flats'!$A$1:$O$69</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O68"/>
+  <dimension ref="A1:O69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -552,147 +552,147 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>2 bedroom flat to rent</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19876910/</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Newton Street, Covent Garden, London, WC2B</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>WC2B</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>4117</v>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>2-Bed</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>Communal / shared</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="n">
+        <v>848</v>
+      </c>
+      <c r="K2" s="4" t="inlineStr"/>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>Stunning 2 bedroom flat arranged on the 1st floor Generous reception room with space to dine; outdoor space is communal/shared; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M2" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N2" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O2" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07 07:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>2 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>https://www.onthemarket.com/details/19318164/</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>Princeton Street, Bloomsbury, London, WC1R</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>WC1R</t>
         </is>
       </c>
-      <c r="F2" s="6" t="n">
+      <c r="F3" s="6" t="n">
         <v>3684</v>
       </c>
-      <c r="G2" s="6" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>2-Bed</t>
         </is>
       </c>
-      <c r="H2" s="6" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>Part Furnished</t>
         </is>
       </c>
-      <c r="I2" s="6" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>Private balcony/terrace</t>
         </is>
       </c>
-      <c r="J2" s="6" t="n">
+      <c r="J3" s="6" t="n">
         <v>649</v>
       </c>
-      <c r="K2" s="6" t="n"/>
-      <c r="L2" s="6" t="inlineStr">
+      <c r="K3" s="6" t="n"/>
+      <c r="L3" s="6" t="inlineStr">
         <is>
           <t>Modern two bedroom, fourth floor flat Bright open plan reception Stylish kitchen featuring a range of modern appliances Two spacious bedrooms with built in stor; under 650 sq ft</t>
         </is>
       </c>
-      <c r="M2" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N2" s="6" t="inlineStr">
+      <c r="M3" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N3" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="O2" s="6" t="inlineStr">
+      <c r="O3" s="6" t="inlineStr">
         <is>
           <t>2026-07-06 20:39</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>1 bedroom flat to rent</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/16574229/</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Casson Square, Waterloo, London, SE1</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>SE1</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="n">
-        <v>3500</v>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>1-Bed</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>Furnished</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>Communal / shared</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="n">
-        <v>548</v>
-      </c>
-      <c r="K3" s="4" t="n"/>
-      <c r="L3" s="4" t="inlineStr">
-        <is>
-          <t>548 sq ft floor area Nearest station 0.1mi.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
-        </is>
-      </c>
-      <c r="M3" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N3" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="O3" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-06 16:39</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -702,25 +702,25 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/13719505/</t>
+          <t>https://www.onthemarket.com/details/16574229/</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Bedford Place, Bloomsbury, WC1B</t>
+          <t>Casson Square, Waterloo, London, SE1</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>WC1B</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F4" s="4" t="n">
-        <v>3878</v>
+        <v>3500</v>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
@@ -730,16 +730,16 @@
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J4" s="4" t="n">
-        <v>961</v>
+        <v>548</v>
       </c>
       <c r="K4" s="4" t="n"/>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>Two Double Bedroom Apartment High Spec; listed furnished — check if flexible</t>
+          <t>548 sq ft floor area Nearest station 0.1mi.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M4" s="4" t="inlineStr">
@@ -754,38 +754,38 @@
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06 15:39</t>
+          <t>2026-07-06 16:39</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Flat</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Rightmove</t>
+          <t>OnTheMarket</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>https://www.rightmove.co.uk/properties/88912341</t>
+          <t>https://www.onthemarket.com/details/13719505/</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Southwark Bridge Road, London, SE1</t>
+          <t>Bedford Place, Bloomsbury, WC1B</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>SE1</t>
+          <t>WC1B</t>
         </is>
       </c>
       <c r="F5" s="4" t="n">
-        <v>4500</v>
+        <v>3878</v>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
@@ -794,168 +794,168 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Furnished</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="J5" s="4" t="n"/>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>961</v>
+      </c>
       <c r="K5" s="4" t="n"/>
       <c r="L5" s="4" t="inlineStr">
         <is>
+          <t>Two Double Bedroom Apartment High Spec; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06 15:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Flat</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Rightmove</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>https://www.rightmove.co.uk/properties/88912341</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Southwark Bridge Road, London, SE1</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>SE1</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>4500</v>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>2-Bed</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Flexible</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="n"/>
+      <c r="K6" s="4" t="n"/>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
           <t>This stunning apartment boasts floor-to-ceiling windows offering breath taking panoramic views across the London skyline, flooding the space with natural light.; verify balcony/terrace; size not stated</t>
         </is>
       </c>
-      <c r="M5" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N5" s="4" t="inlineStr">
+      <c r="M6" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N6" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="O5" s="4" t="inlineStr">
+      <c r="O6" s="4" t="inlineStr">
         <is>
           <t>2026-07-06 14:39</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>2 bedroom flat to rent</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>https://www.onthemarket.com/details/1990566/</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>Endell Street, Covent Garden, London, WC2H</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>WC2H</t>
         </is>
       </c>
-      <c r="F6" s="6" t="n">
+      <c r="F7" s="6" t="n">
         <v>3400</v>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>2-Bed</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>Unfurnished</t>
         </is>
       </c>
-      <c r="I6" s="6" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr">
         <is>
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J6" s="6" t="n"/>
-      <c r="K6" s="6" t="n"/>
-      <c r="L6" s="6" t="inlineStr">
+      <c r="J7" s="6" t="n"/>
+      <c r="K7" s="6" t="n"/>
+      <c r="L7" s="6" t="inlineStr">
         <is>
           <t>Two Bedrooms Two Bathrooms Open plan living room-kitchen First floor; outdoor space is communal/shared; size not stated</t>
         </is>
       </c>
-      <c r="M6" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N6" s="6" t="inlineStr">
+      <c r="M7" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N7" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="O6" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>2 bedroom flat to rent</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/19194043/</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Great Suffolk Street, Southwark, London, SE1</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>SE1</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="n">
-        <v>3100</v>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>2-Bed</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>Furnished</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr">
-        <is>
-          <t>Juliet only</t>
-        </is>
-      </c>
-      <c r="J7" s="4" t="n">
-        <v>638</v>
-      </c>
-      <c r="K7" s="4" t="n"/>
-      <c r="L7" s="4" t="inlineStr">
-        <is>
-          <t>Stylish 2 bedroom flat set on the 5th floor Large reception room with Juliet balcony Modern kitchen 2 lovely double bedroom; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
-        </is>
-      </c>
-      <c r="M7" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N7" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="O7" s="4" t="inlineStr">
+      <c r="O7" s="6" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
@@ -964,7 +964,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -974,25 +974,25 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19099769/</t>
+          <t>https://www.onthemarket.com/details/19194043/</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Fletcher Buildings,, Covent Garden, London, WC2B</t>
+          <t>Great Suffolk Street, Southwark, London, SE1</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>WC2B</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F8" s="4" t="n">
-        <v>3792</v>
+        <v>3100</v>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -1002,16 +1002,16 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Juliet only</t>
         </is>
       </c>
       <c r="J8" s="4" t="n">
-        <v>320</v>
+        <v>638</v>
       </c>
       <c r="K8" s="4" t="n"/>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>Bright and airy one bedroom apartment in a prime Central London location Well proportioned reception with high ceilings and neutral décor Generous double bedroo; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Stylish 2 bedroom flat set on the 5th floor Large reception room with Juliet balcony Modern kitchen 2 lovely double bedroom; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M8" s="4" t="inlineStr">
@@ -1033,7 +1033,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -1043,25 +1043,25 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/6356511/</t>
+          <t>https://www.onthemarket.com/details/19099769/</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Great James Street, Bloomsbury, London, WC1N</t>
+          <t>Fletcher Buildings,, Covent Garden, London, WC2B</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>WC1N</t>
+          <t>WC2B</t>
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>3683</v>
+        <v>3792</v>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1071,16 +1071,16 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J9" s="4" t="n">
-        <v>928</v>
+        <v>320</v>
       </c>
       <c r="K9" s="4" t="n"/>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>Spacious Split Level Apartment Large Terrace Wooden Flooring Nearest tubes: Chancery Lane, Russell Square &amp; Holborn; listed furnished — check if flexible</t>
+          <t>Bright and airy one bedroom apartment in a prime Central London location Well proportioned reception with high ceilings and neutral décor Generous double bedroo; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M9" s="4" t="inlineStr">
@@ -1102,7 +1102,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -1112,25 +1112,25 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19453032/</t>
+          <t>https://www.onthemarket.com/details/6356511/</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Maiden Lane, Covent Garden, London, WC2E</t>
+          <t>Great James Street, Bloomsbury, London, WC1N</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>WC2E</t>
+          <t>WC1N</t>
         </is>
       </c>
       <c r="F10" s="4" t="n">
-        <v>3684</v>
+        <v>3683</v>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -1140,16 +1140,16 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Private balcony/terrace</t>
         </is>
       </c>
       <c r="J10" s="4" t="n">
-        <v>630</v>
+        <v>928</v>
       </c>
       <c r="K10" s="4" t="n"/>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat arranged on the 4th floor Bright and spacious reception room Smart dining room Modern kitchen; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Spacious Split Level Apartment Large Terrace Wooden Flooring Nearest tubes: Chancery Lane, Russell Square &amp; Holborn; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M10" s="4" t="inlineStr">
@@ -1181,21 +1181,21 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19592443/</t>
+          <t>https://www.onthemarket.com/details/19453032/</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Regent Square, Bloomsbury, London, WC1H</t>
+          <t>Maiden Lane, Covent Garden, London, WC2E</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>WC1H</t>
+          <t>WC2E</t>
         </is>
       </c>
       <c r="F11" s="4" t="n">
-        <v>4312</v>
+        <v>3684</v>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
@@ -1209,117 +1209,117 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J11" s="4" t="n">
-        <v>487</v>
+        <v>630</v>
       </c>
       <c r="K11" s="4" t="n"/>
       <c r="L11" s="4" t="inlineStr">
         <is>
+          <t>1 bedroom flat arranged on the 4th floor Bright and spacious reception room Smart dining room Modern kitchen; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M11" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N11" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O11" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>1 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19592443/</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Regent Square, Bloomsbury, London, WC1H</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>WC1H</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>4312</v>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>1-Bed</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>487</v>
+      </c>
+      <c r="K12" s="4" t="n"/>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
           <t>Fantastic one bedroom apartment Set within beautiful period conversion Boasts ample interior space arranged over the second floor Wonderful balcony overlooking ; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
-      <c r="M11" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N11" s="4" t="inlineStr">
+      <c r="M12" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N12" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="O11" s="4" t="inlineStr">
+      <c r="O12" s="4" t="inlineStr">
         <is>
           <t>2026-07-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Apartment</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Rightmove</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>https://www.rightmove.co.uk/properties/89143989</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Waterloo Road, Southwark, SE1</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>SE1</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="n">
-        <v>4346</v>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>2-Bed</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>Part Furnished</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>Private balcony/terrace</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="n">
-        <v>1385</v>
-      </c>
-      <c r="K12" s="2" t="n"/>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>Two bedroom apartment with incredible views Waterloo Road SE1 250 Waterloo Road is an exciting new rental development conveniently located on Waterloo Road, SE1</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="O12" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>Apartment</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>OnTheMarket</t>
+          <t>Rightmove</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/4473051/</t>
+          <t>https://www.rightmove.co.uk/properties/89143989</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1356,7 +1356,7 @@
       <c r="K13" s="2" t="n"/>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Spectacular Views Waterloo</t>
+          <t>Two bedroom apartment with incredible views Waterloo Road SE1 250 Waterloo Road is an exciting new rental development conveniently located on Waterloo Road, SE1</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
@@ -1378,7 +1378,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1388,12 +1388,12 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19728858/</t>
+          <t>https://www.onthemarket.com/details/4473051/</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Waterloo Road, London SE1</t>
+          <t>Waterloo Road, Southwark, SE1</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1402,7 +1402,7 @@
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>4350</v>
+        <v>4346</v>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
@@ -1411,7 +1411,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Part Furnished</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1420,12 +1420,12 @@
         </is>
       </c>
       <c r="J14" s="2" t="n">
-        <v>1140</v>
+        <v>1385</v>
       </c>
       <c r="K14" s="2" t="n"/>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Two Bedrooms Two Bathrooms</t>
+          <t>Spectacular Views Waterloo</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
@@ -1447,7 +1447,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1457,12 +1457,12 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/6248222/</t>
+          <t>https://www.onthemarket.com/details/19728858/</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Nelson Square, Southwark, London, SE1</t>
+          <t>Waterloo Road, London SE1</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1471,7 +1471,7 @@
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>3150</v>
+        <v>4350</v>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
@@ -1480,7 +1480,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -1489,12 +1489,12 @@
         </is>
       </c>
       <c r="J15" s="2" t="n">
-        <v>809</v>
+        <v>1140</v>
       </c>
       <c r="K15" s="2" t="n"/>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Dishwasher Range / Oven</t>
+          <t>Two Bedrooms Two Bathrooms</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
@@ -1516,7 +1516,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1526,21 +1526,21 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19663010/</t>
+          <t>https://www.onthemarket.com/details/6248222/</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Guilford Street, Bloomsbury, London, WC1N</t>
+          <t>Nelson Square, Southwark, London, SE1</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>WC1N</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>3684</v>
+        <v>3150</v>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
@@ -1549,7 +1549,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Part Furnished</t>
+          <t>Unfurnished</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1558,94 +1558,94 @@
         </is>
       </c>
       <c r="J16" s="2" t="n">
-        <v>691</v>
+        <v>809</v>
       </c>
       <c r="K16" s="2" t="n"/>
       <c r="L16" s="2" t="inlineStr">
         <is>
+          <t>Dishwasher Range / Oven</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>2 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19663010/</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Guilford Street, Bloomsbury, London, WC1N</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>WC1N</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>3684</v>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>2-Bed</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Part Furnished</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>691</v>
+      </c>
+      <c r="K17" s="2" t="n"/>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
           <t>Superb 2 bedroom flat on lower ground floor Modern open-plan kitchen with integrated appliance Spacious reception room leading to lovely private patio 2 well-pr</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="O16" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>2 bedroom apartment to rent</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/19809694/</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
-        <is>
-          <t>Shaftesbury Avenue, Soho, W1D</t>
-        </is>
-      </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>W1D</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="n">
-        <v>3553</v>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>2-Bed</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr">
-        <is>
-          <t>Flexible</t>
-        </is>
-      </c>
-      <c r="I17" s="6" t="inlineStr">
-        <is>
-          <t>Communal / shared</t>
-        </is>
-      </c>
-      <c r="J17" s="6" t="n">
-        <v>603</v>
-      </c>
-      <c r="K17" s="6" t="n"/>
-      <c r="L17" s="6" t="inlineStr">
-        <is>
-          <t>Beautifully Refurbished Secondary Glazing; outdoor space is communal/shared; under 650 sq ft</t>
-        </is>
-      </c>
-      <c r="M17" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N17" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O17" s="6" t="inlineStr">
+      <c r="O17" s="2" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
@@ -1664,12 +1664,12 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/13368018/</t>
+          <t>https://www.onthemarket.com/details/19809694/</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>Shaftesbury Avenue , Soho, W1D</t>
+          <t>Shaftesbury Avenue, Soho, W1D</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
@@ -1678,7 +1678,7 @@
         </is>
       </c>
       <c r="F18" s="6" t="n">
-        <v>3987</v>
+        <v>3553</v>
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
@@ -1696,12 +1696,12 @@
         </is>
       </c>
       <c r="J18" s="6" t="n">
-        <v>671</v>
+        <v>603</v>
       </c>
       <c r="K18" s="6" t="n"/>
       <c r="L18" s="6" t="inlineStr">
         <is>
-          <t>Pet friendly Wooden Floors Student; outdoor space is communal/shared</t>
+          <t>Beautifully Refurbished Secondary Glazing; outdoor space is communal/shared; under 650 sq ft</t>
         </is>
       </c>
       <c r="M18" s="6" t="inlineStr">
@@ -1733,12 +1733,12 @@
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19627828/</t>
+          <t>https://www.onthemarket.com/details/13368018/</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Shaftesbury Avenue, Soho, W1D</t>
+          <t>Shaftesbury Avenue , Soho, W1D</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
@@ -1765,12 +1765,12 @@
         </is>
       </c>
       <c r="J19" s="6" t="n">
-        <v>802</v>
+        <v>671</v>
       </c>
       <c r="K19" s="6" t="n"/>
       <c r="L19" s="6" t="inlineStr">
         <is>
-          <t>Built in Storage Pet Friendly; outdoor space is communal/shared</t>
+          <t>Pet friendly Wooden Floors Student; outdoor space is communal/shared</t>
         </is>
       </c>
       <c r="M19" s="6" t="inlineStr">
@@ -1792,7 +1792,7 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
@@ -1802,12 +1802,12 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19600564/</t>
+          <t>https://www.onthemarket.com/details/19627828/</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Rupert Court, Soho, W1D</t>
+          <t>Shaftesbury Avenue, Soho, W1D</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
@@ -1816,11 +1816,11 @@
         </is>
       </c>
       <c r="F20" s="6" t="n">
-        <v>3163</v>
+        <v>3987</v>
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
@@ -1833,11 +1833,13 @@
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J20" s="6" t="n"/>
+      <c r="J20" s="6" t="n">
+        <v>802</v>
+      </c>
       <c r="K20" s="6" t="n"/>
       <c r="L20" s="6" t="inlineStr">
         <is>
-          <t>Beautifully Refurbished Pet friendly; outdoor space is communal/shared; size not stated</t>
+          <t>Built in Storage Pet Friendly; outdoor space is communal/shared</t>
         </is>
       </c>
       <c r="M20" s="6" t="inlineStr">
@@ -1869,17 +1871,17 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/10862827/</t>
+          <t>https://www.onthemarket.com/details/19600564/</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Rupert Court, Soho W1</t>
+          <t>Rupert Court, Soho, W1D</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>W1D</t>
         </is>
       </c>
       <c r="F21" s="6" t="n">
@@ -1892,7 +1894,7 @@
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr">
@@ -1900,13 +1902,11 @@
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J21" s="6" t="n">
-        <v>603</v>
-      </c>
+      <c r="J21" s="6" t="n"/>
       <c r="K21" s="6" t="n"/>
       <c r="L21" s="6" t="inlineStr">
         <is>
-          <t>One bedroom One shower room; outdoor space is communal/shared; under 650 sq ft</t>
+          <t>Beautifully Refurbished Pet friendly; outdoor space is communal/shared; size not stated</t>
         </is>
       </c>
       <c r="M21" s="6" t="inlineStr">
@@ -1928,7 +1928,7 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1938,21 +1938,21 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19845642/</t>
+          <t>https://www.onthemarket.com/details/10862827/</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>Shelton Street, Covent Garden, London, WC2H</t>
+          <t>Rupert Court, Soho W1</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>WC2H</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="F22" s="6" t="n">
-        <v>3142</v>
+        <v>3163</v>
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
@@ -1961,7 +1961,7 @@
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Unfurnished</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr">
@@ -1970,12 +1970,12 @@
         </is>
       </c>
       <c r="J22" s="6" t="n">
-        <v>480</v>
+        <v>603</v>
       </c>
       <c r="K22" s="6" t="n"/>
       <c r="L22" s="6" t="inlineStr">
         <is>
-          <t>Superb one bedroom flat arranged on the second floor Spacious reception/kitchen with ample dining space; outdoor space is communal/shared; under 650 sq ft</t>
+          <t>One bedroom One shower room; outdoor space is communal/shared; under 650 sq ft</t>
         </is>
       </c>
       <c r="M22" s="6" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
@@ -2007,21 +2007,21 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19603496/</t>
+          <t>https://www.onthemarket.com/details/19845642/</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Arne Street, Covent Garden, WC2E</t>
+          <t>Shelton Street, Covent Garden, London, WC2H</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>WC2E</t>
+          <t>WC2H</t>
         </is>
       </c>
       <c r="F23" s="6" t="n">
-        <v>3250</v>
+        <v>3142</v>
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr">
@@ -2039,12 +2039,12 @@
         </is>
       </c>
       <c r="J23" s="6" t="n">
-        <v>514</v>
+        <v>480</v>
       </c>
       <c r="K23" s="6" t="n"/>
       <c r="L23" s="6" t="inlineStr">
         <is>
-          <t>Council Tax Band G 514 sq ft floor area; outdoor space is communal/shared; under 650 sq ft</t>
+          <t>Superb one bedroom flat arranged on the second floor Spacious reception/kitchen with ample dining space; outdoor space is communal/shared; under 650 sq ft</t>
         </is>
       </c>
       <c r="M23" s="6" t="inlineStr">
@@ -2066,7 +2066,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -2076,21 +2076,21 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/14179323/</t>
+          <t>https://www.onthemarket.com/details/19603496/</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>Bloomsbury Square, Bloomsbury, Covent Garden, London, WC1A</t>
+          <t>Arne Street, Covent Garden, WC2E</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>WC1A</t>
+          <t>WC2E</t>
         </is>
       </c>
       <c r="F24" s="6" t="n">
-        <v>3500</v>
+        <v>3250</v>
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
@@ -2099,7 +2099,7 @@
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>Part Furnished</t>
+          <t>Unfurnished</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr">
@@ -2108,12 +2108,12 @@
         </is>
       </c>
       <c r="J24" s="6" t="n">
-        <v>734</v>
+        <v>514</v>
       </c>
       <c r="K24" s="6" t="n"/>
       <c r="L24" s="6" t="inlineStr">
         <is>
-          <t>Stunning Period Conversion Hardwood Flooring Multi-Room Sound System and Mood Lighting Throughout Contemporary Kitchen &amp; Bathroom; outdoor space is communal/shared</t>
+          <t>Council Tax Band G 514 sq ft floor area; outdoor space is communal/shared; under 650 sq ft</t>
         </is>
       </c>
       <c r="M24" s="6" t="inlineStr">
@@ -2145,21 +2145,21 @@
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19823664/</t>
+          <t>https://www.onthemarket.com/details/14179323/</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Bedford Court Mansions, Adeline Place, Bloomsbury, London, WC1B</t>
+          <t>Bloomsbury Square, Bloomsbury, Covent Garden, London, WC1A</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>WC1B</t>
+          <t>WC1A</t>
         </is>
       </c>
       <c r="F25" s="6" t="n">
-        <v>3141</v>
+        <v>3500</v>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
@@ -2168,21 +2168,21 @@
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Part Furnished</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J25" s="6" t="n">
-        <v>573</v>
+        <v>734</v>
       </c>
       <c r="K25" s="6" t="n"/>
       <c r="L25" s="6" t="inlineStr">
         <is>
-          <t>One Bedroom Finished to high standard Lift Access Separate Kitchen; under 650 sq ft</t>
+          <t>Stunning Period Conversion Hardwood Flooring Multi-Room Sound System and Mood Lighting Throughout Contemporary Kitchen &amp; Bathroom; outdoor space is communal/shared</t>
         </is>
       </c>
       <c r="M25" s="6" t="inlineStr">
@@ -2204,7 +2204,7 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -2214,21 +2214,21 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/15813612/</t>
+          <t>https://www.onthemarket.com/details/19823664/</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>Bloomsbury Square, Bloomsbury, WC1A</t>
+          <t>Bedford Court Mansions, Adeline Place, Bloomsbury, London, WC1B</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>WC1A</t>
+          <t>WC1B</t>
         </is>
       </c>
       <c r="F26" s="6" t="n">
-        <v>3142</v>
+        <v>3141</v>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
@@ -2246,12 +2246,12 @@
         </is>
       </c>
       <c r="J26" s="6" t="n">
-        <v>539</v>
+        <v>573</v>
       </c>
       <c r="K26" s="6" t="n"/>
       <c r="L26" s="6" t="inlineStr">
         <is>
-          <t>Large Double Bedroom Period Features Student; under 650 sq ft</t>
+          <t>One Bedroom Finished to high standard Lift Access Separate Kitchen; under 650 sq ft</t>
         </is>
       </c>
       <c r="M26" s="6" t="inlineStr">
@@ -2273,7 +2273,7 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
@@ -2283,17 +2283,17 @@
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19736445/</t>
+          <t>https://www.onthemarket.com/details/15813612/</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>Millman Street, Bloomsbury, London, WC1N</t>
+          <t>Bloomsbury Square, Bloomsbury, WC1A</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>WC1N</t>
+          <t>WC1A</t>
         </is>
       </c>
       <c r="F27" s="6" t="n">
@@ -2306,7 +2306,7 @@
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>Part Furnished</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
@@ -2315,94 +2315,94 @@
         </is>
       </c>
       <c r="J27" s="6" t="n">
-        <v>542</v>
+        <v>539</v>
       </c>
       <c r="K27" s="6" t="n"/>
       <c r="L27" s="6" t="inlineStr">
         <is>
+          <t>Large Double Bedroom Period Features Student; under 650 sq ft</t>
+        </is>
+      </c>
+      <c r="M27" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N27" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O27" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>1 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19736445/</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>Millman Street, Bloomsbury, London, WC1N</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>WC1N</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>3142</v>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>1-Bed</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>Part Furnished</t>
+        </is>
+      </c>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J28" s="6" t="n">
+        <v>542</v>
+      </c>
+      <c r="K28" s="6" t="n"/>
+      <c r="L28" s="6" t="inlineStr">
+        <is>
           <t>Fantastic 1 bedroom flat arranged on the ground floor Set within a lovely residential block; under 650 sq ft</t>
         </is>
       </c>
-      <c r="M27" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N27" s="6" t="inlineStr">
+      <c r="M28" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N28" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="O27" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>Flat</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>Rightmove</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>https://www.rightmove.co.uk/properties/90435384</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>251 SOUTHWARK BRIDGE ROAD, LONDON, SE1, Elephant and Castle, London, SE1</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>SE1</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="n">
-        <v>4250</v>
-      </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>1-Bed</t>
-        </is>
-      </c>
-      <c r="H28" s="4" t="inlineStr">
-        <is>
-          <t>Part Furnished</t>
-        </is>
-      </c>
-      <c r="I28" s="4" t="inlineStr">
-        <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="J28" s="4" t="n">
-        <v>520</v>
-      </c>
-      <c r="K28" s="4" t="n"/>
-      <c r="L28" s="4" t="inlineStr">
-        <is>
-          <t>ZERO DEPOSIT AVAILABLE. SHORT LET. Set on the 21st floor, this 1 bedroom flat boasts well arranged interiors including a large reception room, a modern open-pla; verify balcony/terrace; under 650 sq ft</t>
-        </is>
-      </c>
-      <c r="M28" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N28" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="O28" s="4" t="inlineStr">
+      <c r="O28" s="6" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
@@ -2421,7 +2421,7 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>https://www.rightmove.co.uk/properties/90432648</t>
+          <t>https://www.rightmove.co.uk/properties/90435384</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -2435,7 +2435,7 @@
         </is>
       </c>
       <c r="F29" s="4" t="n">
-        <v>3000</v>
+        <v>4250</v>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
@@ -2458,7 +2458,7 @@
       <c r="K29" s="4" t="n"/>
       <c r="L29" s="4" t="inlineStr">
         <is>
-          <t>ZERO DEPOSIT AVAILABLE. LONG LET. Set on the 21st floor, this 1 bedroom flat boasts well arranged interiors including a large reception room, a modern open-plan; verify balcony/terrace; under 650 sq ft</t>
+          <t>ZERO DEPOSIT AVAILABLE. SHORT LET. Set on the 21st floor, this 1 bedroom flat boasts well arranged interiors including a large reception room, a modern open-pla; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M29" s="4" t="inlineStr">
@@ -2480,31 +2480,31 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>Flat</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>OnTheMarket</t>
+          <t>Rightmove</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/4220060/</t>
+          <t>https://www.rightmove.co.uk/properties/90432648</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Carnaby Street, Soho, W1F</t>
+          <t>251 SOUTHWARK BRIDGE ROAD, LONDON, SE1, Elephant and Castle, London, SE1</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>W1F</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F30" s="4" t="n">
-        <v>3640</v>
+        <v>3000</v>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Part Furnished</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
@@ -2522,12 +2522,12 @@
         </is>
       </c>
       <c r="J30" s="4" t="n">
-        <v>553</v>
+        <v>520</v>
       </c>
       <c r="K30" s="4" t="n"/>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>One bedroom apartment Newly refurbished; verify balcony/terrace; under 650 sq ft</t>
+          <t>ZERO DEPOSIT AVAILABLE. LONG LET. Set on the 21st floor, this 1 bedroom flat boasts well arranged interiors including a large reception room, a modern open-plan; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
@@ -2549,7 +2549,7 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
@@ -2559,12 +2559,12 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/8022324/</t>
+          <t>https://www.onthemarket.com/details/4220060/</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Golden Square, Soho, London, W1F</t>
+          <t>Carnaby Street, Soho, W1F</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
@@ -2573,7 +2573,7 @@
         </is>
       </c>
       <c r="F31" s="4" t="n">
-        <v>3467</v>
+        <v>3640</v>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
@@ -2582,7 +2582,7 @@
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>Furnished</t>
+          <t>Unfurnished</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
@@ -2591,12 +2591,12 @@
         </is>
       </c>
       <c r="J31" s="4" t="n">
-        <v>608</v>
+        <v>553</v>
       </c>
       <c r="K31" s="4" t="n"/>
       <c r="L31" s="4" t="inlineStr">
         <is>
-          <t>608 sq ft floor area Nearest station 0.1mi.; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>One bedroom apartment Newly refurbished; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M31" s="4" t="inlineStr">
@@ -2618,7 +2618,7 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -2628,25 +2628,25 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19852978/</t>
+          <t>https://www.onthemarket.com/details/8022324/</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Newport Court, Covent Garden, London, WC2H</t>
+          <t>Golden Square, Soho, London, W1F</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>WC2H</t>
+          <t>W1F</t>
         </is>
       </c>
       <c r="F32" s="4" t="n">
-        <v>4334</v>
+        <v>3467</v>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
@@ -2656,16 +2656,16 @@
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J32" s="4" t="n">
-        <v>858</v>
+        <v>608</v>
       </c>
       <c r="K32" s="4" t="n"/>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Splendid two bedroom flat Ample interiors; listed furnished — check if flexible</t>
+          <t>608 sq ft floor area Nearest station 0.1mi.; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
@@ -2697,21 +2697,21 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/16157050/</t>
+          <t>https://www.onthemarket.com/details/19852978/</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Brewer Street, Soho, W1F</t>
+          <t>Newport Court, Covent Garden, London, WC2H</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>W1F</t>
+          <t>WC2H</t>
         </is>
       </c>
       <c r="F33" s="4" t="n">
-        <v>3142</v>
+        <v>4334</v>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
@@ -2725,16 +2725,16 @@
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Private balcony/terrace</t>
         </is>
       </c>
       <c r="J33" s="4" t="n">
-        <v>730</v>
+        <v>858</v>
       </c>
       <c r="K33" s="4" t="n"/>
       <c r="L33" s="4" t="inlineStr">
         <is>
-          <t>730 sqft Secure Entrance; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>Splendid two bedroom flat Ample interiors; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M33" s="4" t="inlineStr">
@@ -2756,7 +2756,7 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -2766,25 +2766,25 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/9956499/</t>
+          <t>https://www.onthemarket.com/details/16157050/</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Richmond Buildings, Soho, W1D</t>
+          <t>Brewer Street, Soho, W1F</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>W1D</t>
+          <t>W1F</t>
         </is>
       </c>
       <c r="F34" s="4" t="n">
-        <v>3835</v>
+        <v>3142</v>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
@@ -2794,16 +2794,16 @@
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J34" s="4" t="n">
-        <v>521</v>
+        <v>730</v>
       </c>
       <c r="K34" s="4" t="n"/>
       <c r="L34" s="4" t="inlineStr">
         <is>
-          <t>Council tax band: F 521 sq ft floor area; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>730 sqft Secure Entrance; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M34" s="4" t="inlineStr">
@@ -2825,7 +2825,7 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
@@ -2835,12 +2835,12 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19786051/</t>
+          <t>https://www.onthemarket.com/details/9956499/</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Old Compton Street, Soho, London, W1D</t>
+          <t>Richmond Buildings, Soho, W1D</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
@@ -2849,7 +2849,7 @@
         </is>
       </c>
       <c r="F35" s="4" t="n">
-        <v>3600</v>
+        <v>3835</v>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
@@ -2863,16 +2863,16 @@
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J35" s="4" t="n">
-        <v>432</v>
+        <v>521</v>
       </c>
       <c r="K35" s="4" t="n"/>
       <c r="L35" s="4" t="inlineStr">
         <is>
-          <t>432 sq ft floor area Nearest station 0.1mi. Furnished Nearest school 0.2mi.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Council tax band: F 521 sq ft floor area; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M35" s="4" t="inlineStr">
@@ -2894,7 +2894,7 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -2904,17 +2904,17 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19828226/</t>
+          <t>https://www.onthemarket.com/details/19786051/</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>TCRW SOHO, Fareham Street, W1F</t>
+          <t>Old Compton Street, Soho, London, W1D</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>W1F</t>
+          <t>W1D</t>
         </is>
       </c>
       <c r="F36" s="4" t="n">
@@ -2932,16 +2932,16 @@
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J36" s="4" t="n">
-        <v>656</v>
+        <v>432</v>
       </c>
       <c r="K36" s="4" t="n"/>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Concierge service Highly sought-after Zone 1 location; verify balcony/terrace; listed furnished — check if flexible</t>
+          <t>432 sq ft floor area Nearest station 0.1mi. Furnished Nearest school 0.2mi.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
@@ -2963,7 +2963,7 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
@@ -2973,25 +2973,25 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/11345150/</t>
+          <t>https://www.onthemarket.com/details/19828226/</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Shaftesbury Avenue, Covent Garden, London, WC2H</t>
+          <t>TCRW SOHO, Fareham Street, W1F</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>WC2H</t>
+          <t>W1F</t>
         </is>
       </c>
       <c r="F37" s="4" t="n">
-        <v>3575</v>
+        <v>3600</v>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
@@ -3001,16 +3001,16 @@
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J37" s="4" t="n">
-        <v>870</v>
+        <v>656</v>
       </c>
       <c r="K37" s="4" t="n"/>
       <c r="L37" s="4" t="inlineStr">
         <is>
-          <t>870 sq ft floor area Nearest station 0.1mi.; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>Concierge service Highly sought-after Zone 1 location; verify balcony/terrace; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M37" s="4" t="inlineStr">
@@ -3042,21 +3042,21 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/4747672/</t>
+          <t>https://www.onthemarket.com/details/11345150/</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Townsend House, Deans Street, Soho W1D</t>
+          <t>Shaftesbury Avenue, Covent Garden, London, WC2H</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>W1D</t>
+          <t>WC2H</t>
         </is>
       </c>
       <c r="F38" s="4" t="n">
-        <v>3850</v>
+        <v>3575</v>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
@@ -3070,14 +3070,16 @@
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="J38" s="4" t="n"/>
+          <t>Communal / shared</t>
+        </is>
+      </c>
+      <c r="J38" s="4" t="n">
+        <v>870</v>
+      </c>
       <c r="K38" s="4" t="n"/>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>Close to Local Shops Close to Public Transport; verify balcony/terrace; size not stated; listed furnished — check if flexible</t>
+          <t>870 sq ft floor area Nearest station 0.1mi.; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
@@ -3099,7 +3101,7 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
@@ -3109,30 +3111,30 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19628367/</t>
+          <t>https://www.onthemarket.com/details/4747672/</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Carnaby Street, Soho W1</t>
+          <t>Townsend House, Deans Street, Soho W1D</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>W1D</t>
         </is>
       </c>
       <c r="F39" s="4" t="n">
-        <v>3640</v>
+        <v>3850</v>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Furnished</t>
         </is>
       </c>
       <c r="I39" s="4" t="inlineStr">
@@ -3140,13 +3142,11 @@
           <t>Not stated</t>
         </is>
       </c>
-      <c r="J39" s="4" t="n">
-        <v>549</v>
-      </c>
+      <c r="J39" s="4" t="n"/>
       <c r="K39" s="4" t="n"/>
       <c r="L39" s="4" t="inlineStr">
         <is>
-          <t>One bedroom One shower room, ensuite; verify balcony/terrace; under 650 sq ft</t>
+          <t>Close to Local Shops Close to Public Transport; verify balcony/terrace; size not stated; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M39" s="4" t="inlineStr">
@@ -3178,17 +3178,17 @@
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/13524814/</t>
+          <t>https://www.onthemarket.com/details/19628367/</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Carnaby Street, Soho, W1F</t>
+          <t>Carnaby Street, Soho W1</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>W1F</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="F40" s="4" t="n">
@@ -3201,7 +3201,7 @@
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Unfurnished</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr">
@@ -3210,12 +3210,12 @@
         </is>
       </c>
       <c r="J40" s="4" t="n">
-        <v>552</v>
+        <v>549</v>
       </c>
       <c r="K40" s="4" t="n"/>
       <c r="L40" s="4" t="inlineStr">
         <is>
-          <t>Recently Refurbished Apartment Original Features Student; verify balcony/terrace; under 650 sq ft</t>
+          <t>One bedroom One shower room, ensuite; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M40" s="4" t="inlineStr">
@@ -3247,21 +3247,21 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/18690047/</t>
+          <t>https://www.onthemarket.com/details/13524814/</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Duck Lane, Soho W1</t>
+          <t>Carnaby Street, Soho, W1F</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>W1F</t>
         </is>
       </c>
       <c r="F41" s="4" t="n">
-        <v>3077</v>
+        <v>3640</v>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
@@ -3270,7 +3270,7 @@
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr">
@@ -3279,12 +3279,12 @@
         </is>
       </c>
       <c r="J41" s="4" t="n">
-        <v>581</v>
+        <v>552</v>
       </c>
       <c r="K41" s="4" t="n"/>
       <c r="L41" s="4" t="inlineStr">
         <is>
-          <t>One bedroom One bathroom; verify balcony/terrace; under 650 sq ft</t>
+          <t>Recently Refurbished Apartment Original Features Student; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M41" s="4" t="inlineStr">
@@ -3316,17 +3316,17 @@
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/18690128/</t>
+          <t>https://www.onthemarket.com/details/18690047/</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Duck Lane, Soho, W1F</t>
+          <t>Duck Lane, Soho W1</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>W1F</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="F42" s="4" t="n">
@@ -3348,12 +3348,12 @@
         </is>
       </c>
       <c r="J42" s="4" t="n">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="K42" s="4" t="n"/>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>One Double bedroom Quaint Road; verify balcony/terrace; under 650 sq ft</t>
+          <t>One bedroom One bathroom; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
@@ -3385,12 +3385,12 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/18680649/</t>
+          <t>https://www.onthemarket.com/details/18690128/</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Duck Lane, Soho W1F</t>
+          <t>Duck Lane, Soho, W1F</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Unfurnished</t>
         </is>
       </c>
       <c r="I43" s="4" t="inlineStr">
@@ -3417,12 +3417,12 @@
         </is>
       </c>
       <c r="J43" s="4" t="n">
-        <v>575</v>
+        <v>580</v>
       </c>
       <c r="K43" s="4" t="n"/>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Modern Throughout Wooden Flooring Throughout; verify balcony/terrace; under 650 sq ft</t>
+          <t>One Double bedroom Quaint Road; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
@@ -3454,21 +3454,21 @@
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/15707269/</t>
+          <t>https://www.onthemarket.com/details/18680649/</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Casson Square, London, Waterloo, United Kingdom, SE1</t>
+          <t>Duck Lane, Soho W1F</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>SE1</t>
+          <t>W1F</t>
         </is>
       </c>
       <c r="F44" s="4" t="n">
-        <v>4050</v>
+        <v>3077</v>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
@@ -3477,21 +3477,21 @@
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>Furnished</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J44" s="4" t="n">
-        <v>514</v>
+        <v>575</v>
       </c>
       <c r="K44" s="4" t="n"/>
       <c r="L44" s="4" t="inlineStr">
         <is>
-          <t>Bedroom Bathroom Open-plan reception/kitchen 24 hour concierge; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Modern Throughout Wooden Flooring Throughout; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M44" s="4" t="inlineStr">
@@ -3523,12 +3523,12 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/9568931/</t>
+          <t>https://www.onthemarket.com/details/15707269/</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Casson Square, Waterloo, Southbank Place, London, SE1</t>
+          <t>Casson Square, London, Waterloo, United Kingdom, SE1</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
@@ -3537,7 +3537,7 @@
         </is>
       </c>
       <c r="F45" s="4" t="n">
-        <v>4250</v>
+        <v>4050</v>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
@@ -3551,16 +3551,16 @@
       </c>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J45" s="4" t="n">
-        <v>644</v>
+        <v>514</v>
       </c>
       <c r="K45" s="4" t="n"/>
       <c r="L45" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom 1 bathroom Open-plan reception kitchen 24-hour five-star concierge; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Bedroom Bathroom Open-plan reception/kitchen 24 hour concierge; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M45" s="4" t="inlineStr">
@@ -3582,7 +3582,7 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom end of terrace house to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
@@ -3592,21 +3592,25 @@
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19811489/</t>
+          <t>https://www.onthemarket.com/details/9568931/</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Carlisle Lane, Waterloo</t>
-        </is>
-      </c>
-      <c r="E46" s="4" t="n"/>
+          <t>Casson Square, Waterloo, Southbank Place, London, SE1</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>SE1</t>
+        </is>
+      </c>
       <c r="F46" s="4" t="n">
-        <v>3575</v>
+        <v>4250</v>
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr">
@@ -3620,12 +3624,12 @@
         </is>
       </c>
       <c r="J46" s="4" t="n">
-        <v>904</v>
+        <v>644</v>
       </c>
       <c r="K46" s="4" t="n"/>
       <c r="L46" s="4" t="inlineStr">
         <is>
-          <t>End of Terrace Shared Garden; listed furnished — check if flexible</t>
+          <t>1 bedroom 1 bathroom Open-plan reception kitchen 24-hour five-star concierge; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M46" s="4" t="inlineStr">
@@ -3647,7 +3651,7 @@
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>2 bedroom end of terrace house to rent</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
@@ -3657,21 +3661,17 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/7516361/</t>
+          <t>https://www.onthemarket.com/details/19811489/</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Belvedere Road, Waterloo, London, SE1</t>
-        </is>
-      </c>
-      <c r="E47" s="4" t="inlineStr">
-        <is>
-          <t>SE1</t>
-        </is>
-      </c>
+          <t>Carlisle Lane, Waterloo</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="n"/>
       <c r="F47" s="4" t="n">
-        <v>3350</v>
+        <v>3575</v>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
@@ -3685,16 +3685,16 @@
       </c>
       <c r="I47" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Private balcony/terrace</t>
         </is>
       </c>
       <c r="J47" s="4" t="n">
-        <v>544</v>
+        <v>904</v>
       </c>
       <c r="K47" s="4" t="n"/>
       <c r="L47" s="4" t="inlineStr">
         <is>
-          <t>Residents' swimming pool and gym. Grade II listed period building. 24 hour porters. Set close to the iconic Southbank and London Eye.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>End of Terrace Shared Garden; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M47" s="4" t="inlineStr">
@@ -3716,7 +3716,7 @@
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
@@ -3726,12 +3726,12 @@
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/7589011/</t>
+          <t>https://www.onthemarket.com/details/7516361/</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Belvedere Road, London, Waterloo, SE1</t>
+          <t>Belvedere Road, Waterloo, London, SE1</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
@@ -3740,11 +3740,11 @@
         </is>
       </c>
       <c r="F48" s="4" t="n">
-        <v>4200</v>
+        <v>3350</v>
       </c>
       <c r="G48" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H48" s="4" t="inlineStr">
@@ -3758,12 +3758,12 @@
         </is>
       </c>
       <c r="J48" s="4" t="n">
-        <v>671</v>
+        <v>544</v>
       </c>
       <c r="K48" s="4" t="n"/>
       <c r="L48" s="4" t="inlineStr">
         <is>
-          <t>24-hour five-star concierge 18,000 sq ft gym and spa facilities Set in one of London's most connected locations, opposite Westminster and the Houses of Parliame; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>Residents' swimming pool and gym. Grade II listed period building. 24 hour porters. Set close to the iconic Southbank and London Eye.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M48" s="4" t="inlineStr">
@@ -3785,7 +3785,7 @@
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
@@ -3795,12 +3795,12 @@
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/17616661/</t>
+          <t>https://www.onthemarket.com/details/7589011/</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>The Music Box, 237 Union Street, Southwark, London, SE1</t>
+          <t>Belvedere Road, London, Waterloo, SE1</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
@@ -3809,11 +3809,11 @@
         </is>
       </c>
       <c r="F49" s="4" t="n">
-        <v>3800</v>
+        <v>4200</v>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H49" s="4" t="inlineStr">
@@ -3823,16 +3823,16 @@
       </c>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J49" s="4" t="n">
-        <v>841</v>
+        <v>671</v>
       </c>
       <c r="K49" s="4" t="n"/>
       <c r="L49" s="4" t="inlineStr">
         <is>
-          <t>Two bedrooms Two bathrooms 841 sq. ft. Excellent transport links; verify balcony/terrace; listed furnished — check if flexible</t>
+          <t>24-hour five-star concierge 18,000 sq ft gym and spa facilities Set in one of London's most connected locations, opposite Westminster and the Houses of Parliame; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M49" s="4" t="inlineStr">
@@ -3854,7 +3854,7 @@
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
@@ -3864,25 +3864,25 @@
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19863550/</t>
+          <t>https://www.onthemarket.com/details/17616661/</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>King Street, Covent Garden, London, WC2E</t>
+          <t>The Music Box, 237 Union Street, Southwark, London, SE1</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>WC2E</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F50" s="4" t="n">
-        <v>3358</v>
+        <v>3800</v>
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H50" s="4" t="inlineStr">
@@ -3892,16 +3892,16 @@
       </c>
       <c r="I50" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J50" s="4" t="n">
-        <v>455</v>
+        <v>841</v>
       </c>
       <c r="K50" s="4" t="n"/>
       <c r="L50" s="4" t="inlineStr">
         <is>
-          <t>Iconic Covent Garden location Finished to an excellent standard throughout High ceilings Wooden flooring throughout; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Two bedrooms Two bathrooms 841 sq. ft. Excellent transport links; verify balcony/terrace; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M50" s="4" t="inlineStr">
@@ -3923,7 +3923,7 @@
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
@@ -3933,21 +3933,21 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19860280/</t>
+          <t>https://www.onthemarket.com/details/19863550/</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>Floral Street, Covent Garden WC2</t>
+          <t>King Street, Covent Garden, London, WC2E</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>WC2</t>
+          <t>WC2E</t>
         </is>
       </c>
       <c r="F51" s="4" t="n">
-        <v>3380</v>
+        <v>3358</v>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
@@ -3965,12 +3965,12 @@
         </is>
       </c>
       <c r="J51" s="4" t="n">
-        <v>495</v>
+        <v>455</v>
       </c>
       <c r="K51" s="4" t="n"/>
       <c r="L51" s="4" t="inlineStr">
         <is>
-          <t>One bedroom One bathroom, ensuite; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Iconic Covent Garden location Finished to an excellent standard throughout High ceilings Wooden flooring throughout; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M51" s="4" t="inlineStr">
@@ -4002,21 +4002,21 @@
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/1837052/</t>
+          <t>https://www.onthemarket.com/details/19860280/</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>King Street, Covent Garden, WC2E</t>
+          <t>Floral Street, Covent Garden WC2</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>WC2E</t>
+          <t>WC2</t>
         </is>
       </c>
       <c r="F52" s="4" t="n">
-        <v>3358</v>
+        <v>3380</v>
       </c>
       <c r="G52" s="4" t="inlineStr">
         <is>
@@ -4034,12 +4034,12 @@
         </is>
       </c>
       <c r="J52" s="4" t="n">
-        <v>455</v>
+        <v>495</v>
       </c>
       <c r="K52" s="4" t="n"/>
       <c r="L52" s="4" t="inlineStr">
         <is>
-          <t>Furnished Recently refurbished; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>One bedroom One bathroom, ensuite; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M52" s="4" t="inlineStr">
@@ -4071,12 +4071,12 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/3408032/</t>
+          <t>https://www.onthemarket.com/details/1837052/</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>Floral Street, Covent Garden, WC2E</t>
+          <t>King Street, Covent Garden, WC2E</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
@@ -4085,7 +4085,7 @@
         </is>
       </c>
       <c r="F53" s="4" t="n">
-        <v>3380</v>
+        <v>3358</v>
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
@@ -4103,12 +4103,12 @@
         </is>
       </c>
       <c r="J53" s="4" t="n">
-        <v>398</v>
+        <v>455</v>
       </c>
       <c r="K53" s="4" t="n"/>
       <c r="L53" s="4" t="inlineStr">
         <is>
-          <t>Newly Refurbished Central Location; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Furnished Recently refurbished; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M53" s="4" t="inlineStr">
@@ -4130,7 +4130,7 @@
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
@@ -4140,25 +4140,25 @@
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/3102769/</t>
+          <t>https://www.onthemarket.com/details/3408032/</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>John Adam Street, Covent Garden, WC2N</t>
+          <t>Floral Street, Covent Garden, WC2E</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>WC2N</t>
+          <t>WC2E</t>
         </is>
       </c>
       <c r="F54" s="4" t="n">
-        <v>3185</v>
+        <v>3380</v>
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H54" s="4" t="inlineStr">
@@ -4172,12 +4172,12 @@
         </is>
       </c>
       <c r="J54" s="4" t="n">
-        <v>655</v>
+        <v>398</v>
       </c>
       <c r="K54" s="4" t="n"/>
       <c r="L54" s="4" t="inlineStr">
         <is>
-          <t>Concierge Close to the area's Universities for students and academics; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>Newly Refurbished Central Location; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M54" s="4" t="inlineStr">
@@ -4199,7 +4199,7 @@
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
@@ -4209,25 +4209,25 @@
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19733694/</t>
+          <t>https://www.onthemarket.com/details/3102769/</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>Maiden Lane, Covent Garden, London, WC2E</t>
+          <t>John Adam Street, Covent Garden, WC2N</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>WC2E</t>
+          <t>WC2N</t>
         </is>
       </c>
       <c r="F55" s="4" t="n">
-        <v>3684</v>
+        <v>3185</v>
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H55" s="4" t="inlineStr">
@@ -4241,12 +4241,12 @@
         </is>
       </c>
       <c r="J55" s="4" t="n">
-        <v>630</v>
+        <v>655</v>
       </c>
       <c r="K55" s="4" t="n"/>
       <c r="L55" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat arranged on the 4th floor Bright and spacious reception room; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Concierge Close to the area's Universities for students and academics; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M55" s="4" t="inlineStr">
@@ -4278,21 +4278,21 @@
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19725776/</t>
+          <t>https://www.onthemarket.com/details/19733694/</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>Shelton Street, Covent Garden, London, WC2H</t>
+          <t>Maiden Lane, Covent Garden, London, WC2E</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>WC2H</t>
+          <t>WC2E</t>
         </is>
       </c>
       <c r="F56" s="4" t="n">
-        <v>3500</v>
+        <v>3684</v>
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
@@ -4306,16 +4306,16 @@
       </c>
       <c r="I56" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J56" s="4" t="n">
-        <v>608</v>
+        <v>630</v>
       </c>
       <c r="K56" s="4" t="n"/>
       <c r="L56" s="4" t="inlineStr">
         <is>
-          <t>Stylish one bedroom, third floor apartment Beautifully proportioned open plan reception with balcony access; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>1 bedroom flat arranged on the 4th floor Bright and spacious reception room; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M56" s="4" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
@@ -4347,21 +4347,21 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19591709/</t>
+          <t>https://www.onthemarket.com/details/19725776/</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>King Street, Covent Garden WC2</t>
+          <t>Shelton Street, Covent Garden, London, WC2H</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>WC2</t>
+          <t>WC2H</t>
         </is>
       </c>
       <c r="F57" s="4" t="n">
-        <v>3575</v>
+        <v>3500</v>
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
@@ -4375,16 +4375,16 @@
       </c>
       <c r="I57" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Private balcony/terrace</t>
         </is>
       </c>
       <c r="J57" s="4" t="n">
-        <v>441</v>
+        <v>608</v>
       </c>
       <c r="K57" s="4" t="n"/>
       <c r="L57" s="4" t="inlineStr">
         <is>
-          <t>One double bedroom One bathroom; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Stylish one bedroom, third floor apartment Beautifully proportioned open plan reception with balcony access; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M57" s="4" t="inlineStr">
@@ -4416,7 +4416,7 @@
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19591720/</t>
+          <t>https://www.onthemarket.com/details/19591709/</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
@@ -4430,7 +4430,7 @@
         </is>
       </c>
       <c r="F58" s="4" t="n">
-        <v>4333</v>
+        <v>3575</v>
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
@@ -4448,12 +4448,12 @@
         </is>
       </c>
       <c r="J58" s="4" t="n">
-        <v>667</v>
+        <v>441</v>
       </c>
       <c r="K58" s="4" t="n"/>
       <c r="L58" s="4" t="inlineStr">
         <is>
-          <t>One bedroom One bathroom; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>One double bedroom One bathroom; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M58" s="4" t="inlineStr">
@@ -4475,7 +4475,7 @@
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
@@ -4485,25 +4485,25 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19511649/</t>
+          <t>https://www.onthemarket.com/details/19591720/</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>Broad Court, Covent Garden, London, WC2B</t>
+          <t>King Street, Covent Garden WC2</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>WC2B</t>
+          <t>WC2</t>
         </is>
       </c>
       <c r="F59" s="4" t="n">
-        <v>3684</v>
+        <v>4333</v>
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H59" s="4" t="inlineStr">
@@ -4517,12 +4517,12 @@
         </is>
       </c>
       <c r="J59" s="4" t="n">
-        <v>811</v>
+        <v>667</v>
       </c>
       <c r="K59" s="4" t="n"/>
       <c r="L59" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat arranged on raised ground floor Attractive period building with a sought-after location; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>One bedroom One bathroom; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M59" s="4" t="inlineStr">
@@ -4544,7 +4544,7 @@
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
@@ -4554,25 +4554,25 @@
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19500342/</t>
+          <t>https://www.onthemarket.com/details/19511649/</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>Covent Garden, West End, London, WC2E</t>
+          <t>Broad Court, Covent Garden, London, WC2B</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>WC2E</t>
+          <t>WC2B</t>
         </is>
       </c>
       <c r="F60" s="4" t="n">
-        <v>3700</v>
+        <v>3684</v>
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H60" s="4" t="inlineStr">
@@ -4585,11 +4585,13 @@
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J60" s="4" t="n"/>
+      <c r="J60" s="4" t="n">
+        <v>811</v>
+      </c>
       <c r="K60" s="4" t="n"/>
       <c r="L60" s="4" t="inlineStr">
         <is>
-          <t>Short Term Stay between 1-6 months Furnished Ground Floor of secure block Heart of Covent Garden; outdoor space is communal/shared; size not stated; listed furnished — check if flexible</t>
+          <t>2 bedroom flat arranged on raised ground floor Attractive period building with a sought-after location; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M60" s="4" t="inlineStr">
@@ -4611,7 +4613,7 @@
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
@@ -4621,21 +4623,21 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/9591535/</t>
+          <t>https://www.onthemarket.com/details/19500342/</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>Casson Square, Waterloo, Southbank Place, London, SE1</t>
+          <t>Covent Garden, West End, London, WC2E</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>SE1</t>
+          <t>WC2E</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>4075</v>
+        <v>3700</v>
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
@@ -4649,16 +4651,14 @@
       </c>
       <c r="I61" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
-        </is>
-      </c>
-      <c r="J61" s="4" t="n">
-        <v>641</v>
-      </c>
+          <t>Communal / shared</t>
+        </is>
+      </c>
+      <c r="J61" s="4" t="n"/>
       <c r="K61" s="4" t="n"/>
       <c r="L61" s="4" t="inlineStr">
         <is>
-          <t>*video viewing available* 24-hour five-star concierge 18,000 sq ft gym, pool and spa facilities Bedroom; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Short Term Stay between 1-6 months Furnished Ground Floor of secure block Heart of Covent Garden; outdoor space is communal/shared; size not stated; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M61" s="4" t="inlineStr">
@@ -4680,7 +4680,7 @@
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
@@ -4690,25 +4690,25 @@
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/5166551/</t>
+          <t>https://www.onthemarket.com/details/9591535/</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>Grafton Way, Bloomsbury, London WC1E</t>
+          <t>Casson Square, Waterloo, Southbank Place, London, SE1</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>WC1E</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F62" s="4" t="n">
-        <v>3142</v>
+        <v>4075</v>
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H62" s="4" t="inlineStr">
@@ -4718,16 +4718,16 @@
       </c>
       <c r="I62" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Private balcony/terrace</t>
         </is>
       </c>
       <c r="J62" s="4" t="n">
-        <v>592</v>
+        <v>641</v>
       </c>
       <c r="K62" s="4" t="n"/>
       <c r="L62" s="4" t="inlineStr">
         <is>
-          <t>592 sq ft floor area Nearest station 0.1mi.; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>*video viewing available* 24-hour five-star concierge 18,000 sq ft gym, pool and spa facilities Bedroom; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M62" s="4" t="inlineStr">
@@ -4749,7 +4749,7 @@
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
@@ -4759,21 +4759,21 @@
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/10453057/</t>
+          <t>https://www.onthemarket.com/details/5166551/</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>Doughty Street, Bloomsbury, London, WC1N</t>
+          <t>Grafton Way, Bloomsbury, London WC1E</t>
         </is>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>WC1N</t>
+          <t>WC1E</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>3250</v>
+        <v>3142</v>
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
@@ -4791,12 +4791,12 @@
         </is>
       </c>
       <c r="J63" s="4" t="n">
-        <v>787</v>
+        <v>592</v>
       </c>
       <c r="K63" s="4" t="n"/>
       <c r="L63" s="4" t="inlineStr">
         <is>
-          <t>Two double bedrooms Dine-in kitchen; verify balcony/terrace; listed furnished — check if flexible</t>
+          <t>592 sq ft floor area Nearest station 0.1mi.; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M63" s="4" t="inlineStr">
@@ -4818,7 +4818,7 @@
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
@@ -4828,30 +4828,30 @@
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/13502768/</t>
+          <t>https://www.onthemarket.com/details/10453057/</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>Bedford Court Mansions, Bloomsbury, WC1B</t>
+          <t>Doughty Street, Bloomsbury, London, WC1N</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>WC1B</t>
+          <t>WC1N</t>
         </is>
       </c>
       <c r="F64" s="4" t="n">
-        <v>3142</v>
+        <v>3250</v>
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H64" s="4" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Furnished</t>
         </is>
       </c>
       <c r="I64" s="4" t="inlineStr">
@@ -4860,12 +4860,12 @@
         </is>
       </c>
       <c r="J64" s="4" t="n">
-        <v>587</v>
+        <v>787</v>
       </c>
       <c r="K64" s="4" t="n"/>
       <c r="L64" s="4" t="inlineStr">
         <is>
-          <t>One Bedroom Professionally Managed; verify balcony/terrace; under 650 sq ft</t>
+          <t>Two double bedrooms Dine-in kitchen; verify balcony/terrace; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M64" s="4" t="inlineStr">
@@ -4887,7 +4887,7 @@
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
@@ -4897,21 +4897,21 @@
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19815346/</t>
+          <t>https://www.onthemarket.com/details/13502768/</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>Bloomsbury, London, WC1N</t>
+          <t>Bedford Court Mansions, Bloomsbury, WC1B</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>WC1N</t>
+          <t>WC1B</t>
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>3000</v>
+        <v>3142</v>
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
@@ -4920,19 +4920,21 @@
       </c>
       <c r="H65" s="4" t="inlineStr">
         <is>
-          <t>Furnished</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I65" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
-        </is>
-      </c>
-      <c r="J65" s="4" t="n"/>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="J65" s="4" t="n">
+        <v>587</v>
+      </c>
       <c r="K65" s="4" t="n"/>
       <c r="L65" s="4" t="inlineStr">
         <is>
-          <t>No Agent Fees Property Reference Number: 2942192; size not stated; listed furnished — check if flexible</t>
+          <t>One Bedroom Professionally Managed; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M65" s="4" t="inlineStr">
@@ -4964,21 +4966,21 @@
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/3952850/</t>
+          <t>https://www.onthemarket.com/details/19815346/</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>Bloomsbury Square, Bloomsbury, London, WC1A</t>
+          <t>Bloomsbury, London, WC1N</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>WC1A</t>
+          <t>WC1N</t>
         </is>
       </c>
       <c r="F66" s="4" t="n">
-        <v>3141</v>
+        <v>3000</v>
       </c>
       <c r="G66" s="4" t="inlineStr">
         <is>
@@ -4987,21 +4989,19 @@
       </c>
       <c r="H66" s="4" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Furnished</t>
         </is>
       </c>
       <c r="I66" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="J66" s="4" t="n">
-        <v>609</v>
-      </c>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J66" s="4" t="n"/>
       <c r="K66" s="4" t="n"/>
       <c r="L66" s="4" t="inlineStr">
         <is>
-          <t>One Bedroom High Ceilings Views of Bloomsbury Square Wow Factor; verify balcony/terrace; under 650 sq ft</t>
+          <t>No Agent Fees Property Reference Number: 2942192; size not stated; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M66" s="4" t="inlineStr">
@@ -5023,7 +5023,7 @@
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
@@ -5033,30 +5033,30 @@
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19723779/</t>
+          <t>https://www.onthemarket.com/details/3952850/</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>Mecklenburgh Square, Bloomsbury, London, WC1N</t>
+          <t>Bloomsbury Square, Bloomsbury, London, WC1A</t>
         </is>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>WC1N</t>
+          <t>WC1A</t>
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>3684</v>
+        <v>3141</v>
       </c>
       <c r="G67" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H67" s="4" t="inlineStr">
         <is>
-          <t>Part Furnished</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I67" s="4" t="inlineStr">
@@ -5065,12 +5065,12 @@
         </is>
       </c>
       <c r="J67" s="4" t="n">
-        <v>602</v>
+        <v>609</v>
       </c>
       <c r="K67" s="4" t="n"/>
       <c r="L67" s="4" t="inlineStr">
         <is>
-          <t>Superb 2 bedroom flat Spacious arrangement; verify balcony/terrace; under 650 sq ft</t>
+          <t>One Bedroom High Ceilings Views of Bloomsbury Square Wow Factor; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M67" s="4" t="inlineStr">
@@ -5092,7 +5092,7 @@
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
@@ -5102,64 +5102,133 @@
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19715608/</t>
+          <t>https://www.onthemarket.com/details/19723779/</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>Bloomsbury Square, London WC1A</t>
+          <t>Mecklenburgh Square, Bloomsbury, London, WC1N</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>WC1A</t>
+          <t>WC1N</t>
         </is>
       </c>
       <c r="F68" s="4" t="n">
-        <v>3000</v>
+        <v>3684</v>
       </c>
       <c r="G68" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H68" s="4" t="inlineStr">
         <is>
-          <t>Furnished</t>
+          <t>Part Furnished</t>
         </is>
       </c>
       <c r="I68" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J68" s="4" t="n">
-        <v>581</v>
+        <v>602</v>
       </c>
       <c r="K68" s="4" t="n"/>
       <c r="L68" s="4" t="inlineStr">
         <is>
+          <t>Superb 2 bedroom flat Spacious arrangement; verify balcony/terrace; under 650 sq ft</t>
+        </is>
+      </c>
+      <c r="M68" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N68" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O68" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>1 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19715608/</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>Bloomsbury Square, London WC1A</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>WC1A</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t>1-Bed</t>
+        </is>
+      </c>
+      <c r="H69" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I69" s="4" t="inlineStr">
+        <is>
+          <t>Communal / shared</t>
+        </is>
+      </c>
+      <c r="J69" s="4" t="n">
+        <v>581</v>
+      </c>
+      <c r="K69" s="4" t="n"/>
+      <c r="L69" s="4" t="inlineStr">
+        <is>
           <t>Period Building Concierge; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
-      <c r="M68" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N68" s="4" t="inlineStr">
+      <c r="M69" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N69" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="O68" s="4" t="inlineStr">
+      <c r="O69" s="4" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O68"/>
+  <autoFilter ref="A1:O69"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
@@ -5228,6 +5297,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId65"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C69" r:id="rId68"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily tracker update 2026-07-08
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Flats" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Flats'!$A$1:$O$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Flats'!$A$1:$O$73</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O71"/>
+  <dimension ref="A1:O73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
@@ -564,25 +564,25 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19821591/</t>
+          <t>https://www.onthemarket.com/details/9187629/</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Doughty Street, Bloomsbury WC1</t>
+          <t>Casson Square, Waterloo, Southbank Place, London, SE1</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>WC1</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F2" s="4" t="n">
-        <v>3445</v>
+        <v>3990</v>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -592,16 +592,16 @@
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J2" s="4" t="n">
-        <v>560</v>
-      </c>
-      <c r="K2" s="4" t="n"/>
+        <v>537</v>
+      </c>
+      <c r="K2" s="4" t="inlineStr"/>
       <c r="L2" s="4" t="inlineStr">
         <is>
-          <t>16 apartments spread across two Georgian townhouses Studio, one and two bed layouts Student; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Open plan reception kitchen Bedroom Bathroom 24-hour five-star concierge; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M2" s="4" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="O2" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07 11:38</t>
+          <t>2026-07-08 00:39</t>
         </is>
       </c>
     </row>
@@ -633,12 +633,12 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/7920965/</t>
+          <t>https://www.onthemarket.com/details/11391425/</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Belvedere Road, Waterloo, Southbank Place, London, SE1</t>
+          <t>Casson Square, Waterloo, London, SE1</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -647,7 +647,7 @@
         </is>
       </c>
       <c r="F3" s="4" t="n">
-        <v>3950</v>
+        <v>3033</v>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
@@ -661,16 +661,16 @@
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J3" s="4" t="n">
-        <v>596</v>
-      </c>
-      <c r="K3" s="4" t="n"/>
+        <v>397</v>
+      </c>
+      <c r="K3" s="4" t="inlineStr"/>
       <c r="L3" s="4" t="inlineStr">
         <is>
-          <t>Fully furnished 1 bedroom 24-hour five-star concierge 18,000 sq ft gym and spa facilities; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Studio bedroom Open plan kitchen/ reception room Bathroom 24 hour concierge; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M3" s="4" t="inlineStr">
@@ -685,14 +685,14 @@
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07 08:39</t>
+          <t>2026-07-08 00:39</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -702,21 +702,21 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19876910/</t>
+          <t>https://www.onthemarket.com/details/19821591/</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Newton Street, Covent Garden, London, WC2B</t>
+          <t>Doughty Street, Bloomsbury WC1</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>WC2B</t>
+          <t>WC1</t>
         </is>
       </c>
       <c r="F4" s="4" t="n">
-        <v>4117</v>
+        <v>3445</v>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
@@ -730,16 +730,16 @@
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J4" s="4" t="n">
-        <v>848</v>
+        <v>560</v>
       </c>
       <c r="K4" s="4" t="n"/>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>Stunning 2 bedroom flat arranged on the 1st floor Generous reception room with space to dine; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>16 apartments spread across two Georgian townhouses Studio, one and two bed layouts Student; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M4" s="4" t="inlineStr">
@@ -754,83 +754,83 @@
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07 07:39</t>
+          <t>2026-07-07 11:38</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>2 bedroom flat to rent</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/19318164/</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>Princeton Street, Bloomsbury, London, WC1R</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>WC1R</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="n">
-        <v>3684</v>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>2-Bed</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>Part Furnished</t>
-        </is>
-      </c>
-      <c r="I5" s="6" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>1 bedroom apartment to rent</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/7920965/</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Belvedere Road, Waterloo, Southbank Place, London, SE1</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>SE1</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>3950</v>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>1-Bed</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Private balcony/terrace</t>
         </is>
       </c>
-      <c r="J5" s="6" t="n">
-        <v>649</v>
-      </c>
-      <c r="K5" s="6" t="n"/>
-      <c r="L5" s="6" t="inlineStr">
-        <is>
-          <t>Modern two bedroom, fourth floor flat Bright open plan reception Stylish kitchen featuring a range of modern appliances Two spacious bedrooms with built in stor; under 650 sq ft</t>
-        </is>
-      </c>
-      <c r="M5" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N5" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O5" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-06 20:39</t>
+      <c r="J5" s="4" t="n">
+        <v>596</v>
+      </c>
+      <c r="K5" s="4" t="n"/>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>Fully furnished 1 bedroom 24-hour five-star concierge 18,000 sq ft gym and spa facilities; under 650 sq ft; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07 08:39</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -840,25 +840,25 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/16574229/</t>
+          <t>https://www.onthemarket.com/details/19876910/</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Casson Square, Waterloo, London, SE1</t>
+          <t>Newton Street, Covent Garden, London, WC2B</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>SE1</t>
+          <t>WC2B</t>
         </is>
       </c>
       <c r="F6" s="4" t="n">
-        <v>3500</v>
+        <v>4117</v>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -872,12 +872,12 @@
         </is>
       </c>
       <c r="J6" s="4" t="n">
-        <v>548</v>
+        <v>848</v>
       </c>
       <c r="K6" s="4" t="n"/>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>548 sq ft floor area Nearest station 0.1mi.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Stunning 2 bedroom flat arranged on the 1st floor Generous reception room with space to dine; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M6" s="4" t="inlineStr">
@@ -892,98 +892,98 @@
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06 16:39</t>
+          <t>2026-07-07 07:39</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>2 bedroom apartment to rent</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/13719505/</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Bedford Place, Bloomsbury, WC1B</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>WC1B</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="n">
-        <v>3878</v>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>2 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19318164/</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Princeton Street, Bloomsbury, London, WC1R</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>WC1R</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>3684</v>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>2-Bed</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>Furnished</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>Part Furnished</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
         <is>
           <t>Private balcony/terrace</t>
         </is>
       </c>
-      <c r="J7" s="4" t="n">
-        <v>961</v>
-      </c>
-      <c r="K7" s="4" t="n"/>
-      <c r="L7" s="4" t="inlineStr">
-        <is>
-          <t>Two Double Bedroom Apartment High Spec; listed furnished — check if flexible</t>
-        </is>
-      </c>
-      <c r="M7" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N7" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="O7" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-06 15:39</t>
+      <c r="J7" s="6" t="n">
+        <v>649</v>
+      </c>
+      <c r="K7" s="6" t="n"/>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>Modern two bedroom, fourth floor flat Bright open plan reception Stylish kitchen featuring a range of modern appliances Two spacious bedrooms with built in stor; under 650 sq ft</t>
+        </is>
+      </c>
+      <c r="M7" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N7" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O7" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-06 20:39</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Flat</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Rightmove</t>
+          <t>OnTheMarket</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>https://www.rightmove.co.uk/properties/88912341</t>
+          <t>https://www.onthemarket.com/details/16574229/</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Southwark Bridge Road, London, SE1</t>
+          <t>Casson Square, Waterloo, London, SE1</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -992,28 +992,30 @@
         </is>
       </c>
       <c r="F8" s="4" t="n">
-        <v>4500</v>
+        <v>3500</v>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Furnished</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="J8" s="4" t="n"/>
+          <t>Communal / shared</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>548</v>
+      </c>
       <c r="K8" s="4" t="n"/>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>This stunning apartment boasts floor-to-ceiling windows offering breath taking panoramic views across the London skyline, flooding the space with natural light.; verify balcony/terrace; size not stated</t>
+          <t>548 sq ft floor area Nearest station 0.1mi.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M8" s="4" t="inlineStr">
@@ -1028,96 +1030,98 @@
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06 14:39</t>
+          <t>2026-07-06 16:39</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>2 bedroom flat to rent</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/1990566/</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>Endell Street, Covent Garden, London, WC2H</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>WC2H</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="n">
-        <v>3400</v>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>2 bedroom apartment to rent</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/13719505/</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Bedford Place, Bloomsbury, WC1B</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>WC1B</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>3878</v>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>2-Bed</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>Unfurnished</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="inlineStr">
-        <is>
-          <t>Communal / shared</t>
-        </is>
-      </c>
-      <c r="J9" s="6" t="n"/>
-      <c r="K9" s="6" t="n"/>
-      <c r="L9" s="6" t="inlineStr">
-        <is>
-          <t>Two Bedrooms Two Bathrooms Open plan living room-kitchen First floor; outdoor space is communal/shared; size not stated</t>
-        </is>
-      </c>
-      <c r="M9" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N9" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O9" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-06</t>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>961</v>
+      </c>
+      <c r="K9" s="4" t="n"/>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>Two Double Bedroom Apartment High Spec; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O9" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06 15:39</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>Flat</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>OnTheMarket</t>
+          <t>Rightmove</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19194043/</t>
+          <t>https://www.rightmove.co.uk/properties/88912341</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Great Suffolk Street, Southwark, London, SE1</t>
+          <t>Southwark Bridge Road, London, SE1</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -1126,7 +1130,7 @@
         </is>
       </c>
       <c r="F10" s="4" t="n">
-        <v>3100</v>
+        <v>4500</v>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
@@ -1135,21 +1139,19 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Furnished</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Juliet only</t>
-        </is>
-      </c>
-      <c r="J10" s="4" t="n">
-        <v>638</v>
-      </c>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="n"/>
       <c r="K10" s="4" t="n"/>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>Stylish 2 bedroom flat set on the 5th floor Large reception room with Juliet balcony Modern kitchen 2 lovely double bedroom; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>This stunning apartment boasts floor-to-ceiling windows offering breath taking panoramic views across the London skyline, flooding the space with natural light.; verify balcony/terrace; size not stated</t>
         </is>
       </c>
       <c r="M10" s="4" t="inlineStr">
@@ -1164,74 +1166,72 @@
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-06 14:39</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>1 bedroom flat to rent</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/19099769/</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Fletcher Buildings,, Covent Garden, London, WC2B</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>WC2B</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="n">
-        <v>3792</v>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>1-Bed</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>Furnished</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>2 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/1990566/</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Endell Street, Covent Garden, London, WC2H</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>WC2H</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>3400</v>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>2-Bed</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>Unfurnished</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J11" s="4" t="n">
-        <v>320</v>
-      </c>
-      <c r="K11" s="4" t="n"/>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t>Bright and airy one bedroom apartment in a prime Central London location Well proportioned reception with high ceilings and neutral décor Generous double bedroo; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
-        </is>
-      </c>
-      <c r="M11" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N11" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="O11" s="4" t="inlineStr">
+      <c r="J11" s="6" t="n"/>
+      <c r="K11" s="6" t="n"/>
+      <c r="L11" s="6" t="inlineStr">
+        <is>
+          <t>Two Bedrooms Two Bathrooms Open plan living room-kitchen First floor; outdoor space is communal/shared; size not stated</t>
+        </is>
+      </c>
+      <c r="M11" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N11" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O11" s="6" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
@@ -1250,21 +1250,21 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/6356511/</t>
+          <t>https://www.onthemarket.com/details/19194043/</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Great James Street, Bloomsbury, London, WC1N</t>
+          <t>Great Suffolk Street, Southwark, London, SE1</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>WC1N</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F12" s="4" t="n">
-        <v>3683</v>
+        <v>3100</v>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
@@ -1278,16 +1278,16 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Juliet only</t>
         </is>
       </c>
       <c r="J12" s="4" t="n">
-        <v>928</v>
+        <v>638</v>
       </c>
       <c r="K12" s="4" t="n"/>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t>Spacious Split Level Apartment Large Terrace Wooden Flooring Nearest tubes: Chancery Lane, Russell Square &amp; Holborn; listed furnished — check if flexible</t>
+          <t>Stylish 2 bedroom flat set on the 5th floor Large reception room with Juliet balcony Modern kitchen 2 lovely double bedroom; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M12" s="4" t="inlineStr">
@@ -1319,21 +1319,21 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19453032/</t>
+          <t>https://www.onthemarket.com/details/19099769/</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Maiden Lane, Covent Garden, London, WC2E</t>
+          <t>Fletcher Buildings,, Covent Garden, London, WC2B</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>WC2E</t>
+          <t>WC2B</t>
         </is>
       </c>
       <c r="F13" s="4" t="n">
-        <v>3684</v>
+        <v>3792</v>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
@@ -1351,12 +1351,12 @@
         </is>
       </c>
       <c r="J13" s="4" t="n">
-        <v>630</v>
+        <v>320</v>
       </c>
       <c r="K13" s="4" t="n"/>
       <c r="L13" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat arranged on the 4th floor Bright and spacious reception room Smart dining room Modern kitchen; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Bright and airy one bedroom apartment in a prime Central London location Well proportioned reception with high ceilings and neutral décor Generous double bedroo; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M13" s="4" t="inlineStr">
@@ -1378,7 +1378,7 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -1388,25 +1388,25 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19592443/</t>
+          <t>https://www.onthemarket.com/details/6356511/</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Regent Square, Bloomsbury, London, WC1H</t>
+          <t>Great James Street, Bloomsbury, London, WC1N</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>WC1H</t>
+          <t>WC1N</t>
         </is>
       </c>
       <c r="F14" s="4" t="n">
-        <v>4312</v>
+        <v>3683</v>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -1420,187 +1420,187 @@
         </is>
       </c>
       <c r="J14" s="4" t="n">
-        <v>487</v>
+        <v>928</v>
       </c>
       <c r="K14" s="4" t="n"/>
       <c r="L14" s="4" t="inlineStr">
         <is>
+          <t>Spacious Split Level Apartment Large Terrace Wooden Flooring Nearest tubes: Chancery Lane, Russell Square &amp; Holborn; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M14" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O14" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>1 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19453032/</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Maiden Lane, Covent Garden, London, WC2E</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>WC2E</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>3684</v>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>1-Bed</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>Communal / shared</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="n">
+        <v>630</v>
+      </c>
+      <c r="K15" s="4" t="n"/>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>1 bedroom flat arranged on the 4th floor Bright and spacious reception room Smart dining room Modern kitchen; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N15" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O15" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>1 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19592443/</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Regent Square, Bloomsbury, London, WC1H</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>WC1H</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>4312</v>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>1-Bed</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J16" s="4" t="n">
+        <v>487</v>
+      </c>
+      <c r="K16" s="4" t="n"/>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
           <t>Fantastic one bedroom apartment Set within beautiful period conversion Boasts ample interior space arranged over the second floor Wonderful balcony overlooking ; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
-      <c r="M14" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N14" s="4" t="inlineStr">
+      <c r="M16" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N16" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="O14" s="4" t="inlineStr">
+      <c r="O16" s="4" t="inlineStr">
         <is>
           <t>2026-07-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Apartment</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Rightmove</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>https://www.rightmove.co.uk/properties/89143989</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>Waterloo Road, Southwark, SE1</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>SE1</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="n">
-        <v>4346</v>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>2-Bed</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>Part Furnished</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>Private balcony/terrace</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="n">
-        <v>1385</v>
-      </c>
-      <c r="K15" s="2" t="n"/>
-      <c r="L15" s="2" t="inlineStr">
-        <is>
-          <t>Two bedroom apartment with incredible views Waterloo Road SE1 250 Waterloo Road is an exciting new rental development conveniently located on Waterloo Road, SE1</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="O15" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>2 bedroom apartment to rent</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/4473051/</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Waterloo Road, Southwark, SE1</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>SE1</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="n">
-        <v>4346</v>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>2-Bed</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>Part Furnished</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>Private balcony/terrace</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="n">
-        <v>1385</v>
-      </c>
-      <c r="K16" s="2" t="n"/>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>Spectacular Views Waterloo</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="O16" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>Apartment</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>OnTheMarket</t>
+          <t>Rightmove</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19728858/</t>
+          <t>https://www.rightmove.co.uk/properties/89143989</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Waterloo Road, London SE1</t>
+          <t>Waterloo Road, Southwark, SE1</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1609,7 +1609,7 @@
         </is>
       </c>
       <c r="F17" s="2" t="n">
-        <v>4350</v>
+        <v>4346</v>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
@@ -1618,7 +1618,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Part Furnished</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1627,12 +1627,12 @@
         </is>
       </c>
       <c r="J17" s="2" t="n">
-        <v>1140</v>
+        <v>1385</v>
       </c>
       <c r="K17" s="2" t="n"/>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>Two Bedrooms Two Bathrooms</t>
+          <t>Two bedroom apartment with incredible views Waterloo Road SE1 250 Waterloo Road is an exciting new rental development conveniently located on Waterloo Road, SE1</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
@@ -1664,12 +1664,12 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/6248222/</t>
+          <t>https://www.onthemarket.com/details/4473051/</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Nelson Square, Southwark, London, SE1</t>
+          <t>Waterloo Road, Southwark, SE1</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1678,7 +1678,7 @@
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>3150</v>
+        <v>4346</v>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
@@ -1687,7 +1687,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Part Furnished</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -1696,12 +1696,12 @@
         </is>
       </c>
       <c r="J18" s="2" t="n">
-        <v>809</v>
+        <v>1385</v>
       </c>
       <c r="K18" s="2" t="n"/>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>Dishwasher Range / Oven</t>
+          <t>Spectacular Views Waterloo</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
@@ -1733,21 +1733,21 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19663010/</t>
+          <t>https://www.onthemarket.com/details/19728858/</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Guilford Street, Bloomsbury, London, WC1N</t>
+          <t>Waterloo Road, London SE1</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>WC1N</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>3684</v>
+        <v>4350</v>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
@@ -1756,7 +1756,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Part Furnished</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -1765,163 +1765,163 @@
         </is>
       </c>
       <c r="J19" s="2" t="n">
-        <v>691</v>
+        <v>1140</v>
       </c>
       <c r="K19" s="2" t="n"/>
       <c r="L19" s="2" t="inlineStr">
         <is>
+          <t>Two Bedrooms Two Bathrooms</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>2 bedroom apartment to rent</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/6248222/</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Nelson Square, Southwark, London, SE1</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>SE1</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>3150</v>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>2-Bed</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Unfurnished</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>809</v>
+      </c>
+      <c r="K20" s="2" t="n"/>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Dishwasher Range / Oven</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>2 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19663010/</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Guilford Street, Bloomsbury, London, WC1N</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>WC1N</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>3684</v>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>2-Bed</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Part Furnished</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="n">
+        <v>691</v>
+      </c>
+      <c r="K21" s="2" t="n"/>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
           <t>Superb 2 bedroom flat on lower ground floor Modern open-plan kitchen with integrated appliance Spacious reception room leading to lovely private patio 2 well-pr</t>
         </is>
       </c>
-      <c r="M19" s="2" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="O19" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>2 bedroom apartment to rent</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/19809694/</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>Shaftesbury Avenue, Soho, W1D</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="inlineStr">
-        <is>
-          <t>W1D</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="n">
-        <v>3553</v>
-      </c>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>2-Bed</t>
-        </is>
-      </c>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
-          <t>Flexible</t>
-        </is>
-      </c>
-      <c r="I20" s="6" t="inlineStr">
-        <is>
-          <t>Communal / shared</t>
-        </is>
-      </c>
-      <c r="J20" s="6" t="n">
-        <v>603</v>
-      </c>
-      <c r="K20" s="6" t="n"/>
-      <c r="L20" s="6" t="inlineStr">
-        <is>
-          <t>Beautifully Refurbished Secondary Glazing; outdoor space is communal/shared; under 650 sq ft</t>
-        </is>
-      </c>
-      <c r="M20" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N20" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O20" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>2 bedroom apartment to rent</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/13368018/</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>Shaftesbury Avenue , Soho, W1D</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="inlineStr">
-        <is>
-          <t>W1D</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="n">
-        <v>3987</v>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>2-Bed</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr">
-        <is>
-          <t>Flexible</t>
-        </is>
-      </c>
-      <c r="I21" s="6" t="inlineStr">
-        <is>
-          <t>Communal / shared</t>
-        </is>
-      </c>
-      <c r="J21" s="6" t="n">
-        <v>671</v>
-      </c>
-      <c r="K21" s="6" t="n"/>
-      <c r="L21" s="6" t="inlineStr">
-        <is>
-          <t>Pet friendly Wooden Floors Student; outdoor space is communal/shared</t>
-        </is>
-      </c>
-      <c r="M21" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N21" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O21" s="6" t="inlineStr">
+      <c r="O21" s="2" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
@@ -1940,7 +1940,7 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19627828/</t>
+          <t>https://www.onthemarket.com/details/19809694/</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -1954,7 +1954,7 @@
         </is>
       </c>
       <c r="F22" s="6" t="n">
-        <v>3987</v>
+        <v>3553</v>
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
@@ -1972,12 +1972,12 @@
         </is>
       </c>
       <c r="J22" s="6" t="n">
-        <v>802</v>
+        <v>603</v>
       </c>
       <c r="K22" s="6" t="n"/>
       <c r="L22" s="6" t="inlineStr">
         <is>
-          <t>Built in Storage Pet Friendly; outdoor space is communal/shared</t>
+          <t>Beautifully Refurbished Secondary Glazing; outdoor space is communal/shared; under 650 sq ft</t>
         </is>
       </c>
       <c r="M22" s="6" t="inlineStr">
@@ -1999,7 +1999,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
@@ -2009,12 +2009,12 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19600564/</t>
+          <t>https://www.onthemarket.com/details/13368018/</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Rupert Court, Soho, W1D</t>
+          <t>Shaftesbury Avenue , Soho, W1D</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
@@ -2023,11 +2023,11 @@
         </is>
       </c>
       <c r="F23" s="6" t="n">
-        <v>3163</v>
+        <v>3987</v>
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
@@ -2040,11 +2040,13 @@
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J23" s="6" t="n"/>
+      <c r="J23" s="6" t="n">
+        <v>671</v>
+      </c>
       <c r="K23" s="6" t="n"/>
       <c r="L23" s="6" t="inlineStr">
         <is>
-          <t>Beautifully Refurbished Pet friendly; outdoor space is communal/shared; size not stated</t>
+          <t>Pet friendly Wooden Floors Student; outdoor space is communal/shared</t>
         </is>
       </c>
       <c r="M23" s="6" t="inlineStr">
@@ -2066,7 +2068,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -2076,30 +2078,30 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/10862827/</t>
+          <t>https://www.onthemarket.com/details/19627828/</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>Rupert Court, Soho W1</t>
+          <t>Shaftesbury Avenue, Soho, W1D</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>W1D</t>
         </is>
       </c>
       <c r="F24" s="6" t="n">
-        <v>3163</v>
+        <v>3987</v>
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr">
@@ -2108,12 +2110,12 @@
         </is>
       </c>
       <c r="J24" s="6" t="n">
-        <v>603</v>
+        <v>802</v>
       </c>
       <c r="K24" s="6" t="n"/>
       <c r="L24" s="6" t="inlineStr">
         <is>
-          <t>One bedroom One shower room; outdoor space is communal/shared; under 650 sq ft</t>
+          <t>Built in Storage Pet Friendly; outdoor space is communal/shared</t>
         </is>
       </c>
       <c r="M24" s="6" t="inlineStr">
@@ -2135,7 +2137,7 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
@@ -2145,21 +2147,21 @@
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19845642/</t>
+          <t>https://www.onthemarket.com/details/19600564/</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Shelton Street, Covent Garden, London, WC2H</t>
+          <t>Rupert Court, Soho, W1D</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>WC2H</t>
+          <t>W1D</t>
         </is>
       </c>
       <c r="F25" s="6" t="n">
-        <v>3142</v>
+        <v>3163</v>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
@@ -2168,7 +2170,7 @@
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
@@ -2176,13 +2178,11 @@
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J25" s="6" t="n">
-        <v>480</v>
-      </c>
+      <c r="J25" s="6" t="n"/>
       <c r="K25" s="6" t="n"/>
       <c r="L25" s="6" t="inlineStr">
         <is>
-          <t>Superb one bedroom flat arranged on the second floor Spacious reception/kitchen with ample dining space; outdoor space is communal/shared; under 650 sq ft</t>
+          <t>Beautifully Refurbished Pet friendly; outdoor space is communal/shared; size not stated</t>
         </is>
       </c>
       <c r="M25" s="6" t="inlineStr">
@@ -2214,21 +2214,21 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19603496/</t>
+          <t>https://www.onthemarket.com/details/10862827/</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>Arne Street, Covent Garden, WC2E</t>
+          <t>Rupert Court, Soho W1</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>WC2E</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="F26" s="6" t="n">
-        <v>3250</v>
+        <v>3163</v>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
@@ -2246,12 +2246,12 @@
         </is>
       </c>
       <c r="J26" s="6" t="n">
-        <v>514</v>
+        <v>603</v>
       </c>
       <c r="K26" s="6" t="n"/>
       <c r="L26" s="6" t="inlineStr">
         <is>
-          <t>Council Tax Band G 514 sq ft floor area; outdoor space is communal/shared; under 650 sq ft</t>
+          <t>One bedroom One shower room; outdoor space is communal/shared; under 650 sq ft</t>
         </is>
       </c>
       <c r="M26" s="6" t="inlineStr">
@@ -2283,21 +2283,21 @@
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/14179323/</t>
+          <t>https://www.onthemarket.com/details/19845642/</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>Bloomsbury Square, Bloomsbury, Covent Garden, London, WC1A</t>
+          <t>Shelton Street, Covent Garden, London, WC2H</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>WC1A</t>
+          <t>WC2H</t>
         </is>
       </c>
       <c r="F27" s="6" t="n">
-        <v>3500</v>
+        <v>3142</v>
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
@@ -2306,7 +2306,7 @@
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>Part Furnished</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
@@ -2315,12 +2315,12 @@
         </is>
       </c>
       <c r="J27" s="6" t="n">
-        <v>734</v>
+        <v>480</v>
       </c>
       <c r="K27" s="6" t="n"/>
       <c r="L27" s="6" t="inlineStr">
         <is>
-          <t>Stunning Period Conversion Hardwood Flooring Multi-Room Sound System and Mood Lighting Throughout Contemporary Kitchen &amp; Bathroom; outdoor space is communal/shared</t>
+          <t>Superb one bedroom flat arranged on the second floor Spacious reception/kitchen with ample dining space; outdoor space is communal/shared; under 650 sq ft</t>
         </is>
       </c>
       <c r="M27" s="6" t="inlineStr">
@@ -2342,7 +2342,7 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
@@ -2352,21 +2352,21 @@
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19823664/</t>
+          <t>https://www.onthemarket.com/details/19603496/</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>Bedford Court Mansions, Adeline Place, Bloomsbury, London, WC1B</t>
+          <t>Arne Street, Covent Garden, WC2E</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>WC1B</t>
+          <t>WC2E</t>
         </is>
       </c>
       <c r="F28" s="6" t="n">
-        <v>3141</v>
+        <v>3250</v>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
@@ -2375,21 +2375,21 @@
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Unfurnished</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J28" s="6" t="n">
-        <v>573</v>
+        <v>514</v>
       </c>
       <c r="K28" s="6" t="n"/>
       <c r="L28" s="6" t="inlineStr">
         <is>
-          <t>One Bedroom Finished to high standard Lift Access Separate Kitchen; under 650 sq ft</t>
+          <t>Council Tax Band G 514 sq ft floor area; outdoor space is communal/shared; under 650 sq ft</t>
         </is>
       </c>
       <c r="M28" s="6" t="inlineStr">
@@ -2411,7 +2411,7 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
@@ -2421,12 +2421,12 @@
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/15813612/</t>
+          <t>https://www.onthemarket.com/details/14179323/</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>Bloomsbury Square, Bloomsbury, WC1A</t>
+          <t>Bloomsbury Square, Bloomsbury, Covent Garden, London, WC1A</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
@@ -2435,7 +2435,7 @@
         </is>
       </c>
       <c r="F29" s="6" t="n">
-        <v>3142</v>
+        <v>3500</v>
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
@@ -2444,21 +2444,21 @@
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Part Furnished</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J29" s="6" t="n">
-        <v>539</v>
+        <v>734</v>
       </c>
       <c r="K29" s="6" t="n"/>
       <c r="L29" s="6" t="inlineStr">
         <is>
-          <t>Large Double Bedroom Period Features Student; under 650 sq ft</t>
+          <t>Stunning Period Conversion Hardwood Flooring Multi-Room Sound System and Mood Lighting Throughout Contemporary Kitchen &amp; Bathroom; outdoor space is communal/shared</t>
         </is>
       </c>
       <c r="M29" s="6" t="inlineStr">
@@ -2490,21 +2490,21 @@
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19736445/</t>
+          <t>https://www.onthemarket.com/details/19823664/</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>Millman Street, Bloomsbury, London, WC1N</t>
+          <t>Bedford Court Mansions, Adeline Place, Bloomsbury, London, WC1B</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>WC1N</t>
+          <t>WC1B</t>
         </is>
       </c>
       <c r="F30" s="6" t="n">
-        <v>3142</v>
+        <v>3141</v>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>Part Furnished</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
@@ -2522,163 +2522,163 @@
         </is>
       </c>
       <c r="J30" s="6" t="n">
-        <v>542</v>
+        <v>573</v>
       </c>
       <c r="K30" s="6" t="n"/>
       <c r="L30" s="6" t="inlineStr">
         <is>
+          <t>One Bedroom Finished to high standard Lift Access Separate Kitchen; under 650 sq ft</t>
+        </is>
+      </c>
+      <c r="M30" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N30" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O30" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>1 bedroom apartment to rent</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/15813612/</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>Bloomsbury Square, Bloomsbury, WC1A</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>WC1A</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>3142</v>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>1-Bed</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>Flexible</t>
+        </is>
+      </c>
+      <c r="I31" s="6" t="inlineStr">
+        <is>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J31" s="6" t="n">
+        <v>539</v>
+      </c>
+      <c r="K31" s="6" t="n"/>
+      <c r="L31" s="6" t="inlineStr">
+        <is>
+          <t>Large Double Bedroom Period Features Student; under 650 sq ft</t>
+        </is>
+      </c>
+      <c r="M31" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N31" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O31" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>1 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19736445/</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>Millman Street, Bloomsbury, London, WC1N</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>WC1N</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="n">
+        <v>3142</v>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>1-Bed</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t>Part Furnished</t>
+        </is>
+      </c>
+      <c r="I32" s="6" t="inlineStr">
+        <is>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J32" s="6" t="n">
+        <v>542</v>
+      </c>
+      <c r="K32" s="6" t="n"/>
+      <c r="L32" s="6" t="inlineStr">
+        <is>
           <t>Fantastic 1 bedroom flat arranged on the ground floor Set within a lovely residential block; under 650 sq ft</t>
         </is>
       </c>
-      <c r="M30" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N30" s="6" t="inlineStr">
+      <c r="M32" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N32" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="O30" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>Flat</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>Rightmove</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>https://www.rightmove.co.uk/properties/90435384</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>251 SOUTHWARK BRIDGE ROAD, LONDON, SE1, Elephant and Castle, London, SE1</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>SE1</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="n">
-        <v>4250</v>
-      </c>
-      <c r="G31" s="4" t="inlineStr">
-        <is>
-          <t>1-Bed</t>
-        </is>
-      </c>
-      <c r="H31" s="4" t="inlineStr">
-        <is>
-          <t>Part Furnished</t>
-        </is>
-      </c>
-      <c r="I31" s="4" t="inlineStr">
-        <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="J31" s="4" t="n">
-        <v>520</v>
-      </c>
-      <c r="K31" s="4" t="n"/>
-      <c r="L31" s="4" t="inlineStr">
-        <is>
-          <t>ZERO DEPOSIT AVAILABLE. SHORT LET. Set on the 21st floor, this 1 bedroom flat boasts well arranged interiors including a large reception room, a modern open-pla; verify balcony/terrace; under 650 sq ft</t>
-        </is>
-      </c>
-      <c r="M31" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N31" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="O31" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>Flat</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>Rightmove</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>https://www.rightmove.co.uk/properties/90432648</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>251 SOUTHWARK BRIDGE ROAD, LONDON, SE1, Elephant and Castle, London, SE1</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>SE1</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="n">
-        <v>3000</v>
-      </c>
-      <c r="G32" s="4" t="inlineStr">
-        <is>
-          <t>1-Bed</t>
-        </is>
-      </c>
-      <c r="H32" s="4" t="inlineStr">
-        <is>
-          <t>Part Furnished</t>
-        </is>
-      </c>
-      <c r="I32" s="4" t="inlineStr">
-        <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="J32" s="4" t="n">
-        <v>520</v>
-      </c>
-      <c r="K32" s="4" t="n"/>
-      <c r="L32" s="4" t="inlineStr">
-        <is>
-          <t>ZERO DEPOSIT AVAILABLE. LONG LET. Set on the 21st floor, this 1 bedroom flat boasts well arranged interiors including a large reception room, a modern open-plan; verify balcony/terrace; under 650 sq ft</t>
-        </is>
-      </c>
-      <c r="M32" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N32" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="O32" s="4" t="inlineStr">
+      <c r="O32" s="6" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
@@ -2687,31 +2687,31 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>Flat</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>OnTheMarket</t>
+          <t>Rightmove</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/4220060/</t>
+          <t>https://www.rightmove.co.uk/properties/90435384</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Carnaby Street, Soho, W1F</t>
+          <t>251 SOUTHWARK BRIDGE ROAD, LONDON, SE1, Elephant and Castle, London, SE1</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>W1F</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F33" s="4" t="n">
-        <v>3640</v>
+        <v>4250</v>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
@@ -2720,7 +2720,7 @@
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Part Furnished</t>
         </is>
       </c>
       <c r="I33" s="4" t="inlineStr">
@@ -2729,12 +2729,12 @@
         </is>
       </c>
       <c r="J33" s="4" t="n">
-        <v>553</v>
+        <v>520</v>
       </c>
       <c r="K33" s="4" t="n"/>
       <c r="L33" s="4" t="inlineStr">
         <is>
-          <t>One bedroom apartment Newly refurbished; verify balcony/terrace; under 650 sq ft</t>
+          <t>ZERO DEPOSIT AVAILABLE. SHORT LET. Set on the 21st floor, this 1 bedroom flat boasts well arranged interiors including a large reception room, a modern open-pla; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M33" s="4" t="inlineStr">
@@ -2756,31 +2756,31 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>Flat</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>OnTheMarket</t>
+          <t>Rightmove</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/8022324/</t>
+          <t>https://www.rightmove.co.uk/properties/90432648</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Golden Square, Soho, London, W1F</t>
+          <t>251 SOUTHWARK BRIDGE ROAD, LONDON, SE1, Elephant and Castle, London, SE1</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>W1F</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F34" s="4" t="n">
-        <v>3467</v>
+        <v>3000</v>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
@@ -2789,7 +2789,7 @@
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>Furnished</t>
+          <t>Part Furnished</t>
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr">
@@ -2798,12 +2798,12 @@
         </is>
       </c>
       <c r="J34" s="4" t="n">
-        <v>608</v>
+        <v>520</v>
       </c>
       <c r="K34" s="4" t="n"/>
       <c r="L34" s="4" t="inlineStr">
         <is>
-          <t>608 sq ft floor area Nearest station 0.1mi.; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>ZERO DEPOSIT AVAILABLE. LONG LET. Set on the 21st floor, this 1 bedroom flat boasts well arranged interiors including a large reception room, a modern open-plan; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M34" s="4" t="inlineStr">
@@ -2825,7 +2825,7 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
@@ -2835,44 +2835,44 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19852978/</t>
+          <t>https://www.onthemarket.com/details/4220060/</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Newport Court, Covent Garden, London, WC2H</t>
+          <t>Carnaby Street, Soho, W1F</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>WC2H</t>
+          <t>W1F</t>
         </is>
       </c>
       <c r="F35" s="4" t="n">
-        <v>4334</v>
+        <v>3640</v>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>Furnished</t>
+          <t>Unfurnished</t>
         </is>
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J35" s="4" t="n">
-        <v>858</v>
+        <v>553</v>
       </c>
       <c r="K35" s="4" t="n"/>
       <c r="L35" s="4" t="inlineStr">
         <is>
-          <t>Splendid two bedroom flat Ample interiors; listed furnished — check if flexible</t>
+          <t>One bedroom apartment Newly refurbished; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M35" s="4" t="inlineStr">
@@ -2894,7 +2894,7 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -2904,12 +2904,12 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/16157050/</t>
+          <t>https://www.onthemarket.com/details/8022324/</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Brewer Street, Soho, W1F</t>
+          <t>Golden Square, Soho, London, W1F</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
@@ -2918,11 +2918,11 @@
         </is>
       </c>
       <c r="F36" s="4" t="n">
-        <v>3142</v>
+        <v>3467</v>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
@@ -2932,16 +2932,16 @@
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J36" s="4" t="n">
-        <v>730</v>
+        <v>608</v>
       </c>
       <c r="K36" s="4" t="n"/>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>730 sqft Secure Entrance; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>608 sq ft floor area Nearest station 0.1mi.; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
@@ -2963,7 +2963,7 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
@@ -2973,25 +2973,25 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/9956499/</t>
+          <t>https://www.onthemarket.com/details/19852978/</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Richmond Buildings, Soho, W1D</t>
+          <t>Newport Court, Covent Garden, London, WC2H</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>W1D</t>
+          <t>WC2H</t>
         </is>
       </c>
       <c r="F37" s="4" t="n">
-        <v>3835</v>
+        <v>4334</v>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
@@ -3001,16 +3001,16 @@
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Private balcony/terrace</t>
         </is>
       </c>
       <c r="J37" s="4" t="n">
-        <v>521</v>
+        <v>858</v>
       </c>
       <c r="K37" s="4" t="n"/>
       <c r="L37" s="4" t="inlineStr">
         <is>
-          <t>Council tax band: F 521 sq ft floor area; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Splendid two bedroom flat Ample interiors; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M37" s="4" t="inlineStr">
@@ -3032,7 +3032,7 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
@@ -3042,25 +3042,25 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19786051/</t>
+          <t>https://www.onthemarket.com/details/16157050/</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Old Compton Street, Soho, London, W1D</t>
+          <t>Brewer Street, Soho, W1F</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>W1D</t>
+          <t>W1F</t>
         </is>
       </c>
       <c r="F38" s="4" t="n">
-        <v>3600</v>
+        <v>3142</v>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
@@ -3074,12 +3074,12 @@
         </is>
       </c>
       <c r="J38" s="4" t="n">
-        <v>432</v>
+        <v>730</v>
       </c>
       <c r="K38" s="4" t="n"/>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>432 sq ft floor area Nearest station 0.1mi. Furnished Nearest school 0.2mi.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>730 sqft Secure Entrance; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
@@ -3111,21 +3111,21 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19828226/</t>
+          <t>https://www.onthemarket.com/details/9956499/</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>TCRW SOHO, Fareham Street, W1F</t>
+          <t>Richmond Buildings, Soho, W1D</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>W1F</t>
+          <t>W1D</t>
         </is>
       </c>
       <c r="F39" s="4" t="n">
-        <v>3600</v>
+        <v>3835</v>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
@@ -3143,12 +3143,12 @@
         </is>
       </c>
       <c r="J39" s="4" t="n">
-        <v>656</v>
+        <v>521</v>
       </c>
       <c r="K39" s="4" t="n"/>
       <c r="L39" s="4" t="inlineStr">
         <is>
-          <t>Concierge service Highly sought-after Zone 1 location; verify balcony/terrace; listed furnished — check if flexible</t>
+          <t>Council tax band: F 521 sq ft floor area; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M39" s="4" t="inlineStr">
@@ -3170,7 +3170,7 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
@@ -3180,25 +3180,25 @@
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/11345150/</t>
+          <t>https://www.onthemarket.com/details/19786051/</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Shaftesbury Avenue, Covent Garden, London, WC2H</t>
+          <t>Old Compton Street, Soho, London, W1D</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>WC2H</t>
+          <t>W1D</t>
         </is>
       </c>
       <c r="F40" s="4" t="n">
-        <v>3575</v>
+        <v>3600</v>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
@@ -3212,12 +3212,12 @@
         </is>
       </c>
       <c r="J40" s="4" t="n">
-        <v>870</v>
+        <v>432</v>
       </c>
       <c r="K40" s="4" t="n"/>
       <c r="L40" s="4" t="inlineStr">
         <is>
-          <t>870 sq ft floor area Nearest station 0.1mi.; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>432 sq ft floor area Nearest station 0.1mi. Furnished Nearest school 0.2mi.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M40" s="4" t="inlineStr">
@@ -3239,7 +3239,7 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
@@ -3249,25 +3249,25 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/4747672/</t>
+          <t>https://www.onthemarket.com/details/19828226/</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Townsend House, Deans Street, Soho W1D</t>
+          <t>TCRW SOHO, Fareham Street, W1F</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>W1D</t>
+          <t>W1F</t>
         </is>
       </c>
       <c r="F41" s="4" t="n">
-        <v>3850</v>
+        <v>3600</v>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
@@ -3280,11 +3280,13 @@
           <t>Not stated</t>
         </is>
       </c>
-      <c r="J41" s="4" t="n"/>
+      <c r="J41" s="4" t="n">
+        <v>656</v>
+      </c>
       <c r="K41" s="4" t="n"/>
       <c r="L41" s="4" t="inlineStr">
         <is>
-          <t>Close to Local Shops Close to Public Transport; verify balcony/terrace; size not stated; listed furnished — check if flexible</t>
+          <t>Concierge service Highly sought-after Zone 1 location; verify balcony/terrace; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M41" s="4" t="inlineStr">
@@ -3306,7 +3308,7 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
@@ -3316,44 +3318,44 @@
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19628367/</t>
+          <t>https://www.onthemarket.com/details/11345150/</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Carnaby Street, Soho W1</t>
+          <t>Shaftesbury Avenue, Covent Garden, London, WC2H</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>WC2H</t>
         </is>
       </c>
       <c r="F42" s="4" t="n">
-        <v>3640</v>
+        <v>3575</v>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Furnished</t>
         </is>
       </c>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J42" s="4" t="n">
-        <v>549</v>
+        <v>870</v>
       </c>
       <c r="K42" s="4" t="n"/>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>One bedroom One shower room, ensuite; verify balcony/terrace; under 650 sq ft</t>
+          <t>870 sq ft floor area Nearest station 0.1mi.; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
@@ -3375,7 +3377,7 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
@@ -3385,30 +3387,30 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/13524814/</t>
+          <t>https://www.onthemarket.com/details/4747672/</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Carnaby Street, Soho, W1F</t>
+          <t>Townsend House, Deans Street, Soho W1D</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>W1F</t>
+          <t>W1D</t>
         </is>
       </c>
       <c r="F43" s="4" t="n">
-        <v>3640</v>
+        <v>3850</v>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Furnished</t>
         </is>
       </c>
       <c r="I43" s="4" t="inlineStr">
@@ -3416,13 +3418,11 @@
           <t>Not stated</t>
         </is>
       </c>
-      <c r="J43" s="4" t="n">
-        <v>552</v>
-      </c>
+      <c r="J43" s="4" t="n"/>
       <c r="K43" s="4" t="n"/>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Recently Refurbished Apartment Original Features Student; verify balcony/terrace; under 650 sq ft</t>
+          <t>Close to Local Shops Close to Public Transport; verify balcony/terrace; size not stated; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
@@ -3454,12 +3454,12 @@
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/18690047/</t>
+          <t>https://www.onthemarket.com/details/19628367/</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Duck Lane, Soho W1</t>
+          <t>Carnaby Street, Soho W1</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
@@ -3468,7 +3468,7 @@
         </is>
       </c>
       <c r="F44" s="4" t="n">
-        <v>3077</v>
+        <v>3640</v>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
@@ -3486,12 +3486,12 @@
         </is>
       </c>
       <c r="J44" s="4" t="n">
-        <v>581</v>
+        <v>549</v>
       </c>
       <c r="K44" s="4" t="n"/>
       <c r="L44" s="4" t="inlineStr">
         <is>
-          <t>One bedroom One bathroom; verify balcony/terrace; under 650 sq ft</t>
+          <t>One bedroom One shower room, ensuite; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M44" s="4" t="inlineStr">
@@ -3523,12 +3523,12 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/18690128/</t>
+          <t>https://www.onthemarket.com/details/13524814/</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Duck Lane, Soho, W1F</t>
+          <t>Carnaby Street, Soho, W1F</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
@@ -3537,7 +3537,7 @@
         </is>
       </c>
       <c r="F45" s="4" t="n">
-        <v>3077</v>
+        <v>3640</v>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
@@ -3546,7 +3546,7 @@
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I45" s="4" t="inlineStr">
@@ -3555,12 +3555,12 @@
         </is>
       </c>
       <c r="J45" s="4" t="n">
-        <v>580</v>
+        <v>552</v>
       </c>
       <c r="K45" s="4" t="n"/>
       <c r="L45" s="4" t="inlineStr">
         <is>
-          <t>One Double bedroom Quaint Road; verify balcony/terrace; under 650 sq ft</t>
+          <t>Recently Refurbished Apartment Original Features Student; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M45" s="4" t="inlineStr">
@@ -3592,17 +3592,17 @@
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/18680649/</t>
+          <t>https://www.onthemarket.com/details/18690047/</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Duck Lane, Soho W1F</t>
+          <t>Duck Lane, Soho W1</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>W1F</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="F46" s="4" t="n">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="H46" s="4" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Unfurnished</t>
         </is>
       </c>
       <c r="I46" s="4" t="inlineStr">
@@ -3624,12 +3624,12 @@
         </is>
       </c>
       <c r="J46" s="4" t="n">
-        <v>575</v>
+        <v>581</v>
       </c>
       <c r="K46" s="4" t="n"/>
       <c r="L46" s="4" t="inlineStr">
         <is>
-          <t>Modern Throughout Wooden Flooring Throughout; verify balcony/terrace; under 650 sq ft</t>
+          <t>One bedroom One bathroom; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M46" s="4" t="inlineStr">
@@ -3661,21 +3661,21 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/15707269/</t>
+          <t>https://www.onthemarket.com/details/18690128/</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Casson Square, London, Waterloo, United Kingdom, SE1</t>
+          <t>Duck Lane, Soho, W1F</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>SE1</t>
+          <t>W1F</t>
         </is>
       </c>
       <c r="F47" s="4" t="n">
-        <v>4050</v>
+        <v>3077</v>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
@@ -3684,21 +3684,21 @@
       </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t>Furnished</t>
+          <t>Unfurnished</t>
         </is>
       </c>
       <c r="I47" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J47" s="4" t="n">
-        <v>514</v>
+        <v>580</v>
       </c>
       <c r="K47" s="4" t="n"/>
       <c r="L47" s="4" t="inlineStr">
         <is>
-          <t>Bedroom Bathroom Open-plan reception/kitchen 24 hour concierge; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>One Double bedroom Quaint Road; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M47" s="4" t="inlineStr">
@@ -3730,21 +3730,21 @@
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/9568931/</t>
+          <t>https://www.onthemarket.com/details/18680649/</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Casson Square, Waterloo, Southbank Place, London, SE1</t>
+          <t>Duck Lane, Soho W1F</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>SE1</t>
+          <t>W1F</t>
         </is>
       </c>
       <c r="F48" s="4" t="n">
-        <v>4250</v>
+        <v>3077</v>
       </c>
       <c r="G48" s="4" t="inlineStr">
         <is>
@@ -3753,21 +3753,21 @@
       </c>
       <c r="H48" s="4" t="inlineStr">
         <is>
-          <t>Furnished</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I48" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J48" s="4" t="n">
-        <v>644</v>
+        <v>575</v>
       </c>
       <c r="K48" s="4" t="n"/>
       <c r="L48" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom 1 bathroom Open-plan reception kitchen 24-hour five-star concierge; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Modern Throughout Wooden Flooring Throughout; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M48" s="4" t="inlineStr">
@@ -3789,7 +3789,7 @@
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom end of terrace house to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
@@ -3799,21 +3799,25 @@
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19811489/</t>
+          <t>https://www.onthemarket.com/details/15707269/</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>Carlisle Lane, Waterloo</t>
-        </is>
-      </c>
-      <c r="E49" s="4" t="n"/>
+          <t>Casson Square, London, Waterloo, United Kingdom, SE1</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>SE1</t>
+        </is>
+      </c>
       <c r="F49" s="4" t="n">
-        <v>3575</v>
+        <v>4050</v>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H49" s="4" t="inlineStr">
@@ -3823,16 +3827,16 @@
       </c>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J49" s="4" t="n">
-        <v>904</v>
+        <v>514</v>
       </c>
       <c r="K49" s="4" t="n"/>
       <c r="L49" s="4" t="inlineStr">
         <is>
-          <t>End of Terrace Shared Garden; listed furnished — check if flexible</t>
+          <t>Bedroom Bathroom Open-plan reception/kitchen 24 hour concierge; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M49" s="4" t="inlineStr">
@@ -3854,7 +3858,7 @@
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
@@ -3864,12 +3868,12 @@
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/7516361/</t>
+          <t>https://www.onthemarket.com/details/9568931/</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>Belvedere Road, Waterloo, London, SE1</t>
+          <t>Casson Square, Waterloo, Southbank Place, London, SE1</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
@@ -3878,11 +3882,11 @@
         </is>
       </c>
       <c r="F50" s="4" t="n">
-        <v>3350</v>
+        <v>4250</v>
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H50" s="4" t="inlineStr">
@@ -3892,16 +3896,16 @@
       </c>
       <c r="I50" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Private balcony/terrace</t>
         </is>
       </c>
       <c r="J50" s="4" t="n">
-        <v>544</v>
+        <v>644</v>
       </c>
       <c r="K50" s="4" t="n"/>
       <c r="L50" s="4" t="inlineStr">
         <is>
-          <t>Residents' swimming pool and gym. Grade II listed period building. 24 hour porters. Set close to the iconic Southbank and London Eye.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>1 bedroom 1 bathroom Open-plan reception kitchen 24-hour five-star concierge; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M50" s="4" t="inlineStr">
@@ -3923,7 +3927,7 @@
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom end of terrace house to rent</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
@@ -3933,25 +3937,21 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/7589011/</t>
+          <t>https://www.onthemarket.com/details/19811489/</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>Belvedere Road, London, Waterloo, SE1</t>
-        </is>
-      </c>
-      <c r="E51" s="4" t="inlineStr">
-        <is>
-          <t>SE1</t>
-        </is>
-      </c>
+          <t>Carlisle Lane, Waterloo</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="n"/>
       <c r="F51" s="4" t="n">
-        <v>4200</v>
+        <v>3575</v>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H51" s="4" t="inlineStr">
@@ -3961,16 +3961,16 @@
       </c>
       <c r="I51" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Private balcony/terrace</t>
         </is>
       </c>
       <c r="J51" s="4" t="n">
-        <v>671</v>
+        <v>904</v>
       </c>
       <c r="K51" s="4" t="n"/>
       <c r="L51" s="4" t="inlineStr">
         <is>
-          <t>24-hour five-star concierge 18,000 sq ft gym and spa facilities Set in one of London's most connected locations, opposite Westminster and the Houses of Parliame; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>End of Terrace Shared Garden; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M51" s="4" t="inlineStr">
@@ -3992,7 +3992,7 @@
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
@@ -4002,12 +4002,12 @@
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/17616661/</t>
+          <t>https://www.onthemarket.com/details/7516361/</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>The Music Box, 237 Union Street, Southwark, London, SE1</t>
+          <t>Belvedere Road, Waterloo, London, SE1</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
@@ -4016,7 +4016,7 @@
         </is>
       </c>
       <c r="F52" s="4" t="n">
-        <v>3800</v>
+        <v>3350</v>
       </c>
       <c r="G52" s="4" t="inlineStr">
         <is>
@@ -4030,16 +4030,16 @@
       </c>
       <c r="I52" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J52" s="4" t="n">
-        <v>841</v>
+        <v>544</v>
       </c>
       <c r="K52" s="4" t="n"/>
       <c r="L52" s="4" t="inlineStr">
         <is>
-          <t>Two bedrooms Two bathrooms 841 sq. ft. Excellent transport links; verify balcony/terrace; listed furnished — check if flexible</t>
+          <t>Residents' swimming pool and gym. Grade II listed period building. 24 hour porters. Set close to the iconic Southbank and London Eye.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M52" s="4" t="inlineStr">
@@ -4061,7 +4061,7 @@
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
@@ -4071,21 +4071,21 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19863550/</t>
+          <t>https://www.onthemarket.com/details/7589011/</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>King Street, Covent Garden, London, WC2E</t>
+          <t>Belvedere Road, London, Waterloo, SE1</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>WC2E</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F53" s="4" t="n">
-        <v>3358</v>
+        <v>4200</v>
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
@@ -4103,12 +4103,12 @@
         </is>
       </c>
       <c r="J53" s="4" t="n">
-        <v>455</v>
+        <v>671</v>
       </c>
       <c r="K53" s="4" t="n"/>
       <c r="L53" s="4" t="inlineStr">
         <is>
-          <t>Iconic Covent Garden location Finished to an excellent standard throughout High ceilings Wooden flooring throughout; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>24-hour five-star concierge 18,000 sq ft gym and spa facilities Set in one of London's most connected locations, opposite Westminster and the Houses of Parliame; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M53" s="4" t="inlineStr">
@@ -4130,7 +4130,7 @@
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
@@ -4140,25 +4140,25 @@
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19860280/</t>
+          <t>https://www.onthemarket.com/details/17616661/</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>Floral Street, Covent Garden WC2</t>
+          <t>The Music Box, 237 Union Street, Southwark, London, SE1</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>WC2</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F54" s="4" t="n">
-        <v>3380</v>
+        <v>3800</v>
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H54" s="4" t="inlineStr">
@@ -4168,16 +4168,16 @@
       </c>
       <c r="I54" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J54" s="4" t="n">
-        <v>495</v>
+        <v>841</v>
       </c>
       <c r="K54" s="4" t="n"/>
       <c r="L54" s="4" t="inlineStr">
         <is>
-          <t>One bedroom One bathroom, ensuite; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Two bedrooms Two bathrooms 841 sq. ft. Excellent transport links; verify balcony/terrace; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M54" s="4" t="inlineStr">
@@ -4199,7 +4199,7 @@
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
@@ -4209,12 +4209,12 @@
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/1837052/</t>
+          <t>https://www.onthemarket.com/details/19863550/</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>King Street, Covent Garden, WC2E</t>
+          <t>King Street, Covent Garden, London, WC2E</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
@@ -4246,7 +4246,7 @@
       <c r="K55" s="4" t="n"/>
       <c r="L55" s="4" t="inlineStr">
         <is>
-          <t>Furnished Recently refurbished; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Iconic Covent Garden location Finished to an excellent standard throughout High ceilings Wooden flooring throughout; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M55" s="4" t="inlineStr">
@@ -4278,17 +4278,17 @@
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/3408032/</t>
+          <t>https://www.onthemarket.com/details/19860280/</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>Floral Street, Covent Garden, WC2E</t>
+          <t>Floral Street, Covent Garden WC2</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>WC2E</t>
+          <t>WC2</t>
         </is>
       </c>
       <c r="F56" s="4" t="n">
@@ -4310,12 +4310,12 @@
         </is>
       </c>
       <c r="J56" s="4" t="n">
-        <v>398</v>
+        <v>495</v>
       </c>
       <c r="K56" s="4" t="n"/>
       <c r="L56" s="4" t="inlineStr">
         <is>
-          <t>Newly Refurbished Central Location; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>One bedroom One bathroom, ensuite; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M56" s="4" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
@@ -4347,25 +4347,25 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/3102769/</t>
+          <t>https://www.onthemarket.com/details/1837052/</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>John Adam Street, Covent Garden, WC2N</t>
+          <t>King Street, Covent Garden, WC2E</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>WC2N</t>
+          <t>WC2E</t>
         </is>
       </c>
       <c r="F57" s="4" t="n">
-        <v>3185</v>
+        <v>3358</v>
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H57" s="4" t="inlineStr">
@@ -4379,12 +4379,12 @@
         </is>
       </c>
       <c r="J57" s="4" t="n">
-        <v>655</v>
+        <v>455</v>
       </c>
       <c r="K57" s="4" t="n"/>
       <c r="L57" s="4" t="inlineStr">
         <is>
-          <t>Concierge Close to the area's Universities for students and academics; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>Furnished Recently refurbished; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M57" s="4" t="inlineStr">
@@ -4406,7 +4406,7 @@
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
@@ -4416,12 +4416,12 @@
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19733694/</t>
+          <t>https://www.onthemarket.com/details/3408032/</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>Maiden Lane, Covent Garden, London, WC2E</t>
+          <t>Floral Street, Covent Garden, WC2E</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
@@ -4430,7 +4430,7 @@
         </is>
       </c>
       <c r="F58" s="4" t="n">
-        <v>3684</v>
+        <v>3380</v>
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
@@ -4448,12 +4448,12 @@
         </is>
       </c>
       <c r="J58" s="4" t="n">
-        <v>630</v>
+        <v>398</v>
       </c>
       <c r="K58" s="4" t="n"/>
       <c r="L58" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat arranged on the 4th floor Bright and spacious reception room; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Newly Refurbished Central Location; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M58" s="4" t="inlineStr">
@@ -4475,7 +4475,7 @@
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
@@ -4485,25 +4485,25 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19725776/</t>
+          <t>https://www.onthemarket.com/details/3102769/</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>Shelton Street, Covent Garden, London, WC2H</t>
+          <t>John Adam Street, Covent Garden, WC2N</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>WC2H</t>
+          <t>WC2N</t>
         </is>
       </c>
       <c r="F59" s="4" t="n">
-        <v>3500</v>
+        <v>3185</v>
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H59" s="4" t="inlineStr">
@@ -4513,16 +4513,16 @@
       </c>
       <c r="I59" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J59" s="4" t="n">
-        <v>608</v>
+        <v>655</v>
       </c>
       <c r="K59" s="4" t="n"/>
       <c r="L59" s="4" t="inlineStr">
         <is>
-          <t>Stylish one bedroom, third floor apartment Beautifully proportioned open plan reception with balcony access; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Concierge Close to the area's Universities for students and academics; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M59" s="4" t="inlineStr">
@@ -4544,7 +4544,7 @@
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
@@ -4554,21 +4554,21 @@
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19591709/</t>
+          <t>https://www.onthemarket.com/details/19733694/</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>King Street, Covent Garden WC2</t>
+          <t>Maiden Lane, Covent Garden, London, WC2E</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>WC2</t>
+          <t>WC2E</t>
         </is>
       </c>
       <c r="F60" s="4" t="n">
-        <v>3575</v>
+        <v>3684</v>
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
@@ -4586,12 +4586,12 @@
         </is>
       </c>
       <c r="J60" s="4" t="n">
-        <v>441</v>
+        <v>630</v>
       </c>
       <c r="K60" s="4" t="n"/>
       <c r="L60" s="4" t="inlineStr">
         <is>
-          <t>One double bedroom One bathroom; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>1 bedroom flat arranged on the 4th floor Bright and spacious reception room; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M60" s="4" t="inlineStr">
@@ -4613,7 +4613,7 @@
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
@@ -4623,21 +4623,21 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19591720/</t>
+          <t>https://www.onthemarket.com/details/19725776/</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>King Street, Covent Garden WC2</t>
+          <t>Shelton Street, Covent Garden, London, WC2H</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>WC2</t>
+          <t>WC2H</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>4333</v>
+        <v>3500</v>
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
@@ -4651,16 +4651,16 @@
       </c>
       <c r="I61" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Private balcony/terrace</t>
         </is>
       </c>
       <c r="J61" s="4" t="n">
-        <v>667</v>
+        <v>608</v>
       </c>
       <c r="K61" s="4" t="n"/>
       <c r="L61" s="4" t="inlineStr">
         <is>
-          <t>One bedroom One bathroom; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>Stylish one bedroom, third floor apartment Beautifully proportioned open plan reception with balcony access; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M61" s="4" t="inlineStr">
@@ -4682,7 +4682,7 @@
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
@@ -4692,25 +4692,25 @@
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19511649/</t>
+          <t>https://www.onthemarket.com/details/19591709/</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>Broad Court, Covent Garden, London, WC2B</t>
+          <t>King Street, Covent Garden WC2</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>WC2B</t>
+          <t>WC2</t>
         </is>
       </c>
       <c r="F62" s="4" t="n">
-        <v>3684</v>
+        <v>3575</v>
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H62" s="4" t="inlineStr">
@@ -4724,12 +4724,12 @@
         </is>
       </c>
       <c r="J62" s="4" t="n">
-        <v>811</v>
+        <v>441</v>
       </c>
       <c r="K62" s="4" t="n"/>
       <c r="L62" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat arranged on raised ground floor Attractive period building with a sought-after location; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>One double bedroom One bathroom; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M62" s="4" t="inlineStr">
@@ -4751,7 +4751,7 @@
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
@@ -4761,21 +4761,21 @@
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19500342/</t>
+          <t>https://www.onthemarket.com/details/19591720/</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>Covent Garden, West End, London, WC2E</t>
+          <t>King Street, Covent Garden WC2</t>
         </is>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>WC2E</t>
+          <t>WC2</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>3700</v>
+        <v>4333</v>
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
@@ -4792,11 +4792,13 @@
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J63" s="4" t="n"/>
+      <c r="J63" s="4" t="n">
+        <v>667</v>
+      </c>
       <c r="K63" s="4" t="n"/>
       <c r="L63" s="4" t="inlineStr">
         <is>
-          <t>Short Term Stay between 1-6 months Furnished Ground Floor of secure block Heart of Covent Garden; outdoor space is communal/shared; size not stated; listed furnished — check if flexible</t>
+          <t>One bedroom One bathroom; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M63" s="4" t="inlineStr">
@@ -4818,7 +4820,7 @@
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
@@ -4828,25 +4830,25 @@
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/9591535/</t>
+          <t>https://www.onthemarket.com/details/19511649/</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>Casson Square, Waterloo, Southbank Place, London, SE1</t>
+          <t>Broad Court, Covent Garden, London, WC2B</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>SE1</t>
+          <t>WC2B</t>
         </is>
       </c>
       <c r="F64" s="4" t="n">
-        <v>4075</v>
+        <v>3684</v>
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H64" s="4" t="inlineStr">
@@ -4856,16 +4858,16 @@
       </c>
       <c r="I64" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J64" s="4" t="n">
-        <v>641</v>
+        <v>811</v>
       </c>
       <c r="K64" s="4" t="n"/>
       <c r="L64" s="4" t="inlineStr">
         <is>
-          <t>*video viewing available* 24-hour five-star concierge 18,000 sq ft gym, pool and spa facilities Bedroom; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>2 bedroom flat arranged on raised ground floor Attractive period building with a sought-after location; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M64" s="4" t="inlineStr">
@@ -4887,7 +4889,7 @@
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
@@ -4897,25 +4899,25 @@
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/5166551/</t>
+          <t>https://www.onthemarket.com/details/19500342/</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>Grafton Way, Bloomsbury, London WC1E</t>
+          <t>Covent Garden, West End, London, WC2E</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>WC1E</t>
+          <t>WC2E</t>
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>3142</v>
+        <v>3700</v>
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H65" s="4" t="inlineStr">
@@ -4925,16 +4927,14 @@
       </c>
       <c r="I65" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="J65" s="4" t="n">
-        <v>592</v>
-      </c>
+          <t>Communal / shared</t>
+        </is>
+      </c>
+      <c r="J65" s="4" t="n"/>
       <c r="K65" s="4" t="n"/>
       <c r="L65" s="4" t="inlineStr">
         <is>
-          <t>592 sq ft floor area Nearest station 0.1mi.; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Short Term Stay between 1-6 months Furnished Ground Floor of secure block Heart of Covent Garden; outdoor space is communal/shared; size not stated; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M65" s="4" t="inlineStr">
@@ -4956,7 +4956,7 @@
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
@@ -4966,25 +4966,25 @@
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/10453057/</t>
+          <t>https://www.onthemarket.com/details/9591535/</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>Doughty Street, Bloomsbury, London, WC1N</t>
+          <t>Casson Square, Waterloo, Southbank Place, London, SE1</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>WC1N</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F66" s="4" t="n">
-        <v>3250</v>
+        <v>4075</v>
       </c>
       <c r="G66" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H66" s="4" t="inlineStr">
@@ -4994,16 +4994,16 @@
       </c>
       <c r="I66" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Private balcony/terrace</t>
         </is>
       </c>
       <c r="J66" s="4" t="n">
-        <v>787</v>
+        <v>641</v>
       </c>
       <c r="K66" s="4" t="n"/>
       <c r="L66" s="4" t="inlineStr">
         <is>
-          <t>Two double bedrooms Dine-in kitchen; verify balcony/terrace; listed furnished — check if flexible</t>
+          <t>*video viewing available* 24-hour five-star concierge 18,000 sq ft gym, pool and spa facilities Bedroom; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M66" s="4" t="inlineStr">
@@ -5025,7 +5025,7 @@
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
@@ -5035,17 +5035,17 @@
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/13502768/</t>
+          <t>https://www.onthemarket.com/details/5166551/</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>Bedford Court Mansions, Bloomsbury, WC1B</t>
+          <t>Grafton Way, Bloomsbury, London WC1E</t>
         </is>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>WC1B</t>
+          <t>WC1E</t>
         </is>
       </c>
       <c r="F67" s="4" t="n">
@@ -5053,12 +5053,12 @@
       </c>
       <c r="G67" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H67" s="4" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Furnished</t>
         </is>
       </c>
       <c r="I67" s="4" t="inlineStr">
@@ -5067,12 +5067,12 @@
         </is>
       </c>
       <c r="J67" s="4" t="n">
-        <v>587</v>
+        <v>592</v>
       </c>
       <c r="K67" s="4" t="n"/>
       <c r="L67" s="4" t="inlineStr">
         <is>
-          <t>One Bedroom Professionally Managed; verify balcony/terrace; under 650 sq ft</t>
+          <t>592 sq ft floor area Nearest station 0.1mi.; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M67" s="4" t="inlineStr">
@@ -5094,7 +5094,7 @@
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
@@ -5104,12 +5104,12 @@
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19815346/</t>
+          <t>https://www.onthemarket.com/details/10453057/</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>Bloomsbury, London, WC1N</t>
+          <t>Doughty Street, Bloomsbury, London, WC1N</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
@@ -5118,11 +5118,11 @@
         </is>
       </c>
       <c r="F68" s="4" t="n">
-        <v>3000</v>
+        <v>3250</v>
       </c>
       <c r="G68" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H68" s="4" t="inlineStr">
@@ -5132,14 +5132,16 @@
       </c>
       <c r="I68" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
-        </is>
-      </c>
-      <c r="J68" s="4" t="n"/>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="J68" s="4" t="n">
+        <v>787</v>
+      </c>
       <c r="K68" s="4" t="n"/>
       <c r="L68" s="4" t="inlineStr">
         <is>
-          <t>No Agent Fees Property Reference Number: 2942192; size not stated; listed furnished — check if flexible</t>
+          <t>Two double bedrooms Dine-in kitchen; verify balcony/terrace; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M68" s="4" t="inlineStr">
@@ -5161,7 +5163,7 @@
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
@@ -5171,21 +5173,21 @@
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/3952850/</t>
+          <t>https://www.onthemarket.com/details/13502768/</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>Bloomsbury Square, Bloomsbury, London, WC1A</t>
+          <t>Bedford Court Mansions, Bloomsbury, WC1B</t>
         </is>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>WC1A</t>
+          <t>WC1B</t>
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>3141</v>
+        <v>3142</v>
       </c>
       <c r="G69" s="4" t="inlineStr">
         <is>
@@ -5203,12 +5205,12 @@
         </is>
       </c>
       <c r="J69" s="4" t="n">
-        <v>609</v>
+        <v>587</v>
       </c>
       <c r="K69" s="4" t="n"/>
       <c r="L69" s="4" t="inlineStr">
         <is>
-          <t>One Bedroom High Ceilings Views of Bloomsbury Square Wow Factor; verify balcony/terrace; under 650 sq ft</t>
+          <t>One Bedroom Professionally Managed; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M69" s="4" t="inlineStr">
@@ -5230,7 +5232,7 @@
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
@@ -5240,12 +5242,12 @@
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19723779/</t>
+          <t>https://www.onthemarket.com/details/19815346/</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>Mecklenburgh Square, Bloomsbury, London, WC1N</t>
+          <t>Bloomsbury, London, WC1N</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
@@ -5254,30 +5256,28 @@
         </is>
       </c>
       <c r="F70" s="4" t="n">
-        <v>3684</v>
+        <v>3000</v>
       </c>
       <c r="G70" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H70" s="4" t="inlineStr">
         <is>
-          <t>Part Furnished</t>
+          <t>Furnished</t>
         </is>
       </c>
       <c r="I70" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="J70" s="4" t="n">
-        <v>602</v>
-      </c>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J70" s="4" t="n"/>
       <c r="K70" s="4" t="n"/>
       <c r="L70" s="4" t="inlineStr">
         <is>
-          <t>Superb 2 bedroom flat Spacious arrangement; verify balcony/terrace; under 650 sq ft</t>
+          <t>No Agent Fees Property Reference Number: 2942192; size not stated; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M70" s="4" t="inlineStr">
@@ -5309,12 +5309,12 @@
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19715608/</t>
+          <t>https://www.onthemarket.com/details/3952850/</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>Bloomsbury Square, London WC1A</t>
+          <t>Bloomsbury Square, Bloomsbury, London, WC1A</t>
         </is>
       </c>
       <c r="E71" s="4" t="inlineStr">
@@ -5323,7 +5323,7 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>3000</v>
+        <v>3141</v>
       </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
@@ -5332,41 +5332,179 @@
       </c>
       <c r="H71" s="4" t="inlineStr">
         <is>
-          <t>Furnished</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I71" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J71" s="4" t="n">
-        <v>581</v>
+        <v>609</v>
       </c>
       <c r="K71" s="4" t="n"/>
       <c r="L71" s="4" t="inlineStr">
         <is>
+          <t>One Bedroom High Ceilings Views of Bloomsbury Square Wow Factor; verify balcony/terrace; under 650 sq ft</t>
+        </is>
+      </c>
+      <c r="M71" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N71" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O71" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t>2 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19723779/</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>Mecklenburgh Square, Bloomsbury, London, WC1N</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t>WC1N</t>
+        </is>
+      </c>
+      <c r="F72" s="4" t="n">
+        <v>3684</v>
+      </c>
+      <c r="G72" s="4" t="inlineStr">
+        <is>
+          <t>2-Bed</t>
+        </is>
+      </c>
+      <c r="H72" s="4" t="inlineStr">
+        <is>
+          <t>Part Furnished</t>
+        </is>
+      </c>
+      <c r="I72" s="4" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="J72" s="4" t="n">
+        <v>602</v>
+      </c>
+      <c r="K72" s="4" t="n"/>
+      <c r="L72" s="4" t="inlineStr">
+        <is>
+          <t>Superb 2 bedroom flat Spacious arrangement; verify balcony/terrace; under 650 sq ft</t>
+        </is>
+      </c>
+      <c r="M72" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N72" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O72" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>1 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19715608/</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>Bloomsbury Square, London WC1A</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>WC1A</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G73" s="4" t="inlineStr">
+        <is>
+          <t>1-Bed</t>
+        </is>
+      </c>
+      <c r="H73" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I73" s="4" t="inlineStr">
+        <is>
+          <t>Communal / shared</t>
+        </is>
+      </c>
+      <c r="J73" s="4" t="n">
+        <v>581</v>
+      </c>
+      <c r="K73" s="4" t="n"/>
+      <c r="L73" s="4" t="inlineStr">
+        <is>
           <t>Period Building Concierge; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
-      <c r="M71" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N71" s="4" t="inlineStr">
+      <c r="M73" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N73" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="O71" s="4" t="inlineStr">
+      <c r="O73" s="4" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O71"/>
+  <autoFilter ref="A1:O73"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
@@ -5438,6 +5576,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C69" r:id="rId68"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C70" r:id="rId69"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C73" r:id="rId72"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily tracker update 2026-07-09
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Flats" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Flats'!$A$1:$O$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Flats'!$A$1:$O$77</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O76"/>
+  <dimension ref="A1:O77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -552,111 +552,111 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>1 bedroom apartment to rent</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/19592796/</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
-        <is>
-          <t>Casson Square, Waterloo, SE1 7GU</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>2 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19692817/</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Belvedere Road, Waterloo, London, SE1</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>SE1</t>
         </is>
       </c>
-      <c r="F2" s="6" t="n">
-        <v>3800</v>
-      </c>
-      <c r="G2" s="6" t="inlineStr">
-        <is>
-          <t>1-Bed</t>
-        </is>
-      </c>
-      <c r="H2" s="6" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="I2" s="6" t="inlineStr">
+      <c r="F2" s="4" t="n">
+        <v>3684</v>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>2-Bed</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J2" s="6" t="n">
-        <v>668</v>
-      </c>
-      <c r="K2" s="6" t="n"/>
-      <c r="L2" s="6" t="inlineStr">
-        <is>
-          <t>1 Bedroom and 1 Bathroom South-facing Aspect for Maximum Natural Light; outdoor space is communal/shared</t>
-        </is>
-      </c>
-      <c r="M2" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N2" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O2" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-08 16:39</t>
+      <c r="J2" s="4" t="n">
+        <v>895</v>
+      </c>
+      <c r="K2" s="4" t="inlineStr"/>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>1st Floor apartment set in the prestigious County Hall development Stylish reception filled with natural light and with space to dine Excellent kitchen with int; outdoor space is communal/shared; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M2" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N2" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O2" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-09 02:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Apartment</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Rightmove</t>
+          <t>OnTheMarket</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>https://www.rightmove.co.uk/properties/90623913</t>
+          <t>https://www.onthemarket.com/details/19592796/</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>Shelton Street, Covent Garden, WC2H</t>
+          <t>Casson Square, Waterloo, SE1 7GU</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>WC2H</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F3" s="6" t="n">
-        <v>3358</v>
+        <v>3800</v>
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr">
@@ -665,118 +665,118 @@
         </is>
       </c>
       <c r="J3" s="6" t="n">
-        <v>623</v>
+        <v>668</v>
       </c>
       <c r="K3" s="6" t="n"/>
       <c r="L3" s="6" t="inlineStr">
         <is>
+          <t>1 Bedroom and 1 Bathroom South-facing Aspect for Maximum Natural Light; outdoor space is communal/shared</t>
+        </is>
+      </c>
+      <c r="M3" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N3" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O3" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-08 16:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Apartment</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Rightmove</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>https://www.rightmove.co.uk/properties/90623913</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Shelton Street, Covent Garden, WC2H</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>WC2H</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>3358</v>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>2-Bed</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Unfurnished</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Communal / shared</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="n">
+        <v>623</v>
+      </c>
+      <c r="K4" s="6" t="n"/>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
           <t>Contemporary, spacious 2 bedroom apartment to rent in Covent Garden, WC2 *AVAILABLE SEPTEMBER* A fantastic contemporary two bedroom, two bathroom flat to rent s; outdoor space is communal/shared; under 650 sq ft</t>
         </is>
       </c>
-      <c r="M3" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N3" s="6" t="inlineStr">
+      <c r="M4" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N4" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="O3" s="6" t="inlineStr">
+      <c r="O4" s="6" t="inlineStr">
         <is>
           <t>2026-07-08 10:39</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Flat</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Rightmove</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>https://www.rightmove.co.uk/properties/87966345</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Belvedere Road, Waterloo, London, SE1</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>SE1</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>3250</v>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>2-Bed</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>Part Furnished</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>680</v>
-      </c>
-      <c r="K4" s="4" t="n"/>
-      <c r="L4" s="4" t="inlineStr">
-        <is>
-          <t>ZERO DEPOSIT AVAILABLE. LONG LET. Located on the South Bank just moments from the London Eye and a range of cultural centers, this fabulous 2 bedroom apartment ; verify balcony/terrace</t>
-        </is>
-      </c>
-      <c r="M4" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N4" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="O4" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-08 01:38</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>Flat</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>OnTheMarket</t>
+          <t>Rightmove</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/9187629/</t>
+          <t>https://www.rightmove.co.uk/properties/87966345</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Casson Square, Waterloo, Southbank Place, London, SE1</t>
+          <t>Belvedere Road, Waterloo, London, SE1</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -785,30 +785,30 @@
         </is>
       </c>
       <c r="F5" s="4" t="n">
-        <v>3990</v>
+        <v>3250</v>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Furnished</t>
+          <t>Part Furnished</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J5" s="4" t="n">
-        <v>537</v>
+        <v>680</v>
       </c>
       <c r="K5" s="4" t="n"/>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>Open plan reception kitchen Bedroom Bathroom 24-hour five-star concierge; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>ZERO DEPOSIT AVAILABLE. LONG LET. Located on the South Bank just moments from the London Eye and a range of cultural centers, this fabulous 2 bedroom apartment ; verify balcony/terrace</t>
         </is>
       </c>
       <c r="M5" s="4" t="inlineStr">
@@ -823,7 +823,7 @@
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-08 00:39</t>
+          <t>2026-07-08 01:38</t>
         </is>
       </c>
     </row>
@@ -840,12 +840,12 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/11391425/</t>
+          <t>https://www.onthemarket.com/details/9187629/</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Casson Square, Waterloo, London, SE1</t>
+          <t>Casson Square, Waterloo, Southbank Place, London, SE1</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -854,7 +854,7 @@
         </is>
       </c>
       <c r="F6" s="4" t="n">
-        <v>3033</v>
+        <v>3990</v>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
@@ -872,12 +872,12 @@
         </is>
       </c>
       <c r="J6" s="4" t="n">
-        <v>397</v>
+        <v>537</v>
       </c>
       <c r="K6" s="4" t="n"/>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>Studio bedroom Open plan kitchen/ reception room Bathroom 24 hour concierge; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Open plan reception kitchen Bedroom Bathroom 24-hour five-star concierge; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M6" s="4" t="inlineStr">
@@ -899,7 +899,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -909,25 +909,25 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19821591/</t>
+          <t>https://www.onthemarket.com/details/11391425/</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Doughty Street, Bloomsbury WC1</t>
+          <t>Casson Square, Waterloo, London, SE1</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>WC1</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F7" s="4" t="n">
-        <v>3445</v>
+        <v>3033</v>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -937,16 +937,16 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J7" s="4" t="n">
-        <v>560</v>
+        <v>397</v>
       </c>
       <c r="K7" s="4" t="n"/>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>16 apartments spread across two Georgian townhouses Studio, one and two bed layouts Student; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Studio bedroom Open plan kitchen/ reception room Bathroom 24 hour concierge; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
@@ -961,14 +961,14 @@
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07 11:38</t>
+          <t>2026-07-08 00:39</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -978,25 +978,25 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/7920965/</t>
+          <t>https://www.onthemarket.com/details/19821591/</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Belvedere Road, Waterloo, Southbank Place, London, SE1</t>
+          <t>Doughty Street, Bloomsbury WC1</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>SE1</t>
+          <t>WC1</t>
         </is>
       </c>
       <c r="F8" s="4" t="n">
-        <v>3950</v>
+        <v>3445</v>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -1006,16 +1006,16 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J8" s="4" t="n">
-        <v>596</v>
+        <v>560</v>
       </c>
       <c r="K8" s="4" t="n"/>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>Fully furnished 1 bedroom 24-hour five-star concierge 18,000 sq ft gym and spa facilities; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>16 apartments spread across two Georgian townhouses Studio, one and two bed layouts Student; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M8" s="4" t="inlineStr">
@@ -1030,14 +1030,14 @@
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07 08:39</t>
+          <t>2026-07-07 11:38</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -1047,25 +1047,25 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19876910/</t>
+          <t>https://www.onthemarket.com/details/7920965/</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Newton Street, Covent Garden, London, WC2B</t>
+          <t>Belvedere Road, Waterloo, Southbank Place, London, SE1</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>WC2B</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>4117</v>
+        <v>3950</v>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1075,176 +1075,176 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Private balcony/terrace</t>
         </is>
       </c>
       <c r="J9" s="4" t="n">
-        <v>848</v>
+        <v>596</v>
       </c>
       <c r="K9" s="4" t="n"/>
       <c r="L9" s="4" t="inlineStr">
         <is>
+          <t>Fully furnished 1 bedroom 24-hour five-star concierge 18,000 sq ft gym and spa facilities; under 650 sq ft; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O9" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07 08:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>2 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19876910/</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Newton Street, Covent Garden, London, WC2B</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>WC2B</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>4117</v>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>2-Bed</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>Communal / shared</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>848</v>
+      </c>
+      <c r="K10" s="4" t="n"/>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
           <t>Stunning 2 bedroom flat arranged on the 1st floor Generous reception room with space to dine; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
-      <c r="M9" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N9" s="4" t="inlineStr">
+      <c r="M10" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N10" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="O9" s="4" t="inlineStr">
+      <c r="O10" s="4" t="inlineStr">
         <is>
           <t>2026-07-07 07:39</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>2 bedroom flat to rent</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>https://www.onthemarket.com/details/19318164/</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>Princeton Street, Bloomsbury, London, WC1R</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>WC1R</t>
         </is>
       </c>
-      <c r="F10" s="6" t="n">
+      <c r="F11" s="6" t="n">
         <v>3684</v>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>2-Bed</t>
         </is>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>Part Furnished</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>Private balcony/terrace</t>
         </is>
       </c>
-      <c r="J10" s="6" t="n">
+      <c r="J11" s="6" t="n">
         <v>649</v>
       </c>
-      <c r="K10" s="6" t="n"/>
-      <c r="L10" s="6" t="inlineStr">
+      <c r="K11" s="6" t="n"/>
+      <c r="L11" s="6" t="inlineStr">
         <is>
           <t>Modern two bedroom, fourth floor flat Bright open plan reception Stylish kitchen featuring a range of modern appliances Two spacious bedrooms with built in stor; under 650 sq ft</t>
         </is>
       </c>
-      <c r="M10" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N10" s="6" t="inlineStr">
+      <c r="M11" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N11" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="O10" s="6" t="inlineStr">
+      <c r="O11" s="6" t="inlineStr">
         <is>
           <t>2026-07-06 20:39</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>1 bedroom flat to rent</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/16574229/</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Casson Square, Waterloo, London, SE1</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>SE1</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="n">
-        <v>3500</v>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>1-Bed</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>Furnished</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>Communal / shared</t>
-        </is>
-      </c>
-      <c r="J11" s="4" t="n">
-        <v>548</v>
-      </c>
-      <c r="K11" s="4" t="n"/>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t>548 sq ft floor area Nearest station 0.1mi.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
-        </is>
-      </c>
-      <c r="M11" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N11" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="O11" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-06 16:39</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -1254,25 +1254,25 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/13719505/</t>
+          <t>https://www.onthemarket.com/details/16574229/</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Bedford Place, Bloomsbury, WC1B</t>
+          <t>Casson Square, Waterloo, London, SE1</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>WC1B</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F12" s="4" t="n">
-        <v>3878</v>
+        <v>3500</v>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -1282,16 +1282,16 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J12" s="4" t="n">
-        <v>961</v>
+        <v>548</v>
       </c>
       <c r="K12" s="4" t="n"/>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t>Two Double Bedroom Apartment High Spec; listed furnished — check if flexible</t>
+          <t>548 sq ft floor area Nearest station 0.1mi.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M12" s="4" t="inlineStr">
@@ -1306,38 +1306,38 @@
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06 15:39</t>
+          <t>2026-07-06 16:39</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Flat</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Rightmove</t>
+          <t>OnTheMarket</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>https://www.rightmove.co.uk/properties/88912341</t>
+          <t>https://www.onthemarket.com/details/13719505/</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Southwark Bridge Road, London, SE1</t>
+          <t>Bedford Place, Bloomsbury, WC1B</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>SE1</t>
+          <t>WC1B</t>
         </is>
       </c>
       <c r="F13" s="4" t="n">
-        <v>4500</v>
+        <v>3878</v>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
@@ -1346,168 +1346,168 @@
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Furnished</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="J13" s="4" t="n"/>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="n">
+        <v>961</v>
+      </c>
       <c r="K13" s="4" t="n"/>
       <c r="L13" s="4" t="inlineStr">
         <is>
+          <t>Two Double Bedroom Apartment High Spec; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M13" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N13" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O13" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06 15:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Flat</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Rightmove</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>https://www.rightmove.co.uk/properties/88912341</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Southwark Bridge Road, London, SE1</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>SE1</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>4500</v>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>2-Bed</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Flexible</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="n"/>
+      <c r="K14" s="4" t="n"/>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
           <t>This stunning apartment boasts floor-to-ceiling windows offering breath taking panoramic views across the London skyline, flooding the space with natural light.; verify balcony/terrace; size not stated</t>
         </is>
       </c>
-      <c r="M13" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N13" s="4" t="inlineStr">
+      <c r="M14" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N14" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="O13" s="4" t="inlineStr">
+      <c r="O14" s="4" t="inlineStr">
         <is>
           <t>2026-07-06 14:39</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>2 bedroom flat to rent</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>https://www.onthemarket.com/details/1990566/</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>Endell Street, Covent Garden, London, WC2H</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>WC2H</t>
         </is>
       </c>
-      <c r="F14" s="6" t="n">
+      <c r="F15" s="6" t="n">
         <v>3400</v>
       </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>2-Bed</t>
         </is>
       </c>
-      <c r="H14" s="6" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>Unfurnished</t>
         </is>
       </c>
-      <c r="I14" s="6" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr">
         <is>
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J14" s="6" t="n"/>
-      <c r="K14" s="6" t="n"/>
-      <c r="L14" s="6" t="inlineStr">
+      <c r="J15" s="6" t="n"/>
+      <c r="K15" s="6" t="n"/>
+      <c r="L15" s="6" t="inlineStr">
         <is>
           <t>Two Bedrooms Two Bathrooms Open plan living room-kitchen First floor; outdoor space is communal/shared; size not stated</t>
         </is>
       </c>
-      <c r="M14" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N14" s="6" t="inlineStr">
+      <c r="M15" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N15" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="O14" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>2 bedroom flat to rent</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/19194043/</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>Great Suffolk Street, Southwark, London, SE1</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>SE1</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="n">
-        <v>3100</v>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>2-Bed</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>Furnished</t>
-        </is>
-      </c>
-      <c r="I15" s="4" t="inlineStr">
-        <is>
-          <t>Juliet only</t>
-        </is>
-      </c>
-      <c r="J15" s="4" t="n">
-        <v>638</v>
-      </c>
-      <c r="K15" s="4" t="n"/>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>Stylish 2 bedroom flat set on the 5th floor Large reception room with Juliet balcony Modern kitchen 2 lovely double bedroom; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
-        </is>
-      </c>
-      <c r="M15" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N15" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="O15" s="4" t="inlineStr">
+      <c r="O15" s="6" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
@@ -1516,7 +1516,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -1526,25 +1526,25 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19099769/</t>
+          <t>https://www.onthemarket.com/details/19194043/</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Fletcher Buildings,, Covent Garden, London, WC2B</t>
+          <t>Great Suffolk Street, Southwark, London, SE1</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>WC2B</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F16" s="4" t="n">
-        <v>3792</v>
+        <v>3100</v>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -1554,16 +1554,16 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Juliet only</t>
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>320</v>
+        <v>638</v>
       </c>
       <c r="K16" s="4" t="n"/>
       <c r="L16" s="4" t="inlineStr">
         <is>
-          <t>Bright and airy one bedroom apartment in a prime Central London location Well proportioned reception with high ceilings and neutral décor Generous double bedroo; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Stylish 2 bedroom flat set on the 5th floor Large reception room with Juliet balcony Modern kitchen 2 lovely double bedroom; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M16" s="4" t="inlineStr">
@@ -1585,7 +1585,7 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -1595,25 +1595,25 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/6356511/</t>
+          <t>https://www.onthemarket.com/details/19099769/</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Great James Street, Bloomsbury, London, WC1N</t>
+          <t>Fletcher Buildings,, Covent Garden, London, WC2B</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>WC1N</t>
+          <t>WC2B</t>
         </is>
       </c>
       <c r="F17" s="4" t="n">
-        <v>3683</v>
+        <v>3792</v>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -1623,16 +1623,16 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J17" s="4" t="n">
-        <v>928</v>
+        <v>320</v>
       </c>
       <c r="K17" s="4" t="n"/>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>Spacious Split Level Apartment Large Terrace Wooden Flooring Nearest tubes: Chancery Lane, Russell Square &amp; Holborn; listed furnished — check if flexible</t>
+          <t>Bright and airy one bedroom apartment in a prime Central London location Well proportioned reception with high ceilings and neutral décor Generous double bedroo; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M17" s="4" t="inlineStr">
@@ -1654,7 +1654,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -1664,25 +1664,25 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19453032/</t>
+          <t>https://www.onthemarket.com/details/6356511/</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Maiden Lane, Covent Garden, London, WC2E</t>
+          <t>Great James Street, Bloomsbury, London, WC1N</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>WC2E</t>
+          <t>WC1N</t>
         </is>
       </c>
       <c r="F18" s="4" t="n">
-        <v>3684</v>
+        <v>3683</v>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1692,16 +1692,16 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Private balcony/terrace</t>
         </is>
       </c>
       <c r="J18" s="4" t="n">
-        <v>630</v>
+        <v>928</v>
       </c>
       <c r="K18" s="4" t="n"/>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat arranged on the 4th floor Bright and spacious reception room Smart dining room Modern kitchen; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Spacious Split Level Apartment Large Terrace Wooden Flooring Nearest tubes: Chancery Lane, Russell Square &amp; Holborn; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M18" s="4" t="inlineStr">
@@ -1733,21 +1733,21 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19592443/</t>
+          <t>https://www.onthemarket.com/details/19453032/</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Regent Square, Bloomsbury, London, WC1H</t>
+          <t>Maiden Lane, Covent Garden, London, WC2E</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>WC1H</t>
+          <t>WC2E</t>
         </is>
       </c>
       <c r="F19" s="4" t="n">
-        <v>4312</v>
+        <v>3684</v>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
@@ -1761,117 +1761,117 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J19" s="4" t="n">
-        <v>487</v>
+        <v>630</v>
       </c>
       <c r="K19" s="4" t="n"/>
       <c r="L19" s="4" t="inlineStr">
         <is>
+          <t>1 bedroom flat arranged on the 4th floor Bright and spacious reception room Smart dining room Modern kitchen; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M19" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N19" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O19" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>1 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19592443/</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Regent Square, Bloomsbury, London, WC1H</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>WC1H</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>4312</v>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>1-Bed</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J20" s="4" t="n">
+        <v>487</v>
+      </c>
+      <c r="K20" s="4" t="n"/>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
           <t>Fantastic one bedroom apartment Set within beautiful period conversion Boasts ample interior space arranged over the second floor Wonderful balcony overlooking ; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
-      <c r="M19" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N19" s="4" t="inlineStr">
+      <c r="M20" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N20" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="O19" s="4" t="inlineStr">
+      <c r="O20" s="4" t="inlineStr">
         <is>
           <t>2026-07-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Apartment</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Rightmove</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>https://www.rightmove.co.uk/properties/89143989</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Waterloo Road, Southwark, SE1</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>SE1</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="n">
-        <v>4346</v>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>2-Bed</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>Part Furnished</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>Private balcony/terrace</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="n">
-        <v>1385</v>
-      </c>
-      <c r="K20" s="2" t="n"/>
-      <c r="L20" s="2" t="inlineStr">
-        <is>
-          <t>Two bedroom apartment with incredible views Waterloo Road SE1 250 Waterloo Road is an exciting new rental development conveniently located on Waterloo Road, SE1</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N20" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="O20" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>Apartment</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>OnTheMarket</t>
+          <t>Rightmove</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/4473051/</t>
+          <t>https://www.rightmove.co.uk/properties/89143989</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1908,7 +1908,7 @@
       <c r="K21" s="2" t="n"/>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>Spectacular Views Waterloo</t>
+          <t>Two bedroom apartment with incredible views Waterloo Road SE1 250 Waterloo Road is an exciting new rental development conveniently located on Waterloo Road, SE1</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
@@ -1930,7 +1930,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1940,12 +1940,12 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19728858/</t>
+          <t>https://www.onthemarket.com/details/4473051/</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Waterloo Road, London SE1</t>
+          <t>Waterloo Road, Southwark, SE1</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1954,7 +1954,7 @@
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>4350</v>
+        <v>4346</v>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
@@ -1963,7 +1963,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Part Furnished</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -1972,12 +1972,12 @@
         </is>
       </c>
       <c r="J22" s="2" t="n">
-        <v>1140</v>
+        <v>1385</v>
       </c>
       <c r="K22" s="2" t="n"/>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>Two Bedrooms Two Bathrooms</t>
+          <t>Spectacular Views Waterloo</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
@@ -1999,7 +1999,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -2009,12 +2009,12 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/6248222/</t>
+          <t>https://www.onthemarket.com/details/19728858/</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Nelson Square, Southwark, London, SE1</t>
+          <t>Waterloo Road, London SE1</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -2023,7 +2023,7 @@
         </is>
       </c>
       <c r="F23" s="2" t="n">
-        <v>3150</v>
+        <v>4350</v>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
@@ -2032,7 +2032,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -2041,12 +2041,12 @@
         </is>
       </c>
       <c r="J23" s="2" t="n">
-        <v>809</v>
+        <v>1140</v>
       </c>
       <c r="K23" s="2" t="n"/>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>Dishwasher Range / Oven</t>
+          <t>Two Bedrooms Two Bathrooms</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
@@ -2068,7 +2068,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2078,21 +2078,21 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19663010/</t>
+          <t>https://www.onthemarket.com/details/6248222/</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Guilford Street, Bloomsbury, London, WC1N</t>
+          <t>Nelson Square, Southwark, London, SE1</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>WC1N</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>3684</v>
+        <v>3150</v>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Part Furnished</t>
+          <t>Unfurnished</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -2110,94 +2110,94 @@
         </is>
       </c>
       <c r="J24" s="2" t="n">
-        <v>691</v>
+        <v>809</v>
       </c>
       <c r="K24" s="2" t="n"/>
       <c r="L24" s="2" t="inlineStr">
         <is>
+          <t>Dishwasher Range / Oven</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19663010/</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Guilford Street, Bloomsbury, London, WC1N</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>WC1N</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>3684</v>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>2-Bed</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Part Furnished</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="n">
+        <v>691</v>
+      </c>
+      <c r="K25" s="2" t="n"/>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
           <t>Superb 2 bedroom flat on lower ground floor Modern open-plan kitchen with integrated appliance Spacious reception room leading to lovely private patio 2 well-pr</t>
         </is>
       </c>
-      <c r="M24" s="2" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N24" s="2" t="inlineStr">
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="O24" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>2 bedroom apartment to rent</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/19809694/</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>Shaftesbury Avenue, Soho, W1D</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="inlineStr">
-        <is>
-          <t>W1D</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="n">
-        <v>3553</v>
-      </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>2-Bed</t>
-        </is>
-      </c>
-      <c r="H25" s="6" t="inlineStr">
-        <is>
-          <t>Flexible</t>
-        </is>
-      </c>
-      <c r="I25" s="6" t="inlineStr">
-        <is>
-          <t>Communal / shared</t>
-        </is>
-      </c>
-      <c r="J25" s="6" t="n">
-        <v>603</v>
-      </c>
-      <c r="K25" s="6" t="n"/>
-      <c r="L25" s="6" t="inlineStr">
-        <is>
-          <t>Beautifully Refurbished Secondary Glazing; outdoor space is communal/shared; under 650 sq ft</t>
-        </is>
-      </c>
-      <c r="M25" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N25" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O25" s="6" t="inlineStr">
+      <c r="O25" s="2" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
@@ -2216,12 +2216,12 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/13368018/</t>
+          <t>https://www.onthemarket.com/details/19809694/</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>Shaftesbury Avenue , Soho, W1D</t>
+          <t>Shaftesbury Avenue, Soho, W1D</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
@@ -2230,7 +2230,7 @@
         </is>
       </c>
       <c r="F26" s="6" t="n">
-        <v>3987</v>
+        <v>3553</v>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
@@ -2248,12 +2248,12 @@
         </is>
       </c>
       <c r="J26" s="6" t="n">
-        <v>671</v>
+        <v>603</v>
       </c>
       <c r="K26" s="6" t="n"/>
       <c r="L26" s="6" t="inlineStr">
         <is>
-          <t>Pet friendly Wooden Floors Student; outdoor space is communal/shared</t>
+          <t>Beautifully Refurbished Secondary Glazing; outdoor space is communal/shared; under 650 sq ft</t>
         </is>
       </c>
       <c r="M26" s="6" t="inlineStr">
@@ -2285,12 +2285,12 @@
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19627828/</t>
+          <t>https://www.onthemarket.com/details/13368018/</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>Shaftesbury Avenue, Soho, W1D</t>
+          <t>Shaftesbury Avenue , Soho, W1D</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
@@ -2317,12 +2317,12 @@
         </is>
       </c>
       <c r="J27" s="6" t="n">
-        <v>802</v>
+        <v>671</v>
       </c>
       <c r="K27" s="6" t="n"/>
       <c r="L27" s="6" t="inlineStr">
         <is>
-          <t>Built in Storage Pet Friendly; outdoor space is communal/shared</t>
+          <t>Pet friendly Wooden Floors Student; outdoor space is communal/shared</t>
         </is>
       </c>
       <c r="M27" s="6" t="inlineStr">
@@ -2344,7 +2344,7 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
@@ -2354,12 +2354,12 @@
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19600564/</t>
+          <t>https://www.onthemarket.com/details/19627828/</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>Rupert Court, Soho, W1D</t>
+          <t>Shaftesbury Avenue, Soho, W1D</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
@@ -2368,11 +2368,11 @@
         </is>
       </c>
       <c r="F28" s="6" t="n">
-        <v>3163</v>
+        <v>3987</v>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
@@ -2385,11 +2385,13 @@
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J28" s="6" t="n"/>
+      <c r="J28" s="6" t="n">
+        <v>802</v>
+      </c>
       <c r="K28" s="6" t="n"/>
       <c r="L28" s="6" t="inlineStr">
         <is>
-          <t>Beautifully Refurbished Pet friendly; outdoor space is communal/shared; size not stated</t>
+          <t>Built in Storage Pet Friendly; outdoor space is communal/shared</t>
         </is>
       </c>
       <c r="M28" s="6" t="inlineStr">
@@ -2421,17 +2423,17 @@
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/10862827/</t>
+          <t>https://www.onthemarket.com/details/19600564/</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>Rupert Court, Soho W1</t>
+          <t>Rupert Court, Soho, W1D</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>W1D</t>
         </is>
       </c>
       <c r="F29" s="6" t="n">
@@ -2444,7 +2446,7 @@
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
@@ -2452,13 +2454,11 @@
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J29" s="6" t="n">
-        <v>603</v>
-      </c>
+      <c r="J29" s="6" t="n"/>
       <c r="K29" s="6" t="n"/>
       <c r="L29" s="6" t="inlineStr">
         <is>
-          <t>One bedroom One shower room; outdoor space is communal/shared; under 650 sq ft</t>
+          <t>Beautifully Refurbished Pet friendly; outdoor space is communal/shared; size not stated</t>
         </is>
       </c>
       <c r="M29" s="6" t="inlineStr">
@@ -2480,7 +2480,7 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
@@ -2490,21 +2490,21 @@
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19845642/</t>
+          <t>https://www.onthemarket.com/details/10862827/</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>Shelton Street, Covent Garden, London, WC2H</t>
+          <t>Rupert Court, Soho W1</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>WC2H</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="F30" s="6" t="n">
-        <v>3142</v>
+        <v>3163</v>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Unfurnished</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
@@ -2522,12 +2522,12 @@
         </is>
       </c>
       <c r="J30" s="6" t="n">
-        <v>480</v>
+        <v>603</v>
       </c>
       <c r="K30" s="6" t="n"/>
       <c r="L30" s="6" t="inlineStr">
         <is>
-          <t>Superb one bedroom flat arranged on the second floor Spacious reception/kitchen with ample dining space; outdoor space is communal/shared; under 650 sq ft</t>
+          <t>One bedroom One shower room; outdoor space is communal/shared; under 650 sq ft</t>
         </is>
       </c>
       <c r="M30" s="6" t="inlineStr">
@@ -2549,7 +2549,7 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
@@ -2559,21 +2559,21 @@
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19603496/</t>
+          <t>https://www.onthemarket.com/details/19845642/</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Arne Street, Covent Garden, WC2E</t>
+          <t>Shelton Street, Covent Garden, London, WC2H</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>WC2E</t>
+          <t>WC2H</t>
         </is>
       </c>
       <c r="F31" s="6" t="n">
-        <v>3250</v>
+        <v>3142</v>
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
@@ -2582,7 +2582,7 @@
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr">
@@ -2591,12 +2591,12 @@
         </is>
       </c>
       <c r="J31" s="6" t="n">
-        <v>514</v>
+        <v>480</v>
       </c>
       <c r="K31" s="6" t="n"/>
       <c r="L31" s="6" t="inlineStr">
         <is>
-          <t>Council Tax Band G 514 sq ft floor area; outdoor space is communal/shared; under 650 sq ft</t>
+          <t>Superb one bedroom flat arranged on the second floor Spacious reception/kitchen with ample dining space; outdoor space is communal/shared; under 650 sq ft</t>
         </is>
       </c>
       <c r="M31" s="6" t="inlineStr">
@@ -2618,7 +2618,7 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
@@ -2628,21 +2628,21 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/14179323/</t>
+          <t>https://www.onthemarket.com/details/19603496/</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>Bloomsbury Square, Bloomsbury, Covent Garden, London, WC1A</t>
+          <t>Arne Street, Covent Garden, WC2E</t>
         </is>
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>WC1A</t>
+          <t>WC2E</t>
         </is>
       </c>
       <c r="F32" s="6" t="n">
-        <v>3500</v>
+        <v>3250</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -2651,7 +2651,7 @@
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>Part Furnished</t>
+          <t>Unfurnished</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
@@ -2660,12 +2660,12 @@
         </is>
       </c>
       <c r="J32" s="6" t="n">
-        <v>734</v>
+        <v>514</v>
       </c>
       <c r="K32" s="6" t="n"/>
       <c r="L32" s="6" t="inlineStr">
         <is>
-          <t>Stunning Period Conversion Hardwood Flooring Multi-Room Sound System and Mood Lighting Throughout Contemporary Kitchen &amp; Bathroom; outdoor space is communal/shared</t>
+          <t>Council Tax Band G 514 sq ft floor area; outdoor space is communal/shared; under 650 sq ft</t>
         </is>
       </c>
       <c r="M32" s="6" t="inlineStr">
@@ -2697,21 +2697,21 @@
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19823664/</t>
+          <t>https://www.onthemarket.com/details/14179323/</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>Bedford Court Mansions, Adeline Place, Bloomsbury, London, WC1B</t>
+          <t>Bloomsbury Square, Bloomsbury, Covent Garden, London, WC1A</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>WC1B</t>
+          <t>WC1A</t>
         </is>
       </c>
       <c r="F33" s="6" t="n">
-        <v>3141</v>
+        <v>3500</v>
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
@@ -2720,21 +2720,21 @@
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Part Furnished</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J33" s="6" t="n">
-        <v>573</v>
+        <v>734</v>
       </c>
       <c r="K33" s="6" t="n"/>
       <c r="L33" s="6" t="inlineStr">
         <is>
-          <t>One Bedroom Finished to high standard Lift Access Separate Kitchen; under 650 sq ft</t>
+          <t>Stunning Period Conversion Hardwood Flooring Multi-Room Sound System and Mood Lighting Throughout Contemporary Kitchen &amp; Bathroom; outdoor space is communal/shared</t>
         </is>
       </c>
       <c r="M33" s="6" t="inlineStr">
@@ -2756,7 +2756,7 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
@@ -2766,21 +2766,21 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/15813612/</t>
+          <t>https://www.onthemarket.com/details/19823664/</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>Bloomsbury Square, Bloomsbury, WC1A</t>
+          <t>Bedford Court Mansions, Adeline Place, Bloomsbury, London, WC1B</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>WC1A</t>
+          <t>WC1B</t>
         </is>
       </c>
       <c r="F34" s="6" t="n">
-        <v>3142</v>
+        <v>3141</v>
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
@@ -2798,12 +2798,12 @@
         </is>
       </c>
       <c r="J34" s="6" t="n">
-        <v>539</v>
+        <v>573</v>
       </c>
       <c r="K34" s="6" t="n"/>
       <c r="L34" s="6" t="inlineStr">
         <is>
-          <t>Large Double Bedroom Period Features Student; under 650 sq ft</t>
+          <t>One Bedroom Finished to high standard Lift Access Separate Kitchen; under 650 sq ft</t>
         </is>
       </c>
       <c r="M34" s="6" t="inlineStr">
@@ -2825,7 +2825,7 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
@@ -2835,17 +2835,17 @@
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19736445/</t>
+          <t>https://www.onthemarket.com/details/15813612/</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>Millman Street, Bloomsbury, London, WC1N</t>
+          <t>Bloomsbury Square, Bloomsbury, WC1A</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>WC1N</t>
+          <t>WC1A</t>
         </is>
       </c>
       <c r="F35" s="6" t="n">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>Part Furnished</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
@@ -2867,94 +2867,94 @@
         </is>
       </c>
       <c r="J35" s="6" t="n">
-        <v>542</v>
+        <v>539</v>
       </c>
       <c r="K35" s="6" t="n"/>
       <c r="L35" s="6" t="inlineStr">
         <is>
+          <t>Large Double Bedroom Period Features Student; under 650 sq ft</t>
+        </is>
+      </c>
+      <c r="M35" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N35" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O35" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>1 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19736445/</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>Millman Street, Bloomsbury, London, WC1N</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>WC1N</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="n">
+        <v>3142</v>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>1-Bed</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t>Part Furnished</t>
+        </is>
+      </c>
+      <c r="I36" s="6" t="inlineStr">
+        <is>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J36" s="6" t="n">
+        <v>542</v>
+      </c>
+      <c r="K36" s="6" t="n"/>
+      <c r="L36" s="6" t="inlineStr">
+        <is>
           <t>Fantastic 1 bedroom flat arranged on the ground floor Set within a lovely residential block; under 650 sq ft</t>
         </is>
       </c>
-      <c r="M35" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N35" s="6" t="inlineStr">
+      <c r="M36" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N36" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="O35" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>Flat</t>
-        </is>
-      </c>
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>Rightmove</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>https://www.rightmove.co.uk/properties/90435384</t>
-        </is>
-      </c>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>251 SOUTHWARK BRIDGE ROAD, LONDON, SE1, Elephant and Castle, London, SE1</t>
-        </is>
-      </c>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>SE1</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="n">
-        <v>4250</v>
-      </c>
-      <c r="G36" s="4" t="inlineStr">
-        <is>
-          <t>1-Bed</t>
-        </is>
-      </c>
-      <c r="H36" s="4" t="inlineStr">
-        <is>
-          <t>Part Furnished</t>
-        </is>
-      </c>
-      <c r="I36" s="4" t="inlineStr">
-        <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="J36" s="4" t="n">
-        <v>520</v>
-      </c>
-      <c r="K36" s="4" t="n"/>
-      <c r="L36" s="4" t="inlineStr">
-        <is>
-          <t>ZERO DEPOSIT AVAILABLE. SHORT LET. Set on the 21st floor, this 1 bedroom flat boasts well arranged interiors including a large reception room, a modern open-pla; verify balcony/terrace; under 650 sq ft</t>
-        </is>
-      </c>
-      <c r="M36" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N36" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="O36" s="4" t="inlineStr">
+      <c r="O36" s="6" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
@@ -2973,7 +2973,7 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>https://www.rightmove.co.uk/properties/90432648</t>
+          <t>https://www.rightmove.co.uk/properties/90435384</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -2987,7 +2987,7 @@
         </is>
       </c>
       <c r="F37" s="4" t="n">
-        <v>3000</v>
+        <v>4250</v>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
@@ -3010,7 +3010,7 @@
       <c r="K37" s="4" t="n"/>
       <c r="L37" s="4" t="inlineStr">
         <is>
-          <t>ZERO DEPOSIT AVAILABLE. LONG LET. Set on the 21st floor, this 1 bedroom flat boasts well arranged interiors including a large reception room, a modern open-plan; verify balcony/terrace; under 650 sq ft</t>
+          <t>ZERO DEPOSIT AVAILABLE. SHORT LET. Set on the 21st floor, this 1 bedroom flat boasts well arranged interiors including a large reception room, a modern open-pla; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M37" s="4" t="inlineStr">
@@ -3032,31 +3032,31 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>Flat</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>OnTheMarket</t>
+          <t>Rightmove</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/4220060/</t>
+          <t>https://www.rightmove.co.uk/properties/90432648</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Carnaby Street, Soho, W1F</t>
+          <t>251 SOUTHWARK BRIDGE ROAD, LONDON, SE1, Elephant and Castle, London, SE1</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>W1F</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F38" s="4" t="n">
-        <v>3640</v>
+        <v>3000</v>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
@@ -3065,7 +3065,7 @@
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Part Furnished</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
@@ -3074,12 +3074,12 @@
         </is>
       </c>
       <c r="J38" s="4" t="n">
-        <v>553</v>
+        <v>520</v>
       </c>
       <c r="K38" s="4" t="n"/>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>One bedroom apartment Newly refurbished; verify balcony/terrace; under 650 sq ft</t>
+          <t>ZERO DEPOSIT AVAILABLE. LONG LET. Set on the 21st floor, this 1 bedroom flat boasts well arranged interiors including a large reception room, a modern open-plan; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
@@ -3101,7 +3101,7 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
@@ -3111,12 +3111,12 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/8022324/</t>
+          <t>https://www.onthemarket.com/details/4220060/</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Golden Square, Soho, London, W1F</t>
+          <t>Carnaby Street, Soho, W1F</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
@@ -3125,7 +3125,7 @@
         </is>
       </c>
       <c r="F39" s="4" t="n">
-        <v>3467</v>
+        <v>3640</v>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
@@ -3134,7 +3134,7 @@
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>Furnished</t>
+          <t>Unfurnished</t>
         </is>
       </c>
       <c r="I39" s="4" t="inlineStr">
@@ -3143,12 +3143,12 @@
         </is>
       </c>
       <c r="J39" s="4" t="n">
-        <v>608</v>
+        <v>553</v>
       </c>
       <c r="K39" s="4" t="n"/>
       <c r="L39" s="4" t="inlineStr">
         <is>
-          <t>608 sq ft floor area Nearest station 0.1mi.; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>One bedroom apartment Newly refurbished; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M39" s="4" t="inlineStr">
@@ -3170,7 +3170,7 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
@@ -3180,25 +3180,25 @@
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19852978/</t>
+          <t>https://www.onthemarket.com/details/8022324/</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Newport Court, Covent Garden, London, WC2H</t>
+          <t>Golden Square, Soho, London, W1F</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>WC2H</t>
+          <t>W1F</t>
         </is>
       </c>
       <c r="F40" s="4" t="n">
-        <v>4334</v>
+        <v>3467</v>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
@@ -3208,16 +3208,16 @@
       </c>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J40" s="4" t="n">
-        <v>858</v>
+        <v>608</v>
       </c>
       <c r="K40" s="4" t="n"/>
       <c r="L40" s="4" t="inlineStr">
         <is>
-          <t>Splendid two bedroom flat Ample interiors; listed furnished — check if flexible</t>
+          <t>608 sq ft floor area Nearest station 0.1mi.; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M40" s="4" t="inlineStr">
@@ -3239,7 +3239,7 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
@@ -3249,21 +3249,21 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/16157050/</t>
+          <t>https://www.onthemarket.com/details/19852978/</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Brewer Street, Soho, W1F</t>
+          <t>Newport Court, Covent Garden, London, WC2H</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>W1F</t>
+          <t>WC2H</t>
         </is>
       </c>
       <c r="F41" s="4" t="n">
-        <v>3142</v>
+        <v>4334</v>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
@@ -3277,16 +3277,16 @@
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Private balcony/terrace</t>
         </is>
       </c>
       <c r="J41" s="4" t="n">
-        <v>730</v>
+        <v>858</v>
       </c>
       <c r="K41" s="4" t="n"/>
       <c r="L41" s="4" t="inlineStr">
         <is>
-          <t>730 sqft Secure Entrance; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>Splendid two bedroom flat Ample interiors; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M41" s="4" t="inlineStr">
@@ -3308,7 +3308,7 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
@@ -3318,25 +3318,25 @@
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/9956499/</t>
+          <t>https://www.onthemarket.com/details/16157050/</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Richmond Buildings, Soho, W1D</t>
+          <t>Brewer Street, Soho, W1F</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>W1D</t>
+          <t>W1F</t>
         </is>
       </c>
       <c r="F42" s="4" t="n">
-        <v>3835</v>
+        <v>3142</v>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
@@ -3346,16 +3346,16 @@
       </c>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J42" s="4" t="n">
-        <v>521</v>
+        <v>730</v>
       </c>
       <c r="K42" s="4" t="n"/>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Council tax band: F 521 sq ft floor area; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>730 sqft Secure Entrance; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
@@ -3387,12 +3387,12 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19786051/</t>
+          <t>https://www.onthemarket.com/details/9956499/</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Old Compton Street, Soho, London, W1D</t>
+          <t>Richmond Buildings, Soho, W1D</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
@@ -3401,7 +3401,7 @@
         </is>
       </c>
       <c r="F43" s="4" t="n">
-        <v>3600</v>
+        <v>3835</v>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
@@ -3415,16 +3415,16 @@
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J43" s="4" t="n">
-        <v>432</v>
+        <v>521</v>
       </c>
       <c r="K43" s="4" t="n"/>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>432 sq ft floor area Nearest station 0.1mi. Furnished Nearest school 0.2mi.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Council tax band: F 521 sq ft floor area; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
@@ -3446,7 +3446,7 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
@@ -3456,17 +3456,17 @@
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19828226/</t>
+          <t>https://www.onthemarket.com/details/19786051/</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>TCRW SOHO, Fareham Street, W1F</t>
+          <t>Old Compton Street, Soho, London, W1D</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>W1F</t>
+          <t>W1D</t>
         </is>
       </c>
       <c r="F44" s="4" t="n">
@@ -3484,16 +3484,16 @@
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J44" s="4" t="n">
-        <v>656</v>
+        <v>432</v>
       </c>
       <c r="K44" s="4" t="n"/>
       <c r="L44" s="4" t="inlineStr">
         <is>
-          <t>Concierge service Highly sought-after Zone 1 location; verify balcony/terrace; listed furnished — check if flexible</t>
+          <t>432 sq ft floor area Nearest station 0.1mi. Furnished Nearest school 0.2mi.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M44" s="4" t="inlineStr">
@@ -3515,7 +3515,7 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
@@ -3525,25 +3525,25 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/11345150/</t>
+          <t>https://www.onthemarket.com/details/19828226/</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Shaftesbury Avenue, Covent Garden, London, WC2H</t>
+          <t>TCRW SOHO, Fareham Street, W1F</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>WC2H</t>
+          <t>W1F</t>
         </is>
       </c>
       <c r="F45" s="4" t="n">
-        <v>3575</v>
+        <v>3600</v>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr">
@@ -3553,16 +3553,16 @@
       </c>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J45" s="4" t="n">
-        <v>870</v>
+        <v>656</v>
       </c>
       <c r="K45" s="4" t="n"/>
       <c r="L45" s="4" t="inlineStr">
         <is>
-          <t>870 sq ft floor area Nearest station 0.1mi.; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>Concierge service Highly sought-after Zone 1 location; verify balcony/terrace; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M45" s="4" t="inlineStr">
@@ -3594,21 +3594,21 @@
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/4747672/</t>
+          <t>https://www.onthemarket.com/details/11345150/</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Townsend House, Deans Street, Soho W1D</t>
+          <t>Shaftesbury Avenue, Covent Garden, London, WC2H</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>W1D</t>
+          <t>WC2H</t>
         </is>
       </c>
       <c r="F46" s="4" t="n">
-        <v>3850</v>
+        <v>3575</v>
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
@@ -3622,14 +3622,16 @@
       </c>
       <c r="I46" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="J46" s="4" t="n"/>
+          <t>Communal / shared</t>
+        </is>
+      </c>
+      <c r="J46" s="4" t="n">
+        <v>870</v>
+      </c>
       <c r="K46" s="4" t="n"/>
       <c r="L46" s="4" t="inlineStr">
         <is>
-          <t>Close to Local Shops Close to Public Transport; verify balcony/terrace; size not stated; listed furnished — check if flexible</t>
+          <t>870 sq ft floor area Nearest station 0.1mi.; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M46" s="4" t="inlineStr">
@@ -3651,7 +3653,7 @@
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
@@ -3661,30 +3663,30 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19628367/</t>
+          <t>https://www.onthemarket.com/details/4747672/</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Carnaby Street, Soho W1</t>
+          <t>Townsend House, Deans Street, Soho W1D</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>W1D</t>
         </is>
       </c>
       <c r="F47" s="4" t="n">
-        <v>3640</v>
+        <v>3850</v>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Furnished</t>
         </is>
       </c>
       <c r="I47" s="4" t="inlineStr">
@@ -3692,13 +3694,11 @@
           <t>Not stated</t>
         </is>
       </c>
-      <c r="J47" s="4" t="n">
-        <v>549</v>
-      </c>
+      <c r="J47" s="4" t="n"/>
       <c r="K47" s="4" t="n"/>
       <c r="L47" s="4" t="inlineStr">
         <is>
-          <t>One bedroom One shower room, ensuite; verify balcony/terrace; under 650 sq ft</t>
+          <t>Close to Local Shops Close to Public Transport; verify balcony/terrace; size not stated; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M47" s="4" t="inlineStr">
@@ -3730,17 +3730,17 @@
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/13524814/</t>
+          <t>https://www.onthemarket.com/details/19628367/</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Carnaby Street, Soho, W1F</t>
+          <t>Carnaby Street, Soho W1</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>W1F</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="F48" s="4" t="n">
@@ -3753,7 +3753,7 @@
       </c>
       <c r="H48" s="4" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Unfurnished</t>
         </is>
       </c>
       <c r="I48" s="4" t="inlineStr">
@@ -3762,12 +3762,12 @@
         </is>
       </c>
       <c r="J48" s="4" t="n">
-        <v>552</v>
+        <v>549</v>
       </c>
       <c r="K48" s="4" t="n"/>
       <c r="L48" s="4" t="inlineStr">
         <is>
-          <t>Recently Refurbished Apartment Original Features Student; verify balcony/terrace; under 650 sq ft</t>
+          <t>One bedroom One shower room, ensuite; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M48" s="4" t="inlineStr">
@@ -3799,21 +3799,21 @@
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/18690047/</t>
+          <t>https://www.onthemarket.com/details/13524814/</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>Duck Lane, Soho W1</t>
+          <t>Carnaby Street, Soho, W1F</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>W1F</t>
         </is>
       </c>
       <c r="F49" s="4" t="n">
-        <v>3077</v>
+        <v>3640</v>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
@@ -3822,7 +3822,7 @@
       </c>
       <c r="H49" s="4" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I49" s="4" t="inlineStr">
@@ -3831,12 +3831,12 @@
         </is>
       </c>
       <c r="J49" s="4" t="n">
-        <v>581</v>
+        <v>552</v>
       </c>
       <c r="K49" s="4" t="n"/>
       <c r="L49" s="4" t="inlineStr">
         <is>
-          <t>One bedroom One bathroom; verify balcony/terrace; under 650 sq ft</t>
+          <t>Recently Refurbished Apartment Original Features Student; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M49" s="4" t="inlineStr">
@@ -3868,17 +3868,17 @@
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/18690128/</t>
+          <t>https://www.onthemarket.com/details/18690047/</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>Duck Lane, Soho, W1F</t>
+          <t>Duck Lane, Soho W1</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>W1F</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="F50" s="4" t="n">
@@ -3900,12 +3900,12 @@
         </is>
       </c>
       <c r="J50" s="4" t="n">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="K50" s="4" t="n"/>
       <c r="L50" s="4" t="inlineStr">
         <is>
-          <t>One Double bedroom Quaint Road; verify balcony/terrace; under 650 sq ft</t>
+          <t>One bedroom One bathroom; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M50" s="4" t="inlineStr">
@@ -3937,12 +3937,12 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/18680649/</t>
+          <t>https://www.onthemarket.com/details/18690128/</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>Duck Lane, Soho W1F</t>
+          <t>Duck Lane, Soho, W1F</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="H51" s="4" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Unfurnished</t>
         </is>
       </c>
       <c r="I51" s="4" t="inlineStr">
@@ -3969,12 +3969,12 @@
         </is>
       </c>
       <c r="J51" s="4" t="n">
-        <v>575</v>
+        <v>580</v>
       </c>
       <c r="K51" s="4" t="n"/>
       <c r="L51" s="4" t="inlineStr">
         <is>
-          <t>Modern Throughout Wooden Flooring Throughout; verify balcony/terrace; under 650 sq ft</t>
+          <t>One Double bedroom Quaint Road; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M51" s="4" t="inlineStr">
@@ -4006,21 +4006,21 @@
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/15707269/</t>
+          <t>https://www.onthemarket.com/details/18680649/</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>Casson Square, London, Waterloo, United Kingdom, SE1</t>
+          <t>Duck Lane, Soho W1F</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>SE1</t>
+          <t>W1F</t>
         </is>
       </c>
       <c r="F52" s="4" t="n">
-        <v>4050</v>
+        <v>3077</v>
       </c>
       <c r="G52" s="4" t="inlineStr">
         <is>
@@ -4029,21 +4029,21 @@
       </c>
       <c r="H52" s="4" t="inlineStr">
         <is>
-          <t>Furnished</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I52" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J52" s="4" t="n">
-        <v>514</v>
+        <v>575</v>
       </c>
       <c r="K52" s="4" t="n"/>
       <c r="L52" s="4" t="inlineStr">
         <is>
-          <t>Bedroom Bathroom Open-plan reception/kitchen 24 hour concierge; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Modern Throughout Wooden Flooring Throughout; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M52" s="4" t="inlineStr">
@@ -4075,12 +4075,12 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/9568931/</t>
+          <t>https://www.onthemarket.com/details/15707269/</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>Casson Square, Waterloo, Southbank Place, London, SE1</t>
+          <t>Casson Square, London, Waterloo, United Kingdom, SE1</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
@@ -4089,7 +4089,7 @@
         </is>
       </c>
       <c r="F53" s="4" t="n">
-        <v>4250</v>
+        <v>4050</v>
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
@@ -4103,16 +4103,16 @@
       </c>
       <c r="I53" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J53" s="4" t="n">
-        <v>644</v>
+        <v>514</v>
       </c>
       <c r="K53" s="4" t="n"/>
       <c r="L53" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom 1 bathroom Open-plan reception kitchen 24-hour five-star concierge; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Bedroom Bathroom Open-plan reception/kitchen 24 hour concierge; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M53" s="4" t="inlineStr">
@@ -4134,7 +4134,7 @@
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom end of terrace house to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
@@ -4144,21 +4144,25 @@
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19811489/</t>
+          <t>https://www.onthemarket.com/details/9568931/</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>Carlisle Lane, Waterloo</t>
-        </is>
-      </c>
-      <c r="E54" s="4" t="n"/>
+          <t>Casson Square, Waterloo, Southbank Place, London, SE1</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>SE1</t>
+        </is>
+      </c>
       <c r="F54" s="4" t="n">
-        <v>3575</v>
+        <v>4250</v>
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H54" s="4" t="inlineStr">
@@ -4172,12 +4176,12 @@
         </is>
       </c>
       <c r="J54" s="4" t="n">
-        <v>904</v>
+        <v>644</v>
       </c>
       <c r="K54" s="4" t="n"/>
       <c r="L54" s="4" t="inlineStr">
         <is>
-          <t>End of Terrace Shared Garden; listed furnished — check if flexible</t>
+          <t>1 bedroom 1 bathroom Open-plan reception kitchen 24-hour five-star concierge; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M54" s="4" t="inlineStr">
@@ -4199,7 +4203,7 @@
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>2 bedroom end of terrace house to rent</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
@@ -4209,21 +4213,17 @@
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/7516361/</t>
+          <t>https://www.onthemarket.com/details/19811489/</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>Belvedere Road, Waterloo, London, SE1</t>
-        </is>
-      </c>
-      <c r="E55" s="4" t="inlineStr">
-        <is>
-          <t>SE1</t>
-        </is>
-      </c>
+          <t>Carlisle Lane, Waterloo</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="n"/>
       <c r="F55" s="4" t="n">
-        <v>3350</v>
+        <v>3575</v>
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
@@ -4237,16 +4237,16 @@
       </c>
       <c r="I55" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Private balcony/terrace</t>
         </is>
       </c>
       <c r="J55" s="4" t="n">
-        <v>544</v>
+        <v>904</v>
       </c>
       <c r="K55" s="4" t="n"/>
       <c r="L55" s="4" t="inlineStr">
         <is>
-          <t>Residents' swimming pool and gym. Grade II listed period building. 24 hour porters. Set close to the iconic Southbank and London Eye.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>End of Terrace Shared Garden; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M55" s="4" t="inlineStr">
@@ -4268,7 +4268,7 @@
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
@@ -4278,12 +4278,12 @@
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/7589011/</t>
+          <t>https://www.onthemarket.com/details/7516361/</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>Belvedere Road, London, Waterloo, SE1</t>
+          <t>Belvedere Road, Waterloo, London, SE1</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
@@ -4292,11 +4292,11 @@
         </is>
       </c>
       <c r="F56" s="4" t="n">
-        <v>4200</v>
+        <v>3350</v>
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H56" s="4" t="inlineStr">
@@ -4310,12 +4310,12 @@
         </is>
       </c>
       <c r="J56" s="4" t="n">
-        <v>671</v>
+        <v>544</v>
       </c>
       <c r="K56" s="4" t="n"/>
       <c r="L56" s="4" t="inlineStr">
         <is>
-          <t>24-hour five-star concierge 18,000 sq ft gym and spa facilities Set in one of London's most connected locations, opposite Westminster and the Houses of Parliame; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>Residents' swimming pool and gym. Grade II listed period building. 24 hour porters. Set close to the iconic Southbank and London Eye.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M56" s="4" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
@@ -4347,12 +4347,12 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/17616661/</t>
+          <t>https://www.onthemarket.com/details/7589011/</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>The Music Box, 237 Union Street, Southwark, London, SE1</t>
+          <t>Belvedere Road, London, Waterloo, SE1</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
@@ -4361,11 +4361,11 @@
         </is>
       </c>
       <c r="F57" s="4" t="n">
-        <v>3800</v>
+        <v>4200</v>
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H57" s="4" t="inlineStr">
@@ -4375,16 +4375,16 @@
       </c>
       <c r="I57" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J57" s="4" t="n">
-        <v>841</v>
+        <v>671</v>
       </c>
       <c r="K57" s="4" t="n"/>
       <c r="L57" s="4" t="inlineStr">
         <is>
-          <t>Two bedrooms Two bathrooms 841 sq. ft. Excellent transport links; verify balcony/terrace; listed furnished — check if flexible</t>
+          <t>24-hour five-star concierge 18,000 sq ft gym and spa facilities Set in one of London's most connected locations, opposite Westminster and the Houses of Parliame; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M57" s="4" t="inlineStr">
@@ -4406,7 +4406,7 @@
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
@@ -4416,25 +4416,25 @@
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19863550/</t>
+          <t>https://www.onthemarket.com/details/17616661/</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>King Street, Covent Garden, London, WC2E</t>
+          <t>The Music Box, 237 Union Street, Southwark, London, SE1</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>WC2E</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F58" s="4" t="n">
-        <v>3358</v>
+        <v>3800</v>
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H58" s="4" t="inlineStr">
@@ -4444,16 +4444,16 @@
       </c>
       <c r="I58" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J58" s="4" t="n">
-        <v>455</v>
+        <v>841</v>
       </c>
       <c r="K58" s="4" t="n"/>
       <c r="L58" s="4" t="inlineStr">
         <is>
-          <t>Iconic Covent Garden location Finished to an excellent standard throughout High ceilings Wooden flooring throughout; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Two bedrooms Two bathrooms 841 sq. ft. Excellent transport links; verify balcony/terrace; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M58" s="4" t="inlineStr">
@@ -4475,7 +4475,7 @@
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
@@ -4485,21 +4485,21 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19860280/</t>
+          <t>https://www.onthemarket.com/details/19863550/</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>Floral Street, Covent Garden WC2</t>
+          <t>King Street, Covent Garden, London, WC2E</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>WC2</t>
+          <t>WC2E</t>
         </is>
       </c>
       <c r="F59" s="4" t="n">
-        <v>3380</v>
+        <v>3358</v>
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
@@ -4517,12 +4517,12 @@
         </is>
       </c>
       <c r="J59" s="4" t="n">
-        <v>495</v>
+        <v>455</v>
       </c>
       <c r="K59" s="4" t="n"/>
       <c r="L59" s="4" t="inlineStr">
         <is>
-          <t>One bedroom One bathroom, ensuite; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Iconic Covent Garden location Finished to an excellent standard throughout High ceilings Wooden flooring throughout; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M59" s="4" t="inlineStr">
@@ -4554,21 +4554,21 @@
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/1837052/</t>
+          <t>https://www.onthemarket.com/details/19860280/</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>King Street, Covent Garden, WC2E</t>
+          <t>Floral Street, Covent Garden WC2</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>WC2E</t>
+          <t>WC2</t>
         </is>
       </c>
       <c r="F60" s="4" t="n">
-        <v>3358</v>
+        <v>3380</v>
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
@@ -4586,12 +4586,12 @@
         </is>
       </c>
       <c r="J60" s="4" t="n">
-        <v>455</v>
+        <v>495</v>
       </c>
       <c r="K60" s="4" t="n"/>
       <c r="L60" s="4" t="inlineStr">
         <is>
-          <t>Furnished Recently refurbished; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>One bedroom One bathroom, ensuite; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M60" s="4" t="inlineStr">
@@ -4623,12 +4623,12 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/3408032/</t>
+          <t>https://www.onthemarket.com/details/1837052/</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>Floral Street, Covent Garden, WC2E</t>
+          <t>King Street, Covent Garden, WC2E</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>3380</v>
+        <v>3358</v>
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
@@ -4655,12 +4655,12 @@
         </is>
       </c>
       <c r="J61" s="4" t="n">
-        <v>398</v>
+        <v>455</v>
       </c>
       <c r="K61" s="4" t="n"/>
       <c r="L61" s="4" t="inlineStr">
         <is>
-          <t>Newly Refurbished Central Location; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Furnished Recently refurbished; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M61" s="4" t="inlineStr">
@@ -4682,7 +4682,7 @@
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
@@ -4692,25 +4692,25 @@
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/3102769/</t>
+          <t>https://www.onthemarket.com/details/3408032/</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>John Adam Street, Covent Garden, WC2N</t>
+          <t>Floral Street, Covent Garden, WC2E</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>WC2N</t>
+          <t>WC2E</t>
         </is>
       </c>
       <c r="F62" s="4" t="n">
-        <v>3185</v>
+        <v>3380</v>
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H62" s="4" t="inlineStr">
@@ -4724,12 +4724,12 @@
         </is>
       </c>
       <c r="J62" s="4" t="n">
-        <v>655</v>
+        <v>398</v>
       </c>
       <c r="K62" s="4" t="n"/>
       <c r="L62" s="4" t="inlineStr">
         <is>
-          <t>Concierge Close to the area's Universities for students and academics; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>Newly Refurbished Central Location; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M62" s="4" t="inlineStr">
@@ -4751,7 +4751,7 @@
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
@@ -4761,25 +4761,25 @@
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19733694/</t>
+          <t>https://www.onthemarket.com/details/3102769/</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>Maiden Lane, Covent Garden, London, WC2E</t>
+          <t>John Adam Street, Covent Garden, WC2N</t>
         </is>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>WC2E</t>
+          <t>WC2N</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>3684</v>
+        <v>3185</v>
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H63" s="4" t="inlineStr">
@@ -4793,12 +4793,12 @@
         </is>
       </c>
       <c r="J63" s="4" t="n">
-        <v>630</v>
+        <v>655</v>
       </c>
       <c r="K63" s="4" t="n"/>
       <c r="L63" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat arranged on the 4th floor Bright and spacious reception room; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Concierge Close to the area's Universities for students and academics; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M63" s="4" t="inlineStr">
@@ -4830,21 +4830,21 @@
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19725776/</t>
+          <t>https://www.onthemarket.com/details/19733694/</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>Shelton Street, Covent Garden, London, WC2H</t>
+          <t>Maiden Lane, Covent Garden, London, WC2E</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>WC2H</t>
+          <t>WC2E</t>
         </is>
       </c>
       <c r="F64" s="4" t="n">
-        <v>3500</v>
+        <v>3684</v>
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
@@ -4858,16 +4858,16 @@
       </c>
       <c r="I64" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J64" s="4" t="n">
-        <v>608</v>
+        <v>630</v>
       </c>
       <c r="K64" s="4" t="n"/>
       <c r="L64" s="4" t="inlineStr">
         <is>
-          <t>Stylish one bedroom, third floor apartment Beautifully proportioned open plan reception with balcony access; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>1 bedroom flat arranged on the 4th floor Bright and spacious reception room; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M64" s="4" t="inlineStr">
@@ -4889,7 +4889,7 @@
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
@@ -4899,21 +4899,21 @@
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19591709/</t>
+          <t>https://www.onthemarket.com/details/19725776/</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>King Street, Covent Garden WC2</t>
+          <t>Shelton Street, Covent Garden, London, WC2H</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>WC2</t>
+          <t>WC2H</t>
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>3575</v>
+        <v>3500</v>
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
@@ -4927,16 +4927,16 @@
       </c>
       <c r="I65" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Private balcony/terrace</t>
         </is>
       </c>
       <c r="J65" s="4" t="n">
-        <v>441</v>
+        <v>608</v>
       </c>
       <c r="K65" s="4" t="n"/>
       <c r="L65" s="4" t="inlineStr">
         <is>
-          <t>One double bedroom One bathroom; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Stylish one bedroom, third floor apartment Beautifully proportioned open plan reception with balcony access; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M65" s="4" t="inlineStr">
@@ -4968,7 +4968,7 @@
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19591720/</t>
+          <t>https://www.onthemarket.com/details/19591709/</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
@@ -4982,7 +4982,7 @@
         </is>
       </c>
       <c r="F66" s="4" t="n">
-        <v>4333</v>
+        <v>3575</v>
       </c>
       <c r="G66" s="4" t="inlineStr">
         <is>
@@ -5000,12 +5000,12 @@
         </is>
       </c>
       <c r="J66" s="4" t="n">
-        <v>667</v>
+        <v>441</v>
       </c>
       <c r="K66" s="4" t="n"/>
       <c r="L66" s="4" t="inlineStr">
         <is>
-          <t>One bedroom One bathroom; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>One double bedroom One bathroom; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M66" s="4" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
@@ -5037,25 +5037,25 @@
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19511649/</t>
+          <t>https://www.onthemarket.com/details/19591720/</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>Broad Court, Covent Garden, London, WC2B</t>
+          <t>King Street, Covent Garden WC2</t>
         </is>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>WC2B</t>
+          <t>WC2</t>
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>3684</v>
+        <v>4333</v>
       </c>
       <c r="G67" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H67" s="4" t="inlineStr">
@@ -5069,12 +5069,12 @@
         </is>
       </c>
       <c r="J67" s="4" t="n">
-        <v>811</v>
+        <v>667</v>
       </c>
       <c r="K67" s="4" t="n"/>
       <c r="L67" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat arranged on raised ground floor Attractive period building with a sought-after location; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>One bedroom One bathroom; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M67" s="4" t="inlineStr">
@@ -5096,7 +5096,7 @@
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
@@ -5106,25 +5106,25 @@
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19500342/</t>
+          <t>https://www.onthemarket.com/details/19511649/</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>Covent Garden, West End, London, WC2E</t>
+          <t>Broad Court, Covent Garden, London, WC2B</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>WC2E</t>
+          <t>WC2B</t>
         </is>
       </c>
       <c r="F68" s="4" t="n">
-        <v>3700</v>
+        <v>3684</v>
       </c>
       <c r="G68" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H68" s="4" t="inlineStr">
@@ -5137,11 +5137,13 @@
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J68" s="4" t="n"/>
+      <c r="J68" s="4" t="n">
+        <v>811</v>
+      </c>
       <c r="K68" s="4" t="n"/>
       <c r="L68" s="4" t="inlineStr">
         <is>
-          <t>Short Term Stay between 1-6 months Furnished Ground Floor of secure block Heart of Covent Garden; outdoor space is communal/shared; size not stated; listed furnished — check if flexible</t>
+          <t>2 bedroom flat arranged on raised ground floor Attractive period building with a sought-after location; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M68" s="4" t="inlineStr">
@@ -5163,7 +5165,7 @@
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
@@ -5173,21 +5175,21 @@
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/9591535/</t>
+          <t>https://www.onthemarket.com/details/19500342/</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>Casson Square, Waterloo, Southbank Place, London, SE1</t>
+          <t>Covent Garden, West End, London, WC2E</t>
         </is>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>SE1</t>
+          <t>WC2E</t>
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>4075</v>
+        <v>3700</v>
       </c>
       <c r="G69" s="4" t="inlineStr">
         <is>
@@ -5201,16 +5203,14 @@
       </c>
       <c r="I69" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
-        </is>
-      </c>
-      <c r="J69" s="4" t="n">
-        <v>641</v>
-      </c>
+          <t>Communal / shared</t>
+        </is>
+      </c>
+      <c r="J69" s="4" t="n"/>
       <c r="K69" s="4" t="n"/>
       <c r="L69" s="4" t="inlineStr">
         <is>
-          <t>*video viewing available* 24-hour five-star concierge 18,000 sq ft gym, pool and spa facilities Bedroom; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Short Term Stay between 1-6 months Furnished Ground Floor of secure block Heart of Covent Garden; outdoor space is communal/shared; size not stated; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M69" s="4" t="inlineStr">
@@ -5232,7 +5232,7 @@
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
@@ -5242,25 +5242,25 @@
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/5166551/</t>
+          <t>https://www.onthemarket.com/details/9591535/</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>Grafton Way, Bloomsbury, London WC1E</t>
+          <t>Casson Square, Waterloo, Southbank Place, London, SE1</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>WC1E</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F70" s="4" t="n">
-        <v>3142</v>
+        <v>4075</v>
       </c>
       <c r="G70" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H70" s="4" t="inlineStr">
@@ -5270,16 +5270,16 @@
       </c>
       <c r="I70" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Private balcony/terrace</t>
         </is>
       </c>
       <c r="J70" s="4" t="n">
-        <v>592</v>
+        <v>641</v>
       </c>
       <c r="K70" s="4" t="n"/>
       <c r="L70" s="4" t="inlineStr">
         <is>
-          <t>592 sq ft floor area Nearest station 0.1mi.; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>*video viewing available* 24-hour five-star concierge 18,000 sq ft gym, pool and spa facilities Bedroom; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M70" s="4" t="inlineStr">
@@ -5301,7 +5301,7 @@
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
@@ -5311,21 +5311,21 @@
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/10453057/</t>
+          <t>https://www.onthemarket.com/details/5166551/</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>Doughty Street, Bloomsbury, London, WC1N</t>
+          <t>Grafton Way, Bloomsbury, London WC1E</t>
         </is>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>WC1N</t>
+          <t>WC1E</t>
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>3250</v>
+        <v>3142</v>
       </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
@@ -5343,12 +5343,12 @@
         </is>
       </c>
       <c r="J71" s="4" t="n">
-        <v>787</v>
+        <v>592</v>
       </c>
       <c r="K71" s="4" t="n"/>
       <c r="L71" s="4" t="inlineStr">
         <is>
-          <t>Two double bedrooms Dine-in kitchen; verify balcony/terrace; listed furnished — check if flexible</t>
+          <t>592 sq ft floor area Nearest station 0.1mi.; verify balcony/terrace; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M71" s="4" t="inlineStr">
@@ -5370,7 +5370,7 @@
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
@@ -5380,30 +5380,30 @@
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/13502768/</t>
+          <t>https://www.onthemarket.com/details/10453057/</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>Bedford Court Mansions, Bloomsbury, WC1B</t>
+          <t>Doughty Street, Bloomsbury, London, WC1N</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>WC1B</t>
+          <t>WC1N</t>
         </is>
       </c>
       <c r="F72" s="4" t="n">
-        <v>3142</v>
+        <v>3250</v>
       </c>
       <c r="G72" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H72" s="4" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Furnished</t>
         </is>
       </c>
       <c r="I72" s="4" t="inlineStr">
@@ -5412,12 +5412,12 @@
         </is>
       </c>
       <c r="J72" s="4" t="n">
-        <v>587</v>
+        <v>787</v>
       </c>
       <c r="K72" s="4" t="n"/>
       <c r="L72" s="4" t="inlineStr">
         <is>
-          <t>One Bedroom Professionally Managed; verify balcony/terrace; under 650 sq ft</t>
+          <t>Two double bedrooms Dine-in kitchen; verify balcony/terrace; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M72" s="4" t="inlineStr">
@@ -5439,7 +5439,7 @@
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
@@ -5449,21 +5449,21 @@
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19815346/</t>
+          <t>https://www.onthemarket.com/details/13502768/</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>Bloomsbury, London, WC1N</t>
+          <t>Bedford Court Mansions, Bloomsbury, WC1B</t>
         </is>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>WC1N</t>
+          <t>WC1B</t>
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>3000</v>
+        <v>3142</v>
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
@@ -5472,19 +5472,21 @@
       </c>
       <c r="H73" s="4" t="inlineStr">
         <is>
-          <t>Furnished</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I73" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
-        </is>
-      </c>
-      <c r="J73" s="4" t="n"/>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="J73" s="4" t="n">
+        <v>587</v>
+      </c>
       <c r="K73" s="4" t="n"/>
       <c r="L73" s="4" t="inlineStr">
         <is>
-          <t>No Agent Fees Property Reference Number: 2942192; size not stated; listed furnished — check if flexible</t>
+          <t>One Bedroom Professionally Managed; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M73" s="4" t="inlineStr">
@@ -5516,21 +5518,21 @@
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/3952850/</t>
+          <t>https://www.onthemarket.com/details/19815346/</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>Bloomsbury Square, Bloomsbury, London, WC1A</t>
+          <t>Bloomsbury, London, WC1N</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>WC1A</t>
+          <t>WC1N</t>
         </is>
       </c>
       <c r="F74" s="4" t="n">
-        <v>3141</v>
+        <v>3000</v>
       </c>
       <c r="G74" s="4" t="inlineStr">
         <is>
@@ -5539,21 +5541,19 @@
       </c>
       <c r="H74" s="4" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Furnished</t>
         </is>
       </c>
       <c r="I74" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="J74" s="4" t="n">
-        <v>609</v>
-      </c>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J74" s="4" t="n"/>
       <c r="K74" s="4" t="n"/>
       <c r="L74" s="4" t="inlineStr">
         <is>
-          <t>One Bedroom High Ceilings Views of Bloomsbury Square Wow Factor; verify balcony/terrace; under 650 sq ft</t>
+          <t>No Agent Fees Property Reference Number: 2942192; size not stated; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M74" s="4" t="inlineStr">
@@ -5575,7 +5575,7 @@
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
@@ -5585,30 +5585,30 @@
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19723779/</t>
+          <t>https://www.onthemarket.com/details/3952850/</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>Mecklenburgh Square, Bloomsbury, London, WC1N</t>
+          <t>Bloomsbury Square, Bloomsbury, London, WC1A</t>
         </is>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>WC1N</t>
+          <t>WC1A</t>
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>3684</v>
+        <v>3141</v>
       </c>
       <c r="G75" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H75" s="4" t="inlineStr">
         <is>
-          <t>Part Furnished</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I75" s="4" t="inlineStr">
@@ -5617,12 +5617,12 @@
         </is>
       </c>
       <c r="J75" s="4" t="n">
-        <v>602</v>
+        <v>609</v>
       </c>
       <c r="K75" s="4" t="n"/>
       <c r="L75" s="4" t="inlineStr">
         <is>
-          <t>Superb 2 bedroom flat Spacious arrangement; verify balcony/terrace; under 650 sq ft</t>
+          <t>One Bedroom High Ceilings Views of Bloomsbury Square Wow Factor; verify balcony/terrace; under 650 sq ft</t>
         </is>
       </c>
       <c r="M75" s="4" t="inlineStr">
@@ -5644,7 +5644,7 @@
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
@@ -5654,64 +5654,133 @@
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19715608/</t>
+          <t>https://www.onthemarket.com/details/19723779/</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>Bloomsbury Square, London WC1A</t>
+          <t>Mecklenburgh Square, Bloomsbury, London, WC1N</t>
         </is>
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>WC1A</t>
+          <t>WC1N</t>
         </is>
       </c>
       <c r="F76" s="4" t="n">
-        <v>3000</v>
+        <v>3684</v>
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H76" s="4" t="inlineStr">
         <is>
-          <t>Furnished</t>
+          <t>Part Furnished</t>
         </is>
       </c>
       <c r="I76" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J76" s="4" t="n">
-        <v>581</v>
+        <v>602</v>
       </c>
       <c r="K76" s="4" t="n"/>
       <c r="L76" s="4" t="inlineStr">
         <is>
+          <t>Superb 2 bedroom flat Spacious arrangement; verify balcony/terrace; under 650 sq ft</t>
+        </is>
+      </c>
+      <c r="M76" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N76" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O76" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>1 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19715608/</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>Bloomsbury Square, London WC1A</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>WC1A</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G77" s="4" t="inlineStr">
+        <is>
+          <t>1-Bed</t>
+        </is>
+      </c>
+      <c r="H77" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I77" s="4" t="inlineStr">
+        <is>
+          <t>Communal / shared</t>
+        </is>
+      </c>
+      <c r="J77" s="4" t="n">
+        <v>581</v>
+      </c>
+      <c r="K77" s="4" t="n"/>
+      <c r="L77" s="4" t="inlineStr">
+        <is>
           <t>Period Building Concierge; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
-      <c r="M76" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N76" s="4" t="inlineStr">
+      <c r="M77" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N77" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="O76" s="4" t="inlineStr">
+      <c r="O77" s="4" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O76"/>
+  <autoFilter ref="A1:O77"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
@@ -5788,6 +5857,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C74" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C75" r:id="rId74"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" r:id="rId76"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily tracker update 2026-07-10
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -598,7 +598,7 @@
       <c r="J2" s="2" t="n">
         <v>935</v>
       </c>
-      <c r="K2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="n"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
           <t>ZERO DEPOSIT AVAILABLE. LONG LET. This fantastic 2 bedroom flat is set within a pub conversion and offers spacious accommodation, bright and airy interiors thro</t>
@@ -667,7 +667,7 @@
       <c r="J3" s="4" t="n">
         <v>656</v>
       </c>
-      <c r="K3" s="4" t="inlineStr"/>
+      <c r="K3" s="4" t="n"/>
       <c r="L3" s="4" t="inlineStr">
         <is>
           <t>Large One Bedroom Apartment Large Balcony; listed furnished — check if flexible</t>

</xml_diff>

<commit_message>
Tracker re-tier: furnished is a one-tier demotion (Low -> Medium for otherwise-HIGH flats)
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -621,69 +621,69 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>1 bedroom flat to rent</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>https://www.onthemarket.com/details/19905959/</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>One Casson Square, Waterloo, London, SE1</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>SE1</t>
         </is>
       </c>
-      <c r="F3" s="4" t="n">
+      <c r="F3" s="6" t="n">
         <v>4247</v>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>1-Bed</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>Furnished</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>Private balcony/terrace</t>
         </is>
       </c>
-      <c r="J3" s="4" t="n">
+      <c r="J3" s="6" t="n">
         <v>656</v>
       </c>
-      <c r="K3" s="4" t="n"/>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="K3" s="6" t="n"/>
+      <c r="L3" s="6" t="inlineStr">
         <is>
           <t>Large One Bedroom Apartment Large Balcony; listed furnished — check if flexible</t>
         </is>
       </c>
-      <c r="M3" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N3" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="O3" s="4" t="inlineStr">
+      <c r="M3" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N3" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O3" s="6" t="inlineStr">
         <is>
           <t>2026-07-10 11:39</t>
         </is>
@@ -1725,69 +1725,69 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>2 bedroom apartment to rent</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>https://www.onthemarket.com/details/13719505/</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>Bedford Place, Bloomsbury, WC1B</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>WC1B</t>
         </is>
       </c>
-      <c r="F19" s="4" t="n">
+      <c r="F19" s="6" t="n">
         <v>3878</v>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="G19" s="6" t="inlineStr">
         <is>
           <t>2-Bed</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="H19" s="6" t="inlineStr">
         <is>
           <t>Furnished</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="I19" s="6" t="inlineStr">
         <is>
           <t>Private balcony/terrace</t>
         </is>
       </c>
-      <c r="J19" s="4" t="n">
+      <c r="J19" s="6" t="n">
         <v>961</v>
       </c>
-      <c r="K19" s="4" t="n"/>
-      <c r="L19" s="4" t="inlineStr">
+      <c r="K19" s="6" t="n"/>
+      <c r="L19" s="6" t="inlineStr">
         <is>
           <t>Two Double Bedroom Apartment High Spec; listed furnished — check if flexible</t>
         </is>
       </c>
-      <c r="M19" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N19" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="O19" s="4" t="inlineStr">
+      <c r="M19" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N19" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O19" s="6" t="inlineStr">
         <is>
           <t>2026-07-06 15:39</t>
         </is>
@@ -1861,69 +1861,69 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>1 bedroom flat to rent</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/19099769/</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Fletcher Buildings,, Covent Garden, London, WC2B</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>WC2B</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="n">
-        <v>3792</v>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>1-Bed</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>2 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/6356511/</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Great James Street, Bloomsbury, London, WC1N</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>WC1N</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>3683</v>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>2-Bed</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
         <is>
           <t>Furnished</t>
         </is>
       </c>
-      <c r="I21" s="4" t="inlineStr">
-        <is>
-          <t>Communal / shared</t>
-        </is>
-      </c>
-      <c r="J21" s="4" t="n">
-        <v>320</v>
-      </c>
-      <c r="K21" s="4" t="n"/>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t>Bright and airy one bedroom apartment in a prime Central London location Well proportioned reception with high ceilings and neutral décor Generous double bedroo; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
-        </is>
-      </c>
-      <c r="M21" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N21" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="O21" s="4" t="inlineStr">
+      <c r="I21" s="6" t="inlineStr">
+        <is>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J21" s="6" t="n">
+        <v>928</v>
+      </c>
+      <c r="K21" s="6" t="n"/>
+      <c r="L21" s="6" t="inlineStr">
+        <is>
+          <t>Spacious Split Level Apartment Large Terrace Wooden Flooring Nearest tubes: Chancery Lane, Russell Square &amp; Holborn; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M21" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N21" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O21" s="6" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
@@ -1932,7 +1932,7 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
@@ -1942,25 +1942,25 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/6356511/</t>
+          <t>https://www.onthemarket.com/details/19099769/</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Great James Street, Bloomsbury, London, WC1N</t>
+          <t>Fletcher Buildings,, Covent Garden, London, WC2B</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>WC1N</t>
+          <t>WC2B</t>
         </is>
       </c>
       <c r="F22" s="4" t="n">
-        <v>3683</v>
+        <v>3792</v>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1970,16 +1970,16 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J22" s="4" t="n">
-        <v>928</v>
+        <v>320</v>
       </c>
       <c r="K22" s="4" t="n"/>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Spacious Split Level Apartment Large Terrace Wooden Flooring Nearest tubes: Chancery Lane, Russell Square &amp; Holborn; listed furnished — check if flexible</t>
+          <t>Bright and airy one bedroom apartment in a prime Central London location Well proportioned reception with high ceilings and neutral décor Generous double bedroo; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
@@ -3239,138 +3239,134 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="4" t="inlineStr">
+      <c r="A41" s="6" t="inlineStr">
         <is>
           <t>2 bedroom flat to rent</t>
         </is>
       </c>
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
         <is>
           <t>https://www.onthemarket.com/details/19852978/</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr">
+      <c r="D41" s="6" t="inlineStr">
         <is>
           <t>Newport Court, Covent Garden, London, WC2H</t>
         </is>
       </c>
-      <c r="E41" s="4" t="inlineStr">
+      <c r="E41" s="6" t="inlineStr">
         <is>
           <t>WC2H</t>
         </is>
       </c>
-      <c r="F41" s="4" t="n">
+      <c r="F41" s="6" t="n">
         <v>4334</v>
       </c>
-      <c r="G41" s="4" t="inlineStr">
+      <c r="G41" s="6" t="inlineStr">
         <is>
           <t>2-Bed</t>
         </is>
       </c>
-      <c r="H41" s="4" t="inlineStr">
+      <c r="H41" s="6" t="inlineStr">
         <is>
           <t>Furnished</t>
         </is>
       </c>
-      <c r="I41" s="4" t="inlineStr">
+      <c r="I41" s="6" t="inlineStr">
         <is>
           <t>Private balcony/terrace</t>
         </is>
       </c>
-      <c r="J41" s="4" t="n">
+      <c r="J41" s="6" t="n">
         <v>858</v>
       </c>
-      <c r="K41" s="4" t="n"/>
-      <c r="L41" s="4" t="inlineStr">
+      <c r="K41" s="6" t="n"/>
+      <c r="L41" s="6" t="inlineStr">
         <is>
           <t>Splendid two bedroom flat Ample interiors; listed furnished — check if flexible</t>
         </is>
       </c>
-      <c r="M41" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N41" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="O41" s="4" t="inlineStr">
+      <c r="M41" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N41" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O41" s="6" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>2 bedroom apartment to rent</t>
-        </is>
-      </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/16157050/</t>
-        </is>
-      </c>
-      <c r="D42" s="4" t="inlineStr">
-        <is>
-          <t>Brewer Street, Soho, W1F</t>
-        </is>
-      </c>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t>W1F</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="n">
-        <v>3142</v>
-      </c>
-      <c r="G42" s="4" t="inlineStr">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>2 bedroom end of terrace house to rent</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19811489/</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>Carlisle Lane, Waterloo</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="n"/>
+      <c r="F42" s="6" t="n">
+        <v>3575</v>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
         <is>
           <t>2-Bed</t>
         </is>
       </c>
-      <c r="H42" s="4" t="inlineStr">
+      <c r="H42" s="6" t="inlineStr">
         <is>
           <t>Furnished</t>
         </is>
       </c>
-      <c r="I42" s="4" t="inlineStr">
-        <is>
-          <t>Communal / shared</t>
-        </is>
-      </c>
-      <c r="J42" s="4" t="n">
-        <v>730</v>
-      </c>
-      <c r="K42" s="4" t="n"/>
-      <c r="L42" s="4" t="inlineStr">
-        <is>
-          <t>730 sqft Secure Entrance; outdoor space is communal/shared; listed furnished — check if flexible</t>
-        </is>
-      </c>
-      <c r="M42" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N42" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="O42" s="4" t="inlineStr">
+      <c r="I42" s="6" t="inlineStr">
+        <is>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J42" s="6" t="n">
+        <v>904</v>
+      </c>
+      <c r="K42" s="6" t="n"/>
+      <c r="L42" s="6" t="inlineStr">
+        <is>
+          <t>End of Terrace Shared Garden; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M42" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N42" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O42" s="6" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
@@ -3379,7 +3375,7 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
@@ -3389,25 +3385,25 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19786051/</t>
+          <t>https://www.onthemarket.com/details/16157050/</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Old Compton Street, Soho, London, W1D</t>
+          <t>Brewer Street, Soho, W1F</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>W1D</t>
+          <t>W1F</t>
         </is>
       </c>
       <c r="F43" s="4" t="n">
-        <v>3600</v>
+        <v>3142</v>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
@@ -3421,12 +3417,12 @@
         </is>
       </c>
       <c r="J43" s="4" t="n">
-        <v>432</v>
+        <v>730</v>
       </c>
       <c r="K43" s="4" t="n"/>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>432 sq ft floor area Nearest station 0.1mi. Furnished Nearest school 0.2mi.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>730 sqft Secure Entrance; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
@@ -3448,7 +3444,7 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
@@ -3458,25 +3454,25 @@
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/11345150/</t>
+          <t>https://www.onthemarket.com/details/19786051/</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Shaftesbury Avenue, Covent Garden, London, WC2H</t>
+          <t>Old Compton Street, Soho, London, W1D</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>WC2H</t>
+          <t>W1D</t>
         </is>
       </c>
       <c r="F44" s="4" t="n">
-        <v>3575</v>
+        <v>3600</v>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
@@ -3490,12 +3486,12 @@
         </is>
       </c>
       <c r="J44" s="4" t="n">
-        <v>870</v>
+        <v>432</v>
       </c>
       <c r="K44" s="4" t="n"/>
       <c r="L44" s="4" t="inlineStr">
         <is>
-          <t>870 sq ft floor area Nearest station 0.1mi.; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>432 sq ft floor area Nearest station 0.1mi. Furnished Nearest school 0.2mi.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M44" s="4" t="inlineStr">
@@ -3517,7 +3513,7 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
@@ -3527,25 +3523,25 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/15707269/</t>
+          <t>https://www.onthemarket.com/details/11345150/</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Casson Square, London, Waterloo, United Kingdom, SE1</t>
+          <t>Shaftesbury Avenue, Covent Garden, London, WC2H</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>SE1</t>
+          <t>WC2H</t>
         </is>
       </c>
       <c r="F45" s="4" t="n">
-        <v>4050</v>
+        <v>3575</v>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr">
@@ -3559,12 +3555,12 @@
         </is>
       </c>
       <c r="J45" s="4" t="n">
-        <v>514</v>
+        <v>870</v>
       </c>
       <c r="K45" s="4" t="n"/>
       <c r="L45" s="4" t="inlineStr">
         <is>
-          <t>Bedroom Bathroom Open-plan reception/kitchen 24 hour concierge; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>870 sq ft floor area Nearest station 0.1mi.; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M45" s="4" t="inlineStr">
@@ -3596,12 +3592,12 @@
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/9568931/</t>
+          <t>https://www.onthemarket.com/details/15707269/</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Casson Square, Waterloo, Southbank Place, London, SE1</t>
+          <t>Casson Square, London, Waterloo, United Kingdom, SE1</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
@@ -3610,7 +3606,7 @@
         </is>
       </c>
       <c r="F46" s="4" t="n">
-        <v>4250</v>
+        <v>4050</v>
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
@@ -3624,16 +3620,16 @@
       </c>
       <c r="I46" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J46" s="4" t="n">
-        <v>644</v>
+        <v>514</v>
       </c>
       <c r="K46" s="4" t="n"/>
       <c r="L46" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom 1 bathroom Open-plan reception kitchen 24-hour five-star concierge; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Bedroom Bathroom Open-plan reception/kitchen 24 hour concierge; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M46" s="4" t="inlineStr">
@@ -3655,7 +3651,7 @@
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom end of terrace house to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
@@ -3665,21 +3661,25 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19811489/</t>
+          <t>https://www.onthemarket.com/details/9568931/</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Carlisle Lane, Waterloo</t>
-        </is>
-      </c>
-      <c r="E47" s="4" t="n"/>
+          <t>Casson Square, Waterloo, Southbank Place, London, SE1</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>SE1</t>
+        </is>
+      </c>
       <c r="F47" s="4" t="n">
-        <v>3575</v>
+        <v>4250</v>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr">
@@ -3693,12 +3693,12 @@
         </is>
       </c>
       <c r="J47" s="4" t="n">
-        <v>904</v>
+        <v>644</v>
       </c>
       <c r="K47" s="4" t="n"/>
       <c r="L47" s="4" t="inlineStr">
         <is>
-          <t>End of Terrace Shared Garden; listed furnished — check if flexible</t>
+          <t>1 bedroom 1 bathroom Open-plan reception kitchen 24-hour five-star concierge; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M47" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Daily tracker update 2026-07-11
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -598,7 +598,7 @@
       <c r="J2" s="6" t="n">
         <v>485</v>
       </c>
-      <c r="K2" s="6" t="inlineStr"/>
+      <c r="K2" s="6" t="n"/>
       <c r="L2" s="6" t="inlineStr">
         <is>
           <t>Bright 1 bedroom flat Light and spacious reception room Superb location in vibrant Covent Garden 6th floor of a popular purpose-built block; outdoor space is communal/shared; under 650 sq ft</t>
@@ -667,7 +667,7 @@
       <c r="J3" s="6" t="n">
         <v>522</v>
       </c>
-      <c r="K3" s="6" t="inlineStr"/>
+      <c r="K3" s="6" t="n"/>
       <c r="L3" s="6" t="inlineStr">
         <is>
           <t>Charming one bedroom apartment within an impressive London Townhouse Excellent location close to a range of shops and eateries Bright and airy reception with sa; outdoor space is communal/shared; under 650 sq ft; furnishing not stated</t>

</xml_diff>

<commit_message>
Daily tracker update 2026-07-13
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Flats" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Flats'!$A$1:$O$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Flats'!$A$1:$O$66</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O65"/>
+  <dimension ref="A1:O66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -552,71 +552,71 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>1 bedroom flat to rent</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/19035144/</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
-        <is>
-          <t>Macklin Street, Covent Garden, London, WC2B</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="inlineStr">
-        <is>
-          <t>WC2B</t>
-        </is>
-      </c>
-      <c r="F2" s="6" t="n">
-        <v>3250</v>
-      </c>
-      <c r="G2" s="6" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>1 bedroom apartment to rent</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/4393324/</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Southampton Street, Covent Garden, WC2E</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>WC2E</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>3640</v>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>1-Bed</t>
         </is>
       </c>
-      <c r="H2" s="6" t="inlineStr">
-        <is>
-          <t>Part Furnished</t>
-        </is>
-      </c>
-      <c r="I2" s="6" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J2" s="6" t="n">
-        <v>485</v>
-      </c>
-      <c r="K2" s="6" t="n"/>
-      <c r="L2" s="6" t="inlineStr">
-        <is>
-          <t>Bright 1 bedroom flat Light and spacious reception room Superb location in vibrant Covent Garden 6th floor of a popular purpose-built block; outdoor space is communal/shared; under 650 sq ft</t>
-        </is>
-      </c>
-      <c r="M2" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N2" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O2" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-11 16:39</t>
+      <c r="J2" s="4" t="n">
+        <v>512</v>
+      </c>
+      <c r="K2" s="4" t="inlineStr"/>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>One bedroom Lift within the building Students welcome; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M2" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N2" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O2" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-13 08:39</t>
         </is>
       </c>
     </row>
@@ -633,21 +633,21 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/18441856/</t>
+          <t>https://www.onthemarket.com/details/19035144/</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>Bloomsbury Square, Bloomsbury, London, WC1A</t>
+          <t>Macklin Street, Covent Garden, London, WC2B</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>WC1A</t>
+          <t>WC2B</t>
         </is>
       </c>
       <c r="F3" s="6" t="n">
-        <v>4117</v>
+        <v>3250</v>
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
@@ -656,7 +656,7 @@
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Part Furnished</t>
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr">
@@ -665,163 +665,163 @@
         </is>
       </c>
       <c r="J3" s="6" t="n">
-        <v>522</v>
+        <v>485</v>
       </c>
       <c r="K3" s="6" t="n"/>
       <c r="L3" s="6" t="inlineStr">
         <is>
+          <t>Bright 1 bedroom flat Light and spacious reception room Superb location in vibrant Covent Garden 6th floor of a popular purpose-built block; outdoor space is communal/shared; under 650 sq ft</t>
+        </is>
+      </c>
+      <c r="M3" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N3" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O3" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-11 16:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>1 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/18441856/</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Bloomsbury Square, Bloomsbury, London, WC1A</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>WC1A</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>4117</v>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>1-Bed</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Communal / shared</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="n">
+        <v>522</v>
+      </c>
+      <c r="K4" s="6" t="n"/>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
           <t>Charming one bedroom apartment within an impressive London Townhouse Excellent location close to a range of shops and eateries Bright and airy reception with sa; outdoor space is communal/shared; under 650 sq ft; furnishing not stated</t>
         </is>
       </c>
-      <c r="M3" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N3" s="6" t="inlineStr">
+      <c r="M4" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N4" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="O3" s="6" t="inlineStr">
+      <c r="O4" s="6" t="inlineStr">
         <is>
           <t>2026-07-11 16:39</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Flat</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Rightmove</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>https://www.rightmove.co.uk/properties/90050730</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Southwark Park Road, London Bridge, London, SE16</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>SE16</t>
         </is>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F5" s="2" t="n">
         <v>3000</v>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>2-Bed</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Part Furnished</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Private balcony/terrace</t>
         </is>
       </c>
-      <c r="J4" s="2" t="n">
+      <c r="J5" s="2" t="n">
         <v>935</v>
       </c>
-      <c r="K4" s="2" t="n"/>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="K5" s="2" t="n"/>
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>ZERO DEPOSIT AVAILABLE. LONG LET. This fantastic 2 bedroom flat is set within a pub conversion and offers spacious accommodation, bright and airy interiors thro</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-10 11:39</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>1 bedroom flat to rent</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/19905959/</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>One Casson Square, Waterloo, London, SE1</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>SE1</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="n">
-        <v>4247</v>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>1-Bed</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>Furnished</t>
-        </is>
-      </c>
-      <c r="I5" s="6" t="inlineStr">
-        <is>
-          <t>Private balcony/terrace</t>
-        </is>
-      </c>
-      <c r="J5" s="6" t="n">
-        <v>656</v>
-      </c>
-      <c r="K5" s="6" t="n"/>
-      <c r="L5" s="6" t="inlineStr">
-        <is>
-          <t>Large One Bedroom Apartment Large Balcony; listed furnished — check if flexible</t>
-        </is>
-      </c>
-      <c r="M5" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N5" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O5" s="6" t="inlineStr">
+      <c r="O5" s="2" t="inlineStr">
         <is>
           <t>2026-07-10 11:39</t>
         </is>
@@ -830,7 +830,7 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -840,204 +840,204 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/16575118/</t>
+          <t>https://www.onthemarket.com/details/19905959/</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Brewer Street, Soho, W1F</t>
+          <t>One Casson Square, Waterloo, London, SE1</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>W1F</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F6" s="6" t="n">
-        <v>3358</v>
+        <v>4247</v>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Furnished</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Private balcony/terrace</t>
         </is>
       </c>
       <c r="J6" s="6" t="n">
-        <v>643</v>
+        <v>656</v>
       </c>
       <c r="K6" s="6" t="n"/>
       <c r="L6" s="6" t="inlineStr">
         <is>
+          <t>Large One Bedroom Apartment Large Balcony; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M6" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N6" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O6" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-10 11:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>2 bedroom apartment to rent</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/16575118/</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Brewer Street, Soho, W1F</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>W1F</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>3358</v>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>2-Bed</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>Flexible</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>Communal / shared</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>643</v>
+      </c>
+      <c r="K7" s="6" t="n"/>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
           <t>Pet Friendly Beautifully Refurbished Student; outdoor space is communal/shared; under 650 sq ft</t>
         </is>
       </c>
-      <c r="M6" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N6" s="6" t="inlineStr">
+      <c r="M7" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N7" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="O6" s="6" t="inlineStr">
+      <c r="O7" s="6" t="inlineStr">
         <is>
           <t>2026-07-10 08:38</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Flat</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Rightmove</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>https://www.rightmove.co.uk/properties/89643957</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Saffron Hill, Farringdon, London, EC1N</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>EC1N</t>
         </is>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="F8" s="2" t="n">
         <v>3250</v>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>2-Bed</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Unfurnished</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Private balcony/terrace</t>
         </is>
       </c>
-      <c r="J7" s="2" t="n">
+      <c r="J8" s="2" t="n">
         <v>676</v>
       </c>
-      <c r="K7" s="2" t="n"/>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="K8" s="2" t="n"/>
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">LONG LET. This stunning two bedroom sixth floor flat boasts bright reception room with bi-folding doors leading to large private roof terrace, modern open-plan </t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="O7" s="2" t="inlineStr">
+      <c r="O8" s="2" t="inlineStr">
         <is>
           <t>2026-07-10 05:38</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>2 bedroom flat to rent</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/19476388/</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>Russell Square Mansions, Bloomsbury, London, WC1B</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>WC1B</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="n">
-        <v>3900</v>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>2-Bed</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>Part Furnished</t>
-        </is>
-      </c>
-      <c r="I8" s="6" t="inlineStr">
-        <is>
-          <t>Communal / shared</t>
-        </is>
-      </c>
-      <c r="J8" s="6" t="n">
-        <v>693</v>
-      </c>
-      <c r="K8" s="6" t="n"/>
-      <c r="L8" s="6" t="inlineStr">
-        <is>
-          <t>Fantastic 2 bedroom flat arranged on the 1st floor Offers generous reception room with open-plan kitchen Features two good-sized, well presented bedrooms Provid; outdoor space is communal/shared</t>
-        </is>
-      </c>
-      <c r="M8" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N8" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O8" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-09 16:39</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
@@ -1047,30 +1047,30 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19455974/</t>
+          <t>https://www.onthemarket.com/details/19476388/</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Shaftesbury Avenue, Soho, W1D</t>
+          <t>Russell Square Mansions, Bloomsbury, London, WC1B</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>W1D</t>
+          <t>WC1B</t>
         </is>
       </c>
       <c r="F9" s="6" t="n">
-        <v>3120</v>
+        <v>3900</v>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Part Furnished</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
@@ -1079,103 +1079,103 @@
         </is>
       </c>
       <c r="J9" s="6" t="n">
-        <v>570</v>
+        <v>693</v>
       </c>
       <c r="K9" s="6" t="n"/>
       <c r="L9" s="6" t="inlineStr">
         <is>
+          <t>Fantastic 2 bedroom flat arranged on the 1st floor Offers generous reception room with open-plan kitchen Features two good-sized, well presented bedrooms Provid; outdoor space is communal/shared</t>
+        </is>
+      </c>
+      <c r="M9" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N9" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O9" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-09 16:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>1 bedroom apartment to rent</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19455974/</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Shaftesbury Avenue, Soho, W1D</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>W1D</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>3120</v>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>1-Bed</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>Flexible</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>Communal / shared</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="n">
+        <v>570</v>
+      </c>
+      <c r="K10" s="6" t="n"/>
+      <c r="L10" s="6" t="inlineStr">
+        <is>
           <t>Beautifully Refurbished Built in Storage; outdoor space is communal/shared; under 650 sq ft</t>
         </is>
       </c>
-      <c r="M9" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N9" s="6" t="inlineStr">
+      <c r="M10" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N10" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="O9" s="6" t="inlineStr">
+      <c r="O10" s="6" t="inlineStr">
         <is>
           <t>2026-07-09 11:39</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>1 bedroom apartment to rent</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/8203290/</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Casson Square, Southbank Place, Waterloo, London, SE1</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>SE1</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="n">
-        <v>4350</v>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>1-Bed</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>Furnished</t>
-        </is>
-      </c>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>Communal / shared</t>
-        </is>
-      </c>
-      <c r="J10" s="4" t="n">
-        <v>655</v>
-      </c>
-      <c r="K10" s="4" t="n"/>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>24-hour five-star concierge 18,000 sq ft gym and spa facilities 6th Floor Set in one of London's most connected locations, opposite Westminster and the Houses o; outdoor space is communal/shared; listed furnished — check if flexible</t>
-        </is>
-      </c>
-      <c r="M10" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N10" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="O10" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-09 09:39</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -1185,25 +1185,25 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/2790064/</t>
+          <t>https://www.onthemarket.com/details/8203290/</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>John Adam Street, Covent Garden, WC2N</t>
+          <t>Casson Square, Southbank Place, Waterloo, London, SE1</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>WC2N</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F11" s="4" t="n">
-        <v>3098</v>
+        <v>4350</v>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1217,12 +1217,12 @@
         </is>
       </c>
       <c r="J11" s="4" t="n">
-        <v>597</v>
+        <v>655</v>
       </c>
       <c r="K11" s="4" t="n"/>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>Two double bedrooms 24 hour porter Students welcome; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>24-hour five-star concierge 18,000 sq ft gym and spa facilities 6th Floor Set in one of London's most connected locations, opposite Westminster and the Houses o; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M11" s="4" t="inlineStr">
@@ -1237,14 +1237,14 @@
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>2026-07-09 06:39</t>
+          <t>2026-07-09 09:39</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -1254,21 +1254,21 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19692817/</t>
+          <t>https://www.onthemarket.com/details/2790064/</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Belvedere Road, Waterloo, London, SE1</t>
+          <t>John Adam Street, Covent Garden, WC2N</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>SE1</t>
+          <t>WC2N</t>
         </is>
       </c>
       <c r="F12" s="4" t="n">
-        <v>3684</v>
+        <v>3098</v>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
@@ -1286,136 +1286,136 @@
         </is>
       </c>
       <c r="J12" s="4" t="n">
-        <v>895</v>
+        <v>597</v>
       </c>
       <c r="K12" s="4" t="n"/>
       <c r="L12" s="4" t="inlineStr">
         <is>
+          <t>Two double bedrooms 24 hour porter Students welcome; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M12" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N12" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O12" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-09 06:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>2 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19692817/</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Belvedere Road, Waterloo, London, SE1</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>SE1</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>3684</v>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>2-Bed</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>Communal / shared</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="n">
+        <v>895</v>
+      </c>
+      <c r="K13" s="4" t="n"/>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
           <t>1st Floor apartment set in the prestigious County Hall development Stylish reception filled with natural light and with space to dine Excellent kitchen with int; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
-      <c r="M12" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N12" s="4" t="inlineStr">
+      <c r="M13" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N13" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="O12" s="4" t="inlineStr">
+      <c r="O13" s="4" t="inlineStr">
         <is>
           <t>2026-07-09 02:39</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>1 bedroom apartment to rent</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/19592796/</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>Casson Square, Waterloo, SE1 7GU</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>SE1</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="n">
-        <v>3800</v>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>1-Bed</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="I13" s="6" t="inlineStr">
-        <is>
-          <t>Communal / shared</t>
-        </is>
-      </c>
-      <c r="J13" s="6" t="n">
-        <v>668</v>
-      </c>
-      <c r="K13" s="6" t="n"/>
-      <c r="L13" s="6" t="inlineStr">
-        <is>
-          <t>1 Bedroom and 1 Bathroom South-facing Aspect for Maximum Natural Light; outdoor space is communal/shared</t>
-        </is>
-      </c>
-      <c r="M13" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N13" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O13" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-08 16:39</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Apartment</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Rightmove</t>
+          <t>OnTheMarket</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>https://www.rightmove.co.uk/properties/90623913</t>
+          <t>https://www.onthemarket.com/details/19592796/</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>Shelton Street, Covent Garden, WC2H</t>
+          <t>Casson Square, Waterloo, SE1 7GU</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>WC2H</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F14" s="6" t="n">
-        <v>3358</v>
+        <v>3800</v>
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
@@ -1424,96 +1424,96 @@
         </is>
       </c>
       <c r="J14" s="6" t="n">
-        <v>623</v>
+        <v>668</v>
       </c>
       <c r="K14" s="6" t="n"/>
       <c r="L14" s="6" t="inlineStr">
         <is>
+          <t>1 Bedroom and 1 Bathroom South-facing Aspect for Maximum Natural Light; outdoor space is communal/shared</t>
+        </is>
+      </c>
+      <c r="M14" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N14" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O14" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-08 16:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Apartment</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Rightmove</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>https://www.rightmove.co.uk/properties/90623913</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>Shelton Street, Covent Garden, WC2H</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>WC2H</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>3358</v>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>2-Bed</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>Unfurnished</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>Communal / shared</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>623</v>
+      </c>
+      <c r="K15" s="6" t="n"/>
+      <c r="L15" s="6" t="inlineStr">
+        <is>
           <t>Contemporary, spacious 2 bedroom apartment to rent in Covent Garden, WC2 *AVAILABLE SEPTEMBER* A fantastic contemporary two bedroom, two bathroom flat to rent s; outdoor space is communal/shared; under 650 sq ft</t>
         </is>
       </c>
-      <c r="M14" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N14" s="6" t="inlineStr">
+      <c r="M15" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N15" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="O14" s="6" t="inlineStr">
+      <c r="O15" s="6" t="inlineStr">
         <is>
           <t>2026-07-08 10:39</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>1 bedroom apartment to rent</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/9187629/</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>Casson Square, Waterloo, Southbank Place, London, SE1</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>SE1</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="n">
-        <v>3990</v>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>1-Bed</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>Furnished</t>
-        </is>
-      </c>
-      <c r="I15" s="4" t="inlineStr">
-        <is>
-          <t>Communal / shared</t>
-        </is>
-      </c>
-      <c r="J15" s="4" t="n">
-        <v>537</v>
-      </c>
-      <c r="K15" s="4" t="n"/>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>Open plan reception kitchen Bedroom Bathroom 24-hour five-star concierge; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
-        </is>
-      </c>
-      <c r="M15" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N15" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="O15" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-08 00:39</t>
         </is>
       </c>
     </row>
@@ -1530,12 +1530,12 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/11391425/</t>
+          <t>https://www.onthemarket.com/details/9187629/</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Casson Square, Waterloo, London, SE1</t>
+          <t>Casson Square, Waterloo, Southbank Place, London, SE1</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -1544,7 +1544,7 @@
         </is>
       </c>
       <c r="F16" s="4" t="n">
-        <v>3033</v>
+        <v>3990</v>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
@@ -1562,12 +1562,12 @@
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>397</v>
+        <v>537</v>
       </c>
       <c r="K16" s="4" t="n"/>
       <c r="L16" s="4" t="inlineStr">
         <is>
-          <t>Studio bedroom Open plan kitchen/ reception room Bathroom 24 hour concierge; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Open plan reception kitchen Bedroom Bathroom 24-hour five-star concierge; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M16" s="4" t="inlineStr">
@@ -1599,12 +1599,12 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/7920965/</t>
+          <t>https://www.onthemarket.com/details/11391425/</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Belvedere Road, Waterloo, Southbank Place, London, SE1</t>
+          <t>Casson Square, Waterloo, London, SE1</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -1613,7 +1613,7 @@
         </is>
       </c>
       <c r="F17" s="4" t="n">
-        <v>3950</v>
+        <v>3033</v>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
@@ -1627,16 +1627,16 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J17" s="4" t="n">
-        <v>596</v>
+        <v>397</v>
       </c>
       <c r="K17" s="4" t="n"/>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>Fully furnished 1 bedroom 24-hour five-star concierge 18,000 sq ft gym and spa facilities; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Studio bedroom Open plan kitchen/ reception room Bathroom 24 hour concierge; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M17" s="4" t="inlineStr">
@@ -1651,14 +1651,14 @@
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07 08:39</t>
+          <t>2026-07-08 00:39</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -1668,25 +1668,25 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19876910/</t>
+          <t>https://www.onthemarket.com/details/7920965/</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Newton Street, Covent Garden, London, WC2B</t>
+          <t>Belvedere Road, Waterloo, Southbank Place, London, SE1</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>WC2B</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F18" s="4" t="n">
-        <v>4117</v>
+        <v>3950</v>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1696,245 +1696,245 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Private balcony/terrace</t>
         </is>
       </c>
       <c r="J18" s="4" t="n">
-        <v>848</v>
+        <v>596</v>
       </c>
       <c r="K18" s="4" t="n"/>
       <c r="L18" s="4" t="inlineStr">
         <is>
+          <t>Fully furnished 1 bedroom 24-hour five-star concierge 18,000 sq ft gym and spa facilities; under 650 sq ft; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M18" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N18" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O18" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07 08:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19876910/</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Newton Street, Covent Garden, London, WC2B</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>WC2B</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>4117</v>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>2-Bed</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>Communal / shared</t>
+        </is>
+      </c>
+      <c r="J19" s="4" t="n">
+        <v>848</v>
+      </c>
+      <c r="K19" s="4" t="n"/>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
           <t>Stunning 2 bedroom flat arranged on the 1st floor Generous reception room with space to dine; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
-      <c r="M18" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N18" s="4" t="inlineStr">
+      <c r="M19" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N19" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="O18" s="4" t="inlineStr">
+      <c r="O19" s="4" t="inlineStr">
         <is>
           <t>2026-07-07 07:39</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>2 bedroom flat to rent</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>https://www.onthemarket.com/details/19318164/</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>Princeton Street, Bloomsbury, London, WC1R</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>WC1R</t>
         </is>
       </c>
-      <c r="F19" s="6" t="n">
+      <c r="F20" s="6" t="n">
         <v>3684</v>
       </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="G20" s="6" t="inlineStr">
         <is>
           <t>2-Bed</t>
         </is>
       </c>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="H20" s="6" t="inlineStr">
         <is>
           <t>Part Furnished</t>
         </is>
       </c>
-      <c r="I19" s="6" t="inlineStr">
+      <c r="I20" s="6" t="inlineStr">
         <is>
           <t>Private balcony/terrace</t>
         </is>
       </c>
-      <c r="J19" s="6" t="n">
+      <c r="J20" s="6" t="n">
         <v>649</v>
       </c>
-      <c r="K19" s="6" t="n"/>
-      <c r="L19" s="6" t="inlineStr">
+      <c r="K20" s="6" t="n"/>
+      <c r="L20" s="6" t="inlineStr">
         <is>
           <t>Modern two bedroom, fourth floor flat Bright open plan reception Stylish kitchen featuring a range of modern appliances Two spacious bedrooms with built in stor; under 650 sq ft</t>
         </is>
       </c>
-      <c r="M19" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N19" s="6" t="inlineStr">
+      <c r="M20" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N20" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="O19" s="6" t="inlineStr">
+      <c r="O20" s="6" t="inlineStr">
         <is>
           <t>2026-07-06 20:39</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>1 bedroom flat to rent</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>https://www.onthemarket.com/details/16574229/</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>Casson Square, Waterloo, London, SE1</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>SE1</t>
         </is>
       </c>
-      <c r="F20" s="4" t="n">
+      <c r="F21" s="4" t="n">
         <v>3500</v>
       </c>
-      <c r="G20" s="4" t="inlineStr">
+      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>1-Bed</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="H21" s="4" t="inlineStr">
         <is>
           <t>Furnished</t>
         </is>
       </c>
-      <c r="I20" s="4" t="inlineStr">
+      <c r="I21" s="4" t="inlineStr">
         <is>
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J20" s="4" t="n">
+      <c r="J21" s="4" t="n">
         <v>548</v>
       </c>
-      <c r="K20" s="4" t="n"/>
-      <c r="L20" s="4" t="inlineStr">
+      <c r="K21" s="4" t="n"/>
+      <c r="L21" s="4" t="inlineStr">
         <is>
           <t>548 sq ft floor area Nearest station 0.1mi.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
-      <c r="M20" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N20" s="4" t="inlineStr">
+      <c r="M21" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N21" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="O20" s="4" t="inlineStr">
+      <c r="O21" s="4" t="inlineStr">
         <is>
           <t>2026-07-06 16:39</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>2 bedroom apartment to rent</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/13719505/</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>Bedford Place, Bloomsbury, WC1B</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="inlineStr">
-        <is>
-          <t>WC1B</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="n">
-        <v>3878</v>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>2-Bed</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr">
-        <is>
-          <t>Furnished</t>
-        </is>
-      </c>
-      <c r="I21" s="6" t="inlineStr">
-        <is>
-          <t>Private balcony/terrace</t>
-        </is>
-      </c>
-      <c r="J21" s="6" t="n">
-        <v>961</v>
-      </c>
-      <c r="K21" s="6" t="n"/>
-      <c r="L21" s="6" t="inlineStr">
-        <is>
-          <t>Two Double Bedroom Apartment High Spec; listed furnished — check if flexible</t>
-        </is>
-      </c>
-      <c r="M21" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N21" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O21" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-06 15:39</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1944,21 +1944,21 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/1990566/</t>
+          <t>https://www.onthemarket.com/details/13719505/</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>Endell Street, Covent Garden, London, WC2H</t>
+          <t>Bedford Place, Bloomsbury, WC1B</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>WC2H</t>
+          <t>WC1B</t>
         </is>
       </c>
       <c r="F22" s="6" t="n">
-        <v>3400</v>
+        <v>3878</v>
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
@@ -1967,19 +1967,21 @@
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Furnished</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
-        </is>
-      </c>
-      <c r="J22" s="6" t="n"/>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J22" s="6" t="n">
+        <v>961</v>
+      </c>
       <c r="K22" s="6" t="n"/>
       <c r="L22" s="6" t="inlineStr">
         <is>
-          <t>Two Bedrooms Two Bathrooms Open plan living room-kitchen First floor; outdoor space is communal/shared; size not stated</t>
+          <t>Two Double Bedroom Apartment High Spec; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M22" s="6" t="inlineStr">
@@ -1994,7 +1996,7 @@
       </c>
       <c r="O22" s="6" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-06 15:39</t>
         </is>
       </c>
     </row>
@@ -2011,21 +2013,21 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/6356511/</t>
+          <t>https://www.onthemarket.com/details/1990566/</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Great James Street, Bloomsbury, London, WC1N</t>
+          <t>Endell Street, Covent Garden, London, WC2H</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>WC1N</t>
+          <t>WC2H</t>
         </is>
       </c>
       <c r="F23" s="6" t="n">
-        <v>3683</v>
+        <v>3400</v>
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
@@ -2034,103 +2036,101 @@
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>Furnished</t>
+          <t>Unfurnished</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
-        </is>
-      </c>
-      <c r="J23" s="6" t="n">
-        <v>928</v>
-      </c>
+          <t>Communal / shared</t>
+        </is>
+      </c>
+      <c r="J23" s="6" t="n"/>
       <c r="K23" s="6" t="n"/>
       <c r="L23" s="6" t="inlineStr">
         <is>
+          <t>Two Bedrooms Two Bathrooms Open plan living room-kitchen First floor; outdoor space is communal/shared; size not stated</t>
+        </is>
+      </c>
+      <c r="M23" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N23" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O23" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>2 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/6356511/</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>Great James Street, Bloomsbury, London, WC1N</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>WC1N</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>3683</v>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>2-Bed</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J24" s="6" t="n">
+        <v>928</v>
+      </c>
+      <c r="K24" s="6" t="n"/>
+      <c r="L24" s="6" t="inlineStr">
+        <is>
           <t>Spacious Split Level Apartment Large Terrace Wooden Flooring Nearest tubes: Chancery Lane, Russell Square &amp; Holborn; listed furnished — check if flexible</t>
         </is>
       </c>
-      <c r="M23" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N23" s="6" t="inlineStr">
+      <c r="M24" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N24" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="O23" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>1 bedroom flat to rent</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/19099769/</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>Fletcher Buildings,, Covent Garden, London, WC2B</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>WC2B</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="n">
-        <v>3792</v>
-      </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t>1-Bed</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>Furnished</t>
-        </is>
-      </c>
-      <c r="I24" s="4" t="inlineStr">
-        <is>
-          <t>Communal / shared</t>
-        </is>
-      </c>
-      <c r="J24" s="4" t="n">
-        <v>320</v>
-      </c>
-      <c r="K24" s="4" t="n"/>
-      <c r="L24" s="4" t="inlineStr">
-        <is>
-          <t>Bright and airy one bedroom apartment in a prime Central London location Well proportioned reception with high ceilings and neutral décor Generous double bedroo; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
-        </is>
-      </c>
-      <c r="M24" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N24" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="O24" s="4" t="inlineStr">
+      <c r="O24" s="6" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
@@ -2149,21 +2149,21 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19453032/</t>
+          <t>https://www.onthemarket.com/details/19099769/</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Maiden Lane, Covent Garden, London, WC2E</t>
+          <t>Fletcher Buildings,, Covent Garden, London, WC2B</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>WC2E</t>
+          <t>WC2B</t>
         </is>
       </c>
       <c r="F25" s="4" t="n">
-        <v>3684</v>
+        <v>3792</v>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
@@ -2181,12 +2181,12 @@
         </is>
       </c>
       <c r="J25" s="4" t="n">
-        <v>630</v>
+        <v>320</v>
       </c>
       <c r="K25" s="4" t="n"/>
       <c r="L25" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat arranged on the 4th floor Bright and spacious reception room Smart dining room Modern kitchen; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Bright and airy one bedroom apartment in a prime Central London location Well proportioned reception with high ceilings and neutral décor Generous double bedroo; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M25" s="4" t="inlineStr">
@@ -2218,21 +2218,21 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19592443/</t>
+          <t>https://www.onthemarket.com/details/19453032/</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Regent Square, Bloomsbury, London, WC1H</t>
+          <t>Maiden Lane, Covent Garden, London, WC2E</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>WC1H</t>
+          <t>WC2E</t>
         </is>
       </c>
       <c r="F26" s="4" t="n">
-        <v>4312</v>
+        <v>3684</v>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
@@ -2246,117 +2246,117 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J26" s="4" t="n">
-        <v>487</v>
+        <v>630</v>
       </c>
       <c r="K26" s="4" t="n"/>
       <c r="L26" s="4" t="inlineStr">
         <is>
+          <t>1 bedroom flat arranged on the 4th floor Bright and spacious reception room Smart dining room Modern kitchen; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M26" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N26" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O26" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>1 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19592443/</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Regent Square, Bloomsbury, London, WC1H</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>WC1H</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>4312</v>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>1-Bed</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J27" s="4" t="n">
+        <v>487</v>
+      </c>
+      <c r="K27" s="4" t="n"/>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
           <t>Fantastic one bedroom apartment Set within beautiful period conversion Boasts ample interior space arranged over the second floor Wonderful balcony overlooking ; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
-      <c r="M26" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N26" s="4" t="inlineStr">
+      <c r="M27" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N27" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="O26" s="4" t="inlineStr">
+      <c r="O27" s="4" t="inlineStr">
         <is>
           <t>2026-07-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Apartment</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Rightmove</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>https://www.rightmove.co.uk/properties/89143989</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>Waterloo Road, Southwark, SE1</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>SE1</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="n">
-        <v>4346</v>
-      </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>2-Bed</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>Part Furnished</t>
-        </is>
-      </c>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t>Private balcony/terrace</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="n">
-        <v>1385</v>
-      </c>
-      <c r="K27" s="2" t="n"/>
-      <c r="L27" s="2" t="inlineStr">
-        <is>
-          <t>Two bedroom apartment with incredible views Waterloo Road SE1 250 Waterloo Road is an exciting new rental development conveniently located on Waterloo Road, SE1</t>
-        </is>
-      </c>
-      <c r="M27" s="2" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N27" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="O27" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>Apartment</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>OnTheMarket</t>
+          <t>Rightmove</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/4473051/</t>
+          <t>https://www.rightmove.co.uk/properties/89143989</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -2393,7 +2393,7 @@
       <c r="K28" s="2" t="n"/>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>Spectacular Views Waterloo</t>
+          <t>Two bedroom apartment with incredible views Waterloo Road SE1 250 Waterloo Road is an exciting new rental development conveniently located on Waterloo Road, SE1</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
@@ -2415,7 +2415,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -2425,12 +2425,12 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19728858/</t>
+          <t>https://www.onthemarket.com/details/4473051/</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Waterloo Road, London SE1</t>
+          <t>Waterloo Road, Southwark, SE1</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -2439,7 +2439,7 @@
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>4350</v>
+        <v>4346</v>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Part Furnished</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
@@ -2457,12 +2457,12 @@
         </is>
       </c>
       <c r="J29" s="2" t="n">
-        <v>1140</v>
+        <v>1385</v>
       </c>
       <c r="K29" s="2" t="n"/>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>Two Bedrooms Two Bathrooms</t>
+          <t>Spectacular Views Waterloo</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
@@ -2484,7 +2484,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -2494,12 +2494,12 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/6248222/</t>
+          <t>https://www.onthemarket.com/details/19728858/</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Nelson Square, Southwark, London, SE1</t>
+          <t>Waterloo Road, London SE1</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -2508,7 +2508,7 @@
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>3150</v>
+        <v>4350</v>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
@@ -2517,7 +2517,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -2526,12 +2526,12 @@
         </is>
       </c>
       <c r="J30" s="2" t="n">
-        <v>809</v>
+        <v>1140</v>
       </c>
       <c r="K30" s="2" t="n"/>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>Dishwasher Range / Oven</t>
+          <t>Two Bedrooms Two Bathrooms</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
@@ -2553,7 +2553,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -2563,21 +2563,21 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19663010/</t>
+          <t>https://www.onthemarket.com/details/6248222/</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Guilford Street, Bloomsbury, London, WC1N</t>
+          <t>Nelson Square, Southwark, London, SE1</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>WC1N</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>3684</v>
+        <v>3150</v>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Part Furnished</t>
+          <t>Unfurnished</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -2595,94 +2595,94 @@
         </is>
       </c>
       <c r="J31" s="2" t="n">
-        <v>691</v>
+        <v>809</v>
       </c>
       <c r="K31" s="2" t="n"/>
       <c r="L31" s="2" t="inlineStr">
         <is>
+          <t>Dishwasher Range / Oven</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19663010/</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Guilford Street, Bloomsbury, London, WC1N</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>WC1N</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="n">
+        <v>3684</v>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>2-Bed</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Part Furnished</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="n">
+        <v>691</v>
+      </c>
+      <c r="K32" s="2" t="n"/>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
           <t>Superb 2 bedroom flat on lower ground floor Modern open-plan kitchen with integrated appliance Spacious reception room leading to lovely private patio 2 well-pr</t>
         </is>
       </c>
-      <c r="M31" s="2" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N31" s="2" t="inlineStr">
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="O31" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t>2 bedroom apartment to rent</t>
-        </is>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C32" s="7" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/19809694/</t>
-        </is>
-      </c>
-      <c r="D32" s="6" t="inlineStr">
-        <is>
-          <t>Shaftesbury Avenue, Soho, W1D</t>
-        </is>
-      </c>
-      <c r="E32" s="6" t="inlineStr">
-        <is>
-          <t>W1D</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="n">
-        <v>3553</v>
-      </c>
-      <c r="G32" s="6" t="inlineStr">
-        <is>
-          <t>2-Bed</t>
-        </is>
-      </c>
-      <c r="H32" s="6" t="inlineStr">
-        <is>
-          <t>Flexible</t>
-        </is>
-      </c>
-      <c r="I32" s="6" t="inlineStr">
-        <is>
-          <t>Communal / shared</t>
-        </is>
-      </c>
-      <c r="J32" s="6" t="n">
-        <v>603</v>
-      </c>
-      <c r="K32" s="6" t="n"/>
-      <c r="L32" s="6" t="inlineStr">
-        <is>
-          <t>Beautifully Refurbished Secondary Glazing; outdoor space is communal/shared; under 650 sq ft</t>
-        </is>
-      </c>
-      <c r="M32" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N32" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O32" s="6" t="inlineStr">
+      <c r="O32" s="2" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
@@ -2701,12 +2701,12 @@
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/13368018/</t>
+          <t>https://www.onthemarket.com/details/19809694/</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>Shaftesbury Avenue , Soho, W1D</t>
+          <t>Shaftesbury Avenue, Soho, W1D</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
@@ -2715,7 +2715,7 @@
         </is>
       </c>
       <c r="F33" s="6" t="n">
-        <v>3987</v>
+        <v>3553</v>
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
@@ -2733,12 +2733,12 @@
         </is>
       </c>
       <c r="J33" s="6" t="n">
-        <v>671</v>
+        <v>603</v>
       </c>
       <c r="K33" s="6" t="n"/>
       <c r="L33" s="6" t="inlineStr">
         <is>
-          <t>Pet friendly Wooden Floors Student; outdoor space is communal/shared</t>
+          <t>Beautifully Refurbished Secondary Glazing; outdoor space is communal/shared; under 650 sq ft</t>
         </is>
       </c>
       <c r="M33" s="6" t="inlineStr">
@@ -2770,12 +2770,12 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19627828/</t>
+          <t>https://www.onthemarket.com/details/13368018/</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>Shaftesbury Avenue, Soho, W1D</t>
+          <t>Shaftesbury Avenue , Soho, W1D</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr">
@@ -2802,12 +2802,12 @@
         </is>
       </c>
       <c r="J34" s="6" t="n">
-        <v>802</v>
+        <v>671</v>
       </c>
       <c r="K34" s="6" t="n"/>
       <c r="L34" s="6" t="inlineStr">
         <is>
-          <t>Built in Storage Pet Friendly; outdoor space is communal/shared</t>
+          <t>Pet friendly Wooden Floors Student; outdoor space is communal/shared</t>
         </is>
       </c>
       <c r="M34" s="6" t="inlineStr">
@@ -2829,7 +2829,7 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
@@ -2839,12 +2839,12 @@
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19600564/</t>
+          <t>https://www.onthemarket.com/details/19627828/</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>Rupert Court, Soho, W1D</t>
+          <t>Shaftesbury Avenue, Soho, W1D</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
@@ -2853,11 +2853,11 @@
         </is>
       </c>
       <c r="F35" s="6" t="n">
-        <v>3163</v>
+        <v>3987</v>
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H35" s="6" t="inlineStr">
@@ -2870,11 +2870,13 @@
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J35" s="6" t="n"/>
+      <c r="J35" s="6" t="n">
+        <v>802</v>
+      </c>
       <c r="K35" s="6" t="n"/>
       <c r="L35" s="6" t="inlineStr">
         <is>
-          <t>Beautifully Refurbished Pet friendly; outdoor space is communal/shared; size not stated</t>
+          <t>Built in Storage Pet Friendly; outdoor space is communal/shared</t>
         </is>
       </c>
       <c r="M35" s="6" t="inlineStr">
@@ -2906,17 +2908,17 @@
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/10862827/</t>
+          <t>https://www.onthemarket.com/details/19600564/</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>Rupert Court, Soho W1</t>
+          <t>Rupert Court, Soho, W1D</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>W1D</t>
         </is>
       </c>
       <c r="F36" s="6" t="n">
@@ -2929,7 +2931,7 @@
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
@@ -2937,13 +2939,11 @@
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J36" s="6" t="n">
-        <v>603</v>
-      </c>
+      <c r="J36" s="6" t="n"/>
       <c r="K36" s="6" t="n"/>
       <c r="L36" s="6" t="inlineStr">
         <is>
-          <t>One bedroom One shower room; outdoor space is communal/shared; under 650 sq ft</t>
+          <t>Beautifully Refurbished Pet friendly; outdoor space is communal/shared; size not stated</t>
         </is>
       </c>
       <c r="M36" s="6" t="inlineStr">
@@ -2965,7 +2965,7 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
@@ -2975,21 +2975,21 @@
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19845642/</t>
+          <t>https://www.onthemarket.com/details/10862827/</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>Shelton Street, Covent Garden, London, WC2H</t>
+          <t>Rupert Court, Soho W1</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>WC2H</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="F37" s="6" t="n">
-        <v>3142</v>
+        <v>3163</v>
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Unfurnished</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
@@ -3007,12 +3007,12 @@
         </is>
       </c>
       <c r="J37" s="6" t="n">
-        <v>480</v>
+        <v>603</v>
       </c>
       <c r="K37" s="6" t="n"/>
       <c r="L37" s="6" t="inlineStr">
         <is>
-          <t>Superb one bedroom flat arranged on the second floor Spacious reception/kitchen with ample dining space; outdoor space is communal/shared; under 650 sq ft</t>
+          <t>One bedroom One shower room; outdoor space is communal/shared; under 650 sq ft</t>
         </is>
       </c>
       <c r="M37" s="6" t="inlineStr">
@@ -3034,7 +3034,7 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
@@ -3044,21 +3044,21 @@
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19603496/</t>
+          <t>https://www.onthemarket.com/details/19845642/</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>Arne Street, Covent Garden, WC2E</t>
+          <t>Shelton Street, Covent Garden, London, WC2H</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>WC2E</t>
+          <t>WC2H</t>
         </is>
       </c>
       <c r="F38" s="6" t="n">
-        <v>3250</v>
+        <v>3142</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -3067,7 +3067,7 @@
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>Unfurnished</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr">
@@ -3076,12 +3076,12 @@
         </is>
       </c>
       <c r="J38" s="6" t="n">
-        <v>514</v>
+        <v>480</v>
       </c>
       <c r="K38" s="6" t="n"/>
       <c r="L38" s="6" t="inlineStr">
         <is>
-          <t>Council Tax Band G 514 sq ft floor area; outdoor space is communal/shared; under 650 sq ft</t>
+          <t>Superb one bedroom flat arranged on the second floor Spacious reception/kitchen with ample dining space; outdoor space is communal/shared; under 650 sq ft</t>
         </is>
       </c>
       <c r="M38" s="6" t="inlineStr">
@@ -3103,7 +3103,7 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
@@ -3113,21 +3113,21 @@
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/14179323/</t>
+          <t>https://www.onthemarket.com/details/19603496/</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>Bloomsbury Square, Bloomsbury, Covent Garden, London, WC1A</t>
+          <t>Arne Street, Covent Garden, WC2E</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>WC1A</t>
+          <t>WC2E</t>
         </is>
       </c>
       <c r="F39" s="6" t="n">
-        <v>3500</v>
+        <v>3250</v>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
@@ -3136,7 +3136,7 @@
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>Part Furnished</t>
+          <t>Unfurnished</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr">
@@ -3145,12 +3145,12 @@
         </is>
       </c>
       <c r="J39" s="6" t="n">
-        <v>734</v>
+        <v>514</v>
       </c>
       <c r="K39" s="6" t="n"/>
       <c r="L39" s="6" t="inlineStr">
         <is>
-          <t>Stunning Period Conversion Hardwood Flooring Multi-Room Sound System and Mood Lighting Throughout Contemporary Kitchen &amp; Bathroom; outdoor space is communal/shared</t>
+          <t>Council Tax Band G 514 sq ft floor area; outdoor space is communal/shared; under 650 sq ft</t>
         </is>
       </c>
       <c r="M39" s="6" t="inlineStr">
@@ -3182,21 +3182,21 @@
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19823664/</t>
+          <t>https://www.onthemarket.com/details/14179323/</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>Bedford Court Mansions, Adeline Place, Bloomsbury, London, WC1B</t>
+          <t>Bloomsbury Square, Bloomsbury, Covent Garden, London, WC1A</t>
         </is>
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>WC1B</t>
+          <t>WC1A</t>
         </is>
       </c>
       <c r="F40" s="6" t="n">
-        <v>3141</v>
+        <v>3500</v>
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
@@ -3205,21 +3205,21 @@
       </c>
       <c r="H40" s="6" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Part Furnished</t>
         </is>
       </c>
       <c r="I40" s="6" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J40" s="6" t="n">
-        <v>573</v>
+        <v>734</v>
       </c>
       <c r="K40" s="6" t="n"/>
       <c r="L40" s="6" t="inlineStr">
         <is>
-          <t>One Bedroom Finished to high standard Lift Access Separate Kitchen; under 650 sq ft</t>
+          <t>Stunning Period Conversion Hardwood Flooring Multi-Room Sound System and Mood Lighting Throughout Contemporary Kitchen &amp; Bathroom; outdoor space is communal/shared</t>
         </is>
       </c>
       <c r="M40" s="6" t="inlineStr">
@@ -3241,7 +3241,7 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
@@ -3251,21 +3251,21 @@
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/15813612/</t>
+          <t>https://www.onthemarket.com/details/19823664/</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>Bloomsbury Square, Bloomsbury, WC1A</t>
+          <t>Bedford Court Mansions, Adeline Place, Bloomsbury, London, WC1B</t>
         </is>
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>WC1A</t>
+          <t>WC1B</t>
         </is>
       </c>
       <c r="F41" s="6" t="n">
-        <v>3142</v>
+        <v>3141</v>
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
@@ -3283,12 +3283,12 @@
         </is>
       </c>
       <c r="J41" s="6" t="n">
-        <v>539</v>
+        <v>573</v>
       </c>
       <c r="K41" s="6" t="n"/>
       <c r="L41" s="6" t="inlineStr">
         <is>
-          <t>Large Double Bedroom Period Features Student; under 650 sq ft</t>
+          <t>One Bedroom Finished to high standard Lift Access Separate Kitchen; under 650 sq ft</t>
         </is>
       </c>
       <c r="M41" s="6" t="inlineStr">
@@ -3310,7 +3310,7 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
@@ -3320,17 +3320,17 @@
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19736445/</t>
+          <t>https://www.onthemarket.com/details/15813612/</t>
         </is>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t>Millman Street, Bloomsbury, London, WC1N</t>
+          <t>Bloomsbury Square, Bloomsbury, WC1A</t>
         </is>
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>WC1N</t>
+          <t>WC1A</t>
         </is>
       </c>
       <c r="F42" s="6" t="n">
@@ -3343,7 +3343,7 @@
       </c>
       <c r="H42" s="6" t="inlineStr">
         <is>
-          <t>Part Furnished</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="I42" s="6" t="inlineStr">
@@ -3352,12 +3352,12 @@
         </is>
       </c>
       <c r="J42" s="6" t="n">
-        <v>542</v>
+        <v>539</v>
       </c>
       <c r="K42" s="6" t="n"/>
       <c r="L42" s="6" t="inlineStr">
         <is>
-          <t>Fantastic 1 bedroom flat arranged on the ground floor Set within a lovely residential block; under 650 sq ft</t>
+          <t>Large Double Bedroom Period Features Student; under 650 sq ft</t>
         </is>
       </c>
       <c r="M42" s="6" t="inlineStr">
@@ -3379,7 +3379,7 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
@@ -3389,30 +3389,30 @@
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19852978/</t>
+          <t>https://www.onthemarket.com/details/19736445/</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>Newport Court, Covent Garden, London, WC2H</t>
+          <t>Millman Street, Bloomsbury, London, WC1N</t>
         </is>
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>WC2H</t>
+          <t>WC1N</t>
         </is>
       </c>
       <c r="F43" s="6" t="n">
-        <v>4334</v>
+        <v>3142</v>
       </c>
       <c r="G43" s="6" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H43" s="6" t="inlineStr">
         <is>
-          <t>Furnished</t>
+          <t>Part Furnished</t>
         </is>
       </c>
       <c r="I43" s="6" t="inlineStr">
@@ -3421,12 +3421,12 @@
         </is>
       </c>
       <c r="J43" s="6" t="n">
-        <v>858</v>
+        <v>542</v>
       </c>
       <c r="K43" s="6" t="n"/>
       <c r="L43" s="6" t="inlineStr">
         <is>
-          <t>Splendid two bedroom flat Ample interiors; listed furnished — check if flexible</t>
+          <t>Fantastic 1 bedroom flat arranged on the ground floor Set within a lovely residential block; under 650 sq ft</t>
         </is>
       </c>
       <c r="M43" s="6" t="inlineStr">
@@ -3448,7 +3448,7 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>2 bedroom end of terrace house to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
@@ -3458,17 +3458,21 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19811489/</t>
+          <t>https://www.onthemarket.com/details/19852978/</t>
         </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>Carlisle Lane, Waterloo</t>
-        </is>
-      </c>
-      <c r="E44" s="6" t="n"/>
+          <t>Newport Court, Covent Garden, London, WC2H</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="inlineStr">
+        <is>
+          <t>WC2H</t>
+        </is>
+      </c>
       <c r="F44" s="6" t="n">
-        <v>3575</v>
+        <v>4334</v>
       </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
@@ -3486,94 +3490,90 @@
         </is>
       </c>
       <c r="J44" s="6" t="n">
-        <v>904</v>
+        <v>858</v>
       </c>
       <c r="K44" s="6" t="n"/>
       <c r="L44" s="6" t="inlineStr">
         <is>
+          <t>Splendid two bedroom flat Ample interiors; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M44" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N44" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O44" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>2 bedroom end of terrace house to rent</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19811489/</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="inlineStr">
+        <is>
+          <t>Carlisle Lane, Waterloo</t>
+        </is>
+      </c>
+      <c r="E45" s="6" t="n"/>
+      <c r="F45" s="6" t="n">
+        <v>3575</v>
+      </c>
+      <c r="G45" s="6" t="inlineStr">
+        <is>
+          <t>2-Bed</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I45" s="6" t="inlineStr">
+        <is>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J45" s="6" t="n">
+        <v>904</v>
+      </c>
+      <c r="K45" s="6" t="n"/>
+      <c r="L45" s="6" t="inlineStr">
+        <is>
           <t>End of Terrace Shared Garden; listed furnished — check if flexible</t>
         </is>
       </c>
-      <c r="M44" s="6" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N44" s="6" t="inlineStr">
+      <c r="M45" s="6" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N45" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="O44" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>2 bedroom apartment to rent</t>
-        </is>
-      </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>OnTheMarket</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>https://www.onthemarket.com/details/16157050/</t>
-        </is>
-      </c>
-      <c r="D45" s="4" t="inlineStr">
-        <is>
-          <t>Brewer Street, Soho, W1F</t>
-        </is>
-      </c>
-      <c r="E45" s="4" t="inlineStr">
-        <is>
-          <t>W1F</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="n">
-        <v>3142</v>
-      </c>
-      <c r="G45" s="4" t="inlineStr">
-        <is>
-          <t>2-Bed</t>
-        </is>
-      </c>
-      <c r="H45" s="4" t="inlineStr">
-        <is>
-          <t>Furnished</t>
-        </is>
-      </c>
-      <c r="I45" s="4" t="inlineStr">
-        <is>
-          <t>Communal / shared</t>
-        </is>
-      </c>
-      <c r="J45" s="4" t="n">
-        <v>730</v>
-      </c>
-      <c r="K45" s="4" t="n"/>
-      <c r="L45" s="4" t="inlineStr">
-        <is>
-          <t>730 sqft Secure Entrance; outdoor space is communal/shared; listed furnished — check if flexible</t>
-        </is>
-      </c>
-      <c r="M45" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N45" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="O45" s="4" t="inlineStr">
+      <c r="O45" s="6" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
@@ -3582,7 +3582,7 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
@@ -3592,25 +3592,25 @@
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19786051/</t>
+          <t>https://www.onthemarket.com/details/16157050/</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Old Compton Street, Soho, London, W1D</t>
+          <t>Brewer Street, Soho, W1F</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>W1D</t>
+          <t>W1F</t>
         </is>
       </c>
       <c r="F46" s="4" t="n">
-        <v>3600</v>
+        <v>3142</v>
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr">
@@ -3624,12 +3624,12 @@
         </is>
       </c>
       <c r="J46" s="4" t="n">
-        <v>432</v>
+        <v>730</v>
       </c>
       <c r="K46" s="4" t="n"/>
       <c r="L46" s="4" t="inlineStr">
         <is>
-          <t>432 sq ft floor area Nearest station 0.1mi. Furnished Nearest school 0.2mi.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>730 sqft Secure Entrance; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M46" s="4" t="inlineStr">
@@ -3651,7 +3651,7 @@
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
@@ -3661,25 +3661,25 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/11345150/</t>
+          <t>https://www.onthemarket.com/details/19786051/</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Shaftesbury Avenue, Covent Garden, London, WC2H</t>
+          <t>Old Compton Street, Soho, London, W1D</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>WC2H</t>
+          <t>W1D</t>
         </is>
       </c>
       <c r="F47" s="4" t="n">
-        <v>3575</v>
+        <v>3600</v>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr">
@@ -3693,12 +3693,12 @@
         </is>
       </c>
       <c r="J47" s="4" t="n">
-        <v>870</v>
+        <v>432</v>
       </c>
       <c r="K47" s="4" t="n"/>
       <c r="L47" s="4" t="inlineStr">
         <is>
-          <t>870 sq ft floor area Nearest station 0.1mi.; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>432 sq ft floor area Nearest station 0.1mi. Furnished Nearest school 0.2mi.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M47" s="4" t="inlineStr">
@@ -3720,7 +3720,7 @@
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
@@ -3730,25 +3730,25 @@
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/15707269/</t>
+          <t>https://www.onthemarket.com/details/11345150/</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Casson Square, London, Waterloo, United Kingdom, SE1</t>
+          <t>Shaftesbury Avenue, Covent Garden, London, WC2H</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>SE1</t>
+          <t>WC2H</t>
         </is>
       </c>
       <c r="F48" s="4" t="n">
-        <v>4050</v>
+        <v>3575</v>
       </c>
       <c r="G48" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H48" s="4" t="inlineStr">
@@ -3762,12 +3762,12 @@
         </is>
       </c>
       <c r="J48" s="4" t="n">
-        <v>514</v>
+        <v>870</v>
       </c>
       <c r="K48" s="4" t="n"/>
       <c r="L48" s="4" t="inlineStr">
         <is>
-          <t>Bedroom Bathroom Open-plan reception/kitchen 24 hour concierge; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>870 sq ft floor area Nearest station 0.1mi.; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M48" s="4" t="inlineStr">
@@ -3799,12 +3799,12 @@
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/9568931/</t>
+          <t>https://www.onthemarket.com/details/15707269/</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>Casson Square, Waterloo, Southbank Place, London, SE1</t>
+          <t>Casson Square, London, Waterloo, United Kingdom, SE1</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
@@ -3813,7 +3813,7 @@
         </is>
       </c>
       <c r="F49" s="4" t="n">
-        <v>4250</v>
+        <v>4050</v>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
@@ -3827,16 +3827,16 @@
       </c>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J49" s="4" t="n">
-        <v>644</v>
+        <v>514</v>
       </c>
       <c r="K49" s="4" t="n"/>
       <c r="L49" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom 1 bathroom Open-plan reception kitchen 24-hour five-star concierge; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Bedroom Bathroom Open-plan reception/kitchen 24 hour concierge; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M49" s="4" t="inlineStr">
@@ -3858,7 +3858,7 @@
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
@@ -3868,12 +3868,12 @@
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/7516361/</t>
+          <t>https://www.onthemarket.com/details/9568931/</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>Belvedere Road, Waterloo, London, SE1</t>
+          <t>Casson Square, Waterloo, Southbank Place, London, SE1</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
@@ -3882,11 +3882,11 @@
         </is>
       </c>
       <c r="F50" s="4" t="n">
-        <v>3350</v>
+        <v>4250</v>
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H50" s="4" t="inlineStr">
@@ -3896,16 +3896,16 @@
       </c>
       <c r="I50" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Private balcony/terrace</t>
         </is>
       </c>
       <c r="J50" s="4" t="n">
-        <v>544</v>
+        <v>644</v>
       </c>
       <c r="K50" s="4" t="n"/>
       <c r="L50" s="4" t="inlineStr">
         <is>
-          <t>Residents' swimming pool and gym. Grade II listed period building. 24 hour porters. Set close to the iconic Southbank and London Eye.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>1 bedroom 1 bathroom Open-plan reception kitchen 24-hour five-star concierge; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M50" s="4" t="inlineStr">
@@ -3927,7 +3927,7 @@
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
@@ -3937,12 +3937,12 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/7589011/</t>
+          <t>https://www.onthemarket.com/details/7516361/</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>Belvedere Road, London, Waterloo, SE1</t>
+          <t>Belvedere Road, Waterloo, London, SE1</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
@@ -3951,11 +3951,11 @@
         </is>
       </c>
       <c r="F51" s="4" t="n">
-        <v>4200</v>
+        <v>3350</v>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H51" s="4" t="inlineStr">
@@ -3969,12 +3969,12 @@
         </is>
       </c>
       <c r="J51" s="4" t="n">
-        <v>671</v>
+        <v>544</v>
       </c>
       <c r="K51" s="4" t="n"/>
       <c r="L51" s="4" t="inlineStr">
         <is>
-          <t>24-hour five-star concierge 18,000 sq ft gym and spa facilities Set in one of London's most connected locations, opposite Westminster and the Houses of Parliame; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>Residents' swimming pool and gym. Grade II listed period building. 24 hour porters. Set close to the iconic Southbank and London Eye.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M51" s="4" t="inlineStr">
@@ -3996,7 +3996,7 @@
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
@@ -4006,21 +4006,21 @@
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19863550/</t>
+          <t>https://www.onthemarket.com/details/7589011/</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>King Street, Covent Garden, London, WC2E</t>
+          <t>Belvedere Road, London, Waterloo, SE1</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>WC2E</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F52" s="4" t="n">
-        <v>3358</v>
+        <v>4200</v>
       </c>
       <c r="G52" s="4" t="inlineStr">
         <is>
@@ -4038,12 +4038,12 @@
         </is>
       </c>
       <c r="J52" s="4" t="n">
-        <v>455</v>
+        <v>671</v>
       </c>
       <c r="K52" s="4" t="n"/>
       <c r="L52" s="4" t="inlineStr">
         <is>
-          <t>Iconic Covent Garden location Finished to an excellent standard throughout High ceilings Wooden flooring throughout; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>24-hour five-star concierge 18,000 sq ft gym and spa facilities Set in one of London's most connected locations, opposite Westminster and the Houses of Parliame; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M52" s="4" t="inlineStr">
@@ -4065,7 +4065,7 @@
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
@@ -4075,21 +4075,21 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19860280/</t>
+          <t>https://www.onthemarket.com/details/19863550/</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>Floral Street, Covent Garden WC2</t>
+          <t>King Street, Covent Garden, London, WC2E</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>WC2</t>
+          <t>WC2E</t>
         </is>
       </c>
       <c r="F53" s="4" t="n">
-        <v>3380</v>
+        <v>3358</v>
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
@@ -4107,12 +4107,12 @@
         </is>
       </c>
       <c r="J53" s="4" t="n">
-        <v>495</v>
+        <v>455</v>
       </c>
       <c r="K53" s="4" t="n"/>
       <c r="L53" s="4" t="inlineStr">
         <is>
-          <t>One bedroom One bathroom, ensuite; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Iconic Covent Garden location Finished to an excellent standard throughout High ceilings Wooden flooring throughout; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M53" s="4" t="inlineStr">
@@ -4144,21 +4144,21 @@
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/1837052/</t>
+          <t>https://www.onthemarket.com/details/19860280/</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>King Street, Covent Garden, WC2E</t>
+          <t>Floral Street, Covent Garden WC2</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>WC2E</t>
+          <t>WC2</t>
         </is>
       </c>
       <c r="F54" s="4" t="n">
-        <v>3358</v>
+        <v>3380</v>
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
@@ -4176,12 +4176,12 @@
         </is>
       </c>
       <c r="J54" s="4" t="n">
-        <v>455</v>
+        <v>495</v>
       </c>
       <c r="K54" s="4" t="n"/>
       <c r="L54" s="4" t="inlineStr">
         <is>
-          <t>Furnished Recently refurbished; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>One bedroom One bathroom, ensuite; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M54" s="4" t="inlineStr">
@@ -4213,12 +4213,12 @@
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/3408032/</t>
+          <t>https://www.onthemarket.com/details/1837052/</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>Floral Street, Covent Garden, WC2E</t>
+          <t>King Street, Covent Garden, WC2E</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
@@ -4227,7 +4227,7 @@
         </is>
       </c>
       <c r="F55" s="4" t="n">
-        <v>3380</v>
+        <v>3358</v>
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
@@ -4245,12 +4245,12 @@
         </is>
       </c>
       <c r="J55" s="4" t="n">
-        <v>398</v>
+        <v>455</v>
       </c>
       <c r="K55" s="4" t="n"/>
       <c r="L55" s="4" t="inlineStr">
         <is>
-          <t>Newly Refurbished Central Location; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Furnished Recently refurbished; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M55" s="4" t="inlineStr">
@@ -4272,7 +4272,7 @@
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom apartment to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
@@ -4282,25 +4282,25 @@
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/3102769/</t>
+          <t>https://www.onthemarket.com/details/3408032/</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>John Adam Street, Covent Garden, WC2N</t>
+          <t>Floral Street, Covent Garden, WC2E</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>WC2N</t>
+          <t>WC2E</t>
         </is>
       </c>
       <c r="F56" s="4" t="n">
-        <v>3185</v>
+        <v>3380</v>
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H56" s="4" t="inlineStr">
@@ -4314,12 +4314,12 @@
         </is>
       </c>
       <c r="J56" s="4" t="n">
-        <v>655</v>
+        <v>398</v>
       </c>
       <c r="K56" s="4" t="n"/>
       <c r="L56" s="4" t="inlineStr">
         <is>
-          <t>Concierge Close to the area's Universities for students and academics; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>Newly Refurbished Central Location; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M56" s="4" t="inlineStr">
@@ -4341,7 +4341,7 @@
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>2 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
@@ -4351,25 +4351,25 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19733694/</t>
+          <t>https://www.onthemarket.com/details/3102769/</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>Maiden Lane, Covent Garden, London, WC2E</t>
+          <t>John Adam Street, Covent Garden, WC2N</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>WC2E</t>
+          <t>WC2N</t>
         </is>
       </c>
       <c r="F57" s="4" t="n">
-        <v>3684</v>
+        <v>3185</v>
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H57" s="4" t="inlineStr">
@@ -4383,12 +4383,12 @@
         </is>
       </c>
       <c r="J57" s="4" t="n">
-        <v>630</v>
+        <v>655</v>
       </c>
       <c r="K57" s="4" t="n"/>
       <c r="L57" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat arranged on the 4th floor Bright and spacious reception room; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Concierge Close to the area's Universities for students and academics; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M57" s="4" t="inlineStr">
@@ -4420,21 +4420,21 @@
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19725776/</t>
+          <t>https://www.onthemarket.com/details/19733694/</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>Shelton Street, Covent Garden, London, WC2H</t>
+          <t>Maiden Lane, Covent Garden, London, WC2E</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>WC2H</t>
+          <t>WC2E</t>
         </is>
       </c>
       <c r="F58" s="4" t="n">
-        <v>3500</v>
+        <v>3684</v>
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
@@ -4448,16 +4448,16 @@
       </c>
       <c r="I58" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
+          <t>Communal / shared</t>
         </is>
       </c>
       <c r="J58" s="4" t="n">
-        <v>608</v>
+        <v>630</v>
       </c>
       <c r="K58" s="4" t="n"/>
       <c r="L58" s="4" t="inlineStr">
         <is>
-          <t>Stylish one bedroom, third floor apartment Beautifully proportioned open plan reception with balcony access; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>1 bedroom flat arranged on the 4th floor Bright and spacious reception room; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M58" s="4" t="inlineStr">
@@ -4479,7 +4479,7 @@
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
@@ -4489,21 +4489,21 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19591709/</t>
+          <t>https://www.onthemarket.com/details/19725776/</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>King Street, Covent Garden WC2</t>
+          <t>Shelton Street, Covent Garden, London, WC2H</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>WC2</t>
+          <t>WC2H</t>
         </is>
       </c>
       <c r="F59" s="4" t="n">
-        <v>3575</v>
+        <v>3500</v>
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
@@ -4517,16 +4517,16 @@
       </c>
       <c r="I59" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
+          <t>Private balcony/terrace</t>
         </is>
       </c>
       <c r="J59" s="4" t="n">
-        <v>441</v>
+        <v>608</v>
       </c>
       <c r="K59" s="4" t="n"/>
       <c r="L59" s="4" t="inlineStr">
         <is>
-          <t>One double bedroom One bathroom; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Stylish one bedroom, third floor apartment Beautifully proportioned open plan reception with balcony access; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M59" s="4" t="inlineStr">
@@ -4558,7 +4558,7 @@
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19591720/</t>
+          <t>https://www.onthemarket.com/details/19591709/</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
@@ -4572,7 +4572,7 @@
         </is>
       </c>
       <c r="F60" s="4" t="n">
-        <v>4333</v>
+        <v>3575</v>
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
@@ -4590,12 +4590,12 @@
         </is>
       </c>
       <c r="J60" s="4" t="n">
-        <v>667</v>
+        <v>441</v>
       </c>
       <c r="K60" s="4" t="n"/>
       <c r="L60" s="4" t="inlineStr">
         <is>
-          <t>One bedroom One bathroom; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>One double bedroom One bathroom; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M60" s="4" t="inlineStr">
@@ -4617,7 +4617,7 @@
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
@@ -4627,25 +4627,25 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19511649/</t>
+          <t>https://www.onthemarket.com/details/19591720/</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>Broad Court, Covent Garden, London, WC2B</t>
+          <t>King Street, Covent Garden WC2</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>WC2B</t>
+          <t>WC2</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>3684</v>
+        <v>4333</v>
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
-          <t>2-Bed</t>
+          <t>1-Bed</t>
         </is>
       </c>
       <c r="H61" s="4" t="inlineStr">
@@ -4659,12 +4659,12 @@
         </is>
       </c>
       <c r="J61" s="4" t="n">
-        <v>811</v>
+        <v>667</v>
       </c>
       <c r="K61" s="4" t="n"/>
       <c r="L61" s="4" t="inlineStr">
         <is>
-          <t>2 bedroom flat arranged on raised ground floor Attractive period building with a sought-after location; outdoor space is communal/shared; listed furnished — check if flexible</t>
+          <t>One bedroom One bathroom; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M61" s="4" t="inlineStr">
@@ -4686,7 +4686,7 @@
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>2 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
@@ -4696,25 +4696,25 @@
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19500342/</t>
+          <t>https://www.onthemarket.com/details/19511649/</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>Covent Garden, West End, London, WC2E</t>
+          <t>Broad Court, Covent Garden, London, WC2B</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>WC2E</t>
+          <t>WC2B</t>
         </is>
       </c>
       <c r="F62" s="4" t="n">
-        <v>3700</v>
+        <v>3684</v>
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
-          <t>1-Bed</t>
+          <t>2-Bed</t>
         </is>
       </c>
       <c r="H62" s="4" t="inlineStr">
@@ -4727,11 +4727,13 @@
           <t>Communal / shared</t>
         </is>
       </c>
-      <c r="J62" s="4" t="n"/>
+      <c r="J62" s="4" t="n">
+        <v>811</v>
+      </c>
       <c r="K62" s="4" t="n"/>
       <c r="L62" s="4" t="inlineStr">
         <is>
-          <t>Short Term Stay between 1-6 months Furnished Ground Floor of secure block Heart of Covent Garden; outdoor space is communal/shared; size not stated; listed furnished — check if flexible</t>
+          <t>2 bedroom flat arranged on raised ground floor Attractive period building with a sought-after location; outdoor space is communal/shared; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M62" s="4" t="inlineStr">
@@ -4753,7 +4755,7 @@
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom apartment to rent</t>
+          <t>1 bedroom flat to rent</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
@@ -4763,21 +4765,21 @@
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/9591535/</t>
+          <t>https://www.onthemarket.com/details/19500342/</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>Casson Square, Waterloo, Southbank Place, London, SE1</t>
+          <t>Covent Garden, West End, London, WC2E</t>
         </is>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>SE1</t>
+          <t>WC2E</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>4075</v>
+        <v>3700</v>
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
@@ -4791,16 +4793,14 @@
       </c>
       <c r="I63" s="4" t="inlineStr">
         <is>
-          <t>Private balcony/terrace</t>
-        </is>
-      </c>
-      <c r="J63" s="4" t="n">
-        <v>641</v>
-      </c>
+          <t>Communal / shared</t>
+        </is>
+      </c>
+      <c r="J63" s="4" t="n"/>
       <c r="K63" s="4" t="n"/>
       <c r="L63" s="4" t="inlineStr">
         <is>
-          <t>*video viewing available* 24-hour five-star concierge 18,000 sq ft gym, pool and spa facilities Bedroom; under 650 sq ft; listed furnished — check if flexible</t>
+          <t>Short Term Stay between 1-6 months Furnished Ground Floor of secure block Heart of Covent Garden; outdoor space is communal/shared; size not stated; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M63" s="4" t="inlineStr">
@@ -4822,7 +4822,7 @@
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>1 bedroom flat to rent</t>
+          <t>1 bedroom apartment to rent</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
@@ -4832,21 +4832,21 @@
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19815346/</t>
+          <t>https://www.onthemarket.com/details/9591535/</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>Bloomsbury, London, WC1N</t>
+          <t>Casson Square, Waterloo, Southbank Place, London, SE1</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>WC1N</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="F64" s="4" t="n">
-        <v>3000</v>
+        <v>4075</v>
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
@@ -4863,11 +4863,13 @@
           <t>Private balcony/terrace</t>
         </is>
       </c>
-      <c r="J64" s="4" t="n"/>
+      <c r="J64" s="4" t="n">
+        <v>641</v>
+      </c>
       <c r="K64" s="4" t="n"/>
       <c r="L64" s="4" t="inlineStr">
         <is>
-          <t>No Agent Fees Property Reference Number: 2942192; size not stated; listed furnished — check if flexible</t>
+          <t>*video viewing available* 24-hour five-star concierge 18,000 sq ft gym, pool and spa facilities Bedroom; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
       <c r="M64" s="4" t="inlineStr">
@@ -4899,17 +4901,17 @@
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>https://www.onthemarket.com/details/19715608/</t>
+          <t>https://www.onthemarket.com/details/19815346/</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>Bloomsbury Square, London WC1A</t>
+          <t>Bloomsbury, London, WC1N</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>WC1A</t>
+          <t>WC1N</t>
         </is>
       </c>
       <c r="F65" s="4" t="n">
@@ -4927,36 +4929,103 @@
       </c>
       <c r="I65" s="4" t="inlineStr">
         <is>
-          <t>Communal / shared</t>
-        </is>
-      </c>
-      <c r="J65" s="4" t="n">
-        <v>581</v>
-      </c>
+          <t>Private balcony/terrace</t>
+        </is>
+      </c>
+      <c r="J65" s="4" t="n"/>
       <c r="K65" s="4" t="n"/>
       <c r="L65" s="4" t="inlineStr">
         <is>
+          <t>No Agent Fees Property Reference Number: 2942192; size not stated; listed furnished — check if flexible</t>
+        </is>
+      </c>
+      <c r="M65" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N65" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O65" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>1 bedroom flat to rent</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>OnTheMarket</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19715608/</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>Bloomsbury Square, London WC1A</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>WC1A</t>
+        </is>
+      </c>
+      <c r="F66" s="4" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G66" s="4" t="inlineStr">
+        <is>
+          <t>1-Bed</t>
+        </is>
+      </c>
+      <c r="H66" s="4" t="inlineStr">
+        <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="I66" s="4" t="inlineStr">
+        <is>
+          <t>Communal / shared</t>
+        </is>
+      </c>
+      <c r="J66" s="4" t="n">
+        <v>581</v>
+      </c>
+      <c r="K66" s="4" t="n"/>
+      <c r="L66" s="4" t="inlineStr">
+        <is>
           <t>Period Building Concierge; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
         </is>
       </c>
-      <c r="M65" s="4" t="inlineStr">
-        <is>
-          <t>NEW 🔴</t>
-        </is>
-      </c>
-      <c r="N65" s="4" t="inlineStr">
+      <c r="M66" s="4" t="inlineStr">
+        <is>
+          <t>NEW 🔴</t>
+        </is>
+      </c>
+      <c r="N66" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="O65" s="4" t="inlineStr">
+      <c r="O66" s="4" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O65"/>
+  <autoFilter ref="A1:O66"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
@@ -5022,6 +5091,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId63"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId65"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily tracker update 2026-07-14
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -599,7 +599,7 @@
       <c r="J2" s="6" t="n">
         <v>907</v>
       </c>
-      <c r="K2" s="6" t="inlineStr"/>
+      <c r="K2" s="6" t="n"/>
       <c r="L2" s="6" t="inlineStr">
         <is>
           <t>This elegant two bedroom apartment, with private balcony, luxurious furnishings and excellent finishes is available to lease through Prime London ...; listed furnished — check if flexible</t>
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="J3" s="4" t="n"/>
-      <c r="K3" s="4" t="inlineStr"/>
+      <c r="K3" s="4" t="n"/>
       <c r="L3" s="4" t="inlineStr">
         <is>
           <t>Two Double Bedrooms Two Bathrooms (One En Suite) Open Plan Reception Modern Kitchen; size not stated; listed furnished — check if flexible</t>
@@ -12142,7 +12142,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D304"/>
+  <dimension ref="A1:D305"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18818,6 +18818,28 @@
         </is>
       </c>
     </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>https://www.zoopla.co.uk/to-rent/details/67791860/</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>3142|2-bed|se1</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>2026-07-14 03:39</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily tracker update 2026-07-15
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -599,7 +599,7 @@
       <c r="J2" s="4" t="n">
         <v>597</v>
       </c>
-      <c r="K2" s="4" t="inlineStr"/>
+      <c r="K2" s="4" t="n"/>
       <c r="L2" s="4" t="inlineStr">
         <is>
           <t>597 sq ft floor area Nearest station 0.4mi.; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
@@ -13122,7 +13122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D336"/>
+  <dimension ref="A1:D337"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20502,6 +20502,28 @@
         </is>
       </c>
     </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/3788711/</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>3315|2-bed|w1t</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>2026-07-15 00:40</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily tracker update 2026-07-16
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -14316,7 +14316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D371"/>
+  <dimension ref="A1:D372"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22466,6 +22466,28 @@
         </is>
       </c>
     </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/17634647/</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>3077|1-bed|w1f</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>2026-07-16 01:39</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily tracker update 2026-07-17
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -14874,7 +14874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D397"/>
+  <dimension ref="A1:D398"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23586,6 +23586,28 @@
         </is>
       </c>
     </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>https://www.zoopla.co.uk/to-rent/details/73738221/</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>3888|1-bed|ec1v</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>2026-07-17 00:23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily tracker update 2026-07-18
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -16354,7 +16354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D429"/>
+  <dimension ref="A1:D430"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25760,6 +25760,28 @@
         </is>
       </c>
     </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/9282040/</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>3466|1-bed|ec1v</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>2026-07-18 00:39</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily tracker update 2026-07-19
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -16564,7 +16564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D435"/>
+  <dimension ref="A1:D436"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26102,6 +26102,28 @@
         </is>
       </c>
     </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/1436674/</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>3250|2-bed|wc2e</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>2026-07-19 00:39</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily tracker update 2026-07-20
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="J2" s="4" t="n"/>
-      <c r="K2" s="4" t="inlineStr"/>
+      <c r="K2" s="4" t="n"/>
       <c r="L2" s="4" t="inlineStr">
         <is>
           <t>No Agent Fees Students Can Enquire; size not stated; listed furnished — check if flexible</t>
@@ -666,7 +666,7 @@
       <c r="J3" s="4" t="n">
         <v>635</v>
       </c>
-      <c r="K3" s="4" t="inlineStr"/>
+      <c r="K3" s="4" t="n"/>
       <c r="L3" s="4" t="inlineStr">
         <is>
           <t>Presented in excellent condition throughout Spacious reception room Modern open-plan kitchen Generous bedroom; under 650 sq ft; listed furnished — check if flexible</t>

</xml_diff>

<commit_message>
Daily tracker update 2026-07-21
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -599,7 +599,7 @@
       <c r="J2" s="6" t="n">
         <v>565</v>
       </c>
-      <c r="K2" s="6" t="inlineStr"/>
+      <c r="K2" s="6" t="n"/>
       <c r="L2" s="6" t="inlineStr">
         <is>
           <t>ZERO DEPOSIT AVAILABLE. LONG LET. Set on the 8th floor, this 1 bedroom flat boasts stylish interiors including a large open-plan reception room, a modern kitche; under 650 sq ft</t>
@@ -668,7 +668,7 @@
       <c r="J3" s="6" t="n">
         <v>538</v>
       </c>
-      <c r="K3" s="6" t="inlineStr"/>
+      <c r="K3" s="6" t="n"/>
       <c r="L3" s="6" t="inlineStr">
         <is>
           <t>Regent are excited to present this modern one-bedroom apartment as a part of Brandon House, conveniently located immediately opposite Borough ...; under 650 sq ft; furnishing not stated</t>
@@ -18024,7 +18024,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D478"/>
+  <dimension ref="A1:D479"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28508,6 +28508,28 @@
         </is>
       </c>
     </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>https://www.rightmove.co.uk/properties/91155588</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>3150|2-bed|w1</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>2026-07-21 13:40</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily tracker update 2026-07-22
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -18302,7 +18302,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D487"/>
+  <dimension ref="A1:D488"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28984,6 +28984,28 @@
         </is>
       </c>
     </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>https://www.zoopla.co.uk/to-rent/details/73781519/</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>3179|1-bed|cb1</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>2026-07-22 00:39</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily tracker update 2026-07-23
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -599,7 +599,7 @@
       <c r="J2" s="4" t="n">
         <v>676</v>
       </c>
-      <c r="K2" s="4" t="inlineStr"/>
+      <c r="K2" s="4" t="n"/>
       <c r="L2" s="4" t="inlineStr">
         <is>
           <t>For viewing requests, please email us. Key features: – 2 bedrooms, 1 bathroom – Parking: Underground parking – Furnishings: Furnished – A holding ...; outdoor space is communal/shared; listed furnished — check if flexible</t>
@@ -19220,7 +19220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D510"/>
+  <dimension ref="A1:D512"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30408,6 +30408,50 @@
         </is>
       </c>
     </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>https://www.rightmove.co.uk/properties/89701275</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>4350|2-bed|ec1v</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>2026-07-23 00:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>https://www.zoopla.co.uk/to-rent/details/73792410/</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>4335|1-bed|w1f</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>2026-07-23 00:39</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily tracker update 2026-07-24
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -19916,7 +19916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D533"/>
+  <dimension ref="A1:D534"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31600,6 +31600,28 @@
         </is>
       </c>
     </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>https://www.zoopla.co.uk/to-rent/details/73804145/</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>3185|1-bed|ec1v</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D534" t="inlineStr">
+        <is>
+          <t>2026-07-24 09:39</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily tracker update 2026-07-25
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -20262,7 +20262,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D541"/>
+  <dimension ref="A1:D542"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32122,6 +32122,28 @@
         </is>
       </c>
     </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/19903971/</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>3207|2-bed|w1t</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D542" t="inlineStr">
+        <is>
+          <t>2026-07-25 23:10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily tracker update 2026-07-26
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -20262,7 +20262,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D542"/>
+  <dimension ref="A1:D543"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32144,6 +32144,28 @@
         </is>
       </c>
     </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>https://www.zoopla.co.uk/to-rent/details/73815668/</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>3898|1-bed|ec1v</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>2026-07-26 00:40</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily tracker update 2026-07-27
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -573,7 +573,7 @@
           <t>The Perspective Building, 100 Westminster Bridge Road, Waterloo</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="n">
         <v>3098</v>
       </c>
@@ -595,7 +595,7 @@
       <c r="J2" s="2" t="n">
         <v>774</v>
       </c>
-      <c r="K2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="n"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Two bedroom two bathroom apartment 774 sq ft (71.9 sqm)</t>
@@ -32238,7 +32238,6 @@
           <t>https://www.onthemarket.com/details/14270798/</t>
         </is>
       </c>
-      <c r="B544" t="inlineStr"/>
       <c r="C544" t="inlineStr">
         <is>
           <t>private</t>

</xml_diff>

<commit_message>
Daily tracker update 2026-07-28
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -20748,7 +20748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D557"/>
+  <dimension ref="A1:D558"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32955,6 +32955,28 @@
         </is>
       </c>
     </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/17772141/</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>4100|2-bed|wc1x</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>2026-07-28 01:40</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily tracker update 2026-07-29
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -21102,7 +21102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D576"/>
+  <dimension ref="A1:D577"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33727,6 +33727,28 @@
         </is>
       </c>
     </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>https://www.zoopla.co.uk/to-rent/details/73836927/</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>4247||se1</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>2026-07-29 00:39</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily tracker update 2026-08-01
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -672,7 +672,7 @@
       <c r="J3" s="2" t="n">
         <v>767</v>
       </c>
-      <c r="K3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="n"/>
       <c r="L3" s="2" t="inlineStr">
         <is>
           <t>Zero deposit available. Long let. Set in a wonderful development, this 2 bedroom flat boasts well arranged interiors including a large reception ...</t>
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="J9" s="6" t="n"/>
-      <c r="K9" s="6" t="inlineStr"/>
+      <c r="K9" s="6" t="n"/>
       <c r="L9" s="6" t="inlineStr">
         <is>
           <t>1 bedroom 1 reception room 1 bathroom Concierge; outdoor space is communal/shared; size not stated</t>
@@ -1169,7 +1169,7 @@
       <c r="J10" s="6" t="n">
         <v>1307</v>
       </c>
-      <c r="K10" s="6" t="inlineStr"/>
+      <c r="K10" s="6" t="n"/>
       <c r="L10" s="6" t="inlineStr">
         <is>
           <t>Spacious 2 bedroom flat Separate kitchen; furnishing not stated</t>
@@ -1236,7 +1236,7 @@
         </is>
       </c>
       <c r="J11" s="6" t="n"/>
-      <c r="K11" s="6" t="inlineStr"/>
+      <c r="K11" s="6" t="n"/>
       <c r="L11" s="6" t="inlineStr">
         <is>
           <t>Brand new, high-rise, luxury, furnished apartments in zone 1. Knight Frank are delighted to present Shard Place - a selection of studios, 1,2 &amp; 3 ...; size not stated</t>
@@ -1303,7 +1303,7 @@
         </is>
       </c>
       <c r="J12" s="6" t="n"/>
-      <c r="K12" s="6" t="inlineStr"/>
+      <c r="K12" s="6" t="n"/>
       <c r="L12" s="6" t="inlineStr">
         <is>
           <t>Premium two bedroom apartments in the heart of Elephant Park, offering contemporary homes, exceptional resident amenities and a prime Zone 1 ...; size not stated; furnishing not stated</t>
@@ -1372,7 +1372,7 @@
       <c r="J13" s="6" t="n">
         <v>818</v>
       </c>
-      <c r="K13" s="6" t="inlineStr"/>
+      <c r="K13" s="6" t="n"/>
       <c r="L13" s="6" t="inlineStr">
         <is>
           <t>Modern two bedroom apartment in Brigade Court, Borough, with premium resident amenities and excellent connections across Central London.; listed furnished — check if flexible</t>
@@ -1441,7 +1441,7 @@
       <c r="J14" s="6" t="n">
         <v>861</v>
       </c>
-      <c r="K14" s="6" t="inlineStr"/>
+      <c r="K14" s="6" t="n"/>
       <c r="L14" s="6" t="inlineStr">
         <is>
           <t>A two bedroom, two bathroom property with three balconies set within a sought after development in Farringdon. The property has a large open plan ...; listed furnished — check if flexible</t>
@@ -1510,7 +1510,7 @@
       <c r="J15" s="6" t="n">
         <v>809</v>
       </c>
-      <c r="K15" s="6" t="inlineStr"/>
+      <c r="K15" s="6" t="n"/>
       <c r="L15" s="6" t="inlineStr">
         <is>
           <t>Beautifully presented furnished 2 bedroom 2 bathroom apartment with private balcony in this premium Bloomsbury location. This superior apartment ...; listed furnished — check if flexible</t>
@@ -1579,7 +1579,7 @@
       <c r="J16" s="6" t="n">
         <v>750</v>
       </c>
-      <c r="K16" s="6" t="inlineStr"/>
+      <c r="K16" s="6" t="n"/>
       <c r="L16" s="6" t="inlineStr">
         <is>
           <t>• Short Term • Fully Furnished • Private Underground Parking • Bi-weekly Cleaning Included Available from mid September 2026 3 month minimum ...; listed furnished — check if flexible</t>
@@ -1648,7 +1648,7 @@
       <c r="J17" s="6" t="n">
         <v>829</v>
       </c>
-      <c r="K17" s="6" t="inlineStr"/>
+      <c r="K17" s="6" t="n"/>
       <c r="L17" s="6" t="inlineStr">
         <is>
           <t>Available October 2026 for, a superb lateral two bedroom apartment set within Allen House which was converted in 2002 by Landmark Developments and ...; listed furnished — check if flexible</t>
@@ -1717,7 +1717,7 @@
       <c r="J18" s="6" t="n">
         <v>599</v>
       </c>
-      <c r="K18" s="6" t="inlineStr"/>
+      <c r="K18" s="6" t="n"/>
       <c r="L18" s="6" t="inlineStr">
         <is>
           <t>A spacious one bedroom apartment set within the Atlas Building with fantastic City views and a private balcony.; under 650 sq ft; furnishing not stated</t>
@@ -1784,7 +1784,7 @@
         </is>
       </c>
       <c r="J19" s="4" t="n"/>
-      <c r="K19" s="4" t="inlineStr"/>
+      <c r="K19" s="4" t="n"/>
       <c r="L19" s="4" t="inlineStr">
         <is>
           <t>Short Let One Bedroom Furnished All bills included; size not stated; listed furnished — check if flexible</t>
@@ -1851,7 +1851,7 @@
         </is>
       </c>
       <c r="J20" s="4" t="n"/>
-      <c r="K20" s="4" t="inlineStr"/>
+      <c r="K20" s="4" t="n"/>
       <c r="L20" s="4" t="inlineStr">
         <is>
           <t>Two double bedrooms Two bathrooms; size not stated; listed furnished — check if flexible</t>
@@ -1920,7 +1920,7 @@
       <c r="J21" s="4" t="n">
         <v>786</v>
       </c>
-      <c r="K21" s="4" t="inlineStr"/>
+      <c r="K21" s="4" t="n"/>
       <c r="L21" s="4" t="inlineStr">
         <is>
           <t>Bright Eighteenth Floor Two Bedroom Apartment with Winter Garden, Premium Resident Facilities, Excellent Transport and Iconic London Views.; outdoor space is communal/shared; listed furnished — check if flexible</t>
@@ -1989,7 +1989,7 @@
       <c r="J22" s="4" t="n">
         <v>441</v>
       </c>
-      <c r="K22" s="4" t="inlineStr"/>
+      <c r="K22" s="4" t="n"/>
       <c r="L22" s="4" t="inlineStr">
         <is>
           <t>Modern and spacious 1-bedroom, 1-bathroom furnished apartment in the heart of Bloomsbury with communal rooftop. Featuring high ceilings, excellent ...; outdoor space is communal/shared; under 650 sq ft; listed furnished — check if flexible</t>
@@ -2058,7 +2058,7 @@
       <c r="J23" s="4" t="n">
         <v>538</v>
       </c>
-      <c r="K23" s="4" t="inlineStr"/>
+      <c r="K23" s="4" t="n"/>
       <c r="L23" s="4" t="inlineStr">
         <is>
           <t>A fully furnished, 15th floor 1 bedroom apartment in the Atlas Building, Old Street. EC1 The apartment comprises a large open plan reception with ...; under 650 sq ft; listed furnished — check if flexible</t>
@@ -36262,7 +36262,6 @@
           <t>https://www.rightmove.co.uk/properties/91515501</t>
         </is>
       </c>
-      <c r="B593" t="inlineStr"/>
       <c r="C593" t="inlineStr">
         <is>
           <t>none</t>

</xml_diff>

<commit_message>
Daily tracker update 2026-08-02
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -23492,7 +23492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D633"/>
+  <dimension ref="A1:D634"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37361,6 +37361,28 @@
         </is>
       </c>
     </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>https://www.rightmove.co.uk/properties/91550109</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>3142|2-bed|wc2e</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D634" t="inlineStr">
+        <is>
+          <t>2026-08-02 21:39</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily tracker update 2026-08-03
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -23492,7 +23492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D634"/>
+  <dimension ref="A1:D635"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37383,6 +37383,28 @@
         </is>
       </c>
     </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/12196883/</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>3198|2-bed|ec1v</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>2026-08-03 08:40</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily tracker update 2026-08-04
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -24054,7 +24054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D652"/>
+  <dimension ref="A1:D653"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38336,6 +38336,28 @@
         </is>
       </c>
     </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>https://www.zoopla.co.uk/to-rent/details/73883075/</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>3077|2-bed|ec1v</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>2026-08-04 05:40</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily tracker update 2026-08-05
</commit_message>
<xml_diff>
--- a/tracker/london_flat_hunt.xlsx
+++ b/tracker/london_flat_hunt.xlsx
@@ -599,7 +599,7 @@
       <c r="J2" s="6" t="n">
         <v>852</v>
       </c>
-      <c r="K2" s="6" t="inlineStr"/>
+      <c r="K2" s="6" t="n"/>
       <c r="L2" s="6" t="inlineStr">
         <is>
           <t>ZERO DEPOSIT AVAILABLE. LONG LET. Stunning tenth floor apartment with a spacious open plan living area, two large double bedrooms and a sizable private balcony,; furnishing not stated</t>
@@ -668,7 +668,7 @@
       <c r="J3" s="6" t="n">
         <v>668</v>
       </c>
-      <c r="K3" s="6" t="inlineStr"/>
+      <c r="K3" s="6" t="n"/>
       <c r="L3" s="6" t="inlineStr">
         <is>
           <t>Feel at home wherever you choose to live with Blueground. You’ll love this sophisticated Waterloo furnished two bedroom apartment with its modern ...; listed furnished — check if flexible</t>
@@ -24820,7 +24820,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D675"/>
+  <dimension ref="A1:D676"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -39598,6 +39598,28 @@
         </is>
       </c>
     </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>https://www.onthemarket.com/details/17595131/</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>3300|2-bed|wc1x</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>2026-08-05 13:39</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>